<commit_message>
draft spec for new dose code system
</commit_message>
<xml_diff>
--- a/data/ALAI UP Client-level Reporting Tool Template_4.7.26.xlsx
+++ b/data/ALAI UP Client-level Reporting Tool Template_4.7.26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kmlab\Desktop\Dashboard\alai_up_local_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5B0F360-4449-4B3E-AF31-360D4293B8A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{056D8AEA-C26F-4947-89FB-EE724F37BEC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{500E2EE0-B1C5-4ACF-BC67-EDC8BDABD2D7}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="539">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="540">
   <si>
     <t>INSTRUCTIONS</t>
   </si>
@@ -1805,10 +1805,6 @@
     </r>
   </si>
   <si>
-    <t>Dose of client's first iCAB/RPV injection.
-Note: for icab_rpv_shot1_dose, use code 2 for a typical loading dose. The dashboard code assumes that the next dose has an injection interval of 1 month (since it is a loading dose). If the expected interval is not 1 month (e.g. if a patient came from another clinic already on monthly iCAB/RPV, use code 6.</t>
-  </si>
-  <si>
     <t>The excel sheet provided should be used as a guide for preparing your data. Data can be entered manually, but  extracting data from the electronic medical record and organizing it into the correct format will be easier and more efficient.</t>
   </si>
   <si>
@@ -1840,6 +1836,42 @@
   </si>
   <si>
     <t>1=Satisfaction with previous regimen; 2=Fear/dislike of needles; 3=Frequency of visit schedule; 4=Concerns about cost; 5=Concerns about newness of modality; 6=Failing treatment; 7=Lost to follow up; 8=Concerns about side effects; 9=Switched out of clinic; 10=Change/loss of insurance/payor; 20=Other</t>
+  </si>
+  <si>
+    <t>1 = monthly injection interval, next dose expected to be in 1 month (28 or 31 days, +/-7); 2 = bimonthly injection interval, next dose expected to be in 2 months (56 or 62 days, +-7); 0 = monthly injection interval, to be used if a patient discontinued and is restarting; UNK = Unknown</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Dose of client's first iCAB/RPV injection.
+Note: generally use 1 for loading doses or other monthly injections. 0 is reserved for the special case where a client has discontinued but is restarting injections. The dashboard will process this as a monthly injection interval </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>and</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> it will make sure that this injection is not considered late. If I client is late but requires reloading, use 1.
+Example: 
+Shot 1: 1 (loading dose, next injection in 1 month)
+Shot 2: 2 (bimonthly maintenance dose, next injection in 2 months)
+Shot 3: 2 (bimonthly maintenance dose, next injection in 2 months)
+--Client Discontinues for any reason--
+Shot 4: 0 (loading restart dose, next injection in 1 month. not considered "late")
+Shot 5: 2 (bimonthly maintenance dose, next injection in 2 months)
+</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -3066,7 +3098,7 @@
     </row>
     <row r="9" spans="2:2" ht="41.4" x14ac:dyDescent="0.25">
       <c r="B9" s="89" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.25">
@@ -3204,7 +3236,7 @@
         <v>26</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H1" s="3"/>
       <c r="I1" s="4"/>
@@ -3229,7 +3261,7 @@
         <v>30</v>
       </c>
       <c r="G2" s="110" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="8"/>
@@ -3241,10 +3273,10 @@
         <v>31</v>
       </c>
       <c r="C3" s="111" t="s">
+        <v>534</v>
+      </c>
+      <c r="D3" s="112" t="s">
         <v>535</v>
-      </c>
-      <c r="D3" s="112" t="s">
-        <v>536</v>
       </c>
       <c r="E3" s="112" t="s">
         <v>32</v>
@@ -3253,7 +3285,7 @@
         <v>30</v>
       </c>
       <c r="G3" s="112" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H3" s="12"/>
       <c r="I3" s="8"/>
@@ -3275,7 +3307,7 @@
         <v>36</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H4" s="12"/>
       <c r="I4" s="8"/>
@@ -3297,7 +3329,7 @@
         <v>40</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H5" s="10"/>
       <c r="I5" s="17"/>
@@ -3319,7 +3351,7 @@
         <v>44</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H6" s="12"/>
     </row>
@@ -3340,7 +3372,7 @@
         <v>48</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H7" s="12"/>
     </row>
@@ -3362,7 +3394,7 @@
         <v>52</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H8" s="10"/>
       <c r="I8" s="18"/>
@@ -3386,7 +3418,7 @@
         <v>56</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H9" s="12"/>
     </row>
@@ -3407,7 +3439,7 @@
         <v>60</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H10" s="12"/>
     </row>
@@ -3428,7 +3460,7 @@
         <v>64</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H11" s="12"/>
     </row>
@@ -3449,7 +3481,7 @@
         <v>68</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H12" s="12"/>
     </row>
@@ -3470,7 +3502,7 @@
         <v>72</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H13" s="12"/>
     </row>
@@ -3491,7 +3523,7 @@
         <v>76</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H14" s="12"/>
     </row>
@@ -3512,7 +3544,7 @@
         <v>30</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H15" s="12"/>
     </row>
@@ -3533,7 +3565,7 @@
         <v>83</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H16" s="20"/>
     </row>
@@ -3554,7 +3586,7 @@
         <v>87</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H17" s="12"/>
     </row>
@@ -3575,7 +3607,7 @@
         <v>92</v>
       </c>
       <c r="G18" s="114" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H18" s="12"/>
     </row>
@@ -3596,7 +3628,7 @@
         <v>92</v>
       </c>
       <c r="G19" s="114" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H19" s="12"/>
     </row>
@@ -3617,7 +3649,7 @@
         <v>92</v>
       </c>
       <c r="G20" s="114" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H20" s="12"/>
     </row>
@@ -3638,7 +3670,7 @@
         <v>92</v>
       </c>
       <c r="G21" s="114" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H21" s="12"/>
     </row>
@@ -3659,7 +3691,7 @@
         <v>92</v>
       </c>
       <c r="G22" s="114" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H22" s="12"/>
     </row>
@@ -3680,7 +3712,7 @@
         <v>92</v>
       </c>
       <c r="G23" s="114" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H23" s="12"/>
     </row>
@@ -3701,7 +3733,7 @@
         <v>92</v>
       </c>
       <c r="G24" s="114" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H24" s="12"/>
     </row>
@@ -3722,7 +3754,7 @@
         <v>92</v>
       </c>
       <c r="G25" s="114" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H25" s="12"/>
     </row>
@@ -3743,7 +3775,7 @@
         <v>92</v>
       </c>
       <c r="G26" s="114" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H26" s="12"/>
     </row>
@@ -3764,7 +3796,7 @@
         <v>92</v>
       </c>
       <c r="G27" s="114" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H27" s="12"/>
     </row>
@@ -3785,7 +3817,7 @@
         <v>109</v>
       </c>
       <c r="G28" s="22" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H28" s="12"/>
     </row>
@@ -3806,7 +3838,7 @@
         <v>113</v>
       </c>
       <c r="G29" s="22" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H29" s="12"/>
     </row>
@@ -3827,7 +3859,7 @@
         <v>117</v>
       </c>
       <c r="G30" s="22" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H30" s="12"/>
     </row>
@@ -3859,7 +3891,7 @@
         <v>122</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H32" s="24"/>
     </row>
@@ -3880,7 +3912,7 @@
         <v>125</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H33" s="24"/>
     </row>
@@ -3901,7 +3933,7 @@
         <v>129</v>
       </c>
       <c r="G34" s="23" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H34" s="12"/>
     </row>
@@ -3922,7 +3954,7 @@
         <v>133</v>
       </c>
       <c r="G35" s="23" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H35" s="10"/>
     </row>
@@ -3943,7 +3975,7 @@
         <v>137</v>
       </c>
       <c r="G36" s="23" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H36" s="12"/>
     </row>
@@ -3964,7 +3996,7 @@
         <v>141</v>
       </c>
       <c r="G37" s="23" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H37" s="24"/>
     </row>
@@ -3985,7 +4017,7 @@
         <v>30</v>
       </c>
       <c r="G38" s="23" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H38" s="12"/>
     </row>
@@ -4006,7 +4038,7 @@
         <v>148</v>
       </c>
       <c r="G39" s="23" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H39" s="12"/>
     </row>
@@ -4026,7 +4058,7 @@
       </c>
       <c r="F40" s="117"/>
       <c r="G40" s="117" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H40" s="12"/>
     </row>
@@ -4046,7 +4078,7 @@
       </c>
       <c r="F41" s="117"/>
       <c r="G41" s="117" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H41" s="12"/>
     </row>
@@ -4066,7 +4098,7 @@
       </c>
       <c r="F42" s="117"/>
       <c r="G42" s="117" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H42" s="12"/>
     </row>
@@ -4087,7 +4119,7 @@
         <v>48</v>
       </c>
       <c r="G43" s="119" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H43" s="24"/>
     </row>
@@ -4108,7 +4140,7 @@
         <v>150</v>
       </c>
       <c r="G44" s="119" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H44" s="24"/>
     </row>
@@ -4129,10 +4161,10 @@
         <v>150</v>
       </c>
       <c r="G45" s="119" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H45" s="24" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
     </row>
     <row r="46" spans="1:11" s="136" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
@@ -4153,7 +4185,7 @@
         <v>155</v>
       </c>
       <c r="G46" s="133" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H46" s="134"/>
       <c r="I46" s="135"/>
@@ -4178,7 +4210,7 @@
         <v>150</v>
       </c>
       <c r="G47" s="132" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H47" s="134"/>
       <c r="I47" s="135"/>
@@ -4203,7 +4235,7 @@
         <v>155</v>
       </c>
       <c r="G48" s="119" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H48" s="30"/>
       <c r="I48" s="28"/>
@@ -4228,7 +4260,7 @@
         <v>150</v>
       </c>
       <c r="G49" s="26" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H49" s="30"/>
       <c r="I49" s="28"/>
@@ -4253,7 +4285,7 @@
         <v>155</v>
       </c>
       <c r="G50" s="119" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H50" s="30"/>
       <c r="I50" s="28"/>
@@ -4278,7 +4310,7 @@
         <v>150</v>
       </c>
       <c r="G51" s="26" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H51" s="30"/>
       <c r="I51" s="28"/>
@@ -4303,7 +4335,7 @@
         <v>155</v>
       </c>
       <c r="G52" s="119" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H52" s="30"/>
       <c r="I52" s="28"/>
@@ -4328,7 +4360,7 @@
         <v>150</v>
       </c>
       <c r="G53" s="26" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H53" s="30"/>
       <c r="I53" s="28"/>
@@ -4353,7 +4385,7 @@
         <v>155</v>
       </c>
       <c r="G54" s="119" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H54" s="30"/>
       <c r="I54" s="28"/>
@@ -4378,7 +4410,7 @@
         <v>150</v>
       </c>
       <c r="G55" s="26" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H55" s="30"/>
       <c r="I55" s="28"/>
@@ -4403,7 +4435,7 @@
         <v>155</v>
       </c>
       <c r="G56" s="119" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H56" s="30"/>
       <c r="I56" s="28"/>
@@ -4428,7 +4460,7 @@
         <v>150</v>
       </c>
       <c r="G57" s="26" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H57" s="30"/>
       <c r="I57" s="28"/>
@@ -4453,7 +4485,7 @@
         <v>155</v>
       </c>
       <c r="G58" s="119" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H58" s="30"/>
       <c r="I58" s="28"/>
@@ -4478,7 +4510,7 @@
         <v>150</v>
       </c>
       <c r="G59" s="26" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H59" s="30"/>
       <c r="I59" s="28"/>
@@ -4503,7 +4535,7 @@
         <v>155</v>
       </c>
       <c r="G60" s="119" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H60" s="30"/>
       <c r="I60" s="28"/>
@@ -4528,7 +4560,7 @@
         <v>150</v>
       </c>
       <c r="G61" s="26" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H61" s="30"/>
       <c r="I61" s="28"/>
@@ -4553,7 +4585,7 @@
         <v>155</v>
       </c>
       <c r="G62" s="119" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H62" s="30"/>
       <c r="I62" s="28"/>
@@ -4578,7 +4610,7 @@
         <v>150</v>
       </c>
       <c r="G63" s="26" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H63" s="30"/>
       <c r="I63" s="28"/>
@@ -4603,7 +4635,7 @@
         <v>155</v>
       </c>
       <c r="G64" s="119" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H64" s="30"/>
       <c r="I64" s="28"/>
@@ -4628,7 +4660,7 @@
         <v>150</v>
       </c>
       <c r="G65" s="26" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H65" s="30"/>
       <c r="I65" s="28"/>
@@ -4652,7 +4684,7 @@
         <v>155</v>
       </c>
       <c r="G66" s="119" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H66" s="12"/>
     </row>
@@ -4673,7 +4705,7 @@
         <v>150</v>
       </c>
       <c r="G67" s="26" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H67" s="12"/>
     </row>
@@ -4792,7 +4824,7 @@
         <v>518</v>
       </c>
       <c r="F72" s="36" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="G72" s="36" t="s">
         <v>515</v>
@@ -4892,7 +4924,7 @@
         <v>519</v>
       </c>
       <c r="F76" s="37" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="G76" s="36" t="s">
         <v>515</v>
@@ -4992,7 +5024,7 @@
         <v>520</v>
       </c>
       <c r="F80" s="36" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="G80" s="36" t="s">
         <v>515</v>
@@ -5136,7 +5168,7 @@
         <v>252</v>
       </c>
       <c r="G86" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H86" s="10"/>
     </row>
@@ -5157,7 +5189,7 @@
         <v>150</v>
       </c>
       <c r="G87" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H87" s="12"/>
     </row>
@@ -5179,7 +5211,7 @@
         <v>259</v>
       </c>
       <c r="G88" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H88" s="30"/>
       <c r="I88" s="28"/>
@@ -5204,7 +5236,7 @@
         <v>150</v>
       </c>
       <c r="G89" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H89" s="30"/>
       <c r="I89" s="28"/>
@@ -5229,7 +5261,7 @@
         <v>150</v>
       </c>
       <c r="G90" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H90" s="30"/>
       <c r="I90" s="28"/>
@@ -5254,7 +5286,7 @@
         <v>259</v>
       </c>
       <c r="G91" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H91" s="30"/>
       <c r="I91" s="28"/>
@@ -5279,7 +5311,7 @@
         <v>150</v>
       </c>
       <c r="G92" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H92" s="30"/>
       <c r="I92" s="28"/>
@@ -5304,7 +5336,7 @@
         <v>150</v>
       </c>
       <c r="G93" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H93" s="30"/>
       <c r="I93" s="28"/>
@@ -5329,7 +5361,7 @@
         <v>150</v>
       </c>
       <c r="G94" s="121" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H94" s="30"/>
       <c r="I94" s="28"/>
@@ -5354,7 +5386,7 @@
         <v>155</v>
       </c>
       <c r="G95" s="120" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H95" s="31"/>
       <c r="I95" s="32"/>
@@ -5379,14 +5411,14 @@
         <v>150</v>
       </c>
       <c r="G96" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H96" s="31"/>
       <c r="I96" s="32"/>
       <c r="J96" s="32"/>
       <c r="K96" s="32"/>
     </row>
-    <row r="97" spans="1:11" s="33" customFormat="1" ht="171.6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:11" s="33" customFormat="1" ht="224.4" x14ac:dyDescent="0.3">
       <c r="A97"/>
       <c r="B97" s="36" t="s">
         <v>199</v>
@@ -5398,13 +5430,13 @@
         <v>285</v>
       </c>
       <c r="E97" s="37" t="s">
-        <v>527</v>
+        <v>539</v>
       </c>
       <c r="F97" s="36" t="s">
-        <v>286</v>
+        <v>538</v>
       </c>
       <c r="G97" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H97" s="31"/>
       <c r="I97" s="32"/>
@@ -5429,7 +5461,7 @@
         <v>150</v>
       </c>
       <c r="G98" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H98" s="31"/>
       <c r="I98" s="32"/>
@@ -5454,7 +5486,7 @@
         <v>286</v>
       </c>
       <c r="G99" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H99" s="31"/>
       <c r="I99" s="32"/>
@@ -5479,7 +5511,7 @@
         <v>150</v>
       </c>
       <c r="G100" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H100" s="31"/>
       <c r="I100" s="32"/>
@@ -5504,7 +5536,7 @@
         <v>286</v>
       </c>
       <c r="G101" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H101" s="31"/>
       <c r="I101" s="32"/>
@@ -5529,7 +5561,7 @@
         <v>150</v>
       </c>
       <c r="G102" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H102" s="31"/>
       <c r="I102" s="32"/>
@@ -5554,7 +5586,7 @@
         <v>286</v>
       </c>
       <c r="G103" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H103" s="31"/>
       <c r="I103" s="32"/>
@@ -5579,7 +5611,7 @@
         <v>150</v>
       </c>
       <c r="G104" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H104" s="31"/>
       <c r="I104" s="32"/>
@@ -5604,7 +5636,7 @@
         <v>286</v>
       </c>
       <c r="G105" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H105" s="31"/>
       <c r="I105" s="32"/>
@@ -5629,7 +5661,7 @@
         <v>150</v>
       </c>
       <c r="G106" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H106" s="31"/>
       <c r="I106" s="32"/>
@@ -5654,7 +5686,7 @@
         <v>286</v>
       </c>
       <c r="G107" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H107" s="31"/>
       <c r="I107" s="32"/>
@@ -5679,7 +5711,7 @@
         <v>150</v>
       </c>
       <c r="G108" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H108" s="31"/>
       <c r="I108" s="32"/>
@@ -5704,7 +5736,7 @@
         <v>286</v>
       </c>
       <c r="G109" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H109" s="31"/>
       <c r="I109" s="32"/>
@@ -5729,7 +5761,7 @@
         <v>150</v>
       </c>
       <c r="G110" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H110" s="31"/>
       <c r="I110" s="32"/>
@@ -5754,7 +5786,7 @@
         <v>286</v>
       </c>
       <c r="G111" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H111" s="31"/>
       <c r="I111" s="32"/>
@@ -5779,7 +5811,7 @@
         <v>150</v>
       </c>
       <c r="G112" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H112" s="31"/>
       <c r="I112" s="32"/>
@@ -5804,7 +5836,7 @@
         <v>286</v>
       </c>
       <c r="G113" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H113" s="31"/>
       <c r="I113" s="32"/>
@@ -5829,7 +5861,7 @@
         <v>150</v>
       </c>
       <c r="G114" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H114" s="31"/>
       <c r="I114" s="32"/>
@@ -5854,7 +5886,7 @@
         <v>286</v>
       </c>
       <c r="G115" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H115" s="31"/>
       <c r="I115" s="32"/>
@@ -5879,7 +5911,7 @@
         <v>150</v>
       </c>
       <c r="G116" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H116" s="31"/>
       <c r="I116" s="32"/>
@@ -5904,7 +5936,7 @@
         <v>286</v>
       </c>
       <c r="G117" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H117" s="31"/>
       <c r="I117" s="32"/>
@@ -5929,7 +5961,7 @@
         <v>150</v>
       </c>
       <c r="G118" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H118" s="31"/>
       <c r="I118" s="32"/>
@@ -5954,7 +5986,7 @@
         <v>286</v>
       </c>
       <c r="G119" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H119" s="31"/>
       <c r="I119" s="32"/>
@@ -5979,7 +6011,7 @@
         <v>150</v>
       </c>
       <c r="G120" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H120" s="31"/>
       <c r="I120" s="32"/>
@@ -6004,7 +6036,7 @@
         <v>286</v>
       </c>
       <c r="G121" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H121" s="31"/>
       <c r="I121" s="32"/>
@@ -6029,7 +6061,7 @@
         <v>150</v>
       </c>
       <c r="G122" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H122" s="31"/>
       <c r="I122" s="32"/>
@@ -6054,7 +6086,7 @@
         <v>286</v>
       </c>
       <c r="G123" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H123" s="31"/>
       <c r="I123" s="32"/>
@@ -6079,7 +6111,7 @@
         <v>150</v>
       </c>
       <c r="G124" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H124" s="31"/>
       <c r="I124" s="32"/>
@@ -6104,7 +6136,7 @@
         <v>286</v>
       </c>
       <c r="G125" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H125" s="31"/>
       <c r="I125" s="32"/>
@@ -6129,7 +6161,7 @@
         <v>150</v>
       </c>
       <c r="G126" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H126" s="31"/>
       <c r="I126" s="32"/>
@@ -6154,7 +6186,7 @@
         <v>286</v>
       </c>
       <c r="G127" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H127" s="31"/>
       <c r="I127" s="32"/>
@@ -6179,7 +6211,7 @@
         <v>150</v>
       </c>
       <c r="G128" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H128" s="31"/>
       <c r="I128" s="32"/>
@@ -6204,7 +6236,7 @@
         <v>286</v>
       </c>
       <c r="G129" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H129" s="31"/>
       <c r="I129" s="32"/>
@@ -6229,7 +6261,7 @@
         <v>150</v>
       </c>
       <c r="G130" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H130" s="31"/>
       <c r="I130" s="32"/>
@@ -6254,7 +6286,7 @@
         <v>286</v>
       </c>
       <c r="G131" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H131" s="31"/>
       <c r="I131" s="32"/>
@@ -6279,7 +6311,7 @@
         <v>150</v>
       </c>
       <c r="G132" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H132" s="31"/>
       <c r="I132" s="32"/>
@@ -6304,7 +6336,7 @@
         <v>286</v>
       </c>
       <c r="G133" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H133" s="31"/>
       <c r="I133" s="32"/>
@@ -6329,7 +6361,7 @@
         <v>150</v>
       </c>
       <c r="G134" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H134" s="31"/>
       <c r="I134" s="38"/>
@@ -6354,7 +6386,7 @@
         <v>286</v>
       </c>
       <c r="G135" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H135" s="32"/>
       <c r="I135" s="32"/>
@@ -6379,7 +6411,7 @@
         <v>150</v>
       </c>
       <c r="G136" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H136" s="31"/>
       <c r="I136" s="32"/>
@@ -6404,7 +6436,7 @@
         <v>286</v>
       </c>
       <c r="G137" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H137" s="31"/>
       <c r="I137" s="32"/>
@@ -6429,7 +6461,7 @@
         <v>150</v>
       </c>
       <c r="G138" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H138" s="31"/>
       <c r="I138" s="32"/>
@@ -6454,7 +6486,7 @@
         <v>286</v>
       </c>
       <c r="G139" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H139" s="31"/>
       <c r="I139" s="32"/>
@@ -6479,7 +6511,7 @@
         <v>150</v>
       </c>
       <c r="G140" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H140" s="31"/>
       <c r="I140" s="32"/>
@@ -6504,7 +6536,7 @@
         <v>286</v>
       </c>
       <c r="G141" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H141" s="31"/>
       <c r="I141" s="32"/>
@@ -6529,7 +6561,7 @@
         <v>150</v>
       </c>
       <c r="G142" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H142" s="31"/>
       <c r="I142" s="32"/>
@@ -6554,7 +6586,7 @@
         <v>286</v>
       </c>
       <c r="G143" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H143" s="31"/>
       <c r="I143" s="32"/>
@@ -6579,7 +6611,7 @@
         <v>150</v>
       </c>
       <c r="G144" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H144" s="31"/>
       <c r="I144" s="32"/>
@@ -6604,7 +6636,7 @@
         <v>286</v>
       </c>
       <c r="G145" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H145" s="31"/>
       <c r="I145" s="32"/>
@@ -6629,7 +6661,7 @@
         <v>150</v>
       </c>
       <c r="G146" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H146" s="31"/>
       <c r="I146" s="32"/>
@@ -6654,7 +6686,7 @@
         <v>286</v>
       </c>
       <c r="G147" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H147" s="31"/>
       <c r="I147" s="32"/>
@@ -6679,7 +6711,7 @@
         <v>150</v>
       </c>
       <c r="G148" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H148" s="31"/>
       <c r="I148" s="32"/>
@@ -6704,7 +6736,7 @@
         <v>286</v>
       </c>
       <c r="G149" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H149" s="31"/>
       <c r="I149" s="32"/>
@@ -6729,7 +6761,7 @@
         <v>150</v>
       </c>
       <c r="G150" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H150" s="31"/>
       <c r="I150" s="32"/>
@@ -6754,7 +6786,7 @@
         <v>286</v>
       </c>
       <c r="G151" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H151" s="31"/>
       <c r="I151" s="32"/>
@@ -6778,7 +6810,7 @@
         <v>451</v>
       </c>
       <c r="G152" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
     </row>
     <row r="153" spans="1:11" ht="79.2" x14ac:dyDescent="0.3">
@@ -6798,7 +6830,7 @@
         <v>150</v>
       </c>
       <c r="G153" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
     </row>
     <row r="154" spans="1:11" ht="105.6" x14ac:dyDescent="0.3">
@@ -6815,10 +6847,10 @@
         <v>526</v>
       </c>
       <c r="F154" s="36" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="G154" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
     </row>
     <row r="155" spans="1:11" ht="66" x14ac:dyDescent="0.3">
@@ -6838,7 +6870,7 @@
         <v>30</v>
       </c>
       <c r="G155" s="36" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
     </row>
     <row r="156" spans="1:11" x14ac:dyDescent="0.3">
@@ -6904,7 +6936,7 @@
         <v>28</v>
       </c>
       <c r="B1" s="103" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="C1" s="104" t="s">
         <v>33</v>
@@ -25466,6 +25498,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="42fbd5e6-b175-407a-a25c-5fc6410bf24f" xsi:nil="true"/>
@@ -25474,15 +25515,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -25741,20 +25773,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{286F673D-E70D-4002-B8F5-CAC95B029A7E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E9485EC-5D88-4A1C-961D-0F4FE84359B8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="42fbd5e6-b175-407a-a25c-5fc6410bf24f"/>
     <ds:schemaRef ds:uri="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{286F673D-E70D-4002-B8F5-CAC95B029A7E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
change _oth to _other in not elig
</commit_message>
<xml_diff>
--- a/data/ALAI UP Client-level Reporting Tool Template_4.7.26.xlsx
+++ b/data/ALAI UP Client-level Reporting Tool Template_4.7.26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kmlab\Desktop\Dashboard\alai_up_local_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DB94584-3F37-41E3-A04E-7783E4396F12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF9AAC9B-529C-4EA9-9AAB-3B03C5851854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{500E2EE0-B1C5-4ACF-BC67-EDC8BDABD2D7}"/>
   </bookViews>
@@ -694,10 +694,6 @@
     <t>iCAB/RPV not eligible reason (first screening)</t>
   </si>
   <si>
-    <t xml:space="preserve">icab_rpv_not_elig_1_reason_oth
-</t>
-  </si>
-  <si>
     <t>iCAB/RPV not eligible reason - Other (first screening)</t>
   </si>
   <si>
@@ -754,10 +750,6 @@
     <t>iCAB/RPV not eligible reason (second screening)</t>
   </si>
   <si>
-    <t xml:space="preserve">icab_rpv_not_elig_2_reason_oth
-</t>
-  </si>
-  <si>
     <t>iCAB/RPV not eligible reason - Other (second screening)</t>
   </si>
   <si>
@@ -929,16 +921,10 @@
     <t>icab_rpv_not_elig_1_reason</t>
   </si>
   <si>
-    <t>icab_rpv_not_elig_1_reason_oth</t>
-  </si>
-  <si>
     <t>icab_rpv_screen_2_outcome</t>
   </si>
   <si>
     <t>icab_rpv_not_elig_2_reason</t>
-  </si>
-  <si>
-    <t>icab_rpv_not_elig_2_reason_oth</t>
   </si>
   <si>
     <t>Site name. If you only have 1 site, provide the name. If you have multiple sites, make sure to provide a unique, consistent name for each site.</t>
@@ -1408,6 +1394,20 @@
   </si>
   <si>
     <t>YYYY-MM-DD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">icab_rpv_not_elig_1_reason_other
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">icab_rpv_not_elig_2_reason_other
+</t>
+  </si>
+  <si>
+    <t>icab_rpv_not_elig_1_reason_other</t>
+  </si>
+  <si>
+    <t>icab_rpv_not_elig_2_reason_other</t>
   </si>
 </sst>
 </file>
@@ -2129,13 +2129,13 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2174,7 +2174,7 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2556,7 +2556,7 @@
     </row>
     <row r="7" spans="2:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="B7" s="87" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.25">
@@ -2566,7 +2566,7 @@
     </row>
     <row r="9" spans="2:2" ht="41.4" x14ac:dyDescent="0.25">
       <c r="B9" s="87" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.25">
@@ -2704,7 +2704,7 @@
         <v>26</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="H1" s="3"/>
       <c r="I1" s="4"/>
@@ -2723,13 +2723,13 @@
         <v>29</v>
       </c>
       <c r="E2" s="108" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="F2" s="108" t="s">
         <v>30</v>
       </c>
       <c r="G2" s="108" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="8"/>
@@ -2741,10 +2741,10 @@
         <v>31</v>
       </c>
       <c r="C3" s="109" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="D3" s="110" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="E3" s="110" t="s">
         <v>32</v>
@@ -2753,7 +2753,7 @@
         <v>30</v>
       </c>
       <c r="G3" s="110" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H3" s="12"/>
       <c r="I3" s="8"/>
@@ -2773,7 +2773,7 @@
         <v>36</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="H4" s="12"/>
       <c r="I4" s="8"/>
@@ -2793,7 +2793,7 @@
         <v>40</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="H5" s="10"/>
       <c r="I5" s="17"/>
@@ -2801,19 +2801,19 @@
     <row r="6" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="B6" s="128"/>
       <c r="C6" s="15" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="H6" s="12"/>
     </row>
@@ -2833,7 +2833,7 @@
         <v>45</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H7" s="10"/>
       <c r="I7" s="18"/>
@@ -2855,7 +2855,7 @@
         <v>49</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H8" s="12"/>
     </row>
@@ -2874,7 +2874,7 @@
         <v>53</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H9" s="12"/>
     </row>
@@ -2893,7 +2893,7 @@
         <v>57</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H10" s="12"/>
     </row>
@@ -2912,7 +2912,7 @@
         <v>61</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H11" s="12"/>
     </row>
@@ -2931,7 +2931,7 @@
         <v>65</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H12" s="12"/>
     </row>
@@ -2950,7 +2950,7 @@
         <v>69</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H13" s="12"/>
     </row>
@@ -2969,7 +2969,7 @@
         <v>30</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H14" s="12"/>
     </row>
@@ -2988,7 +2988,7 @@
         <v>76</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="H15" s="20"/>
     </row>
@@ -3007,13 +3007,13 @@
         <v>80</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H16" s="12"/>
     </row>
     <row r="17" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A17" s="139" t="s">
-        <v>345</v>
+      <c r="A17" s="124" t="s">
+        <v>341</v>
       </c>
       <c r="B17" s="130" t="s">
         <v>81</v>
@@ -3031,12 +3031,12 @@
         <v>85</v>
       </c>
       <c r="G17" s="112" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="H17" s="12"/>
     </row>
     <row r="18" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="139"/>
+      <c r="A18" s="124"/>
       <c r="B18" s="131"/>
       <c r="C18" s="111" t="s">
         <v>86</v>
@@ -3051,12 +3051,12 @@
         <v>85</v>
       </c>
       <c r="G18" s="112" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="H18" s="12"/>
     </row>
     <row r="19" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="139"/>
+      <c r="A19" s="124"/>
       <c r="B19" s="131"/>
       <c r="C19" s="111" t="s">
         <v>89</v>
@@ -3071,12 +3071,12 @@
         <v>85</v>
       </c>
       <c r="G19" s="112" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="H19" s="12"/>
     </row>
     <row r="20" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A20" s="139"/>
+      <c r="A20" s="124"/>
       <c r="B20" s="131"/>
       <c r="C20" s="111" t="s">
         <v>92</v>
@@ -3091,12 +3091,12 @@
         <v>85</v>
       </c>
       <c r="G20" s="112" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="H20" s="12"/>
     </row>
     <row r="21" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A21" s="139"/>
+      <c r="A21" s="124"/>
       <c r="B21" s="131"/>
       <c r="C21" s="111" t="s">
         <v>95</v>
@@ -3111,107 +3111,107 @@
         <v>85</v>
       </c>
       <c r="G21" s="112" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="H21" s="12"/>
     </row>
     <row r="22" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A22" s="139"/>
+      <c r="A22" s="124"/>
       <c r="B22" s="131"/>
       <c r="C22" s="111" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="D22" s="112" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="E22" s="112" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="F22" s="112" t="s">
         <v>85</v>
       </c>
       <c r="G22" s="112" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="H22" s="12"/>
     </row>
     <row r="23" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A23" s="139"/>
+      <c r="A23" s="124"/>
       <c r="B23" s="131"/>
       <c r="C23" s="111" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="D23" s="112" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="E23" s="112" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="F23" s="112" t="s">
         <v>85</v>
       </c>
       <c r="G23" s="112" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="H23" s="12"/>
     </row>
     <row r="24" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A24" s="139"/>
+      <c r="A24" s="124"/>
       <c r="B24" s="131"/>
       <c r="C24" s="111" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="D24" s="112" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="E24" s="112" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="F24" s="112" t="s">
         <v>85</v>
       </c>
       <c r="G24" s="112" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="H24" s="12"/>
     </row>
     <row r="25" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A25" s="139"/>
+      <c r="A25" s="124"/>
       <c r="B25" s="131"/>
       <c r="C25" s="111" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D25" s="112" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="E25" s="112" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="F25" s="112" t="s">
         <v>85</v>
       </c>
       <c r="G25" s="112" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="H25" s="12"/>
     </row>
     <row r="26" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A26" s="139"/>
+      <c r="A26" s="124"/>
       <c r="B26" s="132"/>
       <c r="C26" s="111" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="D26" s="112" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="E26" s="112" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="F26" s="112" t="s">
         <v>85</v>
       </c>
       <c r="G26" s="112" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="H26" s="12"/>
     </row>
@@ -3232,7 +3232,7 @@
         <v>102</v>
       </c>
       <c r="G27" s="22" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="H27" s="12"/>
     </row>
@@ -3251,7 +3251,7 @@
         <v>106</v>
       </c>
       <c r="G28" s="22" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="H28" s="12"/>
     </row>
@@ -3270,7 +3270,7 @@
         <v>110</v>
       </c>
       <c r="G29" s="22" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="H29" s="12"/>
     </row>
@@ -3291,7 +3291,7 @@
         <v>115</v>
       </c>
       <c r="G30" s="23" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H30" s="24"/>
     </row>
@@ -3304,13 +3304,13 @@
         <v>117</v>
       </c>
       <c r="E31" s="23" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="F31" s="23" t="s">
         <v>118</v>
       </c>
       <c r="G31" s="23" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="H31" s="24"/>
     </row>
@@ -3329,7 +3329,7 @@
         <v>122</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="H32" s="12"/>
     </row>
@@ -3348,7 +3348,7 @@
         <v>126</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="H33" s="10"/>
     </row>
@@ -3367,7 +3367,7 @@
         <v>130</v>
       </c>
       <c r="G34" s="23" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="H34" s="12"/>
     </row>
@@ -3386,7 +3386,7 @@
         <v>134</v>
       </c>
       <c r="G35" s="23" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="H35" s="24"/>
     </row>
@@ -3405,7 +3405,7 @@
         <v>30</v>
       </c>
       <c r="G36" s="23" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="H36" s="12"/>
     </row>
@@ -3424,7 +3424,7 @@
         <v>141</v>
       </c>
       <c r="G37" s="23" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="H37" s="12"/>
     </row>
@@ -3432,17 +3432,17 @@
       <c r="A38" s="95"/>
       <c r="B38" s="137"/>
       <c r="C38" s="114" t="s">
+        <v>288</v>
+      </c>
+      <c r="D38" s="115" t="s">
+        <v>289</v>
+      </c>
+      <c r="E38" s="115" t="s">
         <v>292</v>
-      </c>
-      <c r="D38" s="115" t="s">
-        <v>293</v>
-      </c>
-      <c r="E38" s="115" t="s">
-        <v>296</v>
       </c>
       <c r="F38" s="115"/>
       <c r="G38" s="115" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="H38" s="12"/>
     </row>
@@ -3450,17 +3450,17 @@
       <c r="A39" s="95"/>
       <c r="B39" s="137"/>
       <c r="C39" s="116" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="D39" s="115" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="E39" s="115" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="F39" s="115"/>
       <c r="G39" s="115" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="H39" s="12"/>
     </row>
@@ -3468,87 +3468,87 @@
       <c r="A40" s="95"/>
       <c r="B40" s="138"/>
       <c r="C40" s="114" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="D40" s="115" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="E40" s="115" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="F40" s="115"/>
       <c r="G40" s="115" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="H40" s="12"/>
     </row>
     <row r="41" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B41" s="124" t="s">
-        <v>340</v>
+      <c r="B41" s="125" t="s">
+        <v>336</v>
       </c>
       <c r="C41" s="26" t="s">
+        <v>278</v>
+      </c>
+      <c r="D41" s="117" t="s">
+        <v>281</v>
+      </c>
+      <c r="E41" s="117" t="s">
         <v>282</v>
-      </c>
-      <c r="D41" s="117" t="s">
-        <v>285</v>
-      </c>
-      <c r="E41" s="117" t="s">
-        <v>286</v>
       </c>
       <c r="F41" s="117" t="s">
         <v>41</v>
       </c>
       <c r="G41" s="117" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="H41" s="24"/>
     </row>
     <row r="42" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B42" s="125"/>
+      <c r="B42" s="126"/>
       <c r="C42" s="26" t="s">
+        <v>279</v>
+      </c>
+      <c r="D42" s="117" t="s">
+        <v>280</v>
+      </c>
+      <c r="E42" s="117" t="s">
         <v>283</v>
-      </c>
-      <c r="D42" s="117" t="s">
-        <v>284</v>
-      </c>
-      <c r="E42" s="117" t="s">
-        <v>287</v>
       </c>
       <c r="F42" s="117" t="s">
         <v>143</v>
       </c>
       <c r="G42" s="117" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="H42" s="24"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B43" s="126"/>
+      <c r="B43" s="139"/>
       <c r="C43" s="26" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D43" s="117" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="E43" s="117" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="F43" s="117" t="s">
         <v>143</v>
       </c>
       <c r="G43" s="117" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H43" s="24" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="44" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A44" s="139" t="s">
-        <v>352</v>
-      </c>
-      <c r="B44" s="124" t="s">
-        <v>346</v>
+      <c r="A44" s="124" t="s">
+        <v>348</v>
+      </c>
+      <c r="B44" s="125" t="s">
+        <v>342</v>
       </c>
       <c r="C44" s="117" t="s">
         <v>147</v>
@@ -3557,13 +3557,13 @@
         <v>148</v>
       </c>
       <c r="E44" s="117" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="F44" s="117" t="s">
         <v>145</v>
       </c>
       <c r="G44" s="117" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H44" s="30"/>
       <c r="I44" s="28"/>
@@ -3571,8 +3571,8 @@
       <c r="K44" s="28"/>
     </row>
     <row r="45" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A45" s="139"/>
-      <c r="B45" s="125"/>
+      <c r="A45" s="124"/>
+      <c r="B45" s="126"/>
       <c r="C45" s="117" t="s">
         <v>149</v>
       </c>
@@ -3580,13 +3580,13 @@
         <v>150</v>
       </c>
       <c r="E45" s="117" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="F45" s="26" t="s">
         <v>143</v>
       </c>
       <c r="G45" s="26" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H45" s="30"/>
       <c r="I45" s="28"/>
@@ -3594,9 +3594,9 @@
       <c r="K45" s="28"/>
     </row>
     <row r="46" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A46" s="139"/>
-      <c r="B46" s="124" t="s">
-        <v>347</v>
+      <c r="A46" s="124"/>
+      <c r="B46" s="125" t="s">
+        <v>343</v>
       </c>
       <c r="C46" s="117" t="s">
         <v>151</v>
@@ -3605,13 +3605,13 @@
         <v>152</v>
       </c>
       <c r="E46" s="117" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="F46" s="117" t="s">
         <v>145</v>
       </c>
       <c r="G46" s="117" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H46" s="30"/>
       <c r="I46" s="28"/>
@@ -3619,8 +3619,8 @@
       <c r="K46" s="28"/>
     </row>
     <row r="47" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A47" s="139"/>
-      <c r="B47" s="125"/>
+      <c r="A47" s="124"/>
+      <c r="B47" s="126"/>
       <c r="C47" s="117" t="s">
         <v>153</v>
       </c>
@@ -3628,13 +3628,13 @@
         <v>154</v>
       </c>
       <c r="E47" s="117" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="F47" s="26" t="s">
         <v>143</v>
       </c>
       <c r="G47" s="26" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H47" s="30"/>
       <c r="I47" s="28"/>
@@ -3659,7 +3659,7 @@
         <v>142</v>
       </c>
       <c r="G48" s="36" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="H48" s="31"/>
       <c r="I48" s="32"/>
@@ -3682,7 +3682,7 @@
         <v>178</v>
       </c>
       <c r="G49" s="36" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="H49" s="31"/>
       <c r="I49" s="32"/>
@@ -3690,11 +3690,11 @@
       <c r="K49" s="32"/>
     </row>
     <row r="50" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A50" s="139" t="s">
-        <v>353</v>
+      <c r="A50" s="124" t="s">
+        <v>349</v>
       </c>
       <c r="B50" s="121" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="C50" s="36" t="s">
         <v>179</v>
@@ -3709,7 +3709,7 @@
         <v>143</v>
       </c>
       <c r="G50" s="36" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="H50" s="31"/>
       <c r="I50" s="32"/>
@@ -3717,7 +3717,7 @@
       <c r="K50" s="32"/>
     </row>
     <row r="51" spans="1:11" s="33" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="139"/>
+      <c r="A51" s="124"/>
       <c r="B51" s="122"/>
       <c r="C51" s="36" t="s">
         <v>182</v>
@@ -3732,7 +3732,7 @@
         <v>185</v>
       </c>
       <c r="G51" s="36" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="H51" s="31"/>
       <c r="I51" s="32"/>
@@ -3740,7 +3740,7 @@
       <c r="K51" s="32"/>
     </row>
     <row r="52" spans="1:11" s="33" customFormat="1" ht="66" x14ac:dyDescent="0.3">
-      <c r="A52" s="139"/>
+      <c r="A52" s="124"/>
       <c r="B52" s="122"/>
       <c r="C52" s="36" t="s">
         <v>186</v>
@@ -3749,13 +3749,13 @@
         <v>187</v>
       </c>
       <c r="E52" s="37" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="F52" s="36" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="G52" s="36" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="H52" s="31"/>
       <c r="I52" s="32"/>
@@ -3763,7 +3763,7 @@
       <c r="K52" s="32"/>
     </row>
     <row r="53" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A53" s="139"/>
+      <c r="A53" s="124"/>
       <c r="B53" s="123"/>
       <c r="C53" s="36" t="s">
         <v>188</v>
@@ -3778,7 +3778,7 @@
         <v>30</v>
       </c>
       <c r="G53" s="36" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="H53" s="31"/>
       <c r="I53" s="32"/>
@@ -3786,11 +3786,11 @@
       <c r="K53" s="32"/>
     </row>
     <row r="54" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A54" s="139" t="s">
-        <v>354</v>
+      <c r="A54" s="124" t="s">
+        <v>350</v>
       </c>
       <c r="B54" s="121" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="C54" s="36" t="s">
         <v>191</v>
@@ -3805,7 +3805,7 @@
         <v>143</v>
       </c>
       <c r="G54" s="36" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="H54" s="31"/>
       <c r="I54" s="32"/>
@@ -3813,7 +3813,7 @@
       <c r="K54" s="32"/>
     </row>
     <row r="55" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A55" s="139"/>
+      <c r="A55" s="124"/>
       <c r="B55" s="122"/>
       <c r="C55" s="36" t="s">
         <v>194</v>
@@ -3828,7 +3828,7 @@
         <v>197</v>
       </c>
       <c r="G55" s="36" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="H55" s="31"/>
       <c r="I55" s="32"/>
@@ -3836,7 +3836,7 @@
       <c r="K55" s="32"/>
     </row>
     <row r="56" spans="1:11" s="33" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
-      <c r="A56" s="139"/>
+      <c r="A56" s="124"/>
       <c r="B56" s="122"/>
       <c r="C56" s="36" t="s">
         <v>198</v>
@@ -3845,13 +3845,13 @@
         <v>199</v>
       </c>
       <c r="E56" s="37" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="F56" s="37" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="G56" s="36" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="H56" s="31"/>
       <c r="I56" s="32"/>
@@ -3859,13 +3859,13 @@
       <c r="K56" s="32"/>
     </row>
     <row r="57" spans="1:11" s="33" customFormat="1" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A57" s="139"/>
+      <c r="A57" s="124"/>
       <c r="B57" s="123"/>
       <c r="C57" s="36" t="s">
+        <v>388</v>
+      </c>
+      <c r="D57" s="37" t="s">
         <v>200</v>
-      </c>
-      <c r="D57" s="37" t="s">
-        <v>201</v>
       </c>
       <c r="E57" s="37" t="s">
         <v>190</v>
@@ -3874,7 +3874,7 @@
         <v>30</v>
       </c>
       <c r="G57" s="36" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="H57" s="31"/>
       <c r="I57" s="32"/>
@@ -3882,26 +3882,26 @@
       <c r="K57" s="32"/>
     </row>
     <row r="58" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A58" s="139" t="s">
-        <v>353</v>
+      <c r="A58" s="124" t="s">
+        <v>349</v>
       </c>
       <c r="B58" s="121" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="C58" s="36" t="s">
+        <v>201</v>
+      </c>
+      <c r="D58" s="37" t="s">
         <v>202</v>
       </c>
-      <c r="D58" s="37" t="s">
+      <c r="E58" s="37" t="s">
         <v>203</v>
-      </c>
-      <c r="E58" s="37" t="s">
-        <v>204</v>
       </c>
       <c r="F58" s="36" t="s">
         <v>143</v>
       </c>
       <c r="G58" s="36" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="H58" s="31"/>
       <c r="I58" s="32"/>
@@ -3909,13 +3909,13 @@
       <c r="K58" s="32"/>
     </row>
     <row r="59" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A59" s="139"/>
+      <c r="A59" s="124"/>
       <c r="B59" s="122"/>
       <c r="C59" s="36" t="s">
+        <v>204</v>
+      </c>
+      <c r="D59" s="37" t="s">
         <v>205</v>
-      </c>
-      <c r="D59" s="37" t="s">
-        <v>206</v>
       </c>
       <c r="E59" s="37" t="s">
         <v>190</v>
@@ -3924,7 +3924,7 @@
         <v>185</v>
       </c>
       <c r="G59" s="36" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="H59" s="31"/>
       <c r="I59" s="32"/>
@@ -3932,22 +3932,22 @@
       <c r="K59" s="32"/>
     </row>
     <row r="60" spans="1:11" s="33" customFormat="1" ht="66" x14ac:dyDescent="0.3">
-      <c r="A60" s="139"/>
+      <c r="A60" s="124"/>
       <c r="B60" s="122"/>
       <c r="C60" s="36" t="s">
+        <v>206</v>
+      </c>
+      <c r="D60" s="37" t="s">
         <v>207</v>
       </c>
-      <c r="D60" s="37" t="s">
-        <v>208</v>
-      </c>
       <c r="E60" s="37" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="F60" s="36" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="G60" s="36" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="H60" s="31"/>
       <c r="I60" s="32"/>
@@ -3955,22 +3955,22 @@
       <c r="K60" s="32"/>
     </row>
     <row r="61" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A61" s="139"/>
+      <c r="A61" s="124"/>
       <c r="B61" s="123"/>
       <c r="C61" s="36" t="s">
+        <v>208</v>
+      </c>
+      <c r="D61" s="37" t="s">
         <v>209</v>
       </c>
-      <c r="D61" s="37" t="s">
-        <v>210</v>
-      </c>
       <c r="E61" s="37" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="F61" s="37" t="s">
         <v>30</v>
       </c>
       <c r="G61" s="36" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="H61" s="31"/>
       <c r="I61" s="32"/>
@@ -3978,26 +3978,26 @@
       <c r="K61" s="32"/>
     </row>
     <row r="62" spans="1:11" s="33" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="139" t="s">
-        <v>354</v>
+      <c r="A62" s="124" t="s">
+        <v>350</v>
       </c>
       <c r="B62" s="121" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
       <c r="C62" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="D62" s="37" t="s">
         <v>211</v>
       </c>
-      <c r="D62" s="37" t="s">
+      <c r="E62" s="37" t="s">
         <v>212</v>
-      </c>
-      <c r="E62" s="37" t="s">
-        <v>213</v>
       </c>
       <c r="F62" s="36" t="s">
         <v>143</v>
       </c>
       <c r="G62" s="36" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="H62" s="31"/>
       <c r="I62" s="32"/>
@@ -4005,22 +4005,22 @@
       <c r="K62" s="32"/>
     </row>
     <row r="63" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A63" s="139"/>
+      <c r="A63" s="124"/>
       <c r="B63" s="122"/>
       <c r="C63" s="36" t="s">
+        <v>213</v>
+      </c>
+      <c r="D63" s="37" t="s">
         <v>214</v>
       </c>
-      <c r="D63" s="37" t="s">
+      <c r="E63" s="37" t="s">
         <v>215</v>
-      </c>
-      <c r="E63" s="37" t="s">
-        <v>216</v>
       </c>
       <c r="F63" s="36" t="s">
         <v>197</v>
       </c>
       <c r="G63" s="36" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="H63" s="31"/>
       <c r="I63" s="32"/>
@@ -4028,33 +4028,33 @@
       <c r="K63" s="32"/>
     </row>
     <row r="64" spans="1:11" ht="105.6" x14ac:dyDescent="0.3">
-      <c r="A64" s="139"/>
+      <c r="A64" s="124"/>
       <c r="B64" s="122"/>
       <c r="C64" s="36" t="s">
+        <v>216</v>
+      </c>
+      <c r="D64" s="37" t="s">
         <v>217</v>
       </c>
-      <c r="D64" s="37" t="s">
-        <v>218</v>
-      </c>
       <c r="E64" s="37" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="F64" s="37" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="G64" s="36" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="H64" s="12"/>
     </row>
     <row r="65" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A65" s="139"/>
+      <c r="A65" s="124"/>
       <c r="B65" s="123"/>
       <c r="C65" s="36" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="D65" s="37" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="E65" s="37" t="s">
         <v>190</v>
@@ -4063,71 +4063,71 @@
         <v>30</v>
       </c>
       <c r="G65" s="36" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="H65" s="12"/>
     </row>
     <row r="66" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="B66" s="121" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="C66" s="36" t="s">
+        <v>219</v>
+      </c>
+      <c r="D66" s="37" t="s">
+        <v>220</v>
+      </c>
+      <c r="E66" s="37" t="s">
         <v>221</v>
       </c>
-      <c r="D66" s="37" t="s">
+      <c r="F66" s="36" t="s">
         <v>222</v>
       </c>
-      <c r="E66" s="37" t="s">
-        <v>223</v>
-      </c>
-      <c r="F66" s="36" t="s">
-        <v>224</v>
-      </c>
       <c r="G66" s="36" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H66" s="10"/>
     </row>
     <row r="67" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B67" s="123"/>
       <c r="C67" s="36" t="s">
+        <v>223</v>
+      </c>
+      <c r="D67" s="37" t="s">
+        <v>224</v>
+      </c>
+      <c r="E67" s="37" t="s">
         <v>225</v>
-      </c>
-      <c r="D67" s="37" t="s">
-        <v>226</v>
-      </c>
-      <c r="E67" s="37" t="s">
-        <v>227</v>
       </c>
       <c r="F67" s="36" t="s">
         <v>143</v>
       </c>
       <c r="G67" s="36" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H67" s="12"/>
     </row>
     <row r="68" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A68" s="139" t="s">
-        <v>355</v>
+      <c r="A68" s="124" t="s">
+        <v>351</v>
       </c>
       <c r="B68" s="121" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="C68" s="36" t="s">
+        <v>226</v>
+      </c>
+      <c r="D68" s="37" t="s">
+        <v>227</v>
+      </c>
+      <c r="E68" s="37" t="s">
         <v>228</v>
       </c>
-      <c r="D68" s="37" t="s">
+      <c r="F68" s="36" t="s">
         <v>229</v>
       </c>
-      <c r="E68" s="37" t="s">
-        <v>230</v>
-      </c>
-      <c r="F68" s="36" t="s">
-        <v>231</v>
-      </c>
       <c r="G68" s="36" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H68" s="30"/>
       <c r="I68" s="28"/>
@@ -4135,22 +4135,22 @@
       <c r="K68" s="28"/>
     </row>
     <row r="69" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A69" s="139"/>
+      <c r="A69" s="124"/>
       <c r="B69" s="122"/>
       <c r="C69" s="36" t="s">
+        <v>230</v>
+      </c>
+      <c r="D69" s="37" t="s">
+        <v>231</v>
+      </c>
+      <c r="E69" s="37" t="s">
         <v>232</v>
-      </c>
-      <c r="D69" s="37" t="s">
-        <v>233</v>
-      </c>
-      <c r="E69" s="37" t="s">
-        <v>234</v>
       </c>
       <c r="F69" s="36" t="s">
         <v>143</v>
       </c>
       <c r="G69" s="36" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H69" s="30"/>
       <c r="I69" s="28"/>
@@ -4158,22 +4158,22 @@
       <c r="K69" s="28"/>
     </row>
     <row r="70" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A70" s="139"/>
+      <c r="A70" s="124"/>
       <c r="B70" s="123"/>
       <c r="C70" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="D70" s="37" t="s">
+        <v>234</v>
+      </c>
+      <c r="E70" s="37" t="s">
         <v>235</v>
-      </c>
-      <c r="D70" s="37" t="s">
-        <v>236</v>
-      </c>
-      <c r="E70" s="37" t="s">
-        <v>237</v>
       </c>
       <c r="F70" s="36" t="s">
         <v>143</v>
       </c>
       <c r="G70" s="36" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H70" s="30"/>
       <c r="I70" s="28"/>
@@ -4181,24 +4181,24 @@
       <c r="K70" s="28"/>
     </row>
     <row r="71" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A71" s="139"/>
+      <c r="A71" s="124"/>
       <c r="B71" s="121" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="C71" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="D71" s="37" t="s">
+        <v>237</v>
+      </c>
+      <c r="E71" s="37" t="s">
         <v>238</v>
       </c>
-      <c r="D71" s="37" t="s">
-        <v>239</v>
-      </c>
-      <c r="E71" s="37" t="s">
-        <v>240</v>
-      </c>
       <c r="F71" s="36" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="G71" s="36" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H71" s="30"/>
       <c r="I71" s="28"/>
@@ -4206,22 +4206,22 @@
       <c r="K71" s="28"/>
     </row>
     <row r="72" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A72" s="139"/>
+      <c r="A72" s="124"/>
       <c r="B72" s="122"/>
       <c r="C72" s="36" t="s">
+        <v>239</v>
+      </c>
+      <c r="D72" s="37" t="s">
+        <v>240</v>
+      </c>
+      <c r="E72" s="37" t="s">
         <v>241</v>
-      </c>
-      <c r="D72" s="37" t="s">
-        <v>242</v>
-      </c>
-      <c r="E72" s="37" t="s">
-        <v>243</v>
       </c>
       <c r="F72" s="36" t="s">
         <v>143</v>
       </c>
       <c r="G72" s="36" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H72" s="30"/>
       <c r="I72" s="28"/>
@@ -4229,22 +4229,22 @@
       <c r="K72" s="28"/>
     </row>
     <row r="73" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A73" s="139"/>
+      <c r="A73" s="124"/>
       <c r="B73" s="123"/>
       <c r="C73" s="36" t="s">
+        <v>242</v>
+      </c>
+      <c r="D73" s="37" t="s">
+        <v>243</v>
+      </c>
+      <c r="E73" s="37" t="s">
         <v>244</v>
-      </c>
-      <c r="D73" s="37" t="s">
-        <v>245</v>
-      </c>
-      <c r="E73" s="37" t="s">
-        <v>246</v>
       </c>
       <c r="F73" s="36" t="s">
         <v>143</v>
       </c>
       <c r="G73" s="36" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H73" s="30"/>
       <c r="I73" s="28"/>
@@ -4254,22 +4254,22 @@
     <row r="74" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A74"/>
       <c r="B74" s="121" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="C74" s="118" t="s">
+        <v>245</v>
+      </c>
+      <c r="D74" s="118" t="s">
+        <v>246</v>
+      </c>
+      <c r="E74" s="118" t="s">
         <v>247</v>
-      </c>
-      <c r="D74" s="118" t="s">
-        <v>248</v>
-      </c>
-      <c r="E74" s="118" t="s">
-        <v>249</v>
       </c>
       <c r="F74" s="119" t="s">
         <v>143</v>
       </c>
       <c r="G74" s="119" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H74" s="30"/>
       <c r="I74" s="28"/>
@@ -4280,19 +4280,19 @@
       <c r="A75"/>
       <c r="B75" s="123"/>
       <c r="C75" s="118" t="s">
+        <v>248</v>
+      </c>
+      <c r="D75" s="118" t="s">
+        <v>249</v>
+      </c>
+      <c r="E75" s="118" t="s">
         <v>250</v>
-      </c>
-      <c r="D75" s="118" t="s">
-        <v>251</v>
-      </c>
-      <c r="E75" s="118" t="s">
-        <v>252</v>
       </c>
       <c r="F75" s="118" t="s">
         <v>145</v>
       </c>
       <c r="G75" s="118" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H75" s="31"/>
       <c r="I75" s="32"/>
@@ -4300,26 +4300,26 @@
       <c r="K75" s="32"/>
     </row>
     <row r="76" spans="1:11" s="33" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="139" t="s">
-        <v>356</v>
+      <c r="A76" s="124" t="s">
+        <v>352</v>
       </c>
       <c r="B76" s="121" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="C76" s="36" t="s">
+        <v>251</v>
+      </c>
+      <c r="D76" s="37" t="s">
+        <v>252</v>
+      </c>
+      <c r="E76" s="118" t="s">
         <v>253</v>
-      </c>
-      <c r="D76" s="37" t="s">
-        <v>254</v>
-      </c>
-      <c r="E76" s="118" t="s">
-        <v>255</v>
       </c>
       <c r="F76" s="36" t="s">
         <v>143</v>
       </c>
       <c r="G76" s="36" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H76" s="31"/>
       <c r="I76" s="32"/>
@@ -4327,22 +4327,22 @@
       <c r="K76" s="32"/>
     </row>
     <row r="77" spans="1:11" s="33" customFormat="1" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="139"/>
+      <c r="A77" s="124"/>
       <c r="B77" s="122"/>
       <c r="C77" s="36" t="s">
+        <v>356</v>
+      </c>
+      <c r="D77" s="37" t="s">
+        <v>357</v>
+      </c>
+      <c r="E77" s="37" t="s">
         <v>360</v>
       </c>
-      <c r="D77" s="37" t="s">
-        <v>361</v>
-      </c>
-      <c r="E77" s="37" t="s">
-        <v>364</v>
-      </c>
       <c r="F77" s="36" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="G77" s="36" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H77" s="31"/>
       <c r="I77" s="32"/>
@@ -4350,19 +4350,19 @@
       <c r="K77" s="32"/>
     </row>
     <row r="78" spans="1:11" s="33" customFormat="1" ht="187.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="139"/>
+      <c r="A78" s="124"/>
       <c r="B78" s="123"/>
       <c r="C78" s="36" t="s">
+        <v>358</v>
+      </c>
+      <c r="D78" s="37" t="s">
+        <v>359</v>
+      </c>
+      <c r="E78" s="37" t="s">
+        <v>361</v>
+      </c>
+      <c r="F78" s="36" t="s">
         <v>362</v>
-      </c>
-      <c r="D78" s="37" t="s">
-        <v>363</v>
-      </c>
-      <c r="E78" s="37" t="s">
-        <v>365</v>
-      </c>
-      <c r="F78" s="36" t="s">
-        <v>366</v>
       </c>
       <c r="G78" s="36"/>
       <c r="H78" s="31"/>
@@ -4371,26 +4371,26 @@
       <c r="K78" s="32"/>
     </row>
     <row r="79" spans="1:11" s="33" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="139" t="s">
-        <v>356</v>
+      <c r="A79" s="124" t="s">
+        <v>352</v>
       </c>
       <c r="B79" s="121" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
       <c r="C79" s="36" t="s">
+        <v>254</v>
+      </c>
+      <c r="D79" s="37" t="s">
+        <v>255</v>
+      </c>
+      <c r="E79" s="118" t="s">
         <v>256</v>
-      </c>
-      <c r="D79" s="37" t="s">
-        <v>257</v>
-      </c>
-      <c r="E79" s="118" t="s">
-        <v>258</v>
       </c>
       <c r="F79" s="36" t="s">
         <v>143</v>
       </c>
       <c r="G79" s="36" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H79" s="31"/>
       <c r="I79" s="32"/>
@@ -4398,22 +4398,22 @@
       <c r="K79" s="32"/>
     </row>
     <row r="80" spans="1:11" s="33" customFormat="1" ht="198" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="139"/>
+      <c r="A80" s="124"/>
       <c r="B80" s="122"/>
       <c r="C80" s="36" t="s">
+        <v>363</v>
+      </c>
+      <c r="D80" s="37" t="s">
+        <v>365</v>
+      </c>
+      <c r="E80" s="37" t="s">
         <v>367</v>
       </c>
-      <c r="D80" s="37" t="s">
-        <v>369</v>
-      </c>
-      <c r="E80" s="37" t="s">
-        <v>371</v>
-      </c>
       <c r="F80" s="36" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="G80" s="36" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="H80" s="31"/>
       <c r="I80" s="32"/>
@@ -4421,19 +4421,19 @@
       <c r="K80" s="32"/>
     </row>
     <row r="81" spans="1:11" s="33" customFormat="1" ht="189" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="139"/>
+      <c r="A81" s="124"/>
       <c r="B81" s="123"/>
       <c r="C81" s="36" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="D81" s="37" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="E81" s="37" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="F81" s="36" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="G81" s="36"/>
       <c r="H81" s="31"/>
@@ -4443,76 +4443,76 @@
     </row>
     <row r="82" spans="1:11" ht="66" x14ac:dyDescent="0.3">
       <c r="B82" s="121" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="C82" s="36" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D82" s="37" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="E82" s="118" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="F82" s="36" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="G82" s="36" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="83" spans="1:11" ht="79.2" x14ac:dyDescent="0.3">
       <c r="B83" s="122"/>
       <c r="C83" s="36" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D83" s="37" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="E83" s="118" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="F83" s="36" t="s">
         <v>143</v>
       </c>
       <c r="G83" s="36" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="84" spans="1:11" ht="105.6" x14ac:dyDescent="0.3">
       <c r="B84" s="122"/>
       <c r="C84" s="36" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D84" s="37" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="E84" s="118" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="F84" s="36" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="G84" s="36" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="85" spans="1:11" ht="66" x14ac:dyDescent="0.3">
       <c r="B85" s="123"/>
       <c r="C85" s="36" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="D85" s="37" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="E85" s="118" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="F85" s="36" t="s">
         <v>30</v>
       </c>
       <c r="G85" s="36" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.3">
@@ -4549,6 +4549,18 @@
     </row>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="B79:B81"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="B54:B57"/>
+    <mergeCell ref="B58:B61"/>
+    <mergeCell ref="B62:B65"/>
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="B3:B16"/>
+    <mergeCell ref="B17:B26"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="B30:B40"/>
+    <mergeCell ref="B50:B53"/>
     <mergeCell ref="B82:B85"/>
     <mergeCell ref="A17:A26"/>
     <mergeCell ref="B44:B45"/>
@@ -4565,18 +4577,6 @@
     <mergeCell ref="A76:A78"/>
     <mergeCell ref="B76:B78"/>
     <mergeCell ref="A79:A81"/>
-    <mergeCell ref="B3:B16"/>
-    <mergeCell ref="B17:B26"/>
-    <mergeCell ref="B27:B29"/>
-    <mergeCell ref="B30:B40"/>
-    <mergeCell ref="B50:B53"/>
-    <mergeCell ref="B79:B81"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="B48:B49"/>
-    <mergeCell ref="B54:B57"/>
-    <mergeCell ref="B58:B61"/>
-    <mergeCell ref="B62:B65"/>
-    <mergeCell ref="B66:B67"/>
   </mergeCells>
   <phoneticPr fontId="29" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4605,7 +4605,7 @@
         <v>28</v>
       </c>
       <c r="B1" s="101" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="C1" s="102" t="s">
         <v>33</v>
@@ -4614,7 +4614,7 @@
         <v>37</v>
       </c>
       <c r="E1" s="102" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="F1" s="102" t="s">
         <v>42</v>
@@ -4662,19 +4662,19 @@
         <v>95</v>
       </c>
       <c r="U1" s="103" t="s">
+        <v>293</v>
+      </c>
+      <c r="V1" s="103" t="s">
+        <v>294</v>
+      </c>
+      <c r="W1" s="103" t="s">
+        <v>295</v>
+      </c>
+      <c r="X1" s="103" t="s">
+        <v>296</v>
+      </c>
+      <c r="Y1" s="103" t="s">
         <v>297</v>
-      </c>
-      <c r="V1" s="103" t="s">
-        <v>298</v>
-      </c>
-      <c r="W1" s="103" t="s">
-        <v>299</v>
-      </c>
-      <c r="X1" s="103" t="s">
-        <v>300</v>
-      </c>
-      <c r="Y1" s="103" t="s">
-        <v>301</v>
       </c>
       <c r="Z1" s="104" t="s">
         <v>99</v>
@@ -4710,22 +4710,22 @@
         <v>138</v>
       </c>
       <c r="AK1" s="104" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="AL1" s="104" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="AM1" s="104" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="AN1" s="105" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="AO1" s="105" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="AP1" s="44" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="AQ1" s="44" t="s">
         <v>144</v>
@@ -4815,169 +4815,169 @@
         <v>191</v>
       </c>
       <c r="BT1" s="45" t="s">
+        <v>273</v>
+      </c>
+      <c r="BU1" s="45" t="s">
+        <v>274</v>
+      </c>
+      <c r="BV1" s="45" t="s">
+        <v>390</v>
+      </c>
+      <c r="BW1" s="45" t="s">
+        <v>201</v>
+      </c>
+      <c r="BX1" s="45" t="s">
+        <v>204</v>
+      </c>
+      <c r="BY1" s="45" t="s">
+        <v>206</v>
+      </c>
+      <c r="BZ1" s="45" t="s">
+        <v>208</v>
+      </c>
+      <c r="CA1" s="45" t="s">
+        <v>210</v>
+      </c>
+      <c r="CB1" s="45" t="s">
         <v>275</v>
       </c>
-      <c r="BU1" s="45" t="s">
+      <c r="CC1" s="45" t="s">
         <v>276</v>
       </c>
-      <c r="BV1" s="45" t="s">
-        <v>277</v>
-      </c>
-      <c r="BW1" s="45" t="s">
-        <v>202</v>
-      </c>
-      <c r="BX1" s="45" t="s">
-        <v>205</v>
-      </c>
-      <c r="BY1" s="45" t="s">
-        <v>207</v>
-      </c>
-      <c r="BZ1" s="45" t="s">
-        <v>209</v>
-      </c>
-      <c r="CA1" s="45" t="s">
-        <v>211</v>
-      </c>
-      <c r="CB1" s="45" t="s">
-        <v>278</v>
-      </c>
-      <c r="CC1" s="45" t="s">
-        <v>279</v>
-      </c>
       <c r="CD1" s="45" t="s">
-        <v>280</v>
+        <v>391</v>
       </c>
       <c r="CE1" s="45" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="CF1" s="45" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="CG1" s="45" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="CH1" s="45" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="CI1" s="45" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="CJ1" s="45" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="CK1" s="45" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="CL1" s="45" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="CM1" s="45" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="CN1" s="45" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="CO1" s="45" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="CP1" s="45" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="CQ1" s="45" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="CR1" s="45" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="CS1" s="45" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="CT1" s="45" t="s">
+        <v>364</v>
+      </c>
+      <c r="CU1" s="45" t="s">
+        <v>257</v>
+      </c>
+      <c r="CV1" s="45" t="s">
         <v>368</v>
       </c>
-      <c r="CU1" s="45" t="s">
+      <c r="CW1" s="45" t="s">
+        <v>376</v>
+      </c>
+      <c r="CX1" s="45" t="s">
+        <v>258</v>
+      </c>
+      <c r="CY1" s="45" t="s">
+        <v>369</v>
+      </c>
+      <c r="CZ1" s="45" t="s">
+        <v>377</v>
+      </c>
+      <c r="DA1" s="45" t="s">
         <v>259</v>
       </c>
-      <c r="CV1" s="45" t="s">
+      <c r="DB1" s="45" t="s">
+        <v>370</v>
+      </c>
+      <c r="DC1" s="45" t="s">
+        <v>378</v>
+      </c>
+      <c r="DD1" s="45" t="s">
+        <v>260</v>
+      </c>
+      <c r="DE1" s="45" t="s">
+        <v>371</v>
+      </c>
+      <c r="DF1" s="45" t="s">
+        <v>379</v>
+      </c>
+      <c r="DG1" s="45" t="s">
+        <v>261</v>
+      </c>
+      <c r="DH1" s="45" t="s">
         <v>372</v>
       </c>
-      <c r="CW1" s="45" t="s">
+      <c r="DI1" s="45" t="s">
         <v>380</v>
       </c>
-      <c r="CX1" s="45" t="s">
-        <v>260</v>
-      </c>
-      <c r="CY1" s="45" t="s">
+      <c r="DJ1" s="45" t="s">
+        <v>262</v>
+      </c>
+      <c r="DK1" s="45" t="s">
         <v>373</v>
       </c>
-      <c r="CZ1" s="45" t="s">
+      <c r="DL1" s="45" t="s">
         <v>381</v>
       </c>
-      <c r="DA1" s="45" t="s">
-        <v>261</v>
-      </c>
-      <c r="DB1" s="45" t="s">
+      <c r="DM1" s="45" t="s">
+        <v>263</v>
+      </c>
+      <c r="DN1" s="45" t="s">
         <v>374</v>
       </c>
-      <c r="DC1" s="45" t="s">
+      <c r="DO1" s="45" t="s">
         <v>382</v>
       </c>
-      <c r="DD1" s="45" t="s">
-        <v>262</v>
-      </c>
-      <c r="DE1" s="45" t="s">
+      <c r="DP1" s="45" t="s">
+        <v>264</v>
+      </c>
+      <c r="DQ1" s="45" t="s">
         <v>375</v>
       </c>
-      <c r="DF1" s="45" t="s">
+      <c r="DR1" s="45" t="s">
         <v>383</v>
       </c>
-      <c r="DG1" s="45" t="s">
-        <v>263</v>
-      </c>
-      <c r="DH1" s="45" t="s">
-        <v>376</v>
-      </c>
-      <c r="DI1" s="45" t="s">
-        <v>384</v>
-      </c>
-      <c r="DJ1" s="45" t="s">
-        <v>264</v>
-      </c>
-      <c r="DK1" s="45" t="s">
-        <v>377</v>
-      </c>
-      <c r="DL1" s="45" t="s">
-        <v>385</v>
-      </c>
-      <c r="DM1" s="45" t="s">
+      <c r="DS1" s="45" t="s">
         <v>265</v>
       </c>
-      <c r="DN1" s="45" t="s">
-        <v>378</v>
-      </c>
-      <c r="DO1" s="45" t="s">
-        <v>386</v>
-      </c>
-      <c r="DP1" s="45" t="s">
-        <v>266</v>
-      </c>
-      <c r="DQ1" s="45" t="s">
-        <v>379</v>
-      </c>
-      <c r="DR1" s="45" t="s">
-        <v>387</v>
-      </c>
-      <c r="DS1" s="45" t="s">
+      <c r="DT1" s="45" t="s">
         <v>267</v>
       </c>
-      <c r="DT1" s="45" t="s">
+      <c r="DU1" s="45" t="s">
         <v>269</v>
       </c>
-      <c r="DU1" s="45" t="s">
+      <c r="DV1" s="45" t="s">
         <v>271</v>
-      </c>
-      <c r="DV1" s="45" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="2" spans="1:126" x14ac:dyDescent="0.3">
@@ -19935,17 +19935,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="42fbd5e6-b175-407a-a25c-5fc6410bf24f" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EE7777BCFCD3E741B5CCCE9A87E98C2C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f7fc7590daec4eb8e38e018938a160ca">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e" xmlns:ns3="42fbd5e6-b175-407a-a25c-5fc6410bf24f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c5ca1b94d4b54616210e83d04e6b3cac" ns2:_="" ns3:_="">
     <xsd:import namespace="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
@@ -20200,6 +20189,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="42fbd5e6-b175-407a-a25c-5fc6410bf24f" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{286F673D-E70D-4002-B8F5-CAC95B029A7E}">
   <ds:schemaRefs>
@@ -20209,17 +20209,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E9485EC-5D88-4A1C-961D-0F4FE84359B8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="42fbd5e6-b175-407a-a25c-5fc6410bf24f"/>
-    <ds:schemaRef ds:uri="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C9C537E-DFD2-4C38-AC8C-930F122DEFFC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -20236,4 +20225,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E9485EC-5D88-4A1C-961D-0F4FE84359B8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="42fbd5e6-b175-407a-a25c-5fc6410bf24f"/>
+    <ds:schemaRef ds:uri="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
adjust data dictionary per discussion
</commit_message>
<xml_diff>
--- a/data/ALAI UP Client-level Reporting Tool Template_4.7.26.xlsx
+++ b/data/ALAI UP Client-level Reporting Tool Template_4.7.26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kmlab\Desktop\Dashboard\alai_up_local_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF9AAC9B-529C-4EA9-9AAB-3B03C5851854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F21A1A49-24D8-402A-885E-3DBC40E77D94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{500E2EE0-B1C5-4ACF-BC67-EDC8BDABD2D7}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{500E2EE0-B1C5-4ACF-BC67-EDC8BDABD2D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="3" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="380">
   <si>
     <t>INSTRUCTIONS</t>
   </si>
@@ -344,9 +344,6 @@
     <t>Active client - 2021</t>
   </si>
   <si>
-    <t>This client accessed clinical HIV services at least once in the 2021 calendar year.</t>
-  </si>
-  <si>
     <t>0=Did not access clinical HIV services; 1=Accessed clinical HIV services</t>
   </si>
   <si>
@@ -356,34 +353,22 @@
     <t>Active client - 2022</t>
   </si>
   <si>
-    <t>This client accessed clinical HIV services at least once in the 2022 calendar year.</t>
-  </si>
-  <si>
     <t>active_2023</t>
   </si>
   <si>
     <t>Active client - 2023</t>
   </si>
   <si>
-    <t>This client accessed clinical HIV services at least once in the 2023 calendar year.</t>
-  </si>
-  <si>
     <t>active_2024</t>
   </si>
   <si>
     <t>Active client - 2024</t>
   </si>
   <si>
-    <t>This client accessed clinical HIV services at least once in the 2024 calendar year.</t>
-  </si>
-  <si>
     <t>active_2025</t>
   </si>
   <si>
     <t>Active client - 2025</t>
-  </si>
-  <si>
-    <t>This client accessed clinical HIV services at least once in the 2025 calendar year.</t>
   </si>
   <si>
     <t>HIV-related behaviors</t>
@@ -759,9 +744,6 @@
     <t>iCAB/RPV prescribed</t>
   </si>
   <si>
-    <t>The client was prescribed iCAB/RPV by a clinical provider.</t>
-  </si>
-  <si>
     <t>0=Client not prescribed iCAB/RPV; 1=Client  prescribed iCAB/RPV; UNK=Unknown</t>
   </si>
   <si>
@@ -771,9 +753,6 @@
     <t>Date iCAB/RPV prescribed</t>
   </si>
   <si>
-    <t>The date the client was prescribed iCAB/RPV.</t>
-  </si>
-  <si>
     <t>icab_rpv_oral_bridge1</t>
   </si>
   <si>
@@ -801,9 +780,6 @@
     <t>Oral bridge1 for planned missed injection end date</t>
   </si>
   <si>
-    <t>Date client ended oral ART for the first time to bridge therapy for planned missed iCAB/RPV injection.</t>
-  </si>
-  <si>
     <t>icab_rpv_oral_bridge2</t>
   </si>
   <si>
@@ -828,9 +804,6 @@
     <t>Oral bridge2 for planned missed injection end date</t>
   </si>
   <si>
-    <t>Date client ended oral ART for the second time to bridge therapy for planned missed iCAB/RPV injection.</t>
-  </si>
-  <si>
     <t>hiv_vl_pre_icab_date</t>
   </si>
   <si>
@@ -846,27 +819,18 @@
     <t>Most recent HIV viral load result on or before first iCAB/RPV injection</t>
   </si>
   <si>
-    <t>Client's most recent viral load result on or before first iCAB/RPV injection.</t>
-  </si>
-  <si>
     <t>icab_rpv_shot1_date</t>
   </si>
   <si>
     <t>Injection 1 date</t>
   </si>
   <si>
-    <t>Date of client's first iCAB/RPV injection. This should be the date of their first loading dose, regardless of whether it occurred before or after the beginning of ALAI UP (3/1/23).</t>
-  </si>
-  <si>
     <t>icab_rpv_shot2_date</t>
   </si>
   <si>
     <t>Injection 2 date</t>
   </si>
   <si>
-    <t xml:space="preserve">Date of client's second iCAB/RPV injection. </t>
-  </si>
-  <si>
     <t>icab_rpv_shot3_date</t>
   </si>
   <si>
@@ -951,15 +915,9 @@
     <t>Client's viral load results at client's first test since the beginning of injectable program</t>
   </si>
   <si>
-    <t>The date of the client's first viral load test since the beginning of injectable program. The date of specimen collected is preferred, but if that cannot be retrieved, then the date of results returned.</t>
-  </si>
-  <si>
     <t>Client's viral load results at client's second test since the beginning of injectable program</t>
   </si>
   <si>
-    <t>The date of the client's second viral load test since the beginning of injectable program. The date of specimen collected is preferred, but if that cannot be retrieved, then the date of results returned.</t>
-  </si>
-  <si>
     <t>SDOH_other_1</t>
   </si>
   <si>
@@ -972,9 +930,6 @@
     <t>SDOH_other_3</t>
   </si>
   <si>
-    <t>Sites are encouraged to report any additional social determinants of health variables (e.g., access to transportation, non-injection drug use) that they collect. Note that these results will show up as text, so ensure that values are consistent.</t>
-  </si>
-  <si>
     <t>active_2026</t>
   </si>
   <si>
@@ -1003,21 +958,6 @@
   </si>
   <si>
     <t>Active client - 2030</t>
-  </si>
-  <si>
-    <t>This client accessed clinical HIV services at least once in the 2026 calendar year.</t>
-  </si>
-  <si>
-    <t>This client accessed clinical HIV services at least once in the 2027 calendar year.</t>
-  </si>
-  <si>
-    <t>This client accessed clinical HIV services at least once in the 2028 calendar year.</t>
-  </si>
-  <si>
-    <t>This client accessed clinical HIV services at least once in the 2029 calendar year.</t>
-  </si>
-  <si>
-    <t>This client accessed clinical HIV services at least once in the 2030 calendar year.</t>
   </si>
   <si>
     <t>hiv_dx_date</t>
@@ -1083,51 +1023,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">If client not interested in iCAB/RPV after first iCAB/RPV counseling, primary reason for disinterest. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>If there are multiple known reasons, please separate them with a comma. If there are "other" reasons, include 20 in the list here and include them in icab_rpv_disinterest_reason_1_other</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">If the client is not eligible for iCAB/RPV at first screening, this is the primary reason why they were determined not eligible. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>If there are multiple known reasons, please separate them with a comma. If there are "other" reasons, include 20 in the list here and include them in icab_rpv_not_elig_1_reason_oth</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">If client not interested in iCAB/RPV after first iCAB/RPV counseling, primary reason for disinterest. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>If there are multiple known reasons, please separate them with a comma. If there are "other" reasons, include 20 in the list here and include them in icab_rpv_disinterest_reason_2_other</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t>If other, please specify.</t>
     </r>
     <r>
@@ -1142,54 +1037,10 @@
     </r>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">If the client is not eligible for iCAB/RPV at first screening, this is the primary reason why they were determined not eligible. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>If there are multiple known reasons, please separate them with a comma. If there are "other" reasons, include 20 in the list here and include them in icab_rpv_not_elig_2_reason_oth</t>
-    </r>
-  </si>
-  <si>
-    <t>Date client decided to discontinue iCAB/RPV.
-If a client was lost to follow up or moved to another clinic, they are considered discontinued (at that clinic), even if they are still on CAB at the new clinic. Assign icab_rpv_discontinued to be 1, and use the last CAB date as the discontinued date if there is no other date</t>
-  </si>
-  <si>
     <t>If other, please specify. 
 Please record any additional information about discontinuation and/or restarts in icab_rpv_discontinued_reason_other (e.g., client discontinued on MM/DD/YYYY due to loss of insurance but restarted at site on MM/DD/YYYY).</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">The client-reported primary reason why they decided to discontinue using iCAB/RPV. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>If there are multiple known reasons, please separate them with a comma. If there are "other" reasons, include 20 in the list here and include them in icab_rpv_discontinued_reason_other</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Please record any additional information about discontinuation and/or restarts in icab_rpv_discontinued_reason_other (e.g., client discontinued on MM/DD/YYYY due to loss of insurance but restarted at site on MM/DD/YYYY).</t>
-    </r>
-  </si>
-  <si>
     <t>The excel sheet provided should be used as a guide for preparing your data. Data can be entered manually, but  extracting data from the electronic medical record and organizing it into the correct format will be easier and more efficient.</t>
   </si>
   <si>
@@ -1226,10 +1077,6 @@
     <t>0=Sustained; 1=Discontinued; UNK=Unknown</t>
   </si>
   <si>
-    <t>A binary measure of whether the client currently discontinued iCAB/RPV.
-Note: only indicate discontinued = 1 if the client is currently NOT on CAB at the clinic. If the client stopped and restarted CAB, they are considered sustained and then stop/restart should be indicated via icab_rpv_shotX_interval=0</t>
-  </si>
-  <si>
     <t>HIV Laboratory - general</t>
   </si>
   <si>
@@ -1302,12 +1149,181 @@
     <t>Injection 1 late exception</t>
   </si>
   <si>
+    <t>0 = maintenance injection or regular loading injection; 1 = do not mark late; Re-loading after discontinuation, or transfer from another clinic already on iCAB/RPV</t>
+  </si>
+  <si>
+    <t>icab_rpv_shot2_interval</t>
+  </si>
+  <si>
+    <t>icab_rpv_shot2_late_exception</t>
+  </si>
+  <si>
+    <t>Injection 2 intended interval</t>
+  </si>
+  <si>
+    <t>Injection 2 late exception</t>
+  </si>
+  <si>
+    <t>icab_rpv_shot3_interval</t>
+  </si>
+  <si>
+    <t>icab_rpv_shot4_interval</t>
+  </si>
+  <si>
+    <t>icab_rpv_shot5_interval</t>
+  </si>
+  <si>
+    <t>icab_rpv_shot6_interval</t>
+  </si>
+  <si>
+    <t>icab_rpv_shot7_interval</t>
+  </si>
+  <si>
+    <t>icab_rpv_shot8_interval</t>
+  </si>
+  <si>
+    <t>icab_rpv_shot9_interval</t>
+  </si>
+  <si>
+    <t>icab_rpv_shot10_interval</t>
+  </si>
+  <si>
+    <t>icab_rpv_shot3_late_exception</t>
+  </si>
+  <si>
+    <t>icab_rpv_shot4_late_exception</t>
+  </si>
+  <si>
+    <t>icab_rpv_shot5_late_exception</t>
+  </si>
+  <si>
+    <t>icab_rpv_shot6_late_exception</t>
+  </si>
+  <si>
+    <t>icab_rpv_shot7_late_exception</t>
+  </si>
+  <si>
+    <t>icab_rpv_shot8_late_exception</t>
+  </si>
+  <si>
+    <t>icab_rpv_shot9_late_exception</t>
+  </si>
+  <si>
+    <t>icab_rpv_shot10_late_exception</t>
+  </si>
+  <si>
+    <t>birth_date</t>
+  </si>
+  <si>
+    <t>Birth date</t>
+  </si>
+  <si>
+    <t>The client's birth date. The value must be on or before all service dates for the client.</t>
+  </si>
+  <si>
+    <t>YYYY-MM-DD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">icab_rpv_not_elig_1_reason_other
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">icab_rpv_not_elig_2_reason_other
+</t>
+  </si>
+  <si>
+    <t>icab_rpv_not_elig_1_reason_other</t>
+  </si>
+  <si>
+    <t>icab_rpv_not_elig_2_reason_other</t>
+  </si>
+  <si>
+    <t>This client accessed clinical HIV services at least once in the given calendar year.
+Clinics can define and code this variable however makes sense for their clinic. For example, a clinic could define and code a client as being active in a given year if they had any clinic visits, any laboratory results, any injection, or any prescriptions.  
+To add future years, follow the same naming format; the Dashboard will detect the years automatically.</t>
+  </si>
+  <si>
+    <t>These variables are available as optional disaggregation variables in the Dashboard that clinics can use as needed. Responses coded under these variables will show up in the Dashboard as text exactly as entered in the template, so ensure that the responses entered are consistent and descriptive.
+Example: If the variable of interest is transportation, sample responses may include:
+-	No reliable transportation
+-	Some reliable transportation
+-	Consistent transportation
+All responses of a given category should have the same spelling and capitalization.</t>
+  </si>
+  <si>
+    <t>The date of the client's second viral load test since the beginning of injectable program. The date of specimen collected is preferred, but if that cannot be retrieved, then the date of results returned.
+Clinics should enter all viral load results for a given patient, starting from the beginning of your site’s injectable program. If that date is unknown, you can approximate, or enter all viral loads since January 2021 when iCAB/RPV was FDA approved.
+Clinics should add as many of these columns as are needed, following the same column naming format with a number instead of the X. 
+Example:
+hiv_vl_1_result
+hiv_vl_1_date
+Example:
+hiv_vl_15_result
+hiv_vl_15_date</t>
+  </si>
+  <si>
+    <t>If client not interested in iCAB/RPV after first iCAB/RPV counseling, primary reason for disinterest.
+The reasons for disinterest in LAI ART are displayed in a bar chart on the Dashboard. If there are multiple reasons for a given client, clinics have 2 options:
+1.	Provide 1 primary reason in the reason column, and list other reasons in the other column. Doing so will make the denominator of the bar chart the number of clients not interested in LAI ART. 
+2.	List all reasons separated by commas. Doing so will make the denominator of the bar chart the total number of reasons provided for LAI ART disinterest among clients counseled about LAI ART.
+Clinics should add as many of these columns (in this block of variables) as are needed, following the same column naming format with a number instead of the X
+Example:
+icab_rpv_counsel_4_date
+icab_rpv_counsel_4_outcome
+icab_rpv_disinterest_reason_4 
+icab_rpv_disinterest_reason_4_other
+If there are "other" reasons, include 20 here and include them in icab_rpv_disinterest_reason_1_other</t>
+  </si>
+  <si>
+    <t>If the client is not eligible for iCAB/RPV at first screening, this is the primary reason why they were determined not eligible. Note that we discourage clinics from categorizing clients as ineligible if they are clinically eligible but do not have a payor that will cover the cost of LAI ART. Coding these clients as eligible but not initiated on LAI ART allow clinics to accurately document the car gap caused by payor access issues. 
+The reasons for not being Eligible for LAI ART are displayed in a bar chart on the Dashboard. If there are multiple reasons for a given client, clinics have 2 options:
+1.	Provide 1 primary reason in the reason column, and list other reasons in the other column. Doing so will make the denominator of the bar chart the number of clients found ineligible for LAI ART. 
+2.	List all reasons separated by commas. Doing so will make the denominator of the bar chart the total number of reasons for not being eligible for LAI ART among clients screened for LAI ART.
+Clinics should add as many of these columns (in this block of variables) as are needed, following the same column naming format with a number instead of the X
+Example:
+icab_rpv_screen_3_date;
+icab_rpv_screen_3_outcome;
+icab_rpv_not_elig_3_reason;
+icab_rpv_not_elig_3_reason_other 
+If there are "other" reasons, include 20 here and include them in icab_rpv_not_elig_1_reason_other</t>
+  </si>
+  <si>
+    <t>The client was prescribed iCAB/RPV by a clinical provider.
+This should be the date the prescription was written and sent to insurance.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The date the client was prescribed iCAB/RPV.
+If this field is left blank but that patient received an injection, ‘prescribed’ will be set to 1=prescribed to ensure consistent denominators. This most often occurs if the patient transfers to your site while already on iCAB/RPV 
+</t>
+  </si>
+  <si>
+    <t>Date client ended oral ART for the first time to bridge therapy for planned missed iCAB/RPV injection.
+For clients on iCAB/RPV, a dose is considered late if it is &gt;38 days between doses for monthly or &gt;69 days between doses for bimonthly dosing. If oral bridging is used during the dates, then the dose is not considered late.
+Make sure that the oral bridging end date is the same date as the next injection date. This will ensure that the client’s injection is not marked as ‘late’
+Clinica should add as many of these columns as needed, following the same column naming format with a number instead of the X
+Example:
+icab_rpv_oral_bridge2; icab_rpv_bridge2_start_date; icab_rpv_bridge2_end_date</t>
+  </si>
+  <si>
+    <t>Date client ended oral ART for the second time to bridge therapy for planned missed iCAB/RPV injection.
+For clients on iCAB/RPV, a dose is considered late if it is &gt;38 days between doses for monthly or &gt;69 days between doses for bimonthly dosing. If oral bridging is used during the dates, then the dose is not considered late.
+Make sure that the oral bridging end date is the same date as the next injection date. This will ensure that the client’s injection is not marked as ‘late’
+Clinica should add as many of these columns as needed, following the same column naming format with a number instead of the X
+Example:
+icab_rpv_oral_bridge2; icab_rpv_bridge2_start_date; icab_rpv_bridge2_end_date</t>
+  </si>
+  <si>
+    <t>Client's most recent viral load result on or before first iCAB/RPV injection.
+If a client came from another clinic already on iCAB/RPV, the most recent viral load may be used. If these variables are left blank, the Dashboard will check the other viral load columns and use the most recent viral load within 3 months before the date of iCAB/RPV initiation to 2 weeks after iCAB/RPV initiation (icab_rpv_shot1_date). However, if these fields are provided, they take priority</t>
+  </si>
+  <si>
     <t xml:space="preserve">Expected interval of next injection, for client's first iCAB/RPV injection.
-Note: use 1 for loading doses or other monthly injections.
+‘1’ should be used for loading doses and for monthly (400mg cabotegravir &amp; 600mg rilpivirine) injections.
+‘2’ should be used for bimonthly (600mg cabotegravir &amp; 900mg rilpivirine) injections.
 </t>
   </si>
   <si>
-    <t>This is a flag to indicate that an injection is not late due to special circumstances. This is typically because the client is re-initiating iCAB/RPV at your site for any reason. This could be due to previous discontinuation or transfer from another clinic. If 1 is indicated, this injection will not be considered late.
+    <t>This is a flag to indicate that an injection is not late due to special circumstances. The late_exception variable should generally be set to ‘0’ or left blank for most loading doses and maintenance injections. ‘1’ should only be used if a client is restarting iCAB/RPV at your clinic following a break. The ‘1’ ensures that this injection will not be marked “late” not matter how long it has been since the previous injection. The two scenarios where this commonly occurs are (a) receiving a reloading (monthly) dose after previously discontinuing or (b) rejoining the clinic from another clinic where the client was also on iCAB/RPV. 
 Example:
 Shot 1: 0 (loading dose)
 Shot 2: 0 (maintenance dose)
@@ -1316,98 +1332,43 @@
 Shot 4: 0 (maintenance dose)</t>
   </si>
   <si>
-    <t>0 = maintenance injection or regular loading injection; 1 = do not mark late; Re-loading after discontinuation, or transfer from another clinic already on iCAB/RPV</t>
-  </si>
-  <si>
-    <t>icab_rpv_shot2_interval</t>
-  </si>
-  <si>
-    <t>icab_rpv_shot2_late_exception</t>
-  </si>
-  <si>
-    <t>Injection 2 intended interval</t>
-  </si>
-  <si>
-    <t>Injection 2 late exception</t>
+    <t>Date of client's first iCAB/RPV injection. This should be the date of their first loading dose, regardless of whether it occurred before or after the beginning of ALAI UP (3/1/23).
+Clinics should add as many of these columns as needed, following the same column naming format with a number instead of the X
+Example: 
+icab_rpv_shot12_date
+icab_rpv_shot12_interval
+icab_rpv_shot12_late_exception</t>
+  </si>
+  <si>
+    <t>Date of client's second iCAB/RPV injection.
+Clinics should add as many of these columns as needed, following the same column naming format with a number instead of the X
+Example: 
+icab_rpv_shot12_date
+icab_rpv_shot12_interval
+icab_rpv_shot12_late_exception</t>
   </si>
   <si>
     <t xml:space="preserve">Expected interval of next injection, for client's second iCAB/RPV injection.
-Note: use 1 for loading doses or other monthly injections.
+‘1’ should be used for loading doses and for monthly (400mg cabotegravir &amp; 600mg rilpivirine) injections.
+‘2’ should be used for bimonthly (600mg cabotegravir &amp; 900mg rilpivirine) injections.
 </t>
   </si>
   <si>
-    <t>icab_rpv_shot3_interval</t>
-  </si>
-  <si>
-    <t>icab_rpv_shot4_interval</t>
-  </si>
-  <si>
-    <t>icab_rpv_shot5_interval</t>
-  </si>
-  <si>
-    <t>icab_rpv_shot6_interval</t>
-  </si>
-  <si>
-    <t>icab_rpv_shot7_interval</t>
-  </si>
-  <si>
-    <t>icab_rpv_shot8_interval</t>
-  </si>
-  <si>
-    <t>icab_rpv_shot9_interval</t>
-  </si>
-  <si>
-    <t>icab_rpv_shot10_interval</t>
-  </si>
-  <si>
-    <t>icab_rpv_shot3_late_exception</t>
-  </si>
-  <si>
-    <t>icab_rpv_shot4_late_exception</t>
-  </si>
-  <si>
-    <t>icab_rpv_shot5_late_exception</t>
-  </si>
-  <si>
-    <t>icab_rpv_shot6_late_exception</t>
-  </si>
-  <si>
-    <t>icab_rpv_shot7_late_exception</t>
-  </si>
-  <si>
-    <t>icab_rpv_shot8_late_exception</t>
-  </si>
-  <si>
-    <t>icab_rpv_shot9_late_exception</t>
-  </si>
-  <si>
-    <t>icab_rpv_shot10_late_exception</t>
-  </si>
-  <si>
-    <t>birth_date</t>
-  </si>
-  <si>
-    <t>Birth date</t>
-  </si>
-  <si>
-    <t>The client's birth date. The value must be on or before all service dates for the client.</t>
-  </si>
-  <si>
-    <t>YYYY-MM-DD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">icab_rpv_not_elig_1_reason_other
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">icab_rpv_not_elig_2_reason_other
-</t>
-  </si>
-  <si>
-    <t>icab_rpv_not_elig_1_reason_other</t>
-  </si>
-  <si>
-    <t>icab_rpv_not_elig_2_reason_other</t>
+    <t>A binary measure of whether the client currently discontinued iCAB/RPV.
+icab_rpv_discontinued should only be ‘1’ if the client initiated iCAB/RPV but has since discontinued for any reason. This could include if the client has switched out of the clinic or back to oral ART; those reasons should be reflected in the reasons column. If a client stopped but restarted iCAB/RPV, make sure this value is ‘0’ (sustained), and the stop/restart should be indicated via icab_rpv_shotX_late_exception
+Note that if this field is left blank, but the client has not received a dose of iCAB/RPV in &gt;90 days since their most recent dose, then they are labeled as ‘discontinued’ by the Dashboard.</t>
+  </si>
+  <si>
+    <t>Date client decided to discontinue iCAB/RPV.
+If a client was lost to follow up or moved to another clinic, they are considered discontinued (at that clinic), even if they are still on CAB at the new clinic. Assign icab_rpv_discontinued to be 1, and use the last CAB date as the discontinued date if there is no other date
+If the date of discontinuation is unknown, the last iCAB/RPV injection date may be used (e.g. if the patient was lost to follow up).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The client-reported primary reason why they decided to discontinue using iCAB/RPV.
+Please record any additional information about discontinuation and/or restarts in icab_rpv_discontinued_reason_other (e.g., client discontinued on MM/DD/YYYY due to loss of insurance but restarted at site on MM/DD/YYYY).
+The reasons for discontinuing LAI ART are displayed in a bar chart on the Dashboard. If there are multiple reasons for a given client, clinics have 2 options:
+1.	Provide 1 primary reason in the reason column, and list other reasons in the other column. Doing so will make the denominator of the bar char the number of clients who have discontinued LAI ART. 
+2.	List the reasons separated by commas. Doing so will make the denominator of the bar chart the total number of reasons for discontinuing LAI ART among client who initiated LAI ART. </t>
   </si>
 </sst>
 </file>
@@ -1792,7 +1753,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="140">
+  <cellXfs count="143">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -2177,6 +2138,15 @@
     <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2556,7 +2526,7 @@
     </row>
     <row r="7" spans="2:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="B7" s="87" t="s">
-        <v>311</v>
+        <v>291</v>
       </c>
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.25">
@@ -2566,7 +2536,7 @@
     </row>
     <row r="9" spans="2:2" ht="41.4" x14ac:dyDescent="0.25">
       <c r="B9" s="87" t="s">
-        <v>323</v>
+        <v>297</v>
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.25">
@@ -2704,7 +2674,7 @@
         <v>26</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>328</v>
+        <v>302</v>
       </c>
       <c r="H1" s="3"/>
       <c r="I1" s="4"/>
@@ -2723,13 +2693,13 @@
         <v>29</v>
       </c>
       <c r="E2" s="108" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
       <c r="F2" s="108" t="s">
         <v>30</v>
       </c>
       <c r="G2" s="108" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="8"/>
@@ -2741,10 +2711,10 @@
         <v>31</v>
       </c>
       <c r="C3" s="109" t="s">
-        <v>330</v>
+        <v>304</v>
       </c>
       <c r="D3" s="110" t="s">
-        <v>331</v>
+        <v>305</v>
       </c>
       <c r="E3" s="110" t="s">
         <v>32</v>
@@ -2753,7 +2723,7 @@
         <v>30</v>
       </c>
       <c r="G3" s="110" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H3" s="12"/>
       <c r="I3" s="8"/>
@@ -2773,7 +2743,7 @@
         <v>36</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="H4" s="12"/>
       <c r="I4" s="8"/>
@@ -2793,7 +2763,7 @@
         <v>40</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="H5" s="10"/>
       <c r="I5" s="17"/>
@@ -2801,19 +2771,19 @@
     <row r="6" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="B6" s="128"/>
       <c r="C6" s="15" t="s">
-        <v>384</v>
+        <v>354</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>385</v>
+        <v>355</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>386</v>
+        <v>356</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>387</v>
+        <v>357</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>326</v>
+        <v>301</v>
       </c>
       <c r="H6" s="12"/>
     </row>
@@ -2833,7 +2803,7 @@
         <v>45</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H7" s="10"/>
       <c r="I7" s="18"/>
@@ -2855,7 +2825,7 @@
         <v>49</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H8" s="12"/>
     </row>
@@ -2874,7 +2844,7 @@
         <v>53</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H9" s="12"/>
     </row>
@@ -2893,7 +2863,7 @@
         <v>57</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H10" s="12"/>
     </row>
@@ -2912,7 +2882,7 @@
         <v>61</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H11" s="12"/>
     </row>
@@ -2931,7 +2901,7 @@
         <v>65</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H12" s="12"/>
     </row>
@@ -2950,7 +2920,7 @@
         <v>69</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H13" s="12"/>
     </row>
@@ -2969,7 +2939,7 @@
         <v>30</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H14" s="12"/>
     </row>
@@ -2988,7 +2958,7 @@
         <v>76</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="H15" s="20"/>
     </row>
@@ -3007,13 +2977,13 @@
         <v>80</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H16" s="12"/>
     </row>
-    <row r="17" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="124" t="s">
-        <v>341</v>
+        <v>314</v>
       </c>
       <c r="B17" s="130" t="s">
         <v>81</v>
@@ -3024,14 +2994,14 @@
       <c r="D17" s="112" t="s">
         <v>83</v>
       </c>
-      <c r="E17" s="112" t="s">
+      <c r="E17" s="130" t="s">
+        <v>362</v>
+      </c>
+      <c r="F17" s="112" t="s">
         <v>84</v>
       </c>
-      <c r="F17" s="112" t="s">
-        <v>85</v>
-      </c>
       <c r="G17" s="112" t="s">
-        <v>329</v>
+        <v>303</v>
       </c>
       <c r="H17" s="12"/>
     </row>
@@ -3039,19 +3009,17 @@
       <c r="A18" s="124"/>
       <c r="B18" s="131"/>
       <c r="C18" s="111" t="s">
+        <v>85</v>
+      </c>
+      <c r="D18" s="112" t="s">
         <v>86</v>
       </c>
-      <c r="D18" s="112" t="s">
-        <v>87</v>
-      </c>
-      <c r="E18" s="112" t="s">
-        <v>88</v>
-      </c>
+      <c r="E18" s="131"/>
       <c r="F18" s="112" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G18" s="112" t="s">
-        <v>329</v>
+        <v>303</v>
       </c>
       <c r="H18" s="12"/>
     </row>
@@ -3059,19 +3027,17 @@
       <c r="A19" s="124"/>
       <c r="B19" s="131"/>
       <c r="C19" s="111" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D19" s="112" t="s">
-        <v>90</v>
-      </c>
-      <c r="E19" s="112" t="s">
-        <v>91</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="E19" s="131"/>
       <c r="F19" s="112" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G19" s="112" t="s">
-        <v>329</v>
+        <v>303</v>
       </c>
       <c r="H19" s="12"/>
     </row>
@@ -3079,19 +3045,17 @@
       <c r="A20" s="124"/>
       <c r="B20" s="131"/>
       <c r="C20" s="111" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D20" s="112" t="s">
-        <v>93</v>
-      </c>
-      <c r="E20" s="112" t="s">
-        <v>94</v>
-      </c>
+        <v>90</v>
+      </c>
+      <c r="E20" s="131"/>
       <c r="F20" s="112" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G20" s="112" t="s">
-        <v>329</v>
+        <v>303</v>
       </c>
       <c r="H20" s="12"/>
     </row>
@@ -3099,19 +3063,17 @@
       <c r="A21" s="124"/>
       <c r="B21" s="131"/>
       <c r="C21" s="111" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="D21" s="112" t="s">
-        <v>96</v>
-      </c>
-      <c r="E21" s="112" t="s">
-        <v>97</v>
-      </c>
+        <v>92</v>
+      </c>
+      <c r="E21" s="131"/>
       <c r="F21" s="112" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G21" s="112" t="s">
-        <v>329</v>
+        <v>303</v>
       </c>
       <c r="H21" s="12"/>
     </row>
@@ -3119,19 +3081,17 @@
       <c r="A22" s="124"/>
       <c r="B22" s="131"/>
       <c r="C22" s="111" t="s">
-        <v>293</v>
+        <v>278</v>
       </c>
       <c r="D22" s="112" t="s">
-        <v>298</v>
-      </c>
-      <c r="E22" s="112" t="s">
+        <v>283</v>
+      </c>
+      <c r="E22" s="131"/>
+      <c r="F22" s="112" t="s">
+        <v>84</v>
+      </c>
+      <c r="G22" s="112" t="s">
         <v>303</v>
-      </c>
-      <c r="F22" s="112" t="s">
-        <v>85</v>
-      </c>
-      <c r="G22" s="112" t="s">
-        <v>329</v>
       </c>
       <c r="H22" s="12"/>
     </row>
@@ -3139,19 +3099,17 @@
       <c r="A23" s="124"/>
       <c r="B23" s="131"/>
       <c r="C23" s="111" t="s">
-        <v>294</v>
+        <v>279</v>
       </c>
       <c r="D23" s="112" t="s">
-        <v>299</v>
-      </c>
-      <c r="E23" s="112" t="s">
-        <v>304</v>
-      </c>
+        <v>284</v>
+      </c>
+      <c r="E23" s="131"/>
       <c r="F23" s="112" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G23" s="112" t="s">
-        <v>329</v>
+        <v>303</v>
       </c>
       <c r="H23" s="12"/>
     </row>
@@ -3159,19 +3117,17 @@
       <c r="A24" s="124"/>
       <c r="B24" s="131"/>
       <c r="C24" s="111" t="s">
-        <v>295</v>
+        <v>280</v>
       </c>
       <c r="D24" s="112" t="s">
-        <v>300</v>
-      </c>
-      <c r="E24" s="112" t="s">
-        <v>305</v>
-      </c>
+        <v>285</v>
+      </c>
+      <c r="E24" s="131"/>
       <c r="F24" s="112" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G24" s="112" t="s">
-        <v>329</v>
+        <v>303</v>
       </c>
       <c r="H24" s="12"/>
     </row>
@@ -3179,19 +3135,17 @@
       <c r="A25" s="124"/>
       <c r="B25" s="131"/>
       <c r="C25" s="111" t="s">
-        <v>296</v>
+        <v>281</v>
       </c>
       <c r="D25" s="112" t="s">
-        <v>301</v>
-      </c>
-      <c r="E25" s="112" t="s">
-        <v>306</v>
-      </c>
+        <v>286</v>
+      </c>
+      <c r="E25" s="131"/>
       <c r="F25" s="112" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G25" s="112" t="s">
-        <v>329</v>
+        <v>303</v>
       </c>
       <c r="H25" s="12"/>
     </row>
@@ -3199,394 +3153,388 @@
       <c r="A26" s="124"/>
       <c r="B26" s="132"/>
       <c r="C26" s="111" t="s">
-        <v>297</v>
+        <v>282</v>
       </c>
       <c r="D26" s="112" t="s">
-        <v>302</v>
-      </c>
-      <c r="E26" s="112" t="s">
-        <v>307</v>
-      </c>
+        <v>287</v>
+      </c>
+      <c r="E26" s="132"/>
       <c r="F26" s="112" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G26" s="112" t="s">
-        <v>329</v>
+        <v>303</v>
       </c>
       <c r="H26" s="12"/>
     </row>
     <row r="27" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="133" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C27" s="113" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="D27" s="22" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="E27" s="22" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="F27" s="22" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="G27" s="22" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="H27" s="12"/>
     </row>
     <row r="28" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="134"/>
       <c r="C28" s="113" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="D28" s="22" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="E28" s="22" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="F28" s="22" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G28" s="22" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="H28" s="12"/>
     </row>
     <row r="29" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="B29" s="135"/>
       <c r="C29" s="113" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="D29" s="22" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="F29" s="22" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="G29" s="22" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="H29" s="12"/>
     </row>
     <row r="30" spans="1:8" ht="52.8" x14ac:dyDescent="0.3">
       <c r="B30" s="136" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="C30" s="114" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="E30" s="23" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="F30" s="23" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="G30" s="23" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H30" s="24"/>
     </row>
     <row r="31" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="137"/>
       <c r="C31" s="114" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="E31" s="23" t="s">
-        <v>314</v>
+        <v>294</v>
       </c>
       <c r="F31" s="23" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="G31" s="23" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="H31" s="24"/>
     </row>
     <row r="32" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="137"/>
       <c r="C32" s="114" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="D32" s="23" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="F32" s="23" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="H32" s="12"/>
     </row>
     <row r="33" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
       <c r="B33" s="137"/>
       <c r="C33" s="114" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="E33" s="23" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="F33" s="23" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="H33" s="10"/>
     </row>
     <row r="34" spans="1:11" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="137"/>
       <c r="C34" s="114" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="D34" s="23" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E34" s="23" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="F34" s="23" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="G34" s="23" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="H34" s="12"/>
     </row>
     <row r="35" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
       <c r="B35" s="137"/>
       <c r="C35" s="114" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="D35" s="23" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="E35" s="23" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="F35" s="23" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="G35" s="23" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="H35" s="24"/>
     </row>
     <row r="36" spans="1:11" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="137"/>
       <c r="C36" s="114" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="D36" s="23" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="E36" s="23" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="F36" s="23" t="s">
         <v>30</v>
       </c>
       <c r="G36" s="23" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="H36" s="12"/>
     </row>
     <row r="37" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
       <c r="B37" s="137"/>
       <c r="C37" s="114" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="D37" s="23" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="E37" s="23" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F37" s="23" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="G37" s="23" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="H37" s="12"/>
     </row>
-    <row r="38" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="95"/>
       <c r="B38" s="137"/>
       <c r="C38" s="114" t="s">
-        <v>288</v>
+        <v>274</v>
       </c>
       <c r="D38" s="115" t="s">
-        <v>289</v>
-      </c>
-      <c r="E38" s="115" t="s">
-        <v>292</v>
+        <v>275</v>
+      </c>
+      <c r="E38" s="140" t="s">
+        <v>363</v>
       </c>
       <c r="F38" s="115"/>
       <c r="G38" s="115" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="H38" s="12"/>
     </row>
-    <row r="39" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="95"/>
       <c r="B39" s="137"/>
       <c r="C39" s="116" t="s">
-        <v>290</v>
+        <v>276</v>
       </c>
       <c r="D39" s="115" t="s">
-        <v>289</v>
-      </c>
-      <c r="E39" s="115" t="s">
-        <v>292</v>
-      </c>
+        <v>275</v>
+      </c>
+      <c r="E39" s="141"/>
       <c r="F39" s="115"/>
       <c r="G39" s="115" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="H39" s="12"/>
     </row>
-    <row r="40" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="95"/>
       <c r="B40" s="138"/>
       <c r="C40" s="114" t="s">
-        <v>291</v>
+        <v>277</v>
       </c>
       <c r="D40" s="115" t="s">
-        <v>289</v>
-      </c>
-      <c r="E40" s="115" t="s">
-        <v>292</v>
-      </c>
+        <v>275</v>
+      </c>
+      <c r="E40" s="142"/>
       <c r="F40" s="115"/>
       <c r="G40" s="115" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="H40" s="12"/>
     </row>
     <row r="41" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="B41" s="125" t="s">
-        <v>336</v>
+        <v>309</v>
       </c>
       <c r="C41" s="26" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="D41" s="117" t="s">
-        <v>281</v>
+        <v>269</v>
       </c>
       <c r="E41" s="117" t="s">
-        <v>282</v>
+        <v>270</v>
       </c>
       <c r="F41" s="117" t="s">
         <v>41</v>
       </c>
       <c r="G41" s="117" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="H41" s="24"/>
     </row>
     <row r="42" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="B42" s="126"/>
       <c r="C42" s="26" t="s">
-        <v>279</v>
+        <v>267</v>
       </c>
       <c r="D42" s="117" t="s">
-        <v>280</v>
+        <v>268</v>
       </c>
       <c r="E42" s="117" t="s">
-        <v>283</v>
+        <v>271</v>
       </c>
       <c r="F42" s="117" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G42" s="117" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="H42" s="24"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B43" s="139"/>
       <c r="C43" s="26" t="s">
-        <v>308</v>
+        <v>288</v>
       </c>
       <c r="D43" s="117" t="s">
-        <v>309</v>
+        <v>289</v>
       </c>
       <c r="E43" s="117" t="s">
-        <v>310</v>
+        <v>290</v>
       </c>
       <c r="F43" s="117" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G43" s="117" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H43" s="24" t="s">
-        <v>324</v>
+        <v>298</v>
       </c>
     </row>
     <row r="44" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A44" s="124" t="s">
-        <v>348</v>
+        <v>321</v>
       </c>
       <c r="B44" s="125" t="s">
-        <v>342</v>
+        <v>315</v>
       </c>
       <c r="C44" s="117" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="D44" s="117" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="E44" s="117" t="s">
-        <v>284</v>
+        <v>272</v>
       </c>
       <c r="F44" s="117" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="G44" s="117" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H44" s="30"/>
       <c r="I44" s="28"/>
       <c r="J44" s="28"/>
       <c r="K44" s="28"/>
     </row>
-    <row r="45" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" s="29" customFormat="1" ht="224.4" x14ac:dyDescent="0.3">
       <c r="A45" s="124"/>
       <c r="B45" s="126"/>
       <c r="C45" s="117" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="D45" s="117" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="E45" s="117" t="s">
-        <v>285</v>
+        <v>364</v>
       </c>
       <c r="F45" s="26" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G45" s="26" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H45" s="30"/>
       <c r="I45" s="28"/>
@@ -3596,45 +3544,45 @@
     <row r="46" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A46" s="124"/>
       <c r="B46" s="125" t="s">
-        <v>343</v>
+        <v>316</v>
       </c>
       <c r="C46" s="117" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="D46" s="117" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="E46" s="117" t="s">
-        <v>286</v>
+        <v>273</v>
       </c>
       <c r="F46" s="117" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="G46" s="117" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H46" s="30"/>
       <c r="I46" s="28"/>
       <c r="J46" s="28"/>
       <c r="K46" s="28"/>
     </row>
-    <row r="47" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" s="29" customFormat="1" ht="224.4" x14ac:dyDescent="0.3">
       <c r="A47" s="124"/>
       <c r="B47" s="126"/>
       <c r="C47" s="117" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="D47" s="117" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E47" s="117" t="s">
-        <v>287</v>
+        <v>364</v>
       </c>
       <c r="F47" s="26" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G47" s="26" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H47" s="30"/>
       <c r="I47" s="28"/>
@@ -3644,22 +3592,22 @@
     <row r="48" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A48"/>
       <c r="B48" s="121" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="C48" s="36" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="D48" s="37" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="E48" s="37" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="F48" s="36" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="G48" s="36" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="H48" s="31"/>
       <c r="I48" s="32"/>
@@ -3670,19 +3618,19 @@
       <c r="A49"/>
       <c r="B49" s="123"/>
       <c r="C49" s="36" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="D49" s="37" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="E49" s="37" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="F49" s="36" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="G49" s="36" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="H49" s="31"/>
       <c r="I49" s="32"/>
@@ -3691,25 +3639,25 @@
     </row>
     <row r="50" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A50" s="124" t="s">
-        <v>349</v>
+        <v>322</v>
       </c>
       <c r="B50" s="121" t="s">
-        <v>344</v>
+        <v>317</v>
       </c>
       <c r="C50" s="36" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D50" s="37" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="E50" s="37" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="F50" s="36" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G50" s="36" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="H50" s="31"/>
       <c r="I50" s="32"/>
@@ -3720,42 +3668,42 @@
       <c r="A51" s="124"/>
       <c r="B51" s="122"/>
       <c r="C51" s="36" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="D51" s="37" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="E51" s="37" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="F51" s="36" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="G51" s="36" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="H51" s="31"/>
       <c r="I51" s="32"/>
       <c r="J51" s="32"/>
       <c r="K51" s="32"/>
     </row>
-    <row r="52" spans="1:11" s="33" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" s="33" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.3">
       <c r="A52" s="124"/>
       <c r="B52" s="122"/>
       <c r="C52" s="36" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="D52" s="37" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="E52" s="37" t="s">
-        <v>315</v>
+        <v>365</v>
       </c>
       <c r="F52" s="36" t="s">
-        <v>332</v>
+        <v>306</v>
       </c>
       <c r="G52" s="36" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="H52" s="31"/>
       <c r="I52" s="32"/>
@@ -3766,19 +3714,19 @@
       <c r="A53" s="124"/>
       <c r="B53" s="123"/>
       <c r="C53" s="36" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="D53" s="37" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="E53" s="37" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="F53" s="37" t="s">
         <v>30</v>
       </c>
       <c r="G53" s="36" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="H53" s="31"/>
       <c r="I53" s="32"/>
@@ -3787,25 +3735,25 @@
     </row>
     <row r="54" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A54" s="124" t="s">
-        <v>350</v>
+        <v>323</v>
       </c>
       <c r="B54" s="121" t="s">
-        <v>347</v>
+        <v>320</v>
       </c>
       <c r="C54" s="36" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="D54" s="37" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="E54" s="37" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="F54" s="36" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G54" s="36" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="H54" s="31"/>
       <c r="I54" s="32"/>
@@ -3816,42 +3764,42 @@
       <c r="A55" s="124"/>
       <c r="B55" s="122"/>
       <c r="C55" s="36" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="D55" s="37" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="E55" s="37" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="F55" s="36" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="G55" s="36" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="H55" s="31"/>
       <c r="I55" s="32"/>
       <c r="J55" s="32"/>
       <c r="K55" s="32"/>
     </row>
-    <row r="56" spans="1:11" s="33" customFormat="1" ht="105.6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" s="33" customFormat="1" ht="343.2" x14ac:dyDescent="0.3">
       <c r="A56" s="124"/>
       <c r="B56" s="122"/>
       <c r="C56" s="36" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="D56" s="37" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="E56" s="37" t="s">
-        <v>316</v>
+        <v>366</v>
       </c>
       <c r="F56" s="37" t="s">
-        <v>325</v>
+        <v>299</v>
       </c>
       <c r="G56" s="36" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="H56" s="31"/>
       <c r="I56" s="32"/>
@@ -3862,19 +3810,19 @@
       <c r="A57" s="124"/>
       <c r="B57" s="123"/>
       <c r="C57" s="36" t="s">
-        <v>388</v>
+        <v>358</v>
       </c>
       <c r="D57" s="37" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="E57" s="37" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="F57" s="36" t="s">
         <v>30</v>
       </c>
       <c r="G57" s="36" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="H57" s="31"/>
       <c r="I57" s="32"/>
@@ -3883,25 +3831,25 @@
     </row>
     <row r="58" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A58" s="124" t="s">
-        <v>349</v>
+        <v>322</v>
       </c>
       <c r="B58" s="121" t="s">
-        <v>346</v>
+        <v>319</v>
       </c>
       <c r="C58" s="36" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="D58" s="37" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="E58" s="37" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="F58" s="36" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G58" s="36" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="H58" s="31"/>
       <c r="I58" s="32"/>
@@ -3912,42 +3860,42 @@
       <c r="A59" s="124"/>
       <c r="B59" s="122"/>
       <c r="C59" s="36" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="D59" s="37" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="E59" s="37" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="F59" s="36" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="G59" s="36" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="H59" s="31"/>
       <c r="I59" s="32"/>
       <c r="J59" s="32"/>
       <c r="K59" s="32"/>
     </row>
-    <row r="60" spans="1:11" s="33" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" s="33" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.3">
       <c r="A60" s="124"/>
       <c r="B60" s="122"/>
       <c r="C60" s="36" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="D60" s="37" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="E60" s="37" t="s">
-        <v>317</v>
+        <v>365</v>
       </c>
       <c r="F60" s="36" t="s">
-        <v>332</v>
+        <v>306</v>
       </c>
       <c r="G60" s="36" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="H60" s="31"/>
       <c r="I60" s="32"/>
@@ -3958,19 +3906,19 @@
       <c r="A61" s="124"/>
       <c r="B61" s="123"/>
       <c r="C61" s="36" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="D61" s="37" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="E61" s="37" t="s">
-        <v>318</v>
+        <v>295</v>
       </c>
       <c r="F61" s="37" t="s">
         <v>30</v>
       </c>
       <c r="G61" s="36" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="H61" s="31"/>
       <c r="I61" s="32"/>
@@ -3979,25 +3927,25 @@
     </row>
     <row r="62" spans="1:11" s="33" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="124" t="s">
-        <v>350</v>
+        <v>323</v>
       </c>
       <c r="B62" s="121" t="s">
-        <v>345</v>
+        <v>318</v>
       </c>
       <c r="C62" s="36" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="D62" s="37" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="E62" s="37" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="F62" s="36" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G62" s="36" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="H62" s="31"/>
       <c r="I62" s="32"/>
@@ -4008,42 +3956,42 @@
       <c r="A63" s="124"/>
       <c r="B63" s="122"/>
       <c r="C63" s="36" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="D63" s="37" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="E63" s="37" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="F63" s="36" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="G63" s="36" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="H63" s="31"/>
       <c r="I63" s="32"/>
       <c r="J63" s="32"/>
       <c r="K63" s="32"/>
     </row>
-    <row r="64" spans="1:11" ht="105.6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:11" ht="343.2" x14ac:dyDescent="0.3">
       <c r="A64" s="124"/>
       <c r="B64" s="122"/>
       <c r="C64" s="36" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="D64" s="37" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="E64" s="37" t="s">
-        <v>319</v>
+        <v>366</v>
       </c>
       <c r="F64" s="37" t="s">
-        <v>313</v>
+        <v>293</v>
       </c>
       <c r="G64" s="36" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="H64" s="12"/>
     </row>
@@ -4051,83 +3999,83 @@
       <c r="A65" s="124"/>
       <c r="B65" s="123"/>
       <c r="C65" s="36" t="s">
-        <v>389</v>
+        <v>359</v>
       </c>
       <c r="D65" s="37" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="E65" s="37" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="F65" s="36" t="s">
         <v>30</v>
       </c>
       <c r="G65" s="36" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="H65" s="12"/>
     </row>
-    <row r="66" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
       <c r="B66" s="121" t="s">
-        <v>337</v>
+        <v>310</v>
       </c>
       <c r="C66" s="36" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="D66" s="37" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="E66" s="37" t="s">
-        <v>221</v>
+        <v>367</v>
       </c>
       <c r="F66" s="36" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="G66" s="36" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H66" s="10"/>
     </row>
-    <row r="67" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:11" ht="93" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B67" s="123"/>
       <c r="C67" s="36" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="D67" s="37" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="E67" s="37" t="s">
-        <v>225</v>
+        <v>368</v>
       </c>
       <c r="F67" s="36" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G67" s="36" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H67" s="12"/>
     </row>
     <row r="68" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A68" s="124" t="s">
-        <v>351</v>
+        <v>324</v>
       </c>
       <c r="B68" s="121" t="s">
-        <v>338</v>
+        <v>311</v>
       </c>
       <c r="C68" s="36" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="D68" s="37" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="E68" s="37" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="F68" s="36" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="G68" s="36" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H68" s="30"/>
       <c r="I68" s="28"/>
@@ -4138,42 +4086,42 @@
       <c r="A69" s="124"/>
       <c r="B69" s="122"/>
       <c r="C69" s="36" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="D69" s="37" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="E69" s="37" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="F69" s="36" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G69" s="36" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H69" s="30"/>
       <c r="I69" s="28"/>
       <c r="J69" s="28"/>
       <c r="K69" s="28"/>
     </row>
-    <row r="70" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:11" s="29" customFormat="1" ht="184.8" x14ac:dyDescent="0.3">
       <c r="A70" s="124"/>
       <c r="B70" s="123"/>
       <c r="C70" s="36" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="D70" s="37" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="E70" s="37" t="s">
-        <v>235</v>
+        <v>369</v>
       </c>
       <c r="F70" s="36" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G70" s="36" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H70" s="30"/>
       <c r="I70" s="28"/>
@@ -4183,22 +4131,22 @@
     <row r="71" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A71" s="124"/>
       <c r="B71" s="121" t="s">
-        <v>338</v>
+        <v>311</v>
       </c>
       <c r="C71" s="36" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="D71" s="37" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="E71" s="37" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="F71" s="36" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="G71" s="36" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H71" s="30"/>
       <c r="I71" s="28"/>
@@ -4209,42 +4157,42 @@
       <c r="A72" s="124"/>
       <c r="B72" s="122"/>
       <c r="C72" s="36" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="D72" s="37" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="E72" s="37" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="F72" s="36" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G72" s="36" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H72" s="30"/>
       <c r="I72" s="28"/>
       <c r="J72" s="28"/>
       <c r="K72" s="28"/>
     </row>
-    <row r="73" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:11" s="29" customFormat="1" ht="184.8" x14ac:dyDescent="0.3">
       <c r="A73" s="124"/>
       <c r="B73" s="123"/>
       <c r="C73" s="36" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="D73" s="37" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="E73" s="37" t="s">
-        <v>244</v>
+        <v>370</v>
       </c>
       <c r="F73" s="36" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G73" s="36" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H73" s="30"/>
       <c r="I73" s="28"/>
@@ -4254,115 +4202,115 @@
     <row r="74" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A74"/>
       <c r="B74" s="121" t="s">
-        <v>339</v>
+        <v>312</v>
       </c>
       <c r="C74" s="118" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="D74" s="118" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
       <c r="E74" s="118" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="F74" s="119" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G74" s="119" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H74" s="30"/>
       <c r="I74" s="28"/>
       <c r="J74" s="28"/>
       <c r="K74" s="28"/>
     </row>
-    <row r="75" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:11" s="33" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A75"/>
       <c r="B75" s="123"/>
       <c r="C75" s="118" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="D75" s="118" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
       <c r="E75" s="118" t="s">
-        <v>250</v>
+        <v>371</v>
       </c>
       <c r="F75" s="118" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="G75" s="118" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H75" s="31"/>
       <c r="I75" s="32"/>
       <c r="J75" s="32"/>
       <c r="K75" s="32"/>
     </row>
-    <row r="76" spans="1:11" s="33" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:11" s="33" customFormat="1" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="124" t="s">
-        <v>352</v>
+        <v>325</v>
       </c>
       <c r="B76" s="121" t="s">
-        <v>353</v>
+        <v>326</v>
       </c>
       <c r="C76" s="36" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="D76" s="37" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="E76" s="118" t="s">
-        <v>253</v>
+        <v>374</v>
       </c>
       <c r="F76" s="36" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G76" s="36" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H76" s="31"/>
       <c r="I76" s="32"/>
       <c r="J76" s="32"/>
       <c r="K76" s="32"/>
     </row>
-    <row r="77" spans="1:11" s="33" customFormat="1" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:11" s="33" customFormat="1" ht="78" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="124"/>
       <c r="B77" s="122"/>
       <c r="C77" s="36" t="s">
-        <v>356</v>
+        <v>329</v>
       </c>
       <c r="D77" s="37" t="s">
-        <v>357</v>
+        <v>330</v>
       </c>
       <c r="E77" s="37" t="s">
-        <v>360</v>
+        <v>372</v>
       </c>
       <c r="F77" s="36" t="s">
-        <v>355</v>
+        <v>328</v>
       </c>
       <c r="G77" s="36" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H77" s="31"/>
       <c r="I77" s="32"/>
       <c r="J77" s="32"/>
       <c r="K77" s="32"/>
     </row>
-    <row r="78" spans="1:11" s="33" customFormat="1" ht="187.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:11" s="33" customFormat="1" ht="212.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="124"/>
       <c r="B78" s="123"/>
       <c r="C78" s="36" t="s">
-        <v>358</v>
+        <v>331</v>
       </c>
       <c r="D78" s="37" t="s">
-        <v>359</v>
+        <v>332</v>
       </c>
       <c r="E78" s="37" t="s">
-        <v>361</v>
+        <v>373</v>
       </c>
       <c r="F78" s="36" t="s">
-        <v>362</v>
+        <v>333</v>
       </c>
       <c r="G78" s="36"/>
       <c r="H78" s="31"/>
@@ -4370,70 +4318,70 @@
       <c r="J78" s="32"/>
       <c r="K78" s="32"/>
     </row>
-    <row r="79" spans="1:11" s="33" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:11" s="33" customFormat="1" ht="117" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="124" t="s">
-        <v>352</v>
+        <v>325</v>
       </c>
       <c r="B79" s="121" t="s">
-        <v>354</v>
+        <v>327</v>
       </c>
       <c r="C79" s="36" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="D79" s="37" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
       <c r="E79" s="118" t="s">
-        <v>256</v>
+        <v>375</v>
       </c>
       <c r="F79" s="36" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G79" s="36" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H79" s="31"/>
       <c r="I79" s="32"/>
       <c r="J79" s="32"/>
       <c r="K79" s="32"/>
     </row>
-    <row r="80" spans="1:11" s="33" customFormat="1" ht="198" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:11" s="33" customFormat="1" ht="83.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="124"/>
       <c r="B80" s="122"/>
       <c r="C80" s="36" t="s">
-        <v>363</v>
+        <v>334</v>
       </c>
       <c r="D80" s="37" t="s">
-        <v>365</v>
+        <v>336</v>
       </c>
       <c r="E80" s="37" t="s">
-        <v>367</v>
+        <v>376</v>
       </c>
       <c r="F80" s="36" t="s">
-        <v>355</v>
+        <v>328</v>
       </c>
       <c r="G80" s="36" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H80" s="31"/>
       <c r="I80" s="32"/>
       <c r="J80" s="32"/>
       <c r="K80" s="32"/>
     </row>
-    <row r="81" spans="1:11" s="33" customFormat="1" ht="189" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:11" s="33" customFormat="1" ht="199.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="124"/>
       <c r="B81" s="123"/>
       <c r="C81" s="36" t="s">
-        <v>364</v>
+        <v>335</v>
       </c>
       <c r="D81" s="37" t="s">
-        <v>366</v>
+        <v>337</v>
       </c>
       <c r="E81" s="37" t="s">
-        <v>361</v>
+        <v>373</v>
       </c>
       <c r="F81" s="36" t="s">
-        <v>362</v>
+        <v>333</v>
       </c>
       <c r="G81" s="36"/>
       <c r="H81" s="31"/>
@@ -4441,78 +4389,78 @@
       <c r="J81" s="32"/>
       <c r="K81" s="32"/>
     </row>
-    <row r="82" spans="1:11" ht="66" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:11" ht="158.4" x14ac:dyDescent="0.3">
       <c r="B82" s="121" t="s">
-        <v>340</v>
+        <v>313</v>
       </c>
       <c r="C82" s="36" t="s">
-        <v>265</v>
+        <v>253</v>
       </c>
       <c r="D82" s="37" t="s">
-        <v>266</v>
+        <v>254</v>
       </c>
       <c r="E82" s="118" t="s">
-        <v>335</v>
+        <v>377</v>
       </c>
       <c r="F82" s="36" t="s">
-        <v>334</v>
+        <v>308</v>
       </c>
       <c r="G82" s="36" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" ht="79.2" x14ac:dyDescent="0.3">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" ht="118.8" x14ac:dyDescent="0.3">
       <c r="B83" s="122"/>
       <c r="C83" s="36" t="s">
-        <v>267</v>
+        <v>255</v>
       </c>
       <c r="D83" s="37" t="s">
-        <v>268</v>
+        <v>256</v>
       </c>
       <c r="E83" s="118" t="s">
-        <v>320</v>
+        <v>378</v>
       </c>
       <c r="F83" s="36" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G83" s="36" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="84" spans="1:11" ht="105.6" x14ac:dyDescent="0.3">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" ht="198" x14ac:dyDescent="0.3">
       <c r="B84" s="122"/>
       <c r="C84" s="36" t="s">
-        <v>269</v>
+        <v>257</v>
       </c>
       <c r="D84" s="37" t="s">
-        <v>270</v>
+        <v>258</v>
       </c>
       <c r="E84" s="118" t="s">
-        <v>322</v>
+        <v>379</v>
       </c>
       <c r="F84" s="36" t="s">
-        <v>333</v>
+        <v>307</v>
       </c>
       <c r="G84" s="36" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
     </row>
     <row r="85" spans="1:11" ht="66" x14ac:dyDescent="0.3">
       <c r="B85" s="123"/>
       <c r="C85" s="36" t="s">
-        <v>271</v>
+        <v>259</v>
       </c>
       <c r="D85" s="37" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
       <c r="E85" s="118" t="s">
-        <v>321</v>
+        <v>296</v>
       </c>
       <c r="F85" s="36" t="s">
         <v>30</v>
       </c>
       <c r="G85" s="36" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.3">
@@ -4548,7 +4496,9 @@
       <c r="G89" s="39"/>
     </row>
   </sheetData>
-  <mergeCells count="28">
+  <mergeCells count="30">
+    <mergeCell ref="E17:E26"/>
+    <mergeCell ref="E38:E40"/>
     <mergeCell ref="B79:B81"/>
     <mergeCell ref="B41:B43"/>
     <mergeCell ref="B48:B49"/>
@@ -4605,7 +4555,7 @@
         <v>28</v>
       </c>
       <c r="B1" s="101" t="s">
-        <v>330</v>
+        <v>304</v>
       </c>
       <c r="C1" s="102" t="s">
         <v>33</v>
@@ -4614,7 +4564,7 @@
         <v>37</v>
       </c>
       <c r="E1" s="102" t="s">
-        <v>384</v>
+        <v>354</v>
       </c>
       <c r="F1" s="102" t="s">
         <v>42</v>
@@ -4650,334 +4600,334 @@
         <v>82</v>
       </c>
       <c r="Q1" s="103" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="R1" s="103" t="s">
+        <v>87</v>
+      </c>
+      <c r="S1" s="103" t="s">
         <v>89</v>
       </c>
-      <c r="S1" s="103" t="s">
-        <v>92</v>
-      </c>
       <c r="T1" s="103" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="U1" s="103" t="s">
-        <v>293</v>
+        <v>278</v>
       </c>
       <c r="V1" s="103" t="s">
-        <v>294</v>
+        <v>279</v>
       </c>
       <c r="W1" s="103" t="s">
-        <v>295</v>
+        <v>280</v>
       </c>
       <c r="X1" s="103" t="s">
-        <v>296</v>
+        <v>281</v>
       </c>
       <c r="Y1" s="103" t="s">
-        <v>297</v>
+        <v>282</v>
       </c>
       <c r="Z1" s="104" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="AA1" s="104" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="AB1" s="104" t="s">
+        <v>102</v>
+      </c>
+      <c r="AC1" s="104" t="s">
         <v>107</v>
       </c>
-      <c r="AC1" s="104" t="s">
-        <v>112</v>
-      </c>
       <c r="AD1" s="104" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="AE1" s="104" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="AF1" s="104" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="AG1" s="104" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="AH1" s="104" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="AI1" s="104" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="AJ1" s="104" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="AK1" s="104" t="s">
+        <v>274</v>
+      </c>
+      <c r="AL1" s="104" t="s">
+        <v>276</v>
+      </c>
+      <c r="AM1" s="104" t="s">
+        <v>277</v>
+      </c>
+      <c r="AN1" s="105" t="s">
+        <v>266</v>
+      </c>
+      <c r="AO1" s="105" t="s">
+        <v>267</v>
+      </c>
+      <c r="AP1" s="44" t="s">
         <v>288</v>
       </c>
-      <c r="AL1" s="104" t="s">
-        <v>290</v>
-      </c>
-      <c r="AM1" s="104" t="s">
-        <v>291</v>
-      </c>
-      <c r="AN1" s="105" t="s">
-        <v>278</v>
-      </c>
-      <c r="AO1" s="105" t="s">
-        <v>279</v>
-      </c>
-      <c r="AP1" s="44" t="s">
-        <v>308</v>
-      </c>
       <c r="AQ1" s="44" t="s">
+        <v>139</v>
+      </c>
+      <c r="AR1" s="44" t="s">
+        <v>141</v>
+      </c>
+      <c r="AS1" s="44" t="s">
+        <v>142</v>
+      </c>
+      <c r="AT1" s="44" t="s">
         <v>144</v>
       </c>
-      <c r="AR1" s="44" t="s">
+      <c r="AU1" s="44" t="s">
         <v>146</v>
       </c>
-      <c r="AS1" s="44" t="s">
-        <v>147</v>
-      </c>
-      <c r="AT1" s="44" t="s">
-        <v>149</v>
-      </c>
-      <c r="AU1" s="44" t="s">
+      <c r="AV1" s="44" t="s">
+        <v>148</v>
+      </c>
+      <c r="AW1" s="44" t="s">
+        <v>150</v>
+      </c>
+      <c r="AX1" s="44" t="s">
         <v>151</v>
       </c>
-      <c r="AV1" s="44" t="s">
+      <c r="AY1" s="44" t="s">
+        <v>152</v>
+      </c>
+      <c r="AZ1" s="44" t="s">
         <v>153</v>
       </c>
-      <c r="AW1" s="44" t="s">
+      <c r="BA1" s="44" t="s">
+        <v>154</v>
+      </c>
+      <c r="BB1" s="44" t="s">
         <v>155</v>
       </c>
-      <c r="AX1" s="44" t="s">
+      <c r="BC1" s="44" t="s">
         <v>156</v>
       </c>
-      <c r="AY1" s="44" t="s">
+      <c r="BD1" s="44" t="s">
         <v>157</v>
       </c>
-      <c r="AZ1" s="44" t="s">
+      <c r="BE1" s="44" t="s">
         <v>158</v>
       </c>
-      <c r="BA1" s="44" t="s">
+      <c r="BF1" s="44" t="s">
         <v>159</v>
       </c>
-      <c r="BB1" s="44" t="s">
+      <c r="BG1" s="44" t="s">
         <v>160</v>
       </c>
-      <c r="BC1" s="44" t="s">
+      <c r="BH1" s="44" t="s">
         <v>161</v>
       </c>
-      <c r="BD1" s="44" t="s">
+      <c r="BI1" s="44" t="s">
         <v>162</v>
       </c>
-      <c r="BE1" s="44" t="s">
+      <c r="BJ1" s="44" t="s">
         <v>163</v>
       </c>
-      <c r="BF1" s="44" t="s">
+      <c r="BK1" s="44" t="s">
         <v>164</v>
       </c>
-      <c r="BG1" s="44" t="s">
+      <c r="BL1" s="44" t="s">
         <v>165</v>
       </c>
-      <c r="BH1" s="44" t="s">
-        <v>166</v>
-      </c>
-      <c r="BI1" s="44" t="s">
+      <c r="BM1" s="45" t="s">
         <v>167</v>
       </c>
-      <c r="BJ1" s="44" t="s">
-        <v>168</v>
-      </c>
-      <c r="BK1" s="44" t="s">
-        <v>169</v>
-      </c>
-      <c r="BL1" s="44" t="s">
+      <c r="BN1" s="45" t="s">
         <v>170</v>
       </c>
-      <c r="BM1" s="45" t="s">
-        <v>172</v>
-      </c>
-      <c r="BN1" s="45" t="s">
-        <v>175</v>
-      </c>
       <c r="BO1" s="45" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="BP1" s="45" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="BQ1" s="45" t="s">
+        <v>181</v>
+      </c>
+      <c r="BR1" s="45" t="s">
+        <v>183</v>
+      </c>
+      <c r="BS1" s="45" t="s">
         <v>186</v>
       </c>
-      <c r="BR1" s="45" t="s">
-        <v>188</v>
-      </c>
-      <c r="BS1" s="45" t="s">
-        <v>191</v>
-      </c>
       <c r="BT1" s="45" t="s">
-        <v>273</v>
+        <v>261</v>
       </c>
       <c r="BU1" s="45" t="s">
-        <v>274</v>
+        <v>262</v>
       </c>
       <c r="BV1" s="45" t="s">
-        <v>390</v>
+        <v>360</v>
       </c>
       <c r="BW1" s="45" t="s">
+        <v>196</v>
+      </c>
+      <c r="BX1" s="45" t="s">
+        <v>199</v>
+      </c>
+      <c r="BY1" s="45" t="s">
         <v>201</v>
       </c>
-      <c r="BX1" s="45" t="s">
-        <v>204</v>
-      </c>
-      <c r="BY1" s="45" t="s">
-        <v>206</v>
-      </c>
       <c r="BZ1" s="45" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="CA1" s="45" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="CB1" s="45" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="CC1" s="45" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="CD1" s="45" t="s">
-        <v>391</v>
+        <v>361</v>
       </c>
       <c r="CE1" s="45" t="s">
+        <v>214</v>
+      </c>
+      <c r="CF1" s="45" t="s">
+        <v>217</v>
+      </c>
+      <c r="CG1" s="45" t="s">
         <v>219</v>
       </c>
-      <c r="CF1" s="45" t="s">
+      <c r="CH1" s="45" t="s">
         <v>223</v>
       </c>
-      <c r="CG1" s="45" t="s">
+      <c r="CI1" s="45" t="s">
         <v>226</v>
       </c>
-      <c r="CH1" s="45" t="s">
-        <v>230</v>
-      </c>
-      <c r="CI1" s="45" t="s">
-        <v>233</v>
-      </c>
       <c r="CJ1" s="45" t="s">
+        <v>228</v>
+      </c>
+      <c r="CK1" s="45" t="s">
+        <v>231</v>
+      </c>
+      <c r="CL1" s="45" t="s">
+        <v>234</v>
+      </c>
+      <c r="CM1" s="45" t="s">
         <v>236</v>
       </c>
-      <c r="CK1" s="45" t="s">
+      <c r="CN1" s="45" t="s">
         <v>239</v>
       </c>
-      <c r="CL1" s="45" t="s">
-        <v>242</v>
-      </c>
-      <c r="CM1" s="45" t="s">
+      <c r="CO1" s="45" t="s">
+        <v>241</v>
+      </c>
+      <c r="CP1" s="45" t="s">
+        <v>329</v>
+      </c>
+      <c r="CQ1" s="45" t="s">
+        <v>331</v>
+      </c>
+      <c r="CR1" s="45" t="s">
+        <v>243</v>
+      </c>
+      <c r="CS1" s="45" t="s">
+        <v>334</v>
+      </c>
+      <c r="CT1" s="45" t="s">
+        <v>335</v>
+      </c>
+      <c r="CU1" s="45" t="s">
         <v>245</v>
       </c>
-      <c r="CN1" s="45" t="s">
+      <c r="CV1" s="45" t="s">
+        <v>338</v>
+      </c>
+      <c r="CW1" s="45" t="s">
+        <v>346</v>
+      </c>
+      <c r="CX1" s="45" t="s">
+        <v>246</v>
+      </c>
+      <c r="CY1" s="45" t="s">
+        <v>339</v>
+      </c>
+      <c r="CZ1" s="45" t="s">
+        <v>347</v>
+      </c>
+      <c r="DA1" s="45" t="s">
+        <v>247</v>
+      </c>
+      <c r="DB1" s="45" t="s">
+        <v>340</v>
+      </c>
+      <c r="DC1" s="45" t="s">
+        <v>348</v>
+      </c>
+      <c r="DD1" s="45" t="s">
         <v>248</v>
       </c>
-      <c r="CO1" s="45" t="s">
+      <c r="DE1" s="45" t="s">
+        <v>341</v>
+      </c>
+      <c r="DF1" s="45" t="s">
+        <v>349</v>
+      </c>
+      <c r="DG1" s="45" t="s">
+        <v>249</v>
+      </c>
+      <c r="DH1" s="45" t="s">
+        <v>342</v>
+      </c>
+      <c r="DI1" s="45" t="s">
+        <v>350</v>
+      </c>
+      <c r="DJ1" s="45" t="s">
+        <v>250</v>
+      </c>
+      <c r="DK1" s="45" t="s">
+        <v>343</v>
+      </c>
+      <c r="DL1" s="45" t="s">
+        <v>351</v>
+      </c>
+      <c r="DM1" s="45" t="s">
         <v>251</v>
       </c>
-      <c r="CP1" s="45" t="s">
-        <v>356</v>
-      </c>
-      <c r="CQ1" s="45" t="s">
-        <v>358</v>
-      </c>
-      <c r="CR1" s="45" t="s">
-        <v>254</v>
-      </c>
-      <c r="CS1" s="45" t="s">
-        <v>363</v>
-      </c>
-      <c r="CT1" s="45" t="s">
-        <v>364</v>
-      </c>
-      <c r="CU1" s="45" t="s">
+      <c r="DN1" s="45" t="s">
+        <v>344</v>
+      </c>
+      <c r="DO1" s="45" t="s">
+        <v>352</v>
+      </c>
+      <c r="DP1" s="45" t="s">
+        <v>252</v>
+      </c>
+      <c r="DQ1" s="45" t="s">
+        <v>345</v>
+      </c>
+      <c r="DR1" s="45" t="s">
+        <v>353</v>
+      </c>
+      <c r="DS1" s="45" t="s">
+        <v>253</v>
+      </c>
+      <c r="DT1" s="45" t="s">
+        <v>255</v>
+      </c>
+      <c r="DU1" s="45" t="s">
         <v>257</v>
       </c>
-      <c r="CV1" s="45" t="s">
-        <v>368</v>
-      </c>
-      <c r="CW1" s="45" t="s">
-        <v>376</v>
-      </c>
-      <c r="CX1" s="45" t="s">
-        <v>258</v>
-      </c>
-      <c r="CY1" s="45" t="s">
-        <v>369</v>
-      </c>
-      <c r="CZ1" s="45" t="s">
-        <v>377</v>
-      </c>
-      <c r="DA1" s="45" t="s">
+      <c r="DV1" s="45" t="s">
         <v>259</v>
-      </c>
-      <c r="DB1" s="45" t="s">
-        <v>370</v>
-      </c>
-      <c r="DC1" s="45" t="s">
-        <v>378</v>
-      </c>
-      <c r="DD1" s="45" t="s">
-        <v>260</v>
-      </c>
-      <c r="DE1" s="45" t="s">
-        <v>371</v>
-      </c>
-      <c r="DF1" s="45" t="s">
-        <v>379</v>
-      </c>
-      <c r="DG1" s="45" t="s">
-        <v>261</v>
-      </c>
-      <c r="DH1" s="45" t="s">
-        <v>372</v>
-      </c>
-      <c r="DI1" s="45" t="s">
-        <v>380</v>
-      </c>
-      <c r="DJ1" s="45" t="s">
-        <v>262</v>
-      </c>
-      <c r="DK1" s="45" t="s">
-        <v>373</v>
-      </c>
-      <c r="DL1" s="45" t="s">
-        <v>381</v>
-      </c>
-      <c r="DM1" s="45" t="s">
-        <v>263</v>
-      </c>
-      <c r="DN1" s="45" t="s">
-        <v>374</v>
-      </c>
-      <c r="DO1" s="45" t="s">
-        <v>382</v>
-      </c>
-      <c r="DP1" s="45" t="s">
-        <v>264</v>
-      </c>
-      <c r="DQ1" s="45" t="s">
-        <v>375</v>
-      </c>
-      <c r="DR1" s="45" t="s">
-        <v>383</v>
-      </c>
-      <c r="DS1" s="45" t="s">
-        <v>265</v>
-      </c>
-      <c r="DT1" s="45" t="s">
-        <v>267</v>
-      </c>
-      <c r="DU1" s="45" t="s">
-        <v>269</v>
-      </c>
-      <c r="DV1" s="45" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="2" spans="1:126" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
draft version of new accessible plot
</commit_message>
<xml_diff>
--- a/data/ALAI UP Client-level Reporting Tool Template_4.7.26.xlsx
+++ b/data/ALAI UP Client-level Reporting Tool Template_4.7.26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kmlab\Desktop\Dashboard\alai_up_local_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FAAE59A-DE41-4D60-8AE0-52A47E059896}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6C66CB2-97D3-4919-95DA-1301A51B6493}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{500E2EE0-B1C5-4ACF-BC67-EDC8BDABD2D7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{500E2EE0-B1C5-4ACF-BC67-EDC8BDABD2D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="3" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Client-level data" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Client-level data'!$A$1:$DV$136</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Client-level data'!$A$1:$DY$136</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="389">
   <si>
     <t>INSTRUCTIONS</t>
   </si>
@@ -1351,9 +1351,6 @@
 </t>
   </si>
   <si>
-    <t>1=Clien does not qualify for PAP; 2=Medication not on payor formulary; 3=Co-pay too expensive for client; 20=Other; UNK=Unknown</t>
-  </si>
-  <si>
     <t>Reason iCAB/RPV is not financially accessible</t>
   </si>
   <si>
@@ -1400,6 +1397,9 @@
 icab_rpv_not_elig_3_reason;
 icab_rpv_not_elig_3_reason_other 
 If there are "other" reasons, include 20 here and include them in icab_rpv_not_elig_1_reason_other</t>
+  </si>
+  <si>
+    <t>1=Client does not qualify for PAP; 2=Medication not on payor formulary; 3=Co-pay too expensive for client; 20=Other; UNK=Unknown</t>
   </si>
 </sst>
 </file>
@@ -1784,7 +1784,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="143">
+  <cellXfs count="144">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -2178,6 +2178,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3726,7 +3729,7 @@
         <v>182</v>
       </c>
       <c r="E52" s="37" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="F52" s="36" t="s">
         <v>305</v>
@@ -3822,7 +3825,7 @@
         <v>194</v>
       </c>
       <c r="E56" s="37" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F56" s="37" t="s">
         <v>298</v>
@@ -3918,7 +3921,7 @@
         <v>202</v>
       </c>
       <c r="E60" s="37" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="F60" s="36" t="s">
         <v>305</v>
@@ -4014,7 +4017,7 @@
         <v>212</v>
       </c>
       <c r="E64" s="37" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F64" s="37" t="s">
         <v>293</v>
@@ -4093,7 +4096,7 @@
         <v>378</v>
       </c>
       <c r="E68" s="37" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F68" s="36" t="s">
         <v>380</v>
@@ -4109,13 +4112,13 @@
         <v>377</v>
       </c>
       <c r="D69" s="37" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E69" s="37" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F69" s="36" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="G69" s="36" t="s">
         <v>299</v>
@@ -4128,7 +4131,7 @@
         <v>379</v>
       </c>
       <c r="D70" s="37" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="E70" s="37" t="s">
         <v>185</v>
@@ -4522,7 +4525,7 @@
         <v>258</v>
       </c>
       <c r="E87" s="118" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="F87" s="36" t="s">
         <v>306</v>
@@ -4622,7 +4625,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9746185-9B90-40DD-9938-E83263BE9444}">
-  <dimension ref="A1:DV175"/>
+  <dimension ref="A1:DY175"/>
   <sheetFormatPr defaultColWidth="8.69921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.3984375" style="69" customWidth="1"/>
@@ -4632,11 +4635,11 @@
     <col min="26" max="39" width="28.19921875" style="100" customWidth="1"/>
     <col min="40" max="41" width="28.19921875" style="71" customWidth="1"/>
     <col min="42" max="64" width="28.19921875" style="73" customWidth="1"/>
-    <col min="65" max="126" width="28.19921875" style="81" customWidth="1"/>
-    <col min="127" max="16384" width="8.69921875" style="83"/>
+    <col min="65" max="129" width="28.19921875" style="81" customWidth="1"/>
+    <col min="130" max="16384" width="8.69921875" style="83"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:126" s="106" customFormat="1" ht="55.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:129" s="106" customFormat="1" ht="55.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="101" t="s">
         <v>28</v>
       </c>
@@ -4889,134 +4892,143 @@
       <c r="CF1" s="45" t="s">
         <v>217</v>
       </c>
-      <c r="CG1" s="45" t="s">
+      <c r="CG1" s="143" t="s">
+        <v>376</v>
+      </c>
+      <c r="CH1" s="143" t="s">
+        <v>377</v>
+      </c>
+      <c r="CI1" s="143" t="s">
+        <v>379</v>
+      </c>
+      <c r="CJ1" s="45" t="s">
         <v>219</v>
       </c>
-      <c r="CH1" s="45" t="s">
+      <c r="CK1" s="45" t="s">
         <v>223</v>
       </c>
-      <c r="CI1" s="45" t="s">
+      <c r="CL1" s="45" t="s">
         <v>226</v>
       </c>
-      <c r="CJ1" s="45" t="s">
+      <c r="CM1" s="45" t="s">
         <v>228</v>
       </c>
-      <c r="CK1" s="45" t="s">
+      <c r="CN1" s="45" t="s">
         <v>231</v>
       </c>
-      <c r="CL1" s="45" t="s">
+      <c r="CO1" s="45" t="s">
         <v>234</v>
       </c>
-      <c r="CM1" s="45" t="s">
+      <c r="CP1" s="45" t="s">
         <v>236</v>
       </c>
-      <c r="CN1" s="45" t="s">
+      <c r="CQ1" s="45" t="s">
         <v>239</v>
       </c>
-      <c r="CO1" s="45" t="s">
+      <c r="CR1" s="45" t="s">
         <v>241</v>
       </c>
-      <c r="CP1" s="45" t="s">
+      <c r="CS1" s="45" t="s">
         <v>328</v>
       </c>
-      <c r="CQ1" s="45" t="s">
+      <c r="CT1" s="45" t="s">
         <v>330</v>
       </c>
-      <c r="CR1" s="45" t="s">
+      <c r="CU1" s="45" t="s">
         <v>243</v>
       </c>
-      <c r="CS1" s="45" t="s">
+      <c r="CV1" s="45" t="s">
         <v>333</v>
       </c>
-      <c r="CT1" s="45" t="s">
+      <c r="CW1" s="45" t="s">
         <v>334</v>
       </c>
-      <c r="CU1" s="45" t="s">
+      <c r="CX1" s="45" t="s">
         <v>245</v>
       </c>
-      <c r="CV1" s="45" t="s">
+      <c r="CY1" s="45" t="s">
         <v>337</v>
       </c>
-      <c r="CW1" s="45" t="s">
+      <c r="CZ1" s="45" t="s">
         <v>345</v>
       </c>
-      <c r="CX1" s="45" t="s">
+      <c r="DA1" s="45" t="s">
         <v>246</v>
       </c>
-      <c r="CY1" s="45" t="s">
+      <c r="DB1" s="45" t="s">
         <v>338</v>
       </c>
-      <c r="CZ1" s="45" t="s">
+      <c r="DC1" s="45" t="s">
         <v>346</v>
       </c>
-      <c r="DA1" s="45" t="s">
+      <c r="DD1" s="45" t="s">
         <v>247</v>
       </c>
-      <c r="DB1" s="45" t="s">
+      <c r="DE1" s="45" t="s">
         <v>339</v>
       </c>
-      <c r="DC1" s="45" t="s">
+      <c r="DF1" s="45" t="s">
         <v>347</v>
       </c>
-      <c r="DD1" s="45" t="s">
+      <c r="DG1" s="45" t="s">
         <v>248</v>
       </c>
-      <c r="DE1" s="45" t="s">
+      <c r="DH1" s="45" t="s">
         <v>340</v>
       </c>
-      <c r="DF1" s="45" t="s">
+      <c r="DI1" s="45" t="s">
         <v>348</v>
       </c>
-      <c r="DG1" s="45" t="s">
+      <c r="DJ1" s="45" t="s">
         <v>249</v>
       </c>
-      <c r="DH1" s="45" t="s">
+      <c r="DK1" s="45" t="s">
         <v>341</v>
       </c>
-      <c r="DI1" s="45" t="s">
+      <c r="DL1" s="45" t="s">
         <v>349</v>
       </c>
-      <c r="DJ1" s="45" t="s">
+      <c r="DM1" s="45" t="s">
         <v>250</v>
       </c>
-      <c r="DK1" s="45" t="s">
+      <c r="DN1" s="45" t="s">
         <v>342</v>
       </c>
-      <c r="DL1" s="45" t="s">
+      <c r="DO1" s="45" t="s">
         <v>350</v>
       </c>
-      <c r="DM1" s="45" t="s">
+      <c r="DP1" s="45" t="s">
         <v>251</v>
       </c>
-      <c r="DN1" s="45" t="s">
+      <c r="DQ1" s="45" t="s">
         <v>343</v>
       </c>
-      <c r="DO1" s="45" t="s">
+      <c r="DR1" s="45" t="s">
         <v>351</v>
       </c>
-      <c r="DP1" s="45" t="s">
+      <c r="DS1" s="45" t="s">
         <v>252</v>
       </c>
-      <c r="DQ1" s="45" t="s">
+      <c r="DT1" s="45" t="s">
         <v>344</v>
       </c>
-      <c r="DR1" s="45" t="s">
+      <c r="DU1" s="45" t="s">
         <v>352</v>
       </c>
-      <c r="DS1" s="45" t="s">
+      <c r="DV1" s="45" t="s">
         <v>253</v>
       </c>
-      <c r="DT1" s="45" t="s">
+      <c r="DW1" s="45" t="s">
         <v>255</v>
       </c>
-      <c r="DU1" s="45" t="s">
+      <c r="DX1" s="45" t="s">
         <v>257</v>
       </c>
-      <c r="DV1" s="45" t="s">
+      <c r="DY1" s="45" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="2" spans="1:126" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A2" s="6"/>
       <c r="B2" s="6"/>
       <c r="C2" s="11"/>
@@ -5107,11 +5119,11 @@
       <c r="CJ2" s="34"/>
       <c r="CK2" s="34"/>
       <c r="CL2" s="34"/>
-      <c r="CM2" s="35"/>
-      <c r="CN2" s="35"/>
-      <c r="CO2" s="49"/>
-      <c r="CP2" s="34"/>
-      <c r="CQ2" s="34"/>
+      <c r="CM2" s="34"/>
+      <c r="CN2" s="34"/>
+      <c r="CO2" s="34"/>
+      <c r="CP2" s="35"/>
+      <c r="CQ2" s="35"/>
       <c r="CR2" s="49"/>
       <c r="CS2" s="34"/>
       <c r="CT2" s="34"/>
@@ -5139,12 +5151,15 @@
       <c r="DP2" s="49"/>
       <c r="DQ2" s="34"/>
       <c r="DR2" s="34"/>
-      <c r="DS2" s="34"/>
-      <c r="DT2" s="49"/>
+      <c r="DS2" s="49"/>
+      <c r="DT2" s="34"/>
       <c r="DU2" s="34"/>
       <c r="DV2" s="34"/>
-    </row>
-    <row r="3" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW2" s="49"/>
+      <c r="DX2" s="34"/>
+      <c r="DY2" s="34"/>
+    </row>
+    <row r="3" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A3" s="6"/>
       <c r="B3" s="6"/>
       <c r="C3" s="11"/>
@@ -5235,11 +5250,11 @@
       <c r="CJ3" s="34"/>
       <c r="CK3" s="34"/>
       <c r="CL3" s="34"/>
-      <c r="CM3" s="35"/>
-      <c r="CN3" s="35"/>
-      <c r="CO3" s="49"/>
-      <c r="CP3" s="34"/>
-      <c r="CQ3" s="34"/>
+      <c r="CM3" s="34"/>
+      <c r="CN3" s="34"/>
+      <c r="CO3" s="34"/>
+      <c r="CP3" s="35"/>
+      <c r="CQ3" s="35"/>
       <c r="CR3" s="49"/>
       <c r="CS3" s="34"/>
       <c r="CT3" s="34"/>
@@ -5267,12 +5282,15 @@
       <c r="DP3" s="49"/>
       <c r="DQ3" s="34"/>
       <c r="DR3" s="34"/>
-      <c r="DS3" s="34"/>
-      <c r="DT3" s="49"/>
+      <c r="DS3" s="49"/>
+      <c r="DT3" s="34"/>
       <c r="DU3" s="34"/>
       <c r="DV3" s="34"/>
-    </row>
-    <row r="4" spans="1:126" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="DW3" s="49"/>
+      <c r="DX3" s="34"/>
+      <c r="DY3" s="34"/>
+    </row>
+    <row r="4" spans="1:129" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="6"/>
       <c r="B4" s="6"/>
       <c r="C4" s="11"/>
@@ -5363,11 +5381,11 @@
       <c r="CJ4" s="34"/>
       <c r="CK4" s="34"/>
       <c r="CL4" s="34"/>
-      <c r="CM4" s="35"/>
-      <c r="CN4" s="35"/>
-      <c r="CO4" s="49"/>
-      <c r="CP4" s="34"/>
-      <c r="CQ4" s="34"/>
+      <c r="CM4" s="34"/>
+      <c r="CN4" s="34"/>
+      <c r="CO4" s="34"/>
+      <c r="CP4" s="35"/>
+      <c r="CQ4" s="35"/>
       <c r="CR4" s="49"/>
       <c r="CS4" s="34"/>
       <c r="CT4" s="34"/>
@@ -5395,12 +5413,15 @@
       <c r="DP4" s="49"/>
       <c r="DQ4" s="34"/>
       <c r="DR4" s="34"/>
-      <c r="DS4" s="34"/>
-      <c r="DT4" s="49"/>
+      <c r="DS4" s="49"/>
+      <c r="DT4" s="34"/>
       <c r="DU4" s="34"/>
       <c r="DV4" s="34"/>
-    </row>
-    <row r="5" spans="1:126" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="DW4" s="49"/>
+      <c r="DX4" s="34"/>
+      <c r="DY4" s="34"/>
+    </row>
+    <row r="5" spans="1:129" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="6"/>
       <c r="B5" s="6"/>
       <c r="C5" s="50"/>
@@ -5475,16 +5496,16 @@
       <c r="CD5" s="60"/>
       <c r="CE5" s="37"/>
       <c r="CF5" s="61"/>
-      <c r="CG5" s="35"/>
-      <c r="CH5" s="35"/>
-      <c r="CI5" s="35"/>
+      <c r="CG5" s="61"/>
+      <c r="CH5" s="61"/>
+      <c r="CI5" s="61"/>
       <c r="CJ5" s="35"/>
       <c r="CK5" s="35"/>
       <c r="CL5" s="35"/>
-      <c r="CM5" s="64"/>
+      <c r="CM5" s="35"/>
       <c r="CN5" s="35"/>
-      <c r="CO5" s="64"/>
-      <c r="CP5" s="35"/>
+      <c r="CO5" s="35"/>
+      <c r="CP5" s="64"/>
       <c r="CQ5" s="35"/>
       <c r="CR5" s="64"/>
       <c r="CS5" s="35"/>
@@ -5504,21 +5525,24 @@
       <c r="DG5" s="64"/>
       <c r="DH5" s="35"/>
       <c r="DI5" s="35"/>
-      <c r="DJ5" s="78"/>
-      <c r="DK5" s="64"/>
+      <c r="DJ5" s="64"/>
+      <c r="DK5" s="35"/>
       <c r="DL5" s="35"/>
-      <c r="DM5" s="64"/>
-      <c r="DN5" s="35"/>
+      <c r="DM5" s="78"/>
+      <c r="DN5" s="64"/>
       <c r="DO5" s="35"/>
       <c r="DP5" s="64"/>
       <c r="DQ5" s="35"/>
       <c r="DR5" s="35"/>
-      <c r="DS5" s="35"/>
+      <c r="DS5" s="64"/>
       <c r="DT5" s="35"/>
       <c r="DU5" s="35"/>
       <c r="DV5" s="35"/>
-    </row>
-    <row r="6" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW5" s="35"/>
+      <c r="DX5" s="35"/>
+      <c r="DY5" s="35"/>
+    </row>
+    <row r="6" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A6" s="6"/>
       <c r="B6" s="6"/>
       <c r="C6" s="50"/>
@@ -5593,9 +5617,9 @@
       <c r="CD6" s="60"/>
       <c r="CE6" s="61"/>
       <c r="CF6" s="37"/>
-      <c r="CG6" s="35"/>
-      <c r="CH6" s="35"/>
-      <c r="CI6" s="35"/>
+      <c r="CG6" s="37"/>
+      <c r="CH6" s="37"/>
+      <c r="CI6" s="37"/>
       <c r="CJ6" s="35"/>
       <c r="CK6" s="35"/>
       <c r="CL6" s="35"/>
@@ -5635,8 +5659,11 @@
       <c r="DT6" s="35"/>
       <c r="DU6" s="35"/>
       <c r="DV6" s="35"/>
-    </row>
-    <row r="7" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW6" s="35"/>
+      <c r="DX6" s="35"/>
+      <c r="DY6" s="35"/>
+    </row>
+    <row r="7" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A7" s="6"/>
       <c r="B7" s="6"/>
       <c r="C7" s="50"/>
@@ -5711,9 +5738,9 @@
       <c r="CD7" s="60"/>
       <c r="CE7" s="37"/>
       <c r="CF7" s="37"/>
-      <c r="CG7" s="35"/>
-      <c r="CH7" s="35"/>
-      <c r="CI7" s="35"/>
+      <c r="CG7" s="37"/>
+      <c r="CH7" s="37"/>
+      <c r="CI7" s="37"/>
       <c r="CJ7" s="35"/>
       <c r="CK7" s="35"/>
       <c r="CL7" s="35"/>
@@ -5753,8 +5780,11 @@
       <c r="DT7" s="35"/>
       <c r="DU7" s="35"/>
       <c r="DV7" s="35"/>
-    </row>
-    <row r="8" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW7" s="35"/>
+      <c r="DX7" s="35"/>
+      <c r="DY7" s="35"/>
+    </row>
+    <row r="8" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
       <c r="C8" s="50"/>
@@ -5829,16 +5859,16 @@
       <c r="CD8" s="60"/>
       <c r="CE8" s="37"/>
       <c r="CF8" s="61"/>
-      <c r="CG8" s="35"/>
-      <c r="CH8" s="35"/>
-      <c r="CI8" s="35"/>
+      <c r="CG8" s="61"/>
+      <c r="CH8" s="61"/>
+      <c r="CI8" s="61"/>
       <c r="CJ8" s="35"/>
       <c r="CK8" s="35"/>
       <c r="CL8" s="35"/>
-      <c r="CM8" s="64"/>
+      <c r="CM8" s="35"/>
       <c r="CN8" s="35"/>
-      <c r="CO8" s="64"/>
-      <c r="CP8" s="35"/>
+      <c r="CO8" s="35"/>
+      <c r="CP8" s="64"/>
       <c r="CQ8" s="35"/>
       <c r="CR8" s="64"/>
       <c r="CS8" s="35"/>
@@ -5867,12 +5897,15 @@
       <c r="DP8" s="64"/>
       <c r="DQ8" s="35"/>
       <c r="DR8" s="35"/>
-      <c r="DS8" s="35"/>
+      <c r="DS8" s="64"/>
       <c r="DT8" s="35"/>
       <c r="DU8" s="35"/>
       <c r="DV8" s="35"/>
-    </row>
-    <row r="9" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW8" s="35"/>
+      <c r="DX8" s="35"/>
+      <c r="DY8" s="35"/>
+    </row>
+    <row r="9" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="50"/>
@@ -5947,15 +5980,15 @@
       <c r="CD9" s="60"/>
       <c r="CE9" s="37"/>
       <c r="CF9" s="61"/>
-      <c r="CG9" s="35"/>
-      <c r="CH9" s="35"/>
-      <c r="CI9" s="35"/>
+      <c r="CG9" s="61"/>
+      <c r="CH9" s="61"/>
+      <c r="CI9" s="61"/>
       <c r="CJ9" s="35"/>
       <c r="CK9" s="35"/>
       <c r="CL9" s="35"/>
       <c r="CM9" s="35"/>
       <c r="CN9" s="35"/>
-      <c r="CO9" s="64"/>
+      <c r="CO9" s="35"/>
       <c r="CP9" s="35"/>
       <c r="CQ9" s="35"/>
       <c r="CR9" s="64"/>
@@ -5985,12 +6018,15 @@
       <c r="DP9" s="64"/>
       <c r="DQ9" s="35"/>
       <c r="DR9" s="35"/>
-      <c r="DS9" s="35"/>
+      <c r="DS9" s="64"/>
       <c r="DT9" s="35"/>
       <c r="DU9" s="35"/>
       <c r="DV9" s="35"/>
-    </row>
-    <row r="10" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW9" s="35"/>
+      <c r="DX9" s="35"/>
+      <c r="DY9" s="35"/>
+    </row>
+    <row r="10" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A10" s="6"/>
       <c r="B10" s="6"/>
       <c r="C10" s="50"/>
@@ -6065,9 +6101,9 @@
       <c r="CD10" s="60"/>
       <c r="CE10" s="37"/>
       <c r="CF10" s="37"/>
-      <c r="CG10" s="35"/>
-      <c r="CH10" s="35"/>
-      <c r="CI10" s="35"/>
+      <c r="CG10" s="37"/>
+      <c r="CH10" s="37"/>
+      <c r="CI10" s="37"/>
       <c r="CJ10" s="35"/>
       <c r="CK10" s="35"/>
       <c r="CL10" s="35"/>
@@ -6107,8 +6143,11 @@
       <c r="DT10" s="35"/>
       <c r="DU10" s="35"/>
       <c r="DV10" s="35"/>
-    </row>
-    <row r="11" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW10" s="35"/>
+      <c r="DX10" s="35"/>
+      <c r="DY10" s="35"/>
+    </row>
+    <row r="11" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A11" s="6"/>
       <c r="B11" s="6"/>
       <c r="C11" s="50"/>
@@ -6183,9 +6222,9 @@
       <c r="CD11" s="60"/>
       <c r="CE11" s="37"/>
       <c r="CF11" s="37"/>
-      <c r="CG11" s="35"/>
-      <c r="CH11" s="35"/>
-      <c r="CI11" s="35"/>
+      <c r="CG11" s="37"/>
+      <c r="CH11" s="37"/>
+      <c r="CI11" s="37"/>
       <c r="CJ11" s="35"/>
       <c r="CK11" s="35"/>
       <c r="CL11" s="35"/>
@@ -6225,8 +6264,11 @@
       <c r="DT11" s="35"/>
       <c r="DU11" s="35"/>
       <c r="DV11" s="35"/>
-    </row>
-    <row r="12" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW11" s="35"/>
+      <c r="DX11" s="35"/>
+      <c r="DY11" s="35"/>
+    </row>
+    <row r="12" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
       <c r="B12" s="6"/>
       <c r="C12" s="50"/>
@@ -6301,9 +6343,9 @@
       <c r="CD12" s="60"/>
       <c r="CE12" s="37"/>
       <c r="CF12" s="37"/>
-      <c r="CG12" s="35"/>
-      <c r="CH12" s="35"/>
-      <c r="CI12" s="35"/>
+      <c r="CG12" s="37"/>
+      <c r="CH12" s="37"/>
+      <c r="CI12" s="37"/>
       <c r="CJ12" s="35"/>
       <c r="CK12" s="35"/>
       <c r="CL12" s="35"/>
@@ -6343,8 +6385,11 @@
       <c r="DT12" s="35"/>
       <c r="DU12" s="35"/>
       <c r="DV12" s="35"/>
-    </row>
-    <row r="13" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW12" s="35"/>
+      <c r="DX12" s="35"/>
+      <c r="DY12" s="35"/>
+    </row>
+    <row r="13" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A13" s="6"/>
       <c r="B13" s="6"/>
       <c r="C13" s="50"/>
@@ -6419,9 +6464,9 @@
       <c r="CD13" s="60"/>
       <c r="CE13" s="37"/>
       <c r="CF13" s="37"/>
-      <c r="CG13" s="35"/>
-      <c r="CH13" s="35"/>
-      <c r="CI13" s="35"/>
+      <c r="CG13" s="37"/>
+      <c r="CH13" s="37"/>
+      <c r="CI13" s="37"/>
       <c r="CJ13" s="35"/>
       <c r="CK13" s="35"/>
       <c r="CL13" s="35"/>
@@ -6461,8 +6506,11 @@
       <c r="DT13" s="35"/>
       <c r="DU13" s="35"/>
       <c r="DV13" s="35"/>
-    </row>
-    <row r="14" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW13" s="35"/>
+      <c r="DX13" s="35"/>
+      <c r="DY13" s="35"/>
+    </row>
+    <row r="14" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A14" s="6"/>
       <c r="B14" s="6"/>
       <c r="C14" s="50"/>
@@ -6537,15 +6585,15 @@
       <c r="CD14" s="60"/>
       <c r="CE14" s="37"/>
       <c r="CF14" s="61"/>
-      <c r="CG14" s="35"/>
-      <c r="CH14" s="64"/>
-      <c r="CI14" s="35"/>
+      <c r="CG14" s="61"/>
+      <c r="CH14" s="61"/>
+      <c r="CI14" s="61"/>
       <c r="CJ14" s="35"/>
-      <c r="CK14" s="35"/>
+      <c r="CK14" s="64"/>
       <c r="CL14" s="35"/>
       <c r="CM14" s="35"/>
       <c r="CN14" s="35"/>
-      <c r="CO14" s="64"/>
+      <c r="CO14" s="35"/>
       <c r="CP14" s="35"/>
       <c r="CQ14" s="35"/>
       <c r="CR14" s="64"/>
@@ -6575,12 +6623,15 @@
       <c r="DP14" s="64"/>
       <c r="DQ14" s="35"/>
       <c r="DR14" s="35"/>
-      <c r="DS14" s="35"/>
+      <c r="DS14" s="64"/>
       <c r="DT14" s="35"/>
       <c r="DU14" s="35"/>
       <c r="DV14" s="35"/>
-    </row>
-    <row r="15" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW14" s="35"/>
+      <c r="DX14" s="35"/>
+      <c r="DY14" s="35"/>
+    </row>
+    <row r="15" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A15" s="6"/>
       <c r="B15" s="6"/>
       <c r="C15" s="50"/>
@@ -6655,9 +6706,9 @@
       <c r="CD15" s="60"/>
       <c r="CE15" s="37"/>
       <c r="CF15" s="37"/>
-      <c r="CG15" s="35"/>
-      <c r="CH15" s="35"/>
-      <c r="CI15" s="35"/>
+      <c r="CG15" s="37"/>
+      <c r="CH15" s="37"/>
+      <c r="CI15" s="37"/>
       <c r="CJ15" s="35"/>
       <c r="CK15" s="35"/>
       <c r="CL15" s="35"/>
@@ -6697,8 +6748,11 @@
       <c r="DT15" s="35"/>
       <c r="DU15" s="35"/>
       <c r="DV15" s="35"/>
-    </row>
-    <row r="16" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW15" s="35"/>
+      <c r="DX15" s="35"/>
+      <c r="DY15" s="35"/>
+    </row>
+    <row r="16" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A16" s="6"/>
       <c r="B16" s="6"/>
       <c r="C16" s="50"/>
@@ -6773,9 +6827,9 @@
       <c r="CD16" s="60"/>
       <c r="CE16" s="37"/>
       <c r="CF16" s="37"/>
-      <c r="CG16" s="35"/>
-      <c r="CH16" s="35"/>
-      <c r="CI16" s="35"/>
+      <c r="CG16" s="37"/>
+      <c r="CH16" s="37"/>
+      <c r="CI16" s="37"/>
       <c r="CJ16" s="35"/>
       <c r="CK16" s="35"/>
       <c r="CL16" s="35"/>
@@ -6815,8 +6869,11 @@
       <c r="DT16" s="35"/>
       <c r="DU16" s="35"/>
       <c r="DV16" s="35"/>
-    </row>
-    <row r="17" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW16" s="35"/>
+      <c r="DX16" s="35"/>
+      <c r="DY16" s="35"/>
+    </row>
+    <row r="17" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A17" s="6"/>
       <c r="B17" s="6"/>
       <c r="C17" s="50"/>
@@ -6891,9 +6948,9 @@
       <c r="CD17" s="60"/>
       <c r="CE17" s="37"/>
       <c r="CF17" s="37"/>
-      <c r="CG17" s="35"/>
-      <c r="CH17" s="35"/>
-      <c r="CI17" s="35"/>
+      <c r="CG17" s="37"/>
+      <c r="CH17" s="37"/>
+      <c r="CI17" s="37"/>
       <c r="CJ17" s="35"/>
       <c r="CK17" s="35"/>
       <c r="CL17" s="35"/>
@@ -6933,8 +6990,11 @@
       <c r="DT17" s="35"/>
       <c r="DU17" s="35"/>
       <c r="DV17" s="35"/>
-    </row>
-    <row r="18" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW17" s="35"/>
+      <c r="DX17" s="35"/>
+      <c r="DY17" s="35"/>
+    </row>
+    <row r="18" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A18" s="6"/>
       <c r="B18" s="6"/>
       <c r="C18" s="50"/>
@@ -7009,9 +7069,9 @@
       <c r="CD18" s="60"/>
       <c r="CE18" s="37"/>
       <c r="CF18" s="37"/>
-      <c r="CG18" s="35"/>
-      <c r="CH18" s="35"/>
-      <c r="CI18" s="35"/>
+      <c r="CG18" s="37"/>
+      <c r="CH18" s="37"/>
+      <c r="CI18" s="37"/>
       <c r="CJ18" s="35"/>
       <c r="CK18" s="35"/>
       <c r="CL18" s="35"/>
@@ -7051,8 +7111,11 @@
       <c r="DT18" s="35"/>
       <c r="DU18" s="35"/>
       <c r="DV18" s="35"/>
-    </row>
-    <row r="19" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW18" s="35"/>
+      <c r="DX18" s="35"/>
+      <c r="DY18" s="35"/>
+    </row>
+    <row r="19" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A19" s="6"/>
       <c r="B19" s="6"/>
       <c r="C19" s="50"/>
@@ -7127,9 +7190,9 @@
       <c r="CD19" s="60"/>
       <c r="CE19" s="37"/>
       <c r="CF19" s="37"/>
-      <c r="CG19" s="35"/>
-      <c r="CH19" s="35"/>
-      <c r="CI19" s="35"/>
+      <c r="CG19" s="37"/>
+      <c r="CH19" s="37"/>
+      <c r="CI19" s="37"/>
       <c r="CJ19" s="35"/>
       <c r="CK19" s="35"/>
       <c r="CL19" s="35"/>
@@ -7169,8 +7232,11 @@
       <c r="DT19" s="35"/>
       <c r="DU19" s="35"/>
       <c r="DV19" s="35"/>
-    </row>
-    <row r="20" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW19" s="35"/>
+      <c r="DX19" s="35"/>
+      <c r="DY19" s="35"/>
+    </row>
+    <row r="20" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A20" s="6"/>
       <c r="B20" s="6"/>
       <c r="C20" s="50"/>
@@ -7245,9 +7311,9 @@
       <c r="CD20" s="60"/>
       <c r="CE20" s="37"/>
       <c r="CF20" s="37"/>
-      <c r="CG20" s="35"/>
-      <c r="CH20" s="35"/>
-      <c r="CI20" s="35"/>
+      <c r="CG20" s="37"/>
+      <c r="CH20" s="37"/>
+      <c r="CI20" s="37"/>
       <c r="CJ20" s="35"/>
       <c r="CK20" s="35"/>
       <c r="CL20" s="35"/>
@@ -7287,8 +7353,11 @@
       <c r="DT20" s="35"/>
       <c r="DU20" s="35"/>
       <c r="DV20" s="35"/>
-    </row>
-    <row r="21" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW20" s="35"/>
+      <c r="DX20" s="35"/>
+      <c r="DY20" s="35"/>
+    </row>
+    <row r="21" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
       <c r="B21" s="6"/>
       <c r="C21" s="50"/>
@@ -7363,9 +7432,9 @@
       <c r="CD21" s="60"/>
       <c r="CE21" s="37"/>
       <c r="CF21" s="37"/>
-      <c r="CG21" s="35"/>
-      <c r="CH21" s="35"/>
-      <c r="CI21" s="35"/>
+      <c r="CG21" s="37"/>
+      <c r="CH21" s="37"/>
+      <c r="CI21" s="37"/>
       <c r="CJ21" s="35"/>
       <c r="CK21" s="35"/>
       <c r="CL21" s="35"/>
@@ -7405,8 +7474,11 @@
       <c r="DT21" s="35"/>
       <c r="DU21" s="35"/>
       <c r="DV21" s="35"/>
-    </row>
-    <row r="22" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW21" s="35"/>
+      <c r="DX21" s="35"/>
+      <c r="DY21" s="35"/>
+    </row>
+    <row r="22" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A22" s="6"/>
       <c r="B22" s="6"/>
       <c r="C22" s="50"/>
@@ -7481,9 +7553,9 @@
       <c r="CD22" s="60"/>
       <c r="CE22" s="37"/>
       <c r="CF22" s="37"/>
-      <c r="CG22" s="35"/>
-      <c r="CH22" s="35"/>
-      <c r="CI22" s="35"/>
+      <c r="CG22" s="37"/>
+      <c r="CH22" s="37"/>
+      <c r="CI22" s="37"/>
       <c r="CJ22" s="35"/>
       <c r="CK22" s="35"/>
       <c r="CL22" s="35"/>
@@ -7523,8 +7595,11 @@
       <c r="DT22" s="35"/>
       <c r="DU22" s="35"/>
       <c r="DV22" s="35"/>
-    </row>
-    <row r="23" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW22" s="35"/>
+      <c r="DX22" s="35"/>
+      <c r="DY22" s="35"/>
+    </row>
+    <row r="23" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A23" s="6"/>
       <c r="B23" s="6"/>
       <c r="C23" s="50"/>
@@ -7599,9 +7674,9 @@
       <c r="CD23" s="60"/>
       <c r="CE23" s="37"/>
       <c r="CF23" s="37"/>
-      <c r="CG23" s="35"/>
-      <c r="CH23" s="35"/>
-      <c r="CI23" s="35"/>
+      <c r="CG23" s="37"/>
+      <c r="CH23" s="37"/>
+      <c r="CI23" s="37"/>
       <c r="CJ23" s="35"/>
       <c r="CK23" s="35"/>
       <c r="CL23" s="35"/>
@@ -7641,8 +7716,11 @@
       <c r="DT23" s="35"/>
       <c r="DU23" s="35"/>
       <c r="DV23" s="35"/>
-    </row>
-    <row r="24" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW23" s="35"/>
+      <c r="DX23" s="35"/>
+      <c r="DY23" s="35"/>
+    </row>
+    <row r="24" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A24" s="6"/>
       <c r="B24" s="6"/>
       <c r="C24" s="50"/>
@@ -7717,9 +7795,9 @@
       <c r="CD24" s="60"/>
       <c r="CE24" s="37"/>
       <c r="CF24" s="37"/>
-      <c r="CG24" s="35"/>
-      <c r="CH24" s="35"/>
-      <c r="CI24" s="35"/>
+      <c r="CG24" s="37"/>
+      <c r="CH24" s="37"/>
+      <c r="CI24" s="37"/>
       <c r="CJ24" s="35"/>
       <c r="CK24" s="35"/>
       <c r="CL24" s="35"/>
@@ -7759,8 +7837,11 @@
       <c r="DT24" s="35"/>
       <c r="DU24" s="35"/>
       <c r="DV24" s="35"/>
-    </row>
-    <row r="25" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW24" s="35"/>
+      <c r="DX24" s="35"/>
+      <c r="DY24" s="35"/>
+    </row>
+    <row r="25" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A25" s="6"/>
       <c r="B25" s="6"/>
       <c r="C25" s="50"/>
@@ -7835,9 +7916,9 @@
       <c r="CD25" s="60"/>
       <c r="CE25" s="37"/>
       <c r="CF25" s="37"/>
-      <c r="CG25" s="35"/>
-      <c r="CH25" s="35"/>
-      <c r="CI25" s="35"/>
+      <c r="CG25" s="37"/>
+      <c r="CH25" s="37"/>
+      <c r="CI25" s="37"/>
       <c r="CJ25" s="35"/>
       <c r="CK25" s="35"/>
       <c r="CL25" s="35"/>
@@ -7877,8 +7958,11 @@
       <c r="DT25" s="35"/>
       <c r="DU25" s="35"/>
       <c r="DV25" s="35"/>
-    </row>
-    <row r="26" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW25" s="35"/>
+      <c r="DX25" s="35"/>
+      <c r="DY25" s="35"/>
+    </row>
+    <row r="26" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
       <c r="C26" s="50"/>
@@ -7953,16 +8037,16 @@
       <c r="CD26" s="60"/>
       <c r="CE26" s="37"/>
       <c r="CF26" s="61"/>
-      <c r="CG26" s="35"/>
-      <c r="CH26" s="64"/>
-      <c r="CI26" s="35"/>
+      <c r="CG26" s="61"/>
+      <c r="CH26" s="61"/>
+      <c r="CI26" s="61"/>
       <c r="CJ26" s="35"/>
-      <c r="CK26" s="35"/>
+      <c r="CK26" s="64"/>
       <c r="CL26" s="35"/>
-      <c r="CM26" s="64"/>
+      <c r="CM26" s="35"/>
       <c r="CN26" s="35"/>
-      <c r="CO26" s="64"/>
-      <c r="CP26" s="35"/>
+      <c r="CO26" s="35"/>
+      <c r="CP26" s="64"/>
       <c r="CQ26" s="35"/>
       <c r="CR26" s="64"/>
       <c r="CS26" s="35"/>
@@ -7982,7 +8066,7 @@
       <c r="DG26" s="64"/>
       <c r="DH26" s="35"/>
       <c r="DI26" s="35"/>
-      <c r="DJ26" s="35"/>
+      <c r="DJ26" s="64"/>
       <c r="DK26" s="35"/>
       <c r="DL26" s="35"/>
       <c r="DM26" s="35"/>
@@ -7992,11 +8076,14 @@
       <c r="DQ26" s="35"/>
       <c r="DR26" s="35"/>
       <c r="DS26" s="35"/>
-      <c r="DT26" s="64"/>
+      <c r="DT26" s="35"/>
       <c r="DU26" s="35"/>
       <c r="DV26" s="35"/>
-    </row>
-    <row r="27" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW26" s="64"/>
+      <c r="DX26" s="35"/>
+      <c r="DY26" s="35"/>
+    </row>
+    <row r="27" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A27" s="6"/>
       <c r="B27" s="6"/>
       <c r="C27" s="50"/>
@@ -8071,15 +8158,15 @@
       <c r="CD27" s="60"/>
       <c r="CE27" s="37"/>
       <c r="CF27" s="61"/>
-      <c r="CG27" s="35"/>
-      <c r="CH27" s="64"/>
-      <c r="CI27" s="35"/>
+      <c r="CG27" s="61"/>
+      <c r="CH27" s="61"/>
+      <c r="CI27" s="61"/>
       <c r="CJ27" s="35"/>
-      <c r="CK27" s="35"/>
+      <c r="CK27" s="64"/>
       <c r="CL27" s="35"/>
       <c r="CM27" s="35"/>
       <c r="CN27" s="35"/>
-      <c r="CO27" s="64"/>
+      <c r="CO27" s="35"/>
       <c r="CP27" s="35"/>
       <c r="CQ27" s="35"/>
       <c r="CR27" s="64"/>
@@ -8094,7 +8181,7 @@
       <c r="DA27" s="64"/>
       <c r="DB27" s="35"/>
       <c r="DC27" s="35"/>
-      <c r="DD27" s="35"/>
+      <c r="DD27" s="64"/>
       <c r="DE27" s="35"/>
       <c r="DF27" s="35"/>
       <c r="DG27" s="35"/>
@@ -8110,11 +8197,14 @@
       <c r="DQ27" s="35"/>
       <c r="DR27" s="35"/>
       <c r="DS27" s="35"/>
-      <c r="DT27" s="64"/>
+      <c r="DT27" s="35"/>
       <c r="DU27" s="35"/>
       <c r="DV27" s="35"/>
-    </row>
-    <row r="28" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW27" s="64"/>
+      <c r="DX27" s="35"/>
+      <c r="DY27" s="35"/>
+    </row>
+    <row r="28" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A28" s="6"/>
       <c r="B28" s="6"/>
       <c r="C28" s="50"/>
@@ -8189,16 +8279,16 @@
       <c r="CD28" s="60"/>
       <c r="CE28" s="37"/>
       <c r="CF28" s="61"/>
-      <c r="CG28" s="35"/>
-      <c r="CH28" s="35"/>
-      <c r="CI28" s="35"/>
+      <c r="CG28" s="61"/>
+      <c r="CH28" s="61"/>
+      <c r="CI28" s="61"/>
       <c r="CJ28" s="35"/>
       <c r="CK28" s="35"/>
       <c r="CL28" s="35"/>
-      <c r="CM28" s="64"/>
+      <c r="CM28" s="35"/>
       <c r="CN28" s="35"/>
-      <c r="CO28" s="64"/>
-      <c r="CP28" s="35"/>
+      <c r="CO28" s="35"/>
+      <c r="CP28" s="64"/>
       <c r="CQ28" s="35"/>
       <c r="CR28" s="64"/>
       <c r="CS28" s="35"/>
@@ -8212,7 +8302,7 @@
       <c r="DA28" s="64"/>
       <c r="DB28" s="35"/>
       <c r="DC28" s="35"/>
-      <c r="DD28" s="35"/>
+      <c r="DD28" s="64"/>
       <c r="DE28" s="35"/>
       <c r="DF28" s="35"/>
       <c r="DG28" s="35"/>
@@ -8231,8 +8321,11 @@
       <c r="DT28" s="35"/>
       <c r="DU28" s="35"/>
       <c r="DV28" s="35"/>
-    </row>
-    <row r="29" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW28" s="35"/>
+      <c r="DX28" s="35"/>
+      <c r="DY28" s="35"/>
+    </row>
+    <row r="29" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A29" s="6"/>
       <c r="B29" s="6"/>
       <c r="C29" s="50"/>
@@ -8307,9 +8400,9 @@
       <c r="CD29" s="60"/>
       <c r="CE29" s="37"/>
       <c r="CF29" s="37"/>
-      <c r="CG29" s="35"/>
-      <c r="CH29" s="35"/>
-      <c r="CI29" s="35"/>
+      <c r="CG29" s="37"/>
+      <c r="CH29" s="37"/>
+      <c r="CI29" s="37"/>
       <c r="CJ29" s="35"/>
       <c r="CK29" s="35"/>
       <c r="CL29" s="35"/>
@@ -8349,8 +8442,11 @@
       <c r="DT29" s="35"/>
       <c r="DU29" s="35"/>
       <c r="DV29" s="35"/>
-    </row>
-    <row r="30" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW29" s="35"/>
+      <c r="DX29" s="35"/>
+      <c r="DY29" s="35"/>
+    </row>
+    <row r="30" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A30" s="6"/>
       <c r="B30" s="6"/>
       <c r="C30" s="50"/>
@@ -8425,9 +8521,9 @@
       <c r="CD30" s="60"/>
       <c r="CE30" s="37"/>
       <c r="CF30" s="37"/>
-      <c r="CG30" s="35"/>
-      <c r="CH30" s="35"/>
-      <c r="CI30" s="35"/>
+      <c r="CG30" s="37"/>
+      <c r="CH30" s="37"/>
+      <c r="CI30" s="37"/>
       <c r="CJ30" s="35"/>
       <c r="CK30" s="35"/>
       <c r="CL30" s="35"/>
@@ -8467,8 +8563,11 @@
       <c r="DT30" s="35"/>
       <c r="DU30" s="35"/>
       <c r="DV30" s="35"/>
-    </row>
-    <row r="31" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW30" s="35"/>
+      <c r="DX30" s="35"/>
+      <c r="DY30" s="35"/>
+    </row>
+    <row r="31" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A31" s="6"/>
       <c r="B31" s="6"/>
       <c r="C31" s="50"/>
@@ -8543,9 +8642,9 @@
       <c r="CD31" s="60"/>
       <c r="CE31" s="37"/>
       <c r="CF31" s="61"/>
-      <c r="CG31" s="35"/>
-      <c r="CH31" s="35"/>
-      <c r="CI31" s="35"/>
+      <c r="CG31" s="61"/>
+      <c r="CH31" s="61"/>
+      <c r="CI31" s="61"/>
       <c r="CJ31" s="35"/>
       <c r="CK31" s="35"/>
       <c r="CL31" s="35"/>
@@ -8585,8 +8684,11 @@
       <c r="DT31" s="35"/>
       <c r="DU31" s="35"/>
       <c r="DV31" s="35"/>
-    </row>
-    <row r="32" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW31" s="35"/>
+      <c r="DX31" s="35"/>
+      <c r="DY31" s="35"/>
+    </row>
+    <row r="32" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A32" s="6"/>
       <c r="B32" s="6"/>
       <c r="C32" s="50"/>
@@ -8661,15 +8763,15 @@
       <c r="CD32" s="60"/>
       <c r="CE32" s="37"/>
       <c r="CF32" s="61"/>
-      <c r="CG32" s="35"/>
-      <c r="CH32" s="35"/>
-      <c r="CI32" s="35"/>
+      <c r="CG32" s="61"/>
+      <c r="CH32" s="61"/>
+      <c r="CI32" s="61"/>
       <c r="CJ32" s="35"/>
       <c r="CK32" s="35"/>
       <c r="CL32" s="35"/>
       <c r="CM32" s="35"/>
       <c r="CN32" s="35"/>
-      <c r="CO32" s="64"/>
+      <c r="CO32" s="35"/>
       <c r="CP32" s="35"/>
       <c r="CQ32" s="35"/>
       <c r="CR32" s="64"/>
@@ -8699,12 +8801,15 @@
       <c r="DP32" s="64"/>
       <c r="DQ32" s="35"/>
       <c r="DR32" s="35"/>
-      <c r="DS32" s="35"/>
+      <c r="DS32" s="64"/>
       <c r="DT32" s="35"/>
       <c r="DU32" s="35"/>
       <c r="DV32" s="35"/>
-    </row>
-    <row r="33" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW32" s="35"/>
+      <c r="DX32" s="35"/>
+      <c r="DY32" s="35"/>
+    </row>
+    <row r="33" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A33" s="6"/>
       <c r="B33" s="6"/>
       <c r="C33" s="50"/>
@@ -8779,9 +8884,9 @@
       <c r="CD33" s="60"/>
       <c r="CE33" s="37"/>
       <c r="CF33" s="37"/>
-      <c r="CG33" s="35"/>
-      <c r="CH33" s="35"/>
-      <c r="CI33" s="35"/>
+      <c r="CG33" s="37"/>
+      <c r="CH33" s="37"/>
+      <c r="CI33" s="37"/>
       <c r="CJ33" s="35"/>
       <c r="CK33" s="35"/>
       <c r="CL33" s="35"/>
@@ -8821,8 +8926,11 @@
       <c r="DT33" s="35"/>
       <c r="DU33" s="35"/>
       <c r="DV33" s="35"/>
-    </row>
-    <row r="34" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW33" s="35"/>
+      <c r="DX33" s="35"/>
+      <c r="DY33" s="35"/>
+    </row>
+    <row r="34" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A34" s="6"/>
       <c r="B34" s="6"/>
       <c r="C34" s="50"/>
@@ -8897,9 +9005,9 @@
       <c r="CD34" s="60"/>
       <c r="CE34" s="37"/>
       <c r="CF34" s="61"/>
-      <c r="CG34" s="35"/>
-      <c r="CH34" s="35"/>
-      <c r="CI34" s="35"/>
+      <c r="CG34" s="61"/>
+      <c r="CH34" s="61"/>
+      <c r="CI34" s="61"/>
       <c r="CJ34" s="35"/>
       <c r="CK34" s="35"/>
       <c r="CL34" s="35"/>
@@ -8939,8 +9047,11 @@
       <c r="DT34" s="35"/>
       <c r="DU34" s="35"/>
       <c r="DV34" s="35"/>
-    </row>
-    <row r="35" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW34" s="35"/>
+      <c r="DX34" s="35"/>
+      <c r="DY34" s="35"/>
+    </row>
+    <row r="35" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A35" s="6"/>
       <c r="B35" s="6"/>
       <c r="C35" s="50"/>
@@ -9015,9 +9126,9 @@
       <c r="CD35" s="60"/>
       <c r="CE35" s="37"/>
       <c r="CF35" s="37"/>
-      <c r="CG35" s="35"/>
-      <c r="CH35" s="35"/>
-      <c r="CI35" s="35"/>
+      <c r="CG35" s="37"/>
+      <c r="CH35" s="37"/>
+      <c r="CI35" s="37"/>
       <c r="CJ35" s="35"/>
       <c r="CK35" s="35"/>
       <c r="CL35" s="35"/>
@@ -9057,8 +9168,11 @@
       <c r="DT35" s="35"/>
       <c r="DU35" s="35"/>
       <c r="DV35" s="35"/>
-    </row>
-    <row r="36" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW35" s="35"/>
+      <c r="DX35" s="35"/>
+      <c r="DY35" s="35"/>
+    </row>
+    <row r="36" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A36" s="6"/>
       <c r="B36" s="6"/>
       <c r="C36" s="50"/>
@@ -9133,9 +9247,9 @@
       <c r="CD36" s="60"/>
       <c r="CE36" s="37"/>
       <c r="CF36" s="37"/>
-      <c r="CG36" s="35"/>
-      <c r="CH36" s="35"/>
-      <c r="CI36" s="35"/>
+      <c r="CG36" s="37"/>
+      <c r="CH36" s="37"/>
+      <c r="CI36" s="37"/>
       <c r="CJ36" s="35"/>
       <c r="CK36" s="35"/>
       <c r="CL36" s="35"/>
@@ -9175,8 +9289,11 @@
       <c r="DT36" s="35"/>
       <c r="DU36" s="35"/>
       <c r="DV36" s="35"/>
-    </row>
-    <row r="37" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW36" s="35"/>
+      <c r="DX36" s="35"/>
+      <c r="DY36" s="35"/>
+    </row>
+    <row r="37" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A37" s="6"/>
       <c r="B37" s="6"/>
       <c r="C37" s="50"/>
@@ -9251,9 +9368,9 @@
       <c r="CD37" s="60"/>
       <c r="CE37" s="37"/>
       <c r="CF37" s="37"/>
-      <c r="CG37" s="35"/>
-      <c r="CH37" s="35"/>
-      <c r="CI37" s="35"/>
+      <c r="CG37" s="37"/>
+      <c r="CH37" s="37"/>
+      <c r="CI37" s="37"/>
       <c r="CJ37" s="35"/>
       <c r="CK37" s="35"/>
       <c r="CL37" s="35"/>
@@ -9293,8 +9410,11 @@
       <c r="DT37" s="35"/>
       <c r="DU37" s="35"/>
       <c r="DV37" s="35"/>
-    </row>
-    <row r="38" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW37" s="35"/>
+      <c r="DX37" s="35"/>
+      <c r="DY37" s="35"/>
+    </row>
+    <row r="38" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A38" s="6"/>
       <c r="B38" s="6"/>
       <c r="C38" s="50"/>
@@ -9369,9 +9489,9 @@
       <c r="CD38" s="60"/>
       <c r="CE38" s="37"/>
       <c r="CF38" s="37"/>
-      <c r="CG38" s="35"/>
-      <c r="CH38" s="35"/>
-      <c r="CI38" s="35"/>
+      <c r="CG38" s="37"/>
+      <c r="CH38" s="37"/>
+      <c r="CI38" s="37"/>
       <c r="CJ38" s="35"/>
       <c r="CK38" s="35"/>
       <c r="CL38" s="35"/>
@@ -9411,8 +9531,11 @@
       <c r="DT38" s="35"/>
       <c r="DU38" s="35"/>
       <c r="DV38" s="35"/>
-    </row>
-    <row r="39" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW38" s="35"/>
+      <c r="DX38" s="35"/>
+      <c r="DY38" s="35"/>
+    </row>
+    <row r="39" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A39" s="6"/>
       <c r="B39" s="6"/>
       <c r="C39" s="50"/>
@@ -9487,15 +9610,15 @@
       <c r="CD39" s="60"/>
       <c r="CE39" s="37"/>
       <c r="CF39" s="61"/>
-      <c r="CG39" s="35"/>
-      <c r="CH39" s="35"/>
-      <c r="CI39" s="35"/>
+      <c r="CG39" s="61"/>
+      <c r="CH39" s="61"/>
+      <c r="CI39" s="61"/>
       <c r="CJ39" s="35"/>
       <c r="CK39" s="35"/>
       <c r="CL39" s="35"/>
       <c r="CM39" s="35"/>
       <c r="CN39" s="35"/>
-      <c r="CO39" s="64"/>
+      <c r="CO39" s="35"/>
       <c r="CP39" s="35"/>
       <c r="CQ39" s="35"/>
       <c r="CR39" s="64"/>
@@ -9504,7 +9627,7 @@
       <c r="CU39" s="64"/>
       <c r="CV39" s="35"/>
       <c r="CW39" s="35"/>
-      <c r="CX39" s="35"/>
+      <c r="CX39" s="64"/>
       <c r="CY39" s="35"/>
       <c r="CZ39" s="35"/>
       <c r="DA39" s="35"/>
@@ -9526,11 +9649,14 @@
       <c r="DQ39" s="35"/>
       <c r="DR39" s="35"/>
       <c r="DS39" s="35"/>
-      <c r="DT39" s="64"/>
+      <c r="DT39" s="35"/>
       <c r="DU39" s="35"/>
       <c r="DV39" s="35"/>
-    </row>
-    <row r="40" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW39" s="64"/>
+      <c r="DX39" s="35"/>
+      <c r="DY39" s="35"/>
+    </row>
+    <row r="40" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A40" s="6"/>
       <c r="B40" s="6"/>
       <c r="C40" s="50"/>
@@ -9605,9 +9731,9 @@
       <c r="CD40" s="60"/>
       <c r="CE40" s="37"/>
       <c r="CF40" s="37"/>
-      <c r="CG40" s="35"/>
-      <c r="CH40" s="35"/>
-      <c r="CI40" s="35"/>
+      <c r="CG40" s="37"/>
+      <c r="CH40" s="37"/>
+      <c r="CI40" s="37"/>
       <c r="CJ40" s="35"/>
       <c r="CK40" s="35"/>
       <c r="CL40" s="35"/>
@@ -9647,8 +9773,11 @@
       <c r="DT40" s="35"/>
       <c r="DU40" s="35"/>
       <c r="DV40" s="35"/>
-    </row>
-    <row r="41" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW40" s="35"/>
+      <c r="DX40" s="35"/>
+      <c r="DY40" s="35"/>
+    </row>
+    <row r="41" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A41" s="6"/>
       <c r="B41" s="6"/>
       <c r="C41" s="50"/>
@@ -9723,9 +9852,9 @@
       <c r="CD41" s="60"/>
       <c r="CE41" s="37"/>
       <c r="CF41" s="37"/>
-      <c r="CG41" s="35"/>
-      <c r="CH41" s="35"/>
-      <c r="CI41" s="35"/>
+      <c r="CG41" s="37"/>
+      <c r="CH41" s="37"/>
+      <c r="CI41" s="37"/>
       <c r="CJ41" s="35"/>
       <c r="CK41" s="35"/>
       <c r="CL41" s="35"/>
@@ -9765,8 +9894,11 @@
       <c r="DT41" s="35"/>
       <c r="DU41" s="35"/>
       <c r="DV41" s="35"/>
-    </row>
-    <row r="42" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW41" s="35"/>
+      <c r="DX41" s="35"/>
+      <c r="DY41" s="35"/>
+    </row>
+    <row r="42" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A42" s="6"/>
       <c r="B42" s="6"/>
       <c r="C42" s="50"/>
@@ -9841,9 +9973,9 @@
       <c r="CD42" s="60"/>
       <c r="CE42" s="37"/>
       <c r="CF42" s="37"/>
-      <c r="CG42" s="35"/>
-      <c r="CH42" s="35"/>
-      <c r="CI42" s="35"/>
+      <c r="CG42" s="37"/>
+      <c r="CH42" s="37"/>
+      <c r="CI42" s="37"/>
       <c r="CJ42" s="35"/>
       <c r="CK42" s="35"/>
       <c r="CL42" s="35"/>
@@ -9883,8 +10015,11 @@
       <c r="DT42" s="35"/>
       <c r="DU42" s="35"/>
       <c r="DV42" s="35"/>
-    </row>
-    <row r="43" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW42" s="35"/>
+      <c r="DX42" s="35"/>
+      <c r="DY42" s="35"/>
+    </row>
+    <row r="43" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A43" s="6"/>
       <c r="B43" s="6"/>
       <c r="C43" s="50"/>
@@ -9959,16 +10094,16 @@
       <c r="CD43" s="60"/>
       <c r="CE43" s="37"/>
       <c r="CF43" s="61"/>
-      <c r="CG43" s="35"/>
-      <c r="CH43" s="35"/>
-      <c r="CI43" s="35"/>
+      <c r="CG43" s="61"/>
+      <c r="CH43" s="61"/>
+      <c r="CI43" s="61"/>
       <c r="CJ43" s="35"/>
       <c r="CK43" s="35"/>
       <c r="CL43" s="35"/>
-      <c r="CM43" s="64"/>
+      <c r="CM43" s="35"/>
       <c r="CN43" s="35"/>
-      <c r="CO43" s="64"/>
-      <c r="CP43" s="35"/>
+      <c r="CO43" s="35"/>
+      <c r="CP43" s="64"/>
       <c r="CQ43" s="35"/>
       <c r="CR43" s="64"/>
       <c r="CS43" s="35"/>
@@ -9997,12 +10132,15 @@
       <c r="DP43" s="64"/>
       <c r="DQ43" s="35"/>
       <c r="DR43" s="35"/>
-      <c r="DS43" s="35"/>
+      <c r="DS43" s="64"/>
       <c r="DT43" s="35"/>
       <c r="DU43" s="35"/>
       <c r="DV43" s="35"/>
-    </row>
-    <row r="44" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW43" s="35"/>
+      <c r="DX43" s="35"/>
+      <c r="DY43" s="35"/>
+    </row>
+    <row r="44" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A44" s="6"/>
       <c r="B44" s="6"/>
       <c r="C44" s="50"/>
@@ -10077,9 +10215,9 @@
       <c r="CD44" s="60"/>
       <c r="CE44" s="61"/>
       <c r="CF44" s="61"/>
-      <c r="CG44" s="35"/>
-      <c r="CH44" s="35"/>
-      <c r="CI44" s="35"/>
+      <c r="CG44" s="61"/>
+      <c r="CH44" s="61"/>
+      <c r="CI44" s="61"/>
       <c r="CJ44" s="35"/>
       <c r="CK44" s="35"/>
       <c r="CL44" s="35"/>
@@ -10119,8 +10257,11 @@
       <c r="DT44" s="35"/>
       <c r="DU44" s="35"/>
       <c r="DV44" s="35"/>
-    </row>
-    <row r="45" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW44" s="35"/>
+      <c r="DX44" s="35"/>
+      <c r="DY44" s="35"/>
+    </row>
+    <row r="45" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A45" s="6"/>
       <c r="B45" s="6"/>
       <c r="C45" s="50"/>
@@ -10195,9 +10336,9 @@
       <c r="CD45" s="60"/>
       <c r="CE45" s="37"/>
       <c r="CF45" s="61"/>
-      <c r="CG45" s="35"/>
-      <c r="CH45" s="35"/>
-      <c r="CI45" s="35"/>
+      <c r="CG45" s="61"/>
+      <c r="CH45" s="61"/>
+      <c r="CI45" s="61"/>
       <c r="CJ45" s="35"/>
       <c r="CK45" s="35"/>
       <c r="CL45" s="35"/>
@@ -10237,8 +10378,11 @@
       <c r="DT45" s="35"/>
       <c r="DU45" s="35"/>
       <c r="DV45" s="35"/>
-    </row>
-    <row r="46" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW45" s="35"/>
+      <c r="DX45" s="35"/>
+      <c r="DY45" s="35"/>
+    </row>
+    <row r="46" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A46" s="6"/>
       <c r="B46" s="6"/>
       <c r="C46" s="50"/>
@@ -10313,9 +10457,9 @@
       <c r="CD46" s="60"/>
       <c r="CE46" s="37"/>
       <c r="CF46" s="37"/>
-      <c r="CG46" s="35"/>
-      <c r="CH46" s="35"/>
-      <c r="CI46" s="35"/>
+      <c r="CG46" s="37"/>
+      <c r="CH46" s="37"/>
+      <c r="CI46" s="37"/>
       <c r="CJ46" s="35"/>
       <c r="CK46" s="35"/>
       <c r="CL46" s="35"/>
@@ -10355,8 +10499,11 @@
       <c r="DT46" s="35"/>
       <c r="DU46" s="35"/>
       <c r="DV46" s="35"/>
-    </row>
-    <row r="47" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW46" s="35"/>
+      <c r="DX46" s="35"/>
+      <c r="DY46" s="35"/>
+    </row>
+    <row r="47" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A47" s="6"/>
       <c r="B47" s="6"/>
       <c r="C47" s="50"/>
@@ -10431,15 +10578,15 @@
       <c r="CD47" s="60"/>
       <c r="CE47" s="37"/>
       <c r="CF47" s="61"/>
-      <c r="CG47" s="35"/>
-      <c r="CH47" s="64"/>
-      <c r="CI47" s="35"/>
+      <c r="CG47" s="61"/>
+      <c r="CH47" s="61"/>
+      <c r="CI47" s="61"/>
       <c r="CJ47" s="35"/>
-      <c r="CK47" s="35"/>
+      <c r="CK47" s="64"/>
       <c r="CL47" s="35"/>
       <c r="CM47" s="35"/>
       <c r="CN47" s="35"/>
-      <c r="CO47" s="64"/>
+      <c r="CO47" s="35"/>
       <c r="CP47" s="35"/>
       <c r="CQ47" s="35"/>
       <c r="CR47" s="64"/>
@@ -10469,12 +10616,15 @@
       <c r="DP47" s="64"/>
       <c r="DQ47" s="35"/>
       <c r="DR47" s="35"/>
-      <c r="DS47" s="35"/>
+      <c r="DS47" s="64"/>
       <c r="DT47" s="35"/>
       <c r="DU47" s="35"/>
       <c r="DV47" s="35"/>
-    </row>
-    <row r="48" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW47" s="35"/>
+      <c r="DX47" s="35"/>
+      <c r="DY47" s="35"/>
+    </row>
+    <row r="48" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A48" s="6"/>
       <c r="B48" s="6"/>
       <c r="C48" s="50"/>
@@ -10549,15 +10699,15 @@
       <c r="CD48" s="60"/>
       <c r="CE48" s="37"/>
       <c r="CF48" s="61"/>
-      <c r="CG48" s="35"/>
-      <c r="CH48" s="35"/>
-      <c r="CI48" s="35"/>
+      <c r="CG48" s="61"/>
+      <c r="CH48" s="61"/>
+      <c r="CI48" s="61"/>
       <c r="CJ48" s="35"/>
       <c r="CK48" s="35"/>
       <c r="CL48" s="35"/>
       <c r="CM48" s="35"/>
       <c r="CN48" s="35"/>
-      <c r="CO48" s="64"/>
+      <c r="CO48" s="35"/>
       <c r="CP48" s="35"/>
       <c r="CQ48" s="35"/>
       <c r="CR48" s="64"/>
@@ -10587,12 +10737,15 @@
       <c r="DP48" s="64"/>
       <c r="DQ48" s="35"/>
       <c r="DR48" s="35"/>
-      <c r="DS48" s="35"/>
+      <c r="DS48" s="64"/>
       <c r="DT48" s="35"/>
       <c r="DU48" s="35"/>
       <c r="DV48" s="35"/>
-    </row>
-    <row r="49" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW48" s="35"/>
+      <c r="DX48" s="35"/>
+      <c r="DY48" s="35"/>
+    </row>
+    <row r="49" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A49" s="6"/>
       <c r="B49" s="6"/>
       <c r="C49" s="50"/>
@@ -10667,9 +10820,9 @@
       <c r="CD49" s="60"/>
       <c r="CE49" s="37"/>
       <c r="CF49" s="61"/>
-      <c r="CG49" s="35"/>
-      <c r="CH49" s="35"/>
-      <c r="CI49" s="35"/>
+      <c r="CG49" s="61"/>
+      <c r="CH49" s="61"/>
+      <c r="CI49" s="61"/>
       <c r="CJ49" s="35"/>
       <c r="CK49" s="35"/>
       <c r="CL49" s="35"/>
@@ -10709,8 +10862,11 @@
       <c r="DT49" s="35"/>
       <c r="DU49" s="35"/>
       <c r="DV49" s="35"/>
-    </row>
-    <row r="50" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW49" s="35"/>
+      <c r="DX49" s="35"/>
+      <c r="DY49" s="35"/>
+    </row>
+    <row r="50" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A50" s="6"/>
       <c r="B50" s="6"/>
       <c r="C50" s="50"/>
@@ -10785,9 +10941,9 @@
       <c r="CD50" s="60"/>
       <c r="CE50" s="37"/>
       <c r="CF50" s="37"/>
-      <c r="CG50" s="35"/>
-      <c r="CH50" s="35"/>
-      <c r="CI50" s="35"/>
+      <c r="CG50" s="37"/>
+      <c r="CH50" s="37"/>
+      <c r="CI50" s="37"/>
       <c r="CJ50" s="35"/>
       <c r="CK50" s="35"/>
       <c r="CL50" s="35"/>
@@ -10827,8 +10983,11 @@
       <c r="DT50" s="35"/>
       <c r="DU50" s="35"/>
       <c r="DV50" s="35"/>
-    </row>
-    <row r="51" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW50" s="35"/>
+      <c r="DX50" s="35"/>
+      <c r="DY50" s="35"/>
+    </row>
+    <row r="51" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A51" s="6"/>
       <c r="B51" s="6"/>
       <c r="C51" s="50"/>
@@ -10903,21 +11062,21 @@
       <c r="CD51" s="60"/>
       <c r="CE51" s="37"/>
       <c r="CF51" s="61"/>
-      <c r="CG51" s="35"/>
-      <c r="CH51" s="35"/>
-      <c r="CI51" s="35"/>
+      <c r="CG51" s="61"/>
+      <c r="CH51" s="61"/>
+      <c r="CI51" s="61"/>
       <c r="CJ51" s="35"/>
       <c r="CK51" s="35"/>
       <c r="CL51" s="35"/>
       <c r="CM51" s="35"/>
       <c r="CN51" s="35"/>
-      <c r="CO51" s="64"/>
+      <c r="CO51" s="35"/>
       <c r="CP51" s="35"/>
       <c r="CQ51" s="35"/>
       <c r="CR51" s="64"/>
       <c r="CS51" s="35"/>
       <c r="CT51" s="35"/>
-      <c r="CU51" s="35"/>
+      <c r="CU51" s="64"/>
       <c r="CV51" s="35"/>
       <c r="CW51" s="35"/>
       <c r="CX51" s="35"/>
@@ -10942,11 +11101,14 @@
       <c r="DQ51" s="35"/>
       <c r="DR51" s="35"/>
       <c r="DS51" s="35"/>
-      <c r="DT51" s="64"/>
+      <c r="DT51" s="35"/>
       <c r="DU51" s="35"/>
       <c r="DV51" s="35"/>
-    </row>
-    <row r="52" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW51" s="64"/>
+      <c r="DX51" s="35"/>
+      <c r="DY51" s="35"/>
+    </row>
+    <row r="52" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A52" s="6"/>
       <c r="B52" s="6"/>
       <c r="C52" s="50"/>
@@ -11021,9 +11183,9 @@
       <c r="CD52" s="60"/>
       <c r="CE52" s="37"/>
       <c r="CF52" s="37"/>
-      <c r="CG52" s="35"/>
-      <c r="CH52" s="35"/>
-      <c r="CI52" s="35"/>
+      <c r="CG52" s="37"/>
+      <c r="CH52" s="37"/>
+      <c r="CI52" s="37"/>
       <c r="CJ52" s="35"/>
       <c r="CK52" s="35"/>
       <c r="CL52" s="35"/>
@@ -11063,8 +11225,11 @@
       <c r="DT52" s="35"/>
       <c r="DU52" s="35"/>
       <c r="DV52" s="35"/>
-    </row>
-    <row r="53" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW52" s="35"/>
+      <c r="DX52" s="35"/>
+      <c r="DY52" s="35"/>
+    </row>
+    <row r="53" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A53" s="6"/>
       <c r="B53" s="6"/>
       <c r="C53" s="50"/>
@@ -11139,9 +11304,9 @@
       <c r="CD53" s="60"/>
       <c r="CE53" s="37"/>
       <c r="CF53" s="37"/>
-      <c r="CG53" s="35"/>
-      <c r="CH53" s="35"/>
-      <c r="CI53" s="35"/>
+      <c r="CG53" s="37"/>
+      <c r="CH53" s="37"/>
+      <c r="CI53" s="37"/>
       <c r="CJ53" s="35"/>
       <c r="CK53" s="35"/>
       <c r="CL53" s="35"/>
@@ -11181,8 +11346,11 @@
       <c r="DT53" s="35"/>
       <c r="DU53" s="35"/>
       <c r="DV53" s="35"/>
-    </row>
-    <row r="54" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW53" s="35"/>
+      <c r="DX53" s="35"/>
+      <c r="DY53" s="35"/>
+    </row>
+    <row r="54" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A54" s="6"/>
       <c r="B54" s="6"/>
       <c r="C54" s="50"/>
@@ -11257,9 +11425,9 @@
       <c r="CD54" s="60"/>
       <c r="CE54" s="37"/>
       <c r="CF54" s="61"/>
-      <c r="CG54" s="35"/>
-      <c r="CH54" s="35"/>
-      <c r="CI54" s="35"/>
+      <c r="CG54" s="61"/>
+      <c r="CH54" s="61"/>
+      <c r="CI54" s="61"/>
       <c r="CJ54" s="35"/>
       <c r="CK54" s="35"/>
       <c r="CL54" s="35"/>
@@ -11299,8 +11467,11 @@
       <c r="DT54" s="35"/>
       <c r="DU54" s="35"/>
       <c r="DV54" s="35"/>
-    </row>
-    <row r="55" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW54" s="35"/>
+      <c r="DX54" s="35"/>
+      <c r="DY54" s="35"/>
+    </row>
+    <row r="55" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A55" s="6"/>
       <c r="B55" s="6"/>
       <c r="C55" s="50"/>
@@ -11375,9 +11546,9 @@
       <c r="CD55" s="60"/>
       <c r="CE55" s="37"/>
       <c r="CF55" s="61"/>
-      <c r="CG55" s="35"/>
-      <c r="CH55" s="35"/>
-      <c r="CI55" s="35"/>
+      <c r="CG55" s="61"/>
+      <c r="CH55" s="61"/>
+      <c r="CI55" s="61"/>
       <c r="CJ55" s="35"/>
       <c r="CK55" s="35"/>
       <c r="CL55" s="35"/>
@@ -11417,8 +11588,11 @@
       <c r="DT55" s="35"/>
       <c r="DU55" s="35"/>
       <c r="DV55" s="35"/>
-    </row>
-    <row r="56" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW55" s="35"/>
+      <c r="DX55" s="35"/>
+      <c r="DY55" s="35"/>
+    </row>
+    <row r="56" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A56" s="6"/>
       <c r="B56" s="6"/>
       <c r="C56" s="50"/>
@@ -11493,9 +11667,9 @@
       <c r="CD56" s="60"/>
       <c r="CE56" s="37"/>
       <c r="CF56" s="37"/>
-      <c r="CG56" s="35"/>
-      <c r="CH56" s="35"/>
-      <c r="CI56" s="35"/>
+      <c r="CG56" s="37"/>
+      <c r="CH56" s="37"/>
+      <c r="CI56" s="37"/>
       <c r="CJ56" s="35"/>
       <c r="CK56" s="35"/>
       <c r="CL56" s="35"/>
@@ -11535,8 +11709,11 @@
       <c r="DT56" s="35"/>
       <c r="DU56" s="35"/>
       <c r="DV56" s="35"/>
-    </row>
-    <row r="57" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW56" s="35"/>
+      <c r="DX56" s="35"/>
+      <c r="DY56" s="35"/>
+    </row>
+    <row r="57" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A57" s="6"/>
       <c r="B57" s="6"/>
       <c r="C57" s="50"/>
@@ -11611,9 +11788,9 @@
       <c r="CD57" s="60"/>
       <c r="CE57" s="37"/>
       <c r="CF57" s="61"/>
-      <c r="CG57" s="35"/>
-      <c r="CH57" s="35"/>
-      <c r="CI57" s="35"/>
+      <c r="CG57" s="61"/>
+      <c r="CH57" s="61"/>
+      <c r="CI57" s="61"/>
       <c r="CJ57" s="35"/>
       <c r="CK57" s="35"/>
       <c r="CL57" s="35"/>
@@ -11653,8 +11830,11 @@
       <c r="DT57" s="35"/>
       <c r="DU57" s="35"/>
       <c r="DV57" s="35"/>
-    </row>
-    <row r="58" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW57" s="35"/>
+      <c r="DX57" s="35"/>
+      <c r="DY57" s="35"/>
+    </row>
+    <row r="58" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A58" s="6"/>
       <c r="B58" s="6"/>
       <c r="C58" s="50"/>
@@ -11729,9 +11909,9 @@
       <c r="CD58" s="60"/>
       <c r="CE58" s="37"/>
       <c r="CF58" s="61"/>
-      <c r="CG58" s="35"/>
-      <c r="CH58" s="35"/>
-      <c r="CI58" s="35"/>
+      <c r="CG58" s="61"/>
+      <c r="CH58" s="61"/>
+      <c r="CI58" s="61"/>
       <c r="CJ58" s="35"/>
       <c r="CK58" s="35"/>
       <c r="CL58" s="35"/>
@@ -11771,8 +11951,11 @@
       <c r="DT58" s="35"/>
       <c r="DU58" s="35"/>
       <c r="DV58" s="35"/>
-    </row>
-    <row r="59" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW58" s="35"/>
+      <c r="DX58" s="35"/>
+      <c r="DY58" s="35"/>
+    </row>
+    <row r="59" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A59" s="6"/>
       <c r="B59" s="6"/>
       <c r="C59" s="50"/>
@@ -11847,9 +12030,9 @@
       <c r="CD59" s="60"/>
       <c r="CE59" s="37"/>
       <c r="CF59" s="37"/>
-      <c r="CG59" s="35"/>
-      <c r="CH59" s="35"/>
-      <c r="CI59" s="35"/>
+      <c r="CG59" s="37"/>
+      <c r="CH59" s="37"/>
+      <c r="CI59" s="37"/>
       <c r="CJ59" s="35"/>
       <c r="CK59" s="35"/>
       <c r="CL59" s="35"/>
@@ -11889,8 +12072,11 @@
       <c r="DT59" s="35"/>
       <c r="DU59" s="35"/>
       <c r="DV59" s="35"/>
-    </row>
-    <row r="60" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW59" s="35"/>
+      <c r="DX59" s="35"/>
+      <c r="DY59" s="35"/>
+    </row>
+    <row r="60" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A60" s="6"/>
       <c r="B60" s="6"/>
       <c r="C60" s="50"/>
@@ -11965,9 +12151,9 @@
       <c r="CD60" s="60"/>
       <c r="CE60" s="37"/>
       <c r="CF60" s="37"/>
-      <c r="CG60" s="35"/>
-      <c r="CH60" s="35"/>
-      <c r="CI60" s="35"/>
+      <c r="CG60" s="37"/>
+      <c r="CH60" s="37"/>
+      <c r="CI60" s="37"/>
       <c r="CJ60" s="35"/>
       <c r="CK60" s="35"/>
       <c r="CL60" s="35"/>
@@ -12007,8 +12193,11 @@
       <c r="DT60" s="35"/>
       <c r="DU60" s="35"/>
       <c r="DV60" s="35"/>
-    </row>
-    <row r="61" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW60" s="35"/>
+      <c r="DX60" s="35"/>
+      <c r="DY60" s="35"/>
+    </row>
+    <row r="61" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A61" s="6"/>
       <c r="B61" s="6"/>
       <c r="C61" s="50"/>
@@ -12083,15 +12272,15 @@
       <c r="CD61" s="60"/>
       <c r="CE61" s="37"/>
       <c r="CF61" s="61"/>
-      <c r="CG61" s="35"/>
-      <c r="CH61" s="35"/>
-      <c r="CI61" s="35"/>
+      <c r="CG61" s="61"/>
+      <c r="CH61" s="61"/>
+      <c r="CI61" s="61"/>
       <c r="CJ61" s="35"/>
       <c r="CK61" s="35"/>
       <c r="CL61" s="35"/>
       <c r="CM61" s="35"/>
       <c r="CN61" s="35"/>
-      <c r="CO61" s="64"/>
+      <c r="CO61" s="35"/>
       <c r="CP61" s="35"/>
       <c r="CQ61" s="35"/>
       <c r="CR61" s="64"/>
@@ -12121,12 +12310,15 @@
       <c r="DP61" s="64"/>
       <c r="DQ61" s="35"/>
       <c r="DR61" s="35"/>
-      <c r="DS61" s="35"/>
+      <c r="DS61" s="64"/>
       <c r="DT61" s="35"/>
       <c r="DU61" s="35"/>
       <c r="DV61" s="35"/>
-    </row>
-    <row r="62" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW61" s="35"/>
+      <c r="DX61" s="35"/>
+      <c r="DY61" s="35"/>
+    </row>
+    <row r="62" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A62" s="6"/>
       <c r="B62" s="6"/>
       <c r="C62" s="50"/>
@@ -12201,16 +12393,16 @@
       <c r="CD62" s="60"/>
       <c r="CE62" s="37"/>
       <c r="CF62" s="61"/>
-      <c r="CG62" s="35"/>
-      <c r="CH62" s="35"/>
-      <c r="CI62" s="35"/>
+      <c r="CG62" s="61"/>
+      <c r="CH62" s="61"/>
+      <c r="CI62" s="61"/>
       <c r="CJ62" s="35"/>
       <c r="CK62" s="35"/>
       <c r="CL62" s="35"/>
-      <c r="CM62" s="64"/>
+      <c r="CM62" s="35"/>
       <c r="CN62" s="35"/>
-      <c r="CO62" s="64"/>
-      <c r="CP62" s="35"/>
+      <c r="CO62" s="35"/>
+      <c r="CP62" s="64"/>
       <c r="CQ62" s="35"/>
       <c r="CR62" s="64"/>
       <c r="CS62" s="35"/>
@@ -12239,12 +12431,15 @@
       <c r="DP62" s="64"/>
       <c r="DQ62" s="35"/>
       <c r="DR62" s="35"/>
-      <c r="DS62" s="35"/>
+      <c r="DS62" s="64"/>
       <c r="DT62" s="35"/>
       <c r="DU62" s="35"/>
       <c r="DV62" s="35"/>
-    </row>
-    <row r="63" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW62" s="35"/>
+      <c r="DX62" s="35"/>
+      <c r="DY62" s="35"/>
+    </row>
+    <row r="63" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A63" s="6"/>
       <c r="B63" s="6"/>
       <c r="C63" s="50"/>
@@ -12319,15 +12514,15 @@
       <c r="CD63" s="60"/>
       <c r="CE63" s="37"/>
       <c r="CF63" s="61"/>
-      <c r="CG63" s="35"/>
-      <c r="CH63" s="35"/>
-      <c r="CI63" s="35"/>
+      <c r="CG63" s="61"/>
+      <c r="CH63" s="61"/>
+      <c r="CI63" s="61"/>
       <c r="CJ63" s="35"/>
       <c r="CK63" s="35"/>
       <c r="CL63" s="35"/>
       <c r="CM63" s="35"/>
       <c r="CN63" s="35"/>
-      <c r="CO63" s="64"/>
+      <c r="CO63" s="35"/>
       <c r="CP63" s="35"/>
       <c r="CQ63" s="35"/>
       <c r="CR63" s="64"/>
@@ -12357,12 +12552,15 @@
       <c r="DP63" s="64"/>
       <c r="DQ63" s="35"/>
       <c r="DR63" s="35"/>
-      <c r="DS63" s="35"/>
+      <c r="DS63" s="64"/>
       <c r="DT63" s="35"/>
       <c r="DU63" s="35"/>
       <c r="DV63" s="35"/>
-    </row>
-    <row r="64" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW63" s="35"/>
+      <c r="DX63" s="35"/>
+      <c r="DY63" s="35"/>
+    </row>
+    <row r="64" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A64" s="6"/>
       <c r="B64" s="6"/>
       <c r="C64" s="50"/>
@@ -12437,21 +12635,21 @@
       <c r="CD64" s="60"/>
       <c r="CE64" s="37"/>
       <c r="CF64" s="61"/>
-      <c r="CG64" s="35"/>
-      <c r="CH64" s="64"/>
-      <c r="CI64" s="35"/>
+      <c r="CG64" s="61"/>
+      <c r="CH64" s="61"/>
+      <c r="CI64" s="61"/>
       <c r="CJ64" s="35"/>
-      <c r="CK64" s="35"/>
+      <c r="CK64" s="64"/>
       <c r="CL64" s="35"/>
       <c r="CM64" s="35"/>
       <c r="CN64" s="35"/>
-      <c r="CO64" s="64"/>
+      <c r="CO64" s="35"/>
       <c r="CP64" s="35"/>
       <c r="CQ64" s="35"/>
       <c r="CR64" s="64"/>
       <c r="CS64" s="35"/>
       <c r="CT64" s="35"/>
-      <c r="CU64" s="35"/>
+      <c r="CU64" s="64"/>
       <c r="CV64" s="35"/>
       <c r="CW64" s="35"/>
       <c r="CX64" s="35"/>
@@ -12476,11 +12674,14 @@
       <c r="DQ64" s="35"/>
       <c r="DR64" s="35"/>
       <c r="DS64" s="35"/>
-      <c r="DT64" s="64"/>
+      <c r="DT64" s="35"/>
       <c r="DU64" s="35"/>
       <c r="DV64" s="35"/>
-    </row>
-    <row r="65" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW64" s="64"/>
+      <c r="DX64" s="35"/>
+      <c r="DY64" s="35"/>
+    </row>
+    <row r="65" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A65" s="6"/>
       <c r="B65" s="6"/>
       <c r="C65" s="50"/>
@@ -12555,15 +12756,15 @@
       <c r="CD65" s="60"/>
       <c r="CE65" s="37"/>
       <c r="CF65" s="61"/>
-      <c r="CG65" s="35"/>
-      <c r="CH65" s="64"/>
-      <c r="CI65" s="35"/>
+      <c r="CG65" s="61"/>
+      <c r="CH65" s="61"/>
+      <c r="CI65" s="61"/>
       <c r="CJ65" s="35"/>
-      <c r="CK65" s="35"/>
+      <c r="CK65" s="64"/>
       <c r="CL65" s="35"/>
       <c r="CM65" s="35"/>
       <c r="CN65" s="35"/>
-      <c r="CO65" s="64"/>
+      <c r="CO65" s="35"/>
       <c r="CP65" s="35"/>
       <c r="CQ65" s="35"/>
       <c r="CR65" s="64"/>
@@ -12584,7 +12785,7 @@
       <c r="DG65" s="64"/>
       <c r="DH65" s="35"/>
       <c r="DI65" s="35"/>
-      <c r="DJ65" s="35"/>
+      <c r="DJ65" s="64"/>
       <c r="DK65" s="35"/>
       <c r="DL65" s="35"/>
       <c r="DM65" s="35"/>
@@ -12594,11 +12795,14 @@
       <c r="DQ65" s="35"/>
       <c r="DR65" s="35"/>
       <c r="DS65" s="35"/>
-      <c r="DT65" s="64"/>
+      <c r="DT65" s="35"/>
       <c r="DU65" s="35"/>
       <c r="DV65" s="35"/>
-    </row>
-    <row r="66" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW65" s="64"/>
+      <c r="DX65" s="35"/>
+      <c r="DY65" s="35"/>
+    </row>
+    <row r="66" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A66" s="6"/>
       <c r="B66" s="6"/>
       <c r="C66" s="50"/>
@@ -12673,9 +12877,9 @@
       <c r="CD66" s="60"/>
       <c r="CE66" s="37"/>
       <c r="CF66" s="37"/>
-      <c r="CG66" s="35"/>
-      <c r="CH66" s="35"/>
-      <c r="CI66" s="35"/>
+      <c r="CG66" s="37"/>
+      <c r="CH66" s="37"/>
+      <c r="CI66" s="37"/>
       <c r="CJ66" s="35"/>
       <c r="CK66" s="35"/>
       <c r="CL66" s="35"/>
@@ -12715,8 +12919,11 @@
       <c r="DT66" s="35"/>
       <c r="DU66" s="35"/>
       <c r="DV66" s="35"/>
-    </row>
-    <row r="67" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW66" s="35"/>
+      <c r="DX66" s="35"/>
+      <c r="DY66" s="35"/>
+    </row>
+    <row r="67" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A67" s="6"/>
       <c r="B67" s="6"/>
       <c r="C67" s="50"/>
@@ -12791,9 +12998,9 @@
       <c r="CD67" s="60"/>
       <c r="CE67" s="37"/>
       <c r="CF67" s="37"/>
-      <c r="CG67" s="35"/>
-      <c r="CH67" s="35"/>
-      <c r="CI67" s="35"/>
+      <c r="CG67" s="37"/>
+      <c r="CH67" s="37"/>
+      <c r="CI67" s="37"/>
       <c r="CJ67" s="35"/>
       <c r="CK67" s="35"/>
       <c r="CL67" s="35"/>
@@ -12833,8 +13040,11 @@
       <c r="DT67" s="35"/>
       <c r="DU67" s="35"/>
       <c r="DV67" s="35"/>
-    </row>
-    <row r="68" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW67" s="35"/>
+      <c r="DX67" s="35"/>
+      <c r="DY67" s="35"/>
+    </row>
+    <row r="68" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A68" s="6"/>
       <c r="B68" s="6"/>
       <c r="C68" s="50"/>
@@ -12909,9 +13119,9 @@
       <c r="CD68" s="60"/>
       <c r="CE68" s="37"/>
       <c r="CF68" s="37"/>
-      <c r="CG68" s="35"/>
-      <c r="CH68" s="35"/>
-      <c r="CI68" s="35"/>
+      <c r="CG68" s="37"/>
+      <c r="CH68" s="37"/>
+      <c r="CI68" s="37"/>
       <c r="CJ68" s="35"/>
       <c r="CK68" s="35"/>
       <c r="CL68" s="35"/>
@@ -12951,8 +13161,11 @@
       <c r="DT68" s="35"/>
       <c r="DU68" s="35"/>
       <c r="DV68" s="35"/>
-    </row>
-    <row r="69" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW68" s="35"/>
+      <c r="DX68" s="35"/>
+      <c r="DY68" s="35"/>
+    </row>
+    <row r="69" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A69" s="6"/>
       <c r="B69" s="6"/>
       <c r="C69" s="50"/>
@@ -13027,9 +13240,9 @@
       <c r="CD69" s="60"/>
       <c r="CE69" s="37"/>
       <c r="CF69" s="37"/>
-      <c r="CG69" s="35"/>
-      <c r="CH69" s="35"/>
-      <c r="CI69" s="35"/>
+      <c r="CG69" s="37"/>
+      <c r="CH69" s="37"/>
+      <c r="CI69" s="37"/>
       <c r="CJ69" s="35"/>
       <c r="CK69" s="35"/>
       <c r="CL69" s="35"/>
@@ -13069,8 +13282,11 @@
       <c r="DT69" s="35"/>
       <c r="DU69" s="35"/>
       <c r="DV69" s="35"/>
-    </row>
-    <row r="70" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW69" s="35"/>
+      <c r="DX69" s="35"/>
+      <c r="DY69" s="35"/>
+    </row>
+    <row r="70" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A70" s="6"/>
       <c r="B70" s="6"/>
       <c r="C70" s="50"/>
@@ -13145,9 +13361,9 @@
       <c r="CD70" s="60"/>
       <c r="CE70" s="37"/>
       <c r="CF70" s="37"/>
-      <c r="CG70" s="35"/>
-      <c r="CH70" s="35"/>
-      <c r="CI70" s="35"/>
+      <c r="CG70" s="37"/>
+      <c r="CH70" s="37"/>
+      <c r="CI70" s="37"/>
       <c r="CJ70" s="35"/>
       <c r="CK70" s="35"/>
       <c r="CL70" s="35"/>
@@ -13187,8 +13403,11 @@
       <c r="DT70" s="35"/>
       <c r="DU70" s="35"/>
       <c r="DV70" s="35"/>
-    </row>
-    <row r="71" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW70" s="35"/>
+      <c r="DX70" s="35"/>
+      <c r="DY70" s="35"/>
+    </row>
+    <row r="71" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A71" s="6"/>
       <c r="B71" s="6"/>
       <c r="C71" s="50"/>
@@ -13263,9 +13482,9 @@
       <c r="CD71" s="60"/>
       <c r="CE71" s="37"/>
       <c r="CF71" s="37"/>
-      <c r="CG71" s="35"/>
-      <c r="CH71" s="35"/>
-      <c r="CI71" s="35"/>
+      <c r="CG71" s="37"/>
+      <c r="CH71" s="37"/>
+      <c r="CI71" s="37"/>
       <c r="CJ71" s="35"/>
       <c r="CK71" s="35"/>
       <c r="CL71" s="35"/>
@@ -13305,8 +13524,11 @@
       <c r="DT71" s="35"/>
       <c r="DU71" s="35"/>
       <c r="DV71" s="35"/>
-    </row>
-    <row r="72" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW71" s="35"/>
+      <c r="DX71" s="35"/>
+      <c r="DY71" s="35"/>
+    </row>
+    <row r="72" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A72" s="6"/>
       <c r="B72" s="6"/>
       <c r="C72" s="50"/>
@@ -13381,9 +13603,9 @@
       <c r="CD72" s="60"/>
       <c r="CE72" s="37"/>
       <c r="CF72" s="37"/>
-      <c r="CG72" s="35"/>
-      <c r="CH72" s="35"/>
-      <c r="CI72" s="35"/>
+      <c r="CG72" s="37"/>
+      <c r="CH72" s="37"/>
+      <c r="CI72" s="37"/>
       <c r="CJ72" s="35"/>
       <c r="CK72" s="35"/>
       <c r="CL72" s="35"/>
@@ -13423,8 +13645,11 @@
       <c r="DT72" s="35"/>
       <c r="DU72" s="35"/>
       <c r="DV72" s="35"/>
-    </row>
-    <row r="73" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW72" s="35"/>
+      <c r="DX72" s="35"/>
+      <c r="DY72" s="35"/>
+    </row>
+    <row r="73" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A73" s="6"/>
       <c r="B73" s="6"/>
       <c r="C73" s="50"/>
@@ -13499,9 +13724,9 @@
       <c r="CD73" s="60"/>
       <c r="CE73" s="37"/>
       <c r="CF73" s="37"/>
-      <c r="CG73" s="35"/>
-      <c r="CH73" s="35"/>
-      <c r="CI73" s="35"/>
+      <c r="CG73" s="37"/>
+      <c r="CH73" s="37"/>
+      <c r="CI73" s="37"/>
       <c r="CJ73" s="35"/>
       <c r="CK73" s="35"/>
       <c r="CL73" s="35"/>
@@ -13541,8 +13766,11 @@
       <c r="DT73" s="35"/>
       <c r="DU73" s="35"/>
       <c r="DV73" s="35"/>
-    </row>
-    <row r="74" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW73" s="35"/>
+      <c r="DX73" s="35"/>
+      <c r="DY73" s="35"/>
+    </row>
+    <row r="74" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A74" s="6"/>
       <c r="B74" s="6"/>
       <c r="C74" s="50"/>
@@ -13617,15 +13845,15 @@
       <c r="CD74" s="60"/>
       <c r="CE74" s="37"/>
       <c r="CF74" s="61"/>
-      <c r="CG74" s="35"/>
-      <c r="CH74" s="35"/>
-      <c r="CI74" s="35"/>
+      <c r="CG74" s="61"/>
+      <c r="CH74" s="61"/>
+      <c r="CI74" s="61"/>
       <c r="CJ74" s="35"/>
       <c r="CK74" s="35"/>
       <c r="CL74" s="35"/>
       <c r="CM74" s="35"/>
       <c r="CN74" s="35"/>
-      <c r="CO74" s="64"/>
+      <c r="CO74" s="35"/>
       <c r="CP74" s="35"/>
       <c r="CQ74" s="35"/>
       <c r="CR74" s="64"/>
@@ -13652,15 +13880,18 @@
       <c r="DM74" s="64"/>
       <c r="DN74" s="35"/>
       <c r="DO74" s="35"/>
-      <c r="DP74" s="35"/>
+      <c r="DP74" s="64"/>
       <c r="DQ74" s="35"/>
       <c r="DR74" s="35"/>
       <c r="DS74" s="35"/>
       <c r="DT74" s="35"/>
       <c r="DU74" s="35"/>
       <c r="DV74" s="35"/>
-    </row>
-    <row r="75" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW74" s="35"/>
+      <c r="DX74" s="35"/>
+      <c r="DY74" s="35"/>
+    </row>
+    <row r="75" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A75" s="6"/>
       <c r="B75" s="6"/>
       <c r="C75" s="50"/>
@@ -13735,9 +13966,9 @@
       <c r="CD75" s="60"/>
       <c r="CE75" s="37"/>
       <c r="CF75" s="37"/>
-      <c r="CG75" s="35"/>
-      <c r="CH75" s="35"/>
-      <c r="CI75" s="35"/>
+      <c r="CG75" s="37"/>
+      <c r="CH75" s="37"/>
+      <c r="CI75" s="37"/>
       <c r="CJ75" s="35"/>
       <c r="CK75" s="35"/>
       <c r="CL75" s="35"/>
@@ -13777,8 +14008,11 @@
       <c r="DT75" s="35"/>
       <c r="DU75" s="35"/>
       <c r="DV75" s="35"/>
-    </row>
-    <row r="76" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW75" s="35"/>
+      <c r="DX75" s="35"/>
+      <c r="DY75" s="35"/>
+    </row>
+    <row r="76" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A76" s="6"/>
       <c r="B76" s="6"/>
       <c r="C76" s="50"/>
@@ -13853,9 +14087,9 @@
       <c r="CD76" s="60"/>
       <c r="CE76" s="37"/>
       <c r="CF76" s="37"/>
-      <c r="CG76" s="35"/>
-      <c r="CH76" s="35"/>
-      <c r="CI76" s="35"/>
+      <c r="CG76" s="37"/>
+      <c r="CH76" s="37"/>
+      <c r="CI76" s="37"/>
       <c r="CJ76" s="35"/>
       <c r="CK76" s="35"/>
       <c r="CL76" s="35"/>
@@ -13895,8 +14129,11 @@
       <c r="DT76" s="35"/>
       <c r="DU76" s="35"/>
       <c r="DV76" s="35"/>
-    </row>
-    <row r="77" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW76" s="35"/>
+      <c r="DX76" s="35"/>
+      <c r="DY76" s="35"/>
+    </row>
+    <row r="77" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A77" s="6"/>
       <c r="B77" s="6"/>
       <c r="C77" s="50"/>
@@ -13971,9 +14208,9 @@
       <c r="CD77" s="60"/>
       <c r="CE77" s="37"/>
       <c r="CF77" s="61"/>
-      <c r="CG77" s="35"/>
-      <c r="CH77" s="35"/>
-      <c r="CI77" s="35"/>
+      <c r="CG77" s="61"/>
+      <c r="CH77" s="61"/>
+      <c r="CI77" s="61"/>
       <c r="CJ77" s="35"/>
       <c r="CK77" s="35"/>
       <c r="CL77" s="35"/>
@@ -14013,8 +14250,11 @@
       <c r="DT77" s="35"/>
       <c r="DU77" s="35"/>
       <c r="DV77" s="35"/>
-    </row>
-    <row r="78" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW77" s="35"/>
+      <c r="DX77" s="35"/>
+      <c r="DY77" s="35"/>
+    </row>
+    <row r="78" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A78" s="6"/>
       <c r="B78" s="6"/>
       <c r="C78" s="50"/>
@@ -14089,9 +14329,9 @@
       <c r="CD78" s="60"/>
       <c r="CE78" s="37"/>
       <c r="CF78" s="37"/>
-      <c r="CG78" s="35"/>
-      <c r="CH78" s="35"/>
-      <c r="CI78" s="35"/>
+      <c r="CG78" s="37"/>
+      <c r="CH78" s="37"/>
+      <c r="CI78" s="37"/>
       <c r="CJ78" s="35"/>
       <c r="CK78" s="35"/>
       <c r="CL78" s="35"/>
@@ -14131,8 +14371,11 @@
       <c r="DT78" s="35"/>
       <c r="DU78" s="35"/>
       <c r="DV78" s="35"/>
-    </row>
-    <row r="79" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW78" s="35"/>
+      <c r="DX78" s="35"/>
+      <c r="DY78" s="35"/>
+    </row>
+    <row r="79" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A79" s="6"/>
       <c r="B79" s="6"/>
       <c r="C79" s="50"/>
@@ -14207,15 +14450,15 @@
       <c r="CD79" s="60"/>
       <c r="CE79" s="37"/>
       <c r="CF79" s="61"/>
-      <c r="CG79" s="35"/>
-      <c r="CH79" s="35"/>
-      <c r="CI79" s="35"/>
+      <c r="CG79" s="61"/>
+      <c r="CH79" s="61"/>
+      <c r="CI79" s="61"/>
       <c r="CJ79" s="35"/>
       <c r="CK79" s="35"/>
       <c r="CL79" s="35"/>
       <c r="CM79" s="35"/>
       <c r="CN79" s="35"/>
-      <c r="CO79" s="64"/>
+      <c r="CO79" s="35"/>
       <c r="CP79" s="35"/>
       <c r="CQ79" s="35"/>
       <c r="CR79" s="64"/>
@@ -14245,12 +14488,15 @@
       <c r="DP79" s="64"/>
       <c r="DQ79" s="35"/>
       <c r="DR79" s="35"/>
-      <c r="DS79" s="35"/>
+      <c r="DS79" s="64"/>
       <c r="DT79" s="35"/>
       <c r="DU79" s="35"/>
       <c r="DV79" s="35"/>
-    </row>
-    <row r="80" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW79" s="35"/>
+      <c r="DX79" s="35"/>
+      <c r="DY79" s="35"/>
+    </row>
+    <row r="80" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A80" s="6"/>
       <c r="B80" s="6"/>
       <c r="C80" s="50"/>
@@ -14325,9 +14571,9 @@
       <c r="CD80" s="60"/>
       <c r="CE80" s="37"/>
       <c r="CF80" s="37"/>
-      <c r="CG80" s="35"/>
-      <c r="CH80" s="35"/>
-      <c r="CI80" s="35"/>
+      <c r="CG80" s="37"/>
+      <c r="CH80" s="37"/>
+      <c r="CI80" s="37"/>
       <c r="CJ80" s="35"/>
       <c r="CK80" s="35"/>
       <c r="CL80" s="35"/>
@@ -14367,8 +14613,11 @@
       <c r="DT80" s="35"/>
       <c r="DU80" s="35"/>
       <c r="DV80" s="35"/>
-    </row>
-    <row r="81" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW80" s="35"/>
+      <c r="DX80" s="35"/>
+      <c r="DY80" s="35"/>
+    </row>
+    <row r="81" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A81" s="6"/>
       <c r="B81" s="6"/>
       <c r="C81" s="50"/>
@@ -14443,16 +14692,16 @@
       <c r="CD81" s="60"/>
       <c r="CE81" s="37"/>
       <c r="CF81" s="61"/>
-      <c r="CG81" s="35"/>
-      <c r="CH81" s="35"/>
-      <c r="CI81" s="35"/>
+      <c r="CG81" s="61"/>
+      <c r="CH81" s="61"/>
+      <c r="CI81" s="61"/>
       <c r="CJ81" s="35"/>
       <c r="CK81" s="35"/>
       <c r="CL81" s="35"/>
-      <c r="CM81" s="64"/>
+      <c r="CM81" s="35"/>
       <c r="CN81" s="35"/>
-      <c r="CO81" s="64"/>
-      <c r="CP81" s="35"/>
+      <c r="CO81" s="35"/>
+      <c r="CP81" s="64"/>
       <c r="CQ81" s="35"/>
       <c r="CR81" s="64"/>
       <c r="CS81" s="35"/>
@@ -14463,7 +14712,7 @@
       <c r="CX81" s="64"/>
       <c r="CY81" s="35"/>
       <c r="CZ81" s="35"/>
-      <c r="DA81" s="35"/>
+      <c r="DA81" s="64"/>
       <c r="DB81" s="35"/>
       <c r="DC81" s="35"/>
       <c r="DD81" s="35"/>
@@ -14485,8 +14734,11 @@
       <c r="DT81" s="35"/>
       <c r="DU81" s="35"/>
       <c r="DV81" s="35"/>
-    </row>
-    <row r="82" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW81" s="35"/>
+      <c r="DX81" s="35"/>
+      <c r="DY81" s="35"/>
+    </row>
+    <row r="82" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A82" s="6"/>
       <c r="B82" s="6"/>
       <c r="C82" s="50"/>
@@ -14561,18 +14813,18 @@
       <c r="CD82" s="60"/>
       <c r="CE82" s="37"/>
       <c r="CF82" s="61"/>
-      <c r="CG82" s="35"/>
-      <c r="CH82" s="35"/>
-      <c r="CI82" s="35"/>
+      <c r="CG82" s="61"/>
+      <c r="CH82" s="61"/>
+      <c r="CI82" s="61"/>
       <c r="CJ82" s="35"/>
       <c r="CK82" s="35"/>
       <c r="CL82" s="35"/>
       <c r="CM82" s="35"/>
       <c r="CN82" s="35"/>
-      <c r="CO82" s="64"/>
+      <c r="CO82" s="35"/>
       <c r="CP82" s="35"/>
       <c r="CQ82" s="35"/>
-      <c r="CR82" s="35"/>
+      <c r="CR82" s="64"/>
       <c r="CS82" s="35"/>
       <c r="CT82" s="35"/>
       <c r="CU82" s="35"/>
@@ -14600,11 +14852,14 @@
       <c r="DQ82" s="35"/>
       <c r="DR82" s="35"/>
       <c r="DS82" s="35"/>
-      <c r="DT82" s="64"/>
+      <c r="DT82" s="35"/>
       <c r="DU82" s="35"/>
       <c r="DV82" s="35"/>
-    </row>
-    <row r="83" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW82" s="64"/>
+      <c r="DX82" s="35"/>
+      <c r="DY82" s="35"/>
+    </row>
+    <row r="83" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A83" s="6"/>
       <c r="B83" s="6"/>
       <c r="C83" s="50"/>
@@ -14679,24 +14934,24 @@
       <c r="CD83" s="60"/>
       <c r="CE83" s="37"/>
       <c r="CF83" s="61"/>
-      <c r="CG83" s="35"/>
-      <c r="CH83" s="35"/>
-      <c r="CI83" s="35"/>
+      <c r="CG83" s="61"/>
+      <c r="CH83" s="61"/>
+      <c r="CI83" s="61"/>
       <c r="CJ83" s="35"/>
       <c r="CK83" s="35"/>
       <c r="CL83" s="35"/>
-      <c r="CM83" s="64"/>
+      <c r="CM83" s="35"/>
       <c r="CN83" s="35"/>
-      <c r="CO83" s="64"/>
-      <c r="CP83" s="35"/>
+      <c r="CO83" s="35"/>
+      <c r="CP83" s="64"/>
       <c r="CQ83" s="35"/>
       <c r="CR83" s="64"/>
       <c r="CS83" s="35"/>
       <c r="CT83" s="35"/>
-      <c r="CU83" s="80"/>
+      <c r="CU83" s="64"/>
+      <c r="CV83" s="35"/>
       <c r="CW83" s="35"/>
-      <c r="CX83" s="64"/>
-      <c r="CY83" s="35"/>
+      <c r="CX83" s="80"/>
       <c r="CZ83" s="35"/>
       <c r="DA83" s="64"/>
       <c r="DB83" s="35"/>
@@ -14716,12 +14971,15 @@
       <c r="DP83" s="64"/>
       <c r="DQ83" s="35"/>
       <c r="DR83" s="35"/>
-      <c r="DS83" s="35"/>
+      <c r="DS83" s="64"/>
       <c r="DT83" s="35"/>
       <c r="DU83" s="35"/>
       <c r="DV83" s="35"/>
-    </row>
-    <row r="84" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW83" s="35"/>
+      <c r="DX83" s="35"/>
+      <c r="DY83" s="35"/>
+    </row>
+    <row r="84" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A84" s="6"/>
       <c r="B84" s="6"/>
       <c r="C84" s="50"/>
@@ -14796,9 +15054,9 @@
       <c r="CD84" s="60"/>
       <c r="CE84" s="37"/>
       <c r="CF84" s="37"/>
-      <c r="CG84" s="35"/>
-      <c r="CH84" s="35"/>
-      <c r="CI84" s="35"/>
+      <c r="CG84" s="37"/>
+      <c r="CH84" s="37"/>
+      <c r="CI84" s="37"/>
       <c r="CJ84" s="35"/>
       <c r="CK84" s="35"/>
       <c r="CL84" s="35"/>
@@ -14838,8 +15096,11 @@
       <c r="DT84" s="35"/>
       <c r="DU84" s="35"/>
       <c r="DV84" s="35"/>
-    </row>
-    <row r="85" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW84" s="35"/>
+      <c r="DX84" s="35"/>
+      <c r="DY84" s="35"/>
+    </row>
+    <row r="85" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A85" s="6"/>
       <c r="B85" s="6"/>
       <c r="C85" s="50"/>
@@ -14914,9 +15175,9 @@
       <c r="CD85" s="60"/>
       <c r="CE85" s="37"/>
       <c r="CF85" s="37"/>
-      <c r="CG85" s="35"/>
-      <c r="CH85" s="35"/>
-      <c r="CI85" s="35"/>
+      <c r="CG85" s="37"/>
+      <c r="CH85" s="37"/>
+      <c r="CI85" s="37"/>
       <c r="CJ85" s="35"/>
       <c r="CK85" s="35"/>
       <c r="CL85" s="35"/>
@@ -14956,8 +15217,11 @@
       <c r="DT85" s="35"/>
       <c r="DU85" s="35"/>
       <c r="DV85" s="35"/>
-    </row>
-    <row r="86" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW85" s="35"/>
+      <c r="DX85" s="35"/>
+      <c r="DY85" s="35"/>
+    </row>
+    <row r="86" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A86" s="6"/>
       <c r="B86" s="6"/>
       <c r="C86" s="50"/>
@@ -15032,9 +15296,9 @@
       <c r="CD86" s="60"/>
       <c r="CE86" s="37"/>
       <c r="CF86" s="37"/>
-      <c r="CG86" s="35"/>
-      <c r="CH86" s="35"/>
-      <c r="CI86" s="35"/>
+      <c r="CG86" s="37"/>
+      <c r="CH86" s="37"/>
+      <c r="CI86" s="37"/>
       <c r="CJ86" s="35"/>
       <c r="CK86" s="35"/>
       <c r="CL86" s="35"/>
@@ -15074,8 +15338,11 @@
       <c r="DT86" s="35"/>
       <c r="DU86" s="35"/>
       <c r="DV86" s="35"/>
-    </row>
-    <row r="87" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW86" s="35"/>
+      <c r="DX86" s="35"/>
+      <c r="DY86" s="35"/>
+    </row>
+    <row r="87" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A87" s="6"/>
       <c r="B87" s="6"/>
       <c r="C87" s="50"/>
@@ -15150,9 +15417,9 @@
       <c r="CD87" s="60"/>
       <c r="CE87" s="37"/>
       <c r="CF87" s="37"/>
-      <c r="CG87" s="35"/>
-      <c r="CH87" s="35"/>
-      <c r="CI87" s="35"/>
+      <c r="CG87" s="37"/>
+      <c r="CH87" s="37"/>
+      <c r="CI87" s="37"/>
       <c r="CJ87" s="35"/>
       <c r="CK87" s="35"/>
       <c r="CL87" s="35"/>
@@ -15192,8 +15459,11 @@
       <c r="DT87" s="35"/>
       <c r="DU87" s="35"/>
       <c r="DV87" s="35"/>
-    </row>
-    <row r="88" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW87" s="35"/>
+      <c r="DX87" s="35"/>
+      <c r="DY87" s="35"/>
+    </row>
+    <row r="88" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A88" s="6"/>
       <c r="B88" s="6"/>
       <c r="C88" s="50"/>
@@ -15268,9 +15538,9 @@
       <c r="CD88" s="60"/>
       <c r="CE88" s="37"/>
       <c r="CF88" s="37"/>
-      <c r="CG88" s="35"/>
-      <c r="CH88" s="35"/>
-      <c r="CI88" s="35"/>
+      <c r="CG88" s="37"/>
+      <c r="CH88" s="37"/>
+      <c r="CI88" s="37"/>
       <c r="CJ88" s="35"/>
       <c r="CK88" s="35"/>
       <c r="CL88" s="35"/>
@@ -15310,8 +15580,11 @@
       <c r="DT88" s="35"/>
       <c r="DU88" s="35"/>
       <c r="DV88" s="35"/>
-    </row>
-    <row r="89" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW88" s="35"/>
+      <c r="DX88" s="35"/>
+      <c r="DY88" s="35"/>
+    </row>
+    <row r="89" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A89" s="6"/>
       <c r="B89" s="6"/>
       <c r="C89" s="50"/>
@@ -15386,9 +15659,9 @@
       <c r="CD89" s="60"/>
       <c r="CE89" s="37"/>
       <c r="CF89" s="37"/>
-      <c r="CG89" s="35"/>
-      <c r="CH89" s="35"/>
-      <c r="CI89" s="35"/>
+      <c r="CG89" s="37"/>
+      <c r="CH89" s="37"/>
+      <c r="CI89" s="37"/>
       <c r="CJ89" s="35"/>
       <c r="CK89" s="35"/>
       <c r="CL89" s="35"/>
@@ -15428,8 +15701,11 @@
       <c r="DT89" s="35"/>
       <c r="DU89" s="35"/>
       <c r="DV89" s="35"/>
-    </row>
-    <row r="90" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW89" s="35"/>
+      <c r="DX89" s="35"/>
+      <c r="DY89" s="35"/>
+    </row>
+    <row r="90" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A90" s="6"/>
       <c r="B90" s="6"/>
       <c r="C90" s="50"/>
@@ -15504,9 +15780,9 @@
       <c r="CD90" s="60"/>
       <c r="CE90" s="37"/>
       <c r="CF90" s="37"/>
-      <c r="CG90" s="35"/>
-      <c r="CH90" s="35"/>
-      <c r="CI90" s="35"/>
+      <c r="CG90" s="37"/>
+      <c r="CH90" s="37"/>
+      <c r="CI90" s="37"/>
       <c r="CJ90" s="35"/>
       <c r="CK90" s="35"/>
       <c r="CL90" s="35"/>
@@ -15546,8 +15822,11 @@
       <c r="DT90" s="35"/>
       <c r="DU90" s="35"/>
       <c r="DV90" s="35"/>
-    </row>
-    <row r="91" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW90" s="35"/>
+      <c r="DX90" s="35"/>
+      <c r="DY90" s="35"/>
+    </row>
+    <row r="91" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A91" s="6"/>
       <c r="B91" s="6"/>
       <c r="C91" s="50"/>
@@ -15622,16 +15901,16 @@
       <c r="CD91" s="60"/>
       <c r="CE91" s="37"/>
       <c r="CF91" s="61"/>
-      <c r="CG91" s="35"/>
-      <c r="CH91" s="35"/>
-      <c r="CI91" s="35"/>
+      <c r="CG91" s="61"/>
+      <c r="CH91" s="61"/>
+      <c r="CI91" s="61"/>
       <c r="CJ91" s="35"/>
       <c r="CK91" s="35"/>
       <c r="CL91" s="35"/>
-      <c r="CM91" s="64"/>
+      <c r="CM91" s="35"/>
       <c r="CN91" s="35"/>
-      <c r="CO91" s="64"/>
-      <c r="CP91" s="35"/>
+      <c r="CO91" s="35"/>
+      <c r="CP91" s="64"/>
       <c r="CQ91" s="35"/>
       <c r="CR91" s="64"/>
       <c r="CS91" s="35"/>
@@ -15651,7 +15930,7 @@
       <c r="DG91" s="64"/>
       <c r="DH91" s="35"/>
       <c r="DI91" s="35"/>
-      <c r="DJ91" s="35"/>
+      <c r="DJ91" s="64"/>
       <c r="DK91" s="35"/>
       <c r="DL91" s="35"/>
       <c r="DM91" s="35"/>
@@ -15664,8 +15943,11 @@
       <c r="DT91" s="35"/>
       <c r="DU91" s="35"/>
       <c r="DV91" s="35"/>
-    </row>
-    <row r="92" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW91" s="35"/>
+      <c r="DX91" s="35"/>
+      <c r="DY91" s="35"/>
+    </row>
+    <row r="92" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A92" s="6"/>
       <c r="B92" s="6"/>
       <c r="C92" s="50"/>
@@ -15740,9 +16022,9 @@
       <c r="CD92" s="60"/>
       <c r="CE92" s="37"/>
       <c r="CF92" s="37"/>
-      <c r="CG92" s="35"/>
-      <c r="CH92" s="35"/>
-      <c r="CI92" s="35"/>
+      <c r="CG92" s="37"/>
+      <c r="CH92" s="37"/>
+      <c r="CI92" s="37"/>
       <c r="CJ92" s="35"/>
       <c r="CK92" s="35"/>
       <c r="CL92" s="35"/>
@@ -15782,8 +16064,11 @@
       <c r="DT92" s="35"/>
       <c r="DU92" s="35"/>
       <c r="DV92" s="35"/>
-    </row>
-    <row r="93" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW92" s="35"/>
+      <c r="DX92" s="35"/>
+      <c r="DY92" s="35"/>
+    </row>
+    <row r="93" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A93" s="6"/>
       <c r="B93" s="6"/>
       <c r="C93" s="50"/>
@@ -15858,15 +16143,15 @@
       <c r="CD93" s="60"/>
       <c r="CE93" s="37"/>
       <c r="CF93" s="61"/>
-      <c r="CG93" s="35"/>
-      <c r="CH93" s="35"/>
-      <c r="CI93" s="35"/>
+      <c r="CG93" s="61"/>
+      <c r="CH93" s="61"/>
+      <c r="CI93" s="61"/>
       <c r="CJ93" s="35"/>
       <c r="CK93" s="35"/>
       <c r="CL93" s="35"/>
       <c r="CM93" s="35"/>
       <c r="CN93" s="35"/>
-      <c r="CO93" s="64"/>
+      <c r="CO93" s="35"/>
       <c r="CP93" s="35"/>
       <c r="CQ93" s="35"/>
       <c r="CR93" s="64"/>
@@ -15893,15 +16178,18 @@
       <c r="DM93" s="64"/>
       <c r="DN93" s="35"/>
       <c r="DO93" s="35"/>
-      <c r="DP93" s="35"/>
+      <c r="DP93" s="64"/>
       <c r="DQ93" s="35"/>
       <c r="DR93" s="35"/>
       <c r="DS93" s="35"/>
       <c r="DT93" s="35"/>
       <c r="DU93" s="35"/>
       <c r="DV93" s="35"/>
-    </row>
-    <row r="94" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW93" s="35"/>
+      <c r="DX93" s="35"/>
+      <c r="DY93" s="35"/>
+    </row>
+    <row r="94" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A94" s="6"/>
       <c r="B94" s="6"/>
       <c r="C94" s="50"/>
@@ -15976,9 +16264,9 @@
       <c r="CD94" s="60"/>
       <c r="CE94" s="37"/>
       <c r="CF94" s="37"/>
-      <c r="CG94" s="35"/>
-      <c r="CH94" s="35"/>
-      <c r="CI94" s="35"/>
+      <c r="CG94" s="37"/>
+      <c r="CH94" s="37"/>
+      <c r="CI94" s="37"/>
       <c r="CJ94" s="35"/>
       <c r="CK94" s="35"/>
       <c r="CL94" s="35"/>
@@ -16018,8 +16306,11 @@
       <c r="DT94" s="35"/>
       <c r="DU94" s="35"/>
       <c r="DV94" s="35"/>
-    </row>
-    <row r="95" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW94" s="35"/>
+      <c r="DX94" s="35"/>
+      <c r="DY94" s="35"/>
+    </row>
+    <row r="95" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A95" s="6"/>
       <c r="B95" s="6"/>
       <c r="C95" s="50"/>
@@ -16094,9 +16385,9 @@
       <c r="CD95" s="60"/>
       <c r="CE95" s="37"/>
       <c r="CF95" s="37"/>
-      <c r="CG95" s="35"/>
-      <c r="CH95" s="35"/>
-      <c r="CI95" s="35"/>
+      <c r="CG95" s="37"/>
+      <c r="CH95" s="37"/>
+      <c r="CI95" s="37"/>
       <c r="CJ95" s="35"/>
       <c r="CK95" s="35"/>
       <c r="CL95" s="35"/>
@@ -16136,8 +16427,11 @@
       <c r="DT95" s="35"/>
       <c r="DU95" s="35"/>
       <c r="DV95" s="35"/>
-    </row>
-    <row r="96" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW95" s="35"/>
+      <c r="DX95" s="35"/>
+      <c r="DY95" s="35"/>
+    </row>
+    <row r="96" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A96" s="6"/>
       <c r="B96" s="6"/>
       <c r="C96" s="50"/>
@@ -16212,9 +16506,9 @@
       <c r="CD96" s="60"/>
       <c r="CE96" s="37"/>
       <c r="CF96" s="37"/>
-      <c r="CG96" s="35"/>
-      <c r="CH96" s="35"/>
-      <c r="CI96" s="35"/>
+      <c r="CG96" s="37"/>
+      <c r="CH96" s="37"/>
+      <c r="CI96" s="37"/>
       <c r="CJ96" s="35"/>
       <c r="CK96" s="35"/>
       <c r="CL96" s="35"/>
@@ -16254,8 +16548,11 @@
       <c r="DT96" s="35"/>
       <c r="DU96" s="35"/>
       <c r="DV96" s="35"/>
-    </row>
-    <row r="97" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW96" s="35"/>
+      <c r="DX96" s="35"/>
+      <c r="DY96" s="35"/>
+    </row>
+    <row r="97" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A97" s="6"/>
       <c r="B97" s="6"/>
       <c r="C97" s="50"/>
@@ -16330,9 +16627,9 @@
       <c r="CD97" s="60"/>
       <c r="CE97" s="37"/>
       <c r="CF97" s="37"/>
-      <c r="CG97" s="35"/>
-      <c r="CH97" s="35"/>
-      <c r="CI97" s="35"/>
+      <c r="CG97" s="37"/>
+      <c r="CH97" s="37"/>
+      <c r="CI97" s="37"/>
       <c r="CJ97" s="35"/>
       <c r="CK97" s="35"/>
       <c r="CL97" s="35"/>
@@ -16372,8 +16669,11 @@
       <c r="DT97" s="35"/>
       <c r="DU97" s="35"/>
       <c r="DV97" s="35"/>
-    </row>
-    <row r="98" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW97" s="35"/>
+      <c r="DX97" s="35"/>
+      <c r="DY97" s="35"/>
+    </row>
+    <row r="98" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A98" s="6"/>
       <c r="B98" s="6"/>
       <c r="C98" s="50"/>
@@ -16448,9 +16748,9 @@
       <c r="CD98" s="60"/>
       <c r="CE98" s="37"/>
       <c r="CF98" s="37"/>
-      <c r="CG98" s="35"/>
-      <c r="CH98" s="35"/>
-      <c r="CI98" s="35"/>
+      <c r="CG98" s="37"/>
+      <c r="CH98" s="37"/>
+      <c r="CI98" s="37"/>
       <c r="CJ98" s="35"/>
       <c r="CK98" s="35"/>
       <c r="CL98" s="35"/>
@@ -16490,8 +16790,11 @@
       <c r="DT98" s="35"/>
       <c r="DU98" s="35"/>
       <c r="DV98" s="35"/>
-    </row>
-    <row r="99" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW98" s="35"/>
+      <c r="DX98" s="35"/>
+      <c r="DY98" s="35"/>
+    </row>
+    <row r="99" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A99" s="6"/>
       <c r="B99" s="6"/>
       <c r="C99" s="50"/>
@@ -16566,9 +16869,9 @@
       <c r="CD99" s="60"/>
       <c r="CE99" s="37"/>
       <c r="CF99" s="37"/>
-      <c r="CG99" s="35"/>
-      <c r="CH99" s="35"/>
-      <c r="CI99" s="35"/>
+      <c r="CG99" s="37"/>
+      <c r="CH99" s="37"/>
+      <c r="CI99" s="37"/>
       <c r="CJ99" s="35"/>
       <c r="CK99" s="35"/>
       <c r="CL99" s="35"/>
@@ -16608,8 +16911,11 @@
       <c r="DT99" s="35"/>
       <c r="DU99" s="35"/>
       <c r="DV99" s="35"/>
-    </row>
-    <row r="100" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW99" s="35"/>
+      <c r="DX99" s="35"/>
+      <c r="DY99" s="35"/>
+    </row>
+    <row r="100" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A100" s="6"/>
       <c r="B100" s="6"/>
       <c r="C100" s="50"/>
@@ -16684,9 +16990,9 @@
       <c r="CD100" s="60"/>
       <c r="CE100" s="37"/>
       <c r="CF100" s="37"/>
-      <c r="CG100" s="35"/>
-      <c r="CH100" s="35"/>
-      <c r="CI100" s="35"/>
+      <c r="CG100" s="37"/>
+      <c r="CH100" s="37"/>
+      <c r="CI100" s="37"/>
       <c r="CJ100" s="35"/>
       <c r="CK100" s="35"/>
       <c r="CL100" s="35"/>
@@ -16726,8 +17032,11 @@
       <c r="DT100" s="35"/>
       <c r="DU100" s="35"/>
       <c r="DV100" s="35"/>
-    </row>
-    <row r="101" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW100" s="35"/>
+      <c r="DX100" s="35"/>
+      <c r="DY100" s="35"/>
+    </row>
+    <row r="101" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A101" s="6"/>
       <c r="B101" s="6"/>
       <c r="C101" s="50"/>
@@ -16802,9 +17111,9 @@
       <c r="CD101" s="60"/>
       <c r="CE101" s="37"/>
       <c r="CF101" s="37"/>
-      <c r="CG101" s="35"/>
-      <c r="CH101" s="35"/>
-      <c r="CI101" s="35"/>
+      <c r="CG101" s="37"/>
+      <c r="CH101" s="37"/>
+      <c r="CI101" s="37"/>
       <c r="CJ101" s="35"/>
       <c r="CK101" s="35"/>
       <c r="CL101" s="35"/>
@@ -16844,8 +17153,11 @@
       <c r="DT101" s="35"/>
       <c r="DU101" s="35"/>
       <c r="DV101" s="35"/>
-    </row>
-    <row r="102" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW101" s="35"/>
+      <c r="DX101" s="35"/>
+      <c r="DY101" s="35"/>
+    </row>
+    <row r="102" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A102" s="6"/>
       <c r="B102" s="6"/>
       <c r="C102" s="50"/>
@@ -16920,9 +17232,9 @@
       <c r="CD102" s="60"/>
       <c r="CE102" s="37"/>
       <c r="CF102" s="61"/>
-      <c r="CG102" s="35"/>
-      <c r="CH102" s="35"/>
-      <c r="CI102" s="35"/>
+      <c r="CG102" s="61"/>
+      <c r="CH102" s="61"/>
+      <c r="CI102" s="61"/>
       <c r="CJ102" s="35"/>
       <c r="CK102" s="35"/>
       <c r="CL102" s="35"/>
@@ -16962,8 +17274,11 @@
       <c r="DT102" s="35"/>
       <c r="DU102" s="35"/>
       <c r="DV102" s="35"/>
-    </row>
-    <row r="103" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW102" s="35"/>
+      <c r="DX102" s="35"/>
+      <c r="DY102" s="35"/>
+    </row>
+    <row r="103" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A103" s="6"/>
       <c r="B103" s="6"/>
       <c r="C103" s="50"/>
@@ -17038,9 +17353,9 @@
       <c r="CD103" s="60"/>
       <c r="CE103" s="37"/>
       <c r="CF103" s="37"/>
-      <c r="CG103" s="35"/>
-      <c r="CH103" s="35"/>
-      <c r="CI103" s="35"/>
+      <c r="CG103" s="37"/>
+      <c r="CH103" s="37"/>
+      <c r="CI103" s="37"/>
       <c r="CJ103" s="35"/>
       <c r="CK103" s="35"/>
       <c r="CL103" s="35"/>
@@ -17080,8 +17395,11 @@
       <c r="DT103" s="35"/>
       <c r="DU103" s="35"/>
       <c r="DV103" s="35"/>
-    </row>
-    <row r="104" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW103" s="35"/>
+      <c r="DX103" s="35"/>
+      <c r="DY103" s="35"/>
+    </row>
+    <row r="104" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A104" s="6"/>
       <c r="B104" s="6"/>
       <c r="C104" s="50"/>
@@ -17156,9 +17474,9 @@
       <c r="CD104" s="60"/>
       <c r="CE104" s="37"/>
       <c r="CF104" s="37"/>
-      <c r="CG104" s="35"/>
-      <c r="CH104" s="35"/>
-      <c r="CI104" s="35"/>
+      <c r="CG104" s="37"/>
+      <c r="CH104" s="37"/>
+      <c r="CI104" s="37"/>
       <c r="CJ104" s="35"/>
       <c r="CK104" s="35"/>
       <c r="CL104" s="35"/>
@@ -17198,8 +17516,11 @@
       <c r="DT104" s="35"/>
       <c r="DU104" s="35"/>
       <c r="DV104" s="35"/>
-    </row>
-    <row r="105" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW104" s="35"/>
+      <c r="DX104" s="35"/>
+      <c r="DY104" s="35"/>
+    </row>
+    <row r="105" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A105" s="6"/>
       <c r="B105" s="6"/>
       <c r="C105" s="50"/>
@@ -17274,9 +17595,9 @@
       <c r="CD105" s="60"/>
       <c r="CE105" s="37"/>
       <c r="CF105" s="37"/>
-      <c r="CG105" s="35"/>
-      <c r="CH105" s="35"/>
-      <c r="CI105" s="35"/>
+      <c r="CG105" s="37"/>
+      <c r="CH105" s="37"/>
+      <c r="CI105" s="37"/>
       <c r="CJ105" s="35"/>
       <c r="CK105" s="35"/>
       <c r="CL105" s="35"/>
@@ -17316,8 +17637,11 @@
       <c r="DT105" s="35"/>
       <c r="DU105" s="35"/>
       <c r="DV105" s="35"/>
-    </row>
-    <row r="106" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW105" s="35"/>
+      <c r="DX105" s="35"/>
+      <c r="DY105" s="35"/>
+    </row>
+    <row r="106" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A106" s="6"/>
       <c r="B106" s="6"/>
       <c r="C106" s="50"/>
@@ -17392,9 +17716,9 @@
       <c r="CD106" s="60"/>
       <c r="CE106" s="37"/>
       <c r="CF106" s="37"/>
-      <c r="CG106" s="35"/>
-      <c r="CH106" s="35"/>
-      <c r="CI106" s="35"/>
+      <c r="CG106" s="37"/>
+      <c r="CH106" s="37"/>
+      <c r="CI106" s="37"/>
       <c r="CJ106" s="35"/>
       <c r="CK106" s="35"/>
       <c r="CL106" s="35"/>
@@ -17434,8 +17758,11 @@
       <c r="DT106" s="35"/>
       <c r="DU106" s="35"/>
       <c r="DV106" s="35"/>
-    </row>
-    <row r="107" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW106" s="35"/>
+      <c r="DX106" s="35"/>
+      <c r="DY106" s="35"/>
+    </row>
+    <row r="107" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A107" s="6"/>
       <c r="B107" s="6"/>
       <c r="C107" s="50"/>
@@ -17510,9 +17837,9 @@
       <c r="CD107" s="60"/>
       <c r="CE107" s="37"/>
       <c r="CF107" s="37"/>
-      <c r="CG107" s="35"/>
-      <c r="CH107" s="35"/>
-      <c r="CI107" s="35"/>
+      <c r="CG107" s="37"/>
+      <c r="CH107" s="37"/>
+      <c r="CI107" s="37"/>
       <c r="CJ107" s="35"/>
       <c r="CK107" s="35"/>
       <c r="CL107" s="35"/>
@@ -17552,8 +17879,11 @@
       <c r="DT107" s="35"/>
       <c r="DU107" s="35"/>
       <c r="DV107" s="35"/>
-    </row>
-    <row r="108" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW107" s="35"/>
+      <c r="DX107" s="35"/>
+      <c r="DY107" s="35"/>
+    </row>
+    <row r="108" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A108" s="6"/>
       <c r="B108" s="6"/>
       <c r="C108" s="50"/>
@@ -17628,9 +17958,9 @@
       <c r="CD108" s="60"/>
       <c r="CE108" s="37"/>
       <c r="CF108" s="37"/>
-      <c r="CG108" s="35"/>
-      <c r="CH108" s="35"/>
-      <c r="CI108" s="35"/>
+      <c r="CG108" s="37"/>
+      <c r="CH108" s="37"/>
+      <c r="CI108" s="37"/>
       <c r="CJ108" s="35"/>
       <c r="CK108" s="35"/>
       <c r="CL108" s="35"/>
@@ -17670,8 +18000,11 @@
       <c r="DT108" s="35"/>
       <c r="DU108" s="35"/>
       <c r="DV108" s="35"/>
-    </row>
-    <row r="109" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW108" s="35"/>
+      <c r="DX108" s="35"/>
+      <c r="DY108" s="35"/>
+    </row>
+    <row r="109" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A109" s="6"/>
       <c r="B109" s="6"/>
       <c r="C109" s="50"/>
@@ -17746,9 +18079,9 @@
       <c r="CD109" s="60"/>
       <c r="CE109" s="37"/>
       <c r="CF109" s="37"/>
-      <c r="CG109" s="35"/>
-      <c r="CH109" s="35"/>
-      <c r="CI109" s="35"/>
+      <c r="CG109" s="37"/>
+      <c r="CH109" s="37"/>
+      <c r="CI109" s="37"/>
       <c r="CJ109" s="35"/>
       <c r="CK109" s="35"/>
       <c r="CL109" s="35"/>
@@ -17788,8 +18121,11 @@
       <c r="DT109" s="35"/>
       <c r="DU109" s="35"/>
       <c r="DV109" s="35"/>
-    </row>
-    <row r="110" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW109" s="35"/>
+      <c r="DX109" s="35"/>
+      <c r="DY109" s="35"/>
+    </row>
+    <row r="110" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A110" s="6"/>
       <c r="B110" s="6"/>
       <c r="C110" s="50"/>
@@ -17864,9 +18200,9 @@
       <c r="CD110" s="60"/>
       <c r="CE110" s="37"/>
       <c r="CF110" s="37"/>
-      <c r="CG110" s="35"/>
-      <c r="CH110" s="35"/>
-      <c r="CI110" s="35"/>
+      <c r="CG110" s="37"/>
+      <c r="CH110" s="37"/>
+      <c r="CI110" s="37"/>
       <c r="CJ110" s="35"/>
       <c r="CK110" s="35"/>
       <c r="CL110" s="35"/>
@@ -17906,8 +18242,11 @@
       <c r="DT110" s="35"/>
       <c r="DU110" s="35"/>
       <c r="DV110" s="35"/>
-    </row>
-    <row r="111" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW110" s="35"/>
+      <c r="DX110" s="35"/>
+      <c r="DY110" s="35"/>
+    </row>
+    <row r="111" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A111" s="6"/>
       <c r="B111" s="6"/>
       <c r="C111" s="50"/>
@@ -17982,9 +18321,9 @@
       <c r="CD111" s="60"/>
       <c r="CE111" s="37"/>
       <c r="CF111" s="37"/>
-      <c r="CG111" s="35"/>
-      <c r="CH111" s="35"/>
-      <c r="CI111" s="35"/>
+      <c r="CG111" s="37"/>
+      <c r="CH111" s="37"/>
+      <c r="CI111" s="37"/>
       <c r="CJ111" s="35"/>
       <c r="CK111" s="35"/>
       <c r="CL111" s="35"/>
@@ -18024,8 +18363,11 @@
       <c r="DT111" s="35"/>
       <c r="DU111" s="35"/>
       <c r="DV111" s="35"/>
-    </row>
-    <row r="112" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW111" s="35"/>
+      <c r="DX111" s="35"/>
+      <c r="DY111" s="35"/>
+    </row>
+    <row r="112" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A112" s="6"/>
       <c r="B112" s="6"/>
       <c r="C112" s="50"/>
@@ -18100,9 +18442,9 @@
       <c r="CD112" s="60"/>
       <c r="CE112" s="37"/>
       <c r="CF112" s="37"/>
-      <c r="CG112" s="35"/>
-      <c r="CH112" s="35"/>
-      <c r="CI112" s="35"/>
+      <c r="CG112" s="37"/>
+      <c r="CH112" s="37"/>
+      <c r="CI112" s="37"/>
       <c r="CJ112" s="35"/>
       <c r="CK112" s="35"/>
       <c r="CL112" s="35"/>
@@ -18142,8 +18484,11 @@
       <c r="DT112" s="35"/>
       <c r="DU112" s="35"/>
       <c r="DV112" s="35"/>
-    </row>
-    <row r="113" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW112" s="35"/>
+      <c r="DX112" s="35"/>
+      <c r="DY112" s="35"/>
+    </row>
+    <row r="113" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A113" s="6"/>
       <c r="B113" s="6"/>
       <c r="C113" s="50"/>
@@ -18218,9 +18563,9 @@
       <c r="CD113" s="60"/>
       <c r="CE113" s="37"/>
       <c r="CF113" s="37"/>
-      <c r="CG113" s="35"/>
-      <c r="CH113" s="35"/>
-      <c r="CI113" s="35"/>
+      <c r="CG113" s="37"/>
+      <c r="CH113" s="37"/>
+      <c r="CI113" s="37"/>
       <c r="CJ113" s="35"/>
       <c r="CK113" s="35"/>
       <c r="CL113" s="35"/>
@@ -18260,8 +18605,11 @@
       <c r="DT113" s="35"/>
       <c r="DU113" s="35"/>
       <c r="DV113" s="35"/>
-    </row>
-    <row r="114" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW113" s="35"/>
+      <c r="DX113" s="35"/>
+      <c r="DY113" s="35"/>
+    </row>
+    <row r="114" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A114" s="6"/>
       <c r="B114" s="6"/>
       <c r="C114" s="50"/>
@@ -18336,9 +18684,9 @@
       <c r="CD114" s="60"/>
       <c r="CE114" s="37"/>
       <c r="CF114" s="37"/>
-      <c r="CG114" s="35"/>
-      <c r="CH114" s="35"/>
-      <c r="CI114" s="35"/>
+      <c r="CG114" s="37"/>
+      <c r="CH114" s="37"/>
+      <c r="CI114" s="37"/>
       <c r="CJ114" s="35"/>
       <c r="CK114" s="35"/>
       <c r="CL114" s="35"/>
@@ -18378,8 +18726,11 @@
       <c r="DT114" s="35"/>
       <c r="DU114" s="35"/>
       <c r="DV114" s="35"/>
-    </row>
-    <row r="115" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW114" s="35"/>
+      <c r="DX114" s="35"/>
+      <c r="DY114" s="35"/>
+    </row>
+    <row r="115" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A115" s="6"/>
       <c r="B115" s="6"/>
       <c r="C115" s="50"/>
@@ -18454,9 +18805,9 @@
       <c r="CD115" s="60"/>
       <c r="CE115" s="37"/>
       <c r="CF115" s="37"/>
-      <c r="CG115" s="35"/>
-      <c r="CH115" s="35"/>
-      <c r="CI115" s="35"/>
+      <c r="CG115" s="37"/>
+      <c r="CH115" s="37"/>
+      <c r="CI115" s="37"/>
       <c r="CJ115" s="35"/>
       <c r="CK115" s="35"/>
       <c r="CL115" s="35"/>
@@ -18496,8 +18847,11 @@
       <c r="DT115" s="35"/>
       <c r="DU115" s="35"/>
       <c r="DV115" s="35"/>
-    </row>
-    <row r="116" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW115" s="35"/>
+      <c r="DX115" s="35"/>
+      <c r="DY115" s="35"/>
+    </row>
+    <row r="116" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A116" s="6"/>
       <c r="B116" s="6"/>
       <c r="C116" s="50"/>
@@ -18572,9 +18926,9 @@
       <c r="CD116" s="60"/>
       <c r="CE116" s="37"/>
       <c r="CF116" s="37"/>
-      <c r="CG116" s="35"/>
-      <c r="CH116" s="35"/>
-      <c r="CI116" s="35"/>
+      <c r="CG116" s="37"/>
+      <c r="CH116" s="37"/>
+      <c r="CI116" s="37"/>
       <c r="CJ116" s="35"/>
       <c r="CK116" s="35"/>
       <c r="CL116" s="35"/>
@@ -18614,8 +18968,11 @@
       <c r="DT116" s="35"/>
       <c r="DU116" s="35"/>
       <c r="DV116" s="35"/>
-    </row>
-    <row r="117" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW116" s="35"/>
+      <c r="DX116" s="35"/>
+      <c r="DY116" s="35"/>
+    </row>
+    <row r="117" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A117" s="6"/>
       <c r="B117" s="6"/>
       <c r="C117" s="50"/>
@@ -18690,9 +19047,9 @@
       <c r="CD117" s="60"/>
       <c r="CE117" s="37"/>
       <c r="CF117" s="37"/>
-      <c r="CG117" s="35"/>
-      <c r="CH117" s="35"/>
-      <c r="CI117" s="35"/>
+      <c r="CG117" s="37"/>
+      <c r="CH117" s="37"/>
+      <c r="CI117" s="37"/>
       <c r="CJ117" s="35"/>
       <c r="CK117" s="35"/>
       <c r="CL117" s="35"/>
@@ -18732,8 +19089,11 @@
       <c r="DT117" s="35"/>
       <c r="DU117" s="35"/>
       <c r="DV117" s="35"/>
-    </row>
-    <row r="118" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DW117" s="35"/>
+      <c r="DX117" s="35"/>
+      <c r="DY117" s="35"/>
+    </row>
+    <row r="118" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A118" s="6"/>
       <c r="B118" s="6"/>
       <c r="AO118" s="72"/>
@@ -18762,7 +19122,7 @@
       <c r="BL118" s="55"/>
       <c r="BO118" s="80"/>
     </row>
-    <row r="119" spans="1:126" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:129" x14ac:dyDescent="0.3">
       <c r="B119" s="6"/>
       <c r="E119" s="70"/>
       <c r="F119" s="50"/>
@@ -18790,7 +19150,7 @@
       <c r="BN119" s="59"/>
       <c r="BO119" s="80"/>
     </row>
-    <row r="120" spans="1:126" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:129" x14ac:dyDescent="0.3">
       <c r="B120" s="6"/>
       <c r="E120" s="70"/>
       <c r="F120" s="50"/>
@@ -18819,7 +19179,7 @@
       <c r="BM120" s="59"/>
       <c r="BN120" s="59"/>
     </row>
-    <row r="121" spans="1:126" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:129" x14ac:dyDescent="0.3">
       <c r="B121" s="6"/>
       <c r="E121" s="70"/>
       <c r="F121" s="50"/>
@@ -18845,7 +19205,7 @@
       <c r="AX121" s="74"/>
       <c r="BN121" s="59"/>
     </row>
-    <row r="122" spans="1:126" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:129" x14ac:dyDescent="0.3">
       <c r="B122" s="6"/>
       <c r="E122" s="70"/>
       <c r="F122" s="50"/>
@@ -18868,7 +19228,7 @@
       <c r="BM122" s="59"/>
       <c r="BN122" s="59"/>
     </row>
-    <row r="123" spans="1:126" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:129" x14ac:dyDescent="0.3">
       <c r="B123" s="6"/>
       <c r="E123" s="70"/>
       <c r="F123" s="50"/>
@@ -18888,7 +19248,7 @@
       <c r="BM123" s="59"/>
       <c r="BN123" s="59"/>
     </row>
-    <row r="124" spans="1:126" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:129" x14ac:dyDescent="0.3">
       <c r="B124" s="6"/>
       <c r="E124" s="70"/>
       <c r="F124" s="50"/>
@@ -18913,7 +19273,7 @@
       <c r="BM124" s="59"/>
       <c r="BN124" s="59"/>
     </row>
-    <row r="125" spans="1:126" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:129" x14ac:dyDescent="0.3">
       <c r="B125" s="6"/>
       <c r="E125" s="70"/>
       <c r="F125" s="50"/>
@@ -18944,14 +19304,17 @@
       <c r="BW125" s="80"/>
       <c r="CE125" s="82"/>
       <c r="CF125" s="80"/>
-      <c r="CM125" s="80"/>
-      <c r="CO125" s="80"/>
+      <c r="CG125" s="80"/>
+      <c r="CH125" s="80"/>
+      <c r="CI125" s="80"/>
+      <c r="CP125" s="80"/>
       <c r="CR125" s="80"/>
       <c r="CU125" s="80"/>
       <c r="CX125" s="80"/>
       <c r="DA125" s="80"/>
-    </row>
-    <row r="126" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="DD125" s="80"/>
+    </row>
+    <row r="126" spans="1:129" x14ac:dyDescent="0.3">
       <c r="B126" s="6"/>
       <c r="E126" s="70"/>
       <c r="F126" s="50"/>
@@ -18975,7 +19338,7 @@
       <c r="BM126" s="59"/>
       <c r="BN126" s="59"/>
     </row>
-    <row r="127" spans="1:126" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:129" x14ac:dyDescent="0.3">
       <c r="B127" s="6"/>
       <c r="E127" s="70"/>
       <c r="F127" s="50"/>
@@ -19002,11 +19365,14 @@
       <c r="BS127" s="80"/>
       <c r="CE127" s="82"/>
       <c r="CF127" s="80"/>
-      <c r="CM127" s="80"/>
-      <c r="CO127" s="80"/>
-      <c r="DT127" s="80"/>
-    </row>
-    <row r="128" spans="1:126" x14ac:dyDescent="0.3">
+      <c r="CG127" s="80"/>
+      <c r="CH127" s="80"/>
+      <c r="CI127" s="80"/>
+      <c r="CP127" s="80"/>
+      <c r="CR127" s="80"/>
+      <c r="DW127" s="80"/>
+    </row>
+    <row r="128" spans="1:129" x14ac:dyDescent="0.3">
       <c r="B128" s="6"/>
       <c r="E128" s="70"/>
       <c r="F128" s="50"/>
@@ -19029,7 +19395,7 @@
       <c r="BM128" s="59"/>
       <c r="BN128" s="59"/>
     </row>
-    <row r="129" spans="2:124" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:127" x14ac:dyDescent="0.3">
       <c r="B129" s="6"/>
       <c r="E129" s="70"/>
       <c r="F129" s="50"/>
@@ -19064,7 +19430,7 @@
       <c r="BM129" s="59"/>
       <c r="BN129" s="59"/>
     </row>
-    <row r="130" spans="2:124" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:127" x14ac:dyDescent="0.3">
       <c r="B130" s="6"/>
       <c r="E130" s="70"/>
       <c r="F130" s="50"/>
@@ -19090,7 +19456,7 @@
       <c r="BM130" s="59"/>
       <c r="BN130" s="59"/>
     </row>
-    <row r="131" spans="2:124" x14ac:dyDescent="0.3">
+    <row r="131" spans="2:127" x14ac:dyDescent="0.3">
       <c r="B131" s="6"/>
       <c r="E131" s="70"/>
       <c r="F131" s="50"/>
@@ -19114,11 +19480,14 @@
       <c r="BS131" s="80"/>
       <c r="CE131" s="82"/>
       <c r="CF131" s="80"/>
-      <c r="CM131" s="80"/>
-      <c r="CO131" s="80"/>
-      <c r="DT131" s="80"/>
-    </row>
-    <row r="132" spans="2:124" x14ac:dyDescent="0.3">
+      <c r="CG131" s="80"/>
+      <c r="CH131" s="80"/>
+      <c r="CI131" s="80"/>
+      <c r="CP131" s="80"/>
+      <c r="CR131" s="80"/>
+      <c r="DW131" s="80"/>
+    </row>
+    <row r="132" spans="2:127" x14ac:dyDescent="0.3">
       <c r="B132" s="6"/>
       <c r="E132" s="70"/>
       <c r="F132" s="50"/>
@@ -19139,7 +19508,7 @@
       <c r="BM132" s="59"/>
       <c r="BN132" s="59"/>
     </row>
-    <row r="133" spans="2:124" x14ac:dyDescent="0.3">
+    <row r="133" spans="2:127" x14ac:dyDescent="0.3">
       <c r="B133" s="6"/>
       <c r="E133" s="70"/>
       <c r="F133" s="50"/>
@@ -19160,7 +19529,7 @@
       <c r="BM133" s="59"/>
       <c r="BN133" s="59"/>
     </row>
-    <row r="134" spans="2:124" x14ac:dyDescent="0.3">
+    <row r="134" spans="2:127" x14ac:dyDescent="0.3">
       <c r="B134" s="6"/>
       <c r="E134" s="70"/>
       <c r="F134" s="50"/>
@@ -19186,13 +19555,16 @@
       <c r="BO134" s="80"/>
       <c r="BS134" s="80"/>
       <c r="CF134" s="80"/>
-      <c r="CM134" s="80"/>
-      <c r="CO134" s="80"/>
+      <c r="CG134" s="80"/>
+      <c r="CH134" s="80"/>
+      <c r="CI134" s="80"/>
+      <c r="CP134" s="80"/>
       <c r="CR134" s="80"/>
       <c r="CU134" s="80"/>
       <c r="CX134" s="80"/>
-    </row>
-    <row r="135" spans="2:124" x14ac:dyDescent="0.3">
+      <c r="DA134" s="80"/>
+    </row>
+    <row r="135" spans="2:127" x14ac:dyDescent="0.3">
       <c r="B135" s="6"/>
       <c r="E135" s="70"/>
       <c r="O135" s="50"/>
@@ -19215,7 +19587,7 @@
       <c r="BM135" s="59"/>
       <c r="BN135" s="59"/>
     </row>
-    <row r="136" spans="2:124" x14ac:dyDescent="0.3">
+    <row r="136" spans="2:127" x14ac:dyDescent="0.3">
       <c r="B136" s="6"/>
       <c r="E136" s="70"/>
       <c r="F136" s="50"/>
@@ -19241,7 +19613,7 @@
       <c r="BM136" s="59"/>
       <c r="BN136" s="59"/>
     </row>
-    <row r="137" spans="2:124" x14ac:dyDescent="0.3">
+    <row r="137" spans="2:127" x14ac:dyDescent="0.3">
       <c r="E137" s="70"/>
       <c r="F137" s="50"/>
       <c r="L137" s="50"/>
@@ -19259,7 +19631,7 @@
       <c r="BO137" s="80"/>
       <c r="BS137" s="80"/>
     </row>
-    <row r="138" spans="2:124" x14ac:dyDescent="0.3">
+    <row r="138" spans="2:127" x14ac:dyDescent="0.3">
       <c r="B138" s="6"/>
       <c r="E138" s="70"/>
       <c r="F138" s="50"/>
@@ -19276,7 +19648,7 @@
       <c r="BN138" s="59"/>
       <c r="BO138" s="80"/>
     </row>
-    <row r="139" spans="2:124" x14ac:dyDescent="0.3">
+    <row r="139" spans="2:127" x14ac:dyDescent="0.3">
       <c r="E139" s="70"/>
       <c r="F139" s="50"/>
       <c r="L139" s="50"/>
@@ -19297,7 +19669,7 @@
       <c r="BO139" s="80"/>
       <c r="BS139" s="80"/>
     </row>
-    <row r="140" spans="2:124" x14ac:dyDescent="0.3">
+    <row r="140" spans="2:127" x14ac:dyDescent="0.3">
       <c r="B140" s="6"/>
       <c r="E140" s="70"/>
       <c r="F140" s="50"/>
@@ -19317,7 +19689,7 @@
       <c r="BN140" s="59"/>
       <c r="BO140" s="80"/>
     </row>
-    <row r="141" spans="2:124" x14ac:dyDescent="0.3">
+    <row r="141" spans="2:127" x14ac:dyDescent="0.3">
       <c r="E141" s="70"/>
       <c r="F141" s="50"/>
       <c r="L141" s="50"/>
@@ -19337,7 +19709,7 @@
       <c r="BN141" s="59"/>
       <c r="BO141" s="80"/>
     </row>
-    <row r="142" spans="2:124" x14ac:dyDescent="0.3">
+    <row r="142" spans="2:127" x14ac:dyDescent="0.3">
       <c r="B142" s="6"/>
       <c r="E142" s="70"/>
       <c r="F142" s="50"/>
@@ -19357,7 +19729,7 @@
       <c r="BN142" s="59"/>
       <c r="BO142" s="80"/>
     </row>
-    <row r="143" spans="2:124" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:127" x14ac:dyDescent="0.3">
       <c r="E143" s="70"/>
       <c r="AC143" s="97"/>
       <c r="AD143" s="97"/>
@@ -19377,7 +19749,7 @@
       <c r="BN143" s="59"/>
       <c r="BO143" s="80"/>
     </row>
-    <row r="144" spans="2:124" x14ac:dyDescent="0.3">
+    <row r="144" spans="2:127" x14ac:dyDescent="0.3">
       <c r="B144" s="6"/>
       <c r="E144" s="70"/>
       <c r="L144" s="50"/>
@@ -19952,36 +20324,16 @@
       <c r="BO175" s="80"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:DV136" xr:uid="{0DA90007-303F-4AED-8AB9-2CF07A0AFD4B}"/>
+  <autoFilter ref="A1:DY136" xr:uid="{0DA90007-303F-4AED-8AB9-2CF07A0AFD4B}"/>
   <phoneticPr fontId="29" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:DV4" xr:uid="{2A892EB8-2528-4AEA-96E4-FE721A55DBFB}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:DY4" xr:uid="{2A892EB8-2528-4AEA-96E4-FE721A55DBFB}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="42fbd5e6-b175-407a-a25c-5fc6410bf24f" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EE7777BCFCD3E741B5CCCE9A87E98C2C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f7fc7590daec4eb8e38e018938a160ca">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e" xmlns:ns3="42fbd5e6-b175-407a-a25c-5fc6410bf24f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c5ca1b94d4b54616210e83d04e6b3cac" ns2:_="" ns3:_="">
     <xsd:import namespace="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
@@ -20236,26 +20588,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{286F673D-E70D-4002-B8F5-CAC95B029A7E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E9485EC-5D88-4A1C-961D-0F4FE84359B8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="42fbd5e6-b175-407a-a25c-5fc6410bf24f"/>
-    <ds:schemaRef ds:uri="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="42fbd5e6-b175-407a-a25c-5fc6410bf24f" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C9C537E-DFD2-4C38-AC8C-930F122DEFFC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -20272,4 +20625,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{286F673D-E70D-4002-B8F5-CAC95B029A7E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E9485EC-5D88-4A1C-961D-0F4FE84359B8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="42fbd5e6-b175-407a-a25c-5fc6410bf24f"/>
+    <ds:schemaRef ds:uri="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
update patient to client
</commit_message>
<xml_diff>
--- a/data/ALAI UP Client-level Reporting Tool Template_4.7.26.xlsx
+++ b/data/ALAI UP Client-level Reporting Tool Template_4.7.26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kmlab\Desktop\Dashboard\alai_up_local_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6C66CB2-97D3-4919-95DA-1301A51B6493}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68C4B550-B271-4962-B815-2E5EAA6AF2FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{500E2EE0-B1C5-4ACF-BC67-EDC8BDABD2D7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{500E2EE0-B1C5-4ACF-BC67-EDC8BDABD2D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="3" r:id="rId1"/>
@@ -476,9 +476,6 @@
     <t>Primary language</t>
   </si>
   <si>
-    <t>The primary language patient prefers for communication</t>
-  </si>
-  <si>
     <t>1=English; 2=Spanish; 3=Chinese; 4=Haitian Creole; 5=Tagalog; 6=Vietnamese; 7=Arabic; 8=Amharic; 20=Other; UNK=Unknown</t>
   </si>
   <si>
@@ -1248,24 +1245,8 @@
 All responses of a given category should have the same spelling and capitalization.</t>
   </si>
   <si>
-    <t>The date of the client's second viral load test since the beginning of injectable program. The date of specimen collected is preferred, but if that cannot be retrieved, then the date of results returned.
-Clinics should enter all viral load results for a given patient, starting from the beginning of your site’s injectable program. If that date is unknown, you can approximate, or enter all viral loads since January 2021 when iCAB/RPV was FDA approved.
-Clinics should add as many of these columns as are needed, following the same column naming format with a number instead of the X. 
-Example:
-hiv_vl_1_result
-hiv_vl_1_date
-Example:
-hiv_vl_15_result
-hiv_vl_15_date</t>
-  </si>
-  <si>
     <t>The client was prescribed iCAB/RPV by a clinical provider.
 This should be the date the prescription was written and sent to insurance.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The date the client was prescribed iCAB/RPV.
-If this field is left blank but that patient received an injection, ‘prescribed’ will be set to 1=prescribed to ensure consistent denominators. This most often occurs if the patient transfers to your site while already on iCAB/RPV 
-</t>
   </si>
   <si>
     <t>Date client ended oral ART for the first time to bridge therapy for planned missed iCAB/RPV injection.
@@ -1328,11 +1309,6 @@
     <t>A binary measure of whether the client currently discontinued iCAB/RPV.
 icab_rpv_discontinued should only be ‘1’ if the client initiated iCAB/RPV but has since discontinued for any reason. This could include if the client has switched out of the clinic or back to oral ART; those reasons should be reflected in the reasons column. If a client stopped but restarted iCAB/RPV, make sure this value is ‘0’ (sustained), and the stop/restart should be indicated via icab_rpv_shotX_late_exception
 Note that if this field is left blank, but the client has not received a dose of iCAB/RPV in &gt;90 days since their most recent dose, then they are labeled as ‘discontinued’ by the Dashboard.</t>
-  </si>
-  <si>
-    <t>Date client decided to discontinue iCAB/RPV.
-If a client was lost to follow up or moved to another clinic, they are considered discontinued (at that clinic), even if they are still on CAB at the new clinic. Assign icab_rpv_discontinued to be 1, and use the last CAB date as the discontinued date if there is no other date
-If the date of discontinuation is unknown, the last iCAB/RPV injection date may be used (e.g. if the patient was lost to follow up).</t>
   </si>
   <si>
     <t>icab_rpv_accessible</t>
@@ -1400,6 +1376,30 @@
   </si>
   <si>
     <t>1=Client does not qualify for PAP; 2=Medication not on payor formulary; 3=Co-pay too expensive for client; 20=Other; UNK=Unknown</t>
+  </si>
+  <si>
+    <t>Date client decided to discontinue iCAB/RPV.
+If a client was lost to follow up or moved to another clinic, they are considered discontinued (at that clinic), even if they are still on CAB at the new clinic. Assign icab_rpv_discontinued to be 1, and use the last CAB date as the discontinued date if there is no other date
+If the date of discontinuation is unknown, the last iCAB/RPV injection date may be used (e.g. if the client was lost to follow up).</t>
+  </si>
+  <si>
+    <t>The primary language client prefers for communication</t>
+  </si>
+  <si>
+    <t>The date of the client's second viral load test since the beginning of injectable program. The date of specimen collected is preferred, but if that cannot be retrieved, then the date of results returned.
+Clinics should enter all viral load results for a given client, starting from the beginning of your site’s injectable program. If that date is unknown, you can approximate, or enter all viral loads since January 2021 when iCAB/RPV was FDA approved.
+Clinics should add as many of these columns as are needed, following the same column naming format with a number instead of the X. 
+Example:
+hiv_vl_1_result
+hiv_vl_1_date
+Example:
+hiv_vl_15_result
+hiv_vl_15_date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The date the client was prescribed iCAB/RPV.
+If this field is left blank but that client received an injection, ‘prescribed’ will be set to 1=prescribed to ensure consistent denominators. This most often occurs if the client transfers to your site while already on iCAB/RPV 
+</t>
   </si>
 </sst>
 </file>
@@ -2112,23 +2112,8 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2139,13 +2124,13 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2155,6 +2140,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2175,11 +2169,17 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2560,7 +2560,7 @@
     </row>
     <row r="7" spans="2:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="B7" s="87" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.25">
@@ -2570,7 +2570,7 @@
     </row>
     <row r="9" spans="2:2" ht="41.4" x14ac:dyDescent="0.25">
       <c r="B9" s="87" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.25">
@@ -2708,7 +2708,7 @@
         <v>26</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H1" s="3"/>
       <c r="I1" s="4"/>
@@ -2727,13 +2727,13 @@
         <v>29</v>
       </c>
       <c r="E2" s="108" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F2" s="108" t="s">
         <v>30</v>
       </c>
       <c r="G2" s="108" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="8"/>
@@ -2741,14 +2741,14 @@
       <c r="K2" s="4"/>
     </row>
     <row r="3" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="133" t="s">
+      <c r="B3" s="128" t="s">
         <v>31</v>
       </c>
       <c r="C3" s="109" t="s">
+        <v>302</v>
+      </c>
+      <c r="D3" s="110" t="s">
         <v>303</v>
-      </c>
-      <c r="D3" s="110" t="s">
-        <v>304</v>
       </c>
       <c r="E3" s="110" t="s">
         <v>32</v>
@@ -2757,13 +2757,13 @@
         <v>30</v>
       </c>
       <c r="G3" s="110" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H3" s="12"/>
       <c r="I3" s="8"/>
     </row>
     <row r="4" spans="1:11" ht="67.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="134"/>
+      <c r="B4" s="129"/>
       <c r="C4" s="15" t="s">
         <v>33</v>
       </c>
@@ -2777,13 +2777,13 @@
         <v>36</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H4" s="12"/>
       <c r="I4" s="8"/>
     </row>
     <row r="5" spans="1:11" ht="44.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="134"/>
+      <c r="B5" s="129"/>
       <c r="C5" s="15" t="s">
         <v>37</v>
       </c>
@@ -2797,33 +2797,33 @@
         <v>40</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H5" s="10"/>
       <c r="I5" s="17"/>
     </row>
     <row r="6" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B6" s="134"/>
+      <c r="B6" s="129"/>
       <c r="C6" s="15" t="s">
+        <v>352</v>
+      </c>
+      <c r="D6" s="16" t="s">
         <v>353</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="E6" s="16" t="s">
         <v>354</v>
       </c>
-      <c r="E6" s="16" t="s">
+      <c r="F6" s="16" t="s">
         <v>355</v>
       </c>
-      <c r="F6" s="16" t="s">
-        <v>356</v>
-      </c>
       <c r="G6" s="16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H6" s="12"/>
     </row>
     <row r="7" spans="1:11" s="19" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A7"/>
-      <c r="B7" s="134"/>
+      <c r="B7" s="129"/>
       <c r="C7" s="15" t="s">
         <v>42</v>
       </c>
@@ -2837,7 +2837,7 @@
         <v>45</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H7" s="10"/>
       <c r="I7" s="18"/>
@@ -2845,7 +2845,7 @@
       <c r="K7" s="18"/>
     </row>
     <row r="8" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B8" s="134"/>
+      <c r="B8" s="129"/>
       <c r="C8" s="15" t="s">
         <v>46</v>
       </c>
@@ -2859,12 +2859,12 @@
         <v>49</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H8" s="12"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B9" s="134"/>
+      <c r="B9" s="129"/>
       <c r="C9" s="15" t="s">
         <v>50</v>
       </c>
@@ -2878,12 +2878,12 @@
         <v>53</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H9" s="12"/>
     </row>
     <row r="10" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B10" s="134"/>
+      <c r="B10" s="129"/>
       <c r="C10" s="15" t="s">
         <v>54</v>
       </c>
@@ -2897,12 +2897,12 @@
         <v>57</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H10" s="12"/>
     </row>
     <row r="11" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B11" s="134"/>
+      <c r="B11" s="129"/>
       <c r="C11" s="15" t="s">
         <v>58</v>
       </c>
@@ -2916,12 +2916,12 @@
         <v>61</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H11" s="12"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B12" s="134"/>
+      <c r="B12" s="129"/>
       <c r="C12" s="15" t="s">
         <v>62</v>
       </c>
@@ -2935,12 +2935,12 @@
         <v>65</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H12" s="12"/>
     </row>
     <row r="13" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B13" s="134"/>
+      <c r="B13" s="129"/>
       <c r="C13" s="15" t="s">
         <v>66</v>
       </c>
@@ -2954,12 +2954,12 @@
         <v>69</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H13" s="12"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B14" s="134"/>
+      <c r="B14" s="129"/>
       <c r="C14" s="15" t="s">
         <v>70</v>
       </c>
@@ -2973,12 +2973,12 @@
         <v>30</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H14" s="12"/>
     </row>
     <row r="15" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B15" s="134"/>
+      <c r="B15" s="129"/>
       <c r="C15" s="15" t="s">
         <v>73</v>
       </c>
@@ -2992,12 +2992,12 @@
         <v>76</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H15" s="20"/>
     </row>
     <row r="16" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B16" s="135"/>
+      <c r="B16" s="130"/>
       <c r="C16" s="15" t="s">
         <v>77</v>
       </c>
@@ -3011,15 +3011,15 @@
         <v>80</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H16" s="12"/>
     </row>
     <row r="17" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="142" t="s">
-        <v>313</v>
-      </c>
-      <c r="B17" s="121" t="s">
+      <c r="A17" s="125" t="s">
+        <v>312</v>
+      </c>
+      <c r="B17" s="131" t="s">
         <v>81</v>
       </c>
       <c r="C17" s="111" t="s">
@@ -3028,181 +3028,181 @@
       <c r="D17" s="112" t="s">
         <v>83</v>
       </c>
-      <c r="E17" s="121" t="s">
-        <v>361</v>
+      <c r="E17" s="131" t="s">
+        <v>360</v>
       </c>
       <c r="F17" s="112" t="s">
         <v>84</v>
       </c>
       <c r="G17" s="112" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H17" s="12"/>
     </row>
     <row r="18" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="142"/>
-      <c r="B18" s="122"/>
+      <c r="A18" s="125"/>
+      <c r="B18" s="132"/>
       <c r="C18" s="111" t="s">
         <v>85</v>
       </c>
       <c r="D18" s="112" t="s">
         <v>86</v>
       </c>
-      <c r="E18" s="122"/>
+      <c r="E18" s="132"/>
       <c r="F18" s="112" t="s">
         <v>84</v>
       </c>
       <c r="G18" s="112" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H18" s="12"/>
     </row>
     <row r="19" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="142"/>
-      <c r="B19" s="122"/>
+      <c r="A19" s="125"/>
+      <c r="B19" s="132"/>
       <c r="C19" s="111" t="s">
         <v>87</v>
       </c>
       <c r="D19" s="112" t="s">
         <v>88</v>
       </c>
-      <c r="E19" s="122"/>
+      <c r="E19" s="132"/>
       <c r="F19" s="112" t="s">
         <v>84</v>
       </c>
       <c r="G19" s="112" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H19" s="12"/>
     </row>
     <row r="20" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A20" s="142"/>
-      <c r="B20" s="122"/>
+      <c r="A20" s="125"/>
+      <c r="B20" s="132"/>
       <c r="C20" s="111" t="s">
         <v>89</v>
       </c>
       <c r="D20" s="112" t="s">
         <v>90</v>
       </c>
-      <c r="E20" s="122"/>
+      <c r="E20" s="132"/>
       <c r="F20" s="112" t="s">
         <v>84</v>
       </c>
       <c r="G20" s="112" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H20" s="12"/>
     </row>
     <row r="21" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A21" s="142"/>
-      <c r="B21" s="122"/>
+      <c r="A21" s="125"/>
+      <c r="B21" s="132"/>
       <c r="C21" s="111" t="s">
         <v>91</v>
       </c>
       <c r="D21" s="112" t="s">
         <v>92</v>
       </c>
-      <c r="E21" s="122"/>
+      <c r="E21" s="132"/>
       <c r="F21" s="112" t="s">
         <v>84</v>
       </c>
       <c r="G21" s="112" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H21" s="12"/>
     </row>
     <row r="22" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A22" s="142"/>
-      <c r="B22" s="122"/>
+      <c r="A22" s="125"/>
+      <c r="B22" s="132"/>
       <c r="C22" s="111" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D22" s="112" t="s">
-        <v>283</v>
-      </c>
-      <c r="E22" s="122"/>
+        <v>282</v>
+      </c>
+      <c r="E22" s="132"/>
       <c r="F22" s="112" t="s">
         <v>84</v>
       </c>
       <c r="G22" s="112" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H22" s="12"/>
     </row>
     <row r="23" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A23" s="142"/>
-      <c r="B23" s="122"/>
+      <c r="A23" s="125"/>
+      <c r="B23" s="132"/>
       <c r="C23" s="111" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D23" s="112" t="s">
-        <v>284</v>
-      </c>
-      <c r="E23" s="122"/>
+        <v>283</v>
+      </c>
+      <c r="E23" s="132"/>
       <c r="F23" s="112" t="s">
         <v>84</v>
       </c>
       <c r="G23" s="112" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H23" s="12"/>
     </row>
     <row r="24" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A24" s="142"/>
-      <c r="B24" s="122"/>
+      <c r="A24" s="125"/>
+      <c r="B24" s="132"/>
       <c r="C24" s="111" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D24" s="112" t="s">
-        <v>285</v>
-      </c>
-      <c r="E24" s="122"/>
+        <v>284</v>
+      </c>
+      <c r="E24" s="132"/>
       <c r="F24" s="112" t="s">
         <v>84</v>
       </c>
       <c r="G24" s="112" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H24" s="12"/>
     </row>
     <row r="25" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A25" s="142"/>
-      <c r="B25" s="122"/>
+      <c r="A25" s="125"/>
+      <c r="B25" s="132"/>
       <c r="C25" s="111" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D25" s="112" t="s">
-        <v>286</v>
-      </c>
-      <c r="E25" s="122"/>
+        <v>285</v>
+      </c>
+      <c r="E25" s="132"/>
       <c r="F25" s="112" t="s">
         <v>84</v>
       </c>
       <c r="G25" s="112" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H25" s="12"/>
     </row>
     <row r="26" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A26" s="142"/>
-      <c r="B26" s="123"/>
+      <c r="A26" s="125"/>
+      <c r="B26" s="133"/>
       <c r="C26" s="111" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D26" s="112" t="s">
-        <v>287</v>
-      </c>
-      <c r="E26" s="123"/>
+        <v>286</v>
+      </c>
+      <c r="E26" s="133"/>
       <c r="F26" s="112" t="s">
         <v>84</v>
       </c>
       <c r="G26" s="112" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H26" s="12"/>
     </row>
     <row r="27" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="136" t="s">
+      <c r="B27" s="134" t="s">
         <v>93</v>
       </c>
       <c r="C27" s="113" t="s">
@@ -3218,12 +3218,12 @@
         <v>97</v>
       </c>
       <c r="G27" s="22" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H27" s="12"/>
     </row>
     <row r="28" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="137"/>
+      <c r="B28" s="135"/>
       <c r="C28" s="113" t="s">
         <v>98</v>
       </c>
@@ -3237,12 +3237,12 @@
         <v>101</v>
       </c>
       <c r="G28" s="22" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H28" s="12"/>
     </row>
     <row r="29" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B29" s="138"/>
+      <c r="B29" s="136"/>
       <c r="C29" s="113" t="s">
         <v>102</v>
       </c>
@@ -3256,12 +3256,12 @@
         <v>105</v>
       </c>
       <c r="G29" s="22" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H29" s="12"/>
     </row>
     <row r="30" spans="1:8" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="B30" s="139" t="s">
+      <c r="B30" s="137" t="s">
         <v>106</v>
       </c>
       <c r="C30" s="114" t="s">
@@ -3277,12 +3277,12 @@
         <v>110</v>
       </c>
       <c r="G30" s="23" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H30" s="24"/>
     </row>
     <row r="31" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="140"/>
+      <c r="B31" s="138"/>
       <c r="C31" s="114" t="s">
         <v>111</v>
       </c>
@@ -3290,18 +3290,18 @@
         <v>112</v>
       </c>
       <c r="E31" s="23" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F31" s="23" t="s">
         <v>113</v>
       </c>
       <c r="G31" s="23" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H31" s="24"/>
     </row>
     <row r="32" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="140"/>
+      <c r="B32" s="138"/>
       <c r="C32" s="114" t="s">
         <v>114</v>
       </c>
@@ -3315,12 +3315,12 @@
         <v>117</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H32" s="12"/>
     </row>
     <row r="33" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B33" s="140"/>
+      <c r="B33" s="138"/>
       <c r="C33" s="114" t="s">
         <v>118</v>
       </c>
@@ -3334,12 +3334,12 @@
         <v>121</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H33" s="10"/>
     </row>
     <row r="34" spans="1:11" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="140"/>
+      <c r="B34" s="138"/>
       <c r="C34" s="114" t="s">
         <v>122</v>
       </c>
@@ -3353,12 +3353,12 @@
         <v>125</v>
       </c>
       <c r="G34" s="23" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H34" s="12"/>
     </row>
     <row r="35" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B35" s="140"/>
+      <c r="B35" s="138"/>
       <c r="C35" s="114" t="s">
         <v>126</v>
       </c>
@@ -3366,184 +3366,184 @@
         <v>127</v>
       </c>
       <c r="E35" s="23" t="s">
+        <v>386</v>
+      </c>
+      <c r="F35" s="23" t="s">
         <v>128</v>
       </c>
-      <c r="F35" s="23" t="s">
+      <c r="G35" s="23" t="s">
+        <v>298</v>
+      </c>
+      <c r="H35" s="24"/>
+    </row>
+    <row r="36" spans="1:11" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="138"/>
+      <c r="C36" s="114" t="s">
         <v>129</v>
       </c>
-      <c r="G35" s="23" t="s">
-        <v>299</v>
-      </c>
-      <c r="H35" s="24"/>
-    </row>
-    <row r="36" spans="1:11" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="140"/>
-      <c r="C36" s="114" t="s">
+      <c r="D36" s="23" t="s">
         <v>130</v>
       </c>
-      <c r="D36" s="23" t="s">
+      <c r="E36" s="23" t="s">
         <v>131</v>
-      </c>
-      <c r="E36" s="23" t="s">
-        <v>132</v>
       </c>
       <c r="F36" s="23" t="s">
         <v>30</v>
       </c>
       <c r="G36" s="23" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H36" s="12"/>
     </row>
     <row r="37" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="B37" s="140"/>
+      <c r="B37" s="138"/>
       <c r="C37" s="114" t="s">
+        <v>132</v>
+      </c>
+      <c r="D37" s="23" t="s">
         <v>133</v>
       </c>
-      <c r="D37" s="23" t="s">
+      <c r="E37" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="E37" s="23" t="s">
+      <c r="F37" s="23" t="s">
         <v>135</v>
       </c>
-      <c r="F37" s="23" t="s">
-        <v>136</v>
-      </c>
       <c r="G37" s="23" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H37" s="12"/>
     </row>
     <row r="38" spans="1:11" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="95"/>
-      <c r="B38" s="140"/>
+      <c r="B38" s="138"/>
       <c r="C38" s="114" t="s">
+        <v>273</v>
+      </c>
+      <c r="D38" s="115" t="s">
         <v>274</v>
       </c>
-      <c r="D38" s="115" t="s">
-        <v>275</v>
-      </c>
-      <c r="E38" s="124" t="s">
-        <v>362</v>
+      <c r="E38" s="140" t="s">
+        <v>361</v>
       </c>
       <c r="F38" s="115"/>
       <c r="G38" s="115" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H38" s="12"/>
     </row>
     <row r="39" spans="1:11" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="95"/>
-      <c r="B39" s="140"/>
+      <c r="B39" s="138"/>
       <c r="C39" s="116" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D39" s="115" t="s">
-        <v>275</v>
-      </c>
-      <c r="E39" s="125"/>
+        <v>274</v>
+      </c>
+      <c r="E39" s="141"/>
       <c r="F39" s="115"/>
       <c r="G39" s="115" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H39" s="12"/>
     </row>
     <row r="40" spans="1:11" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="95"/>
-      <c r="B40" s="141"/>
+      <c r="B40" s="139"/>
       <c r="C40" s="114" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D40" s="115" t="s">
-        <v>275</v>
-      </c>
-      <c r="E40" s="126"/>
+        <v>274</v>
+      </c>
+      <c r="E40" s="142"/>
       <c r="F40" s="115"/>
       <c r="G40" s="115" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H40" s="12"/>
     </row>
     <row r="41" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B41" s="130" t="s">
-        <v>308</v>
+      <c r="B41" s="126" t="s">
+        <v>307</v>
       </c>
       <c r="C41" s="26" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D41" s="117" t="s">
+        <v>268</v>
+      </c>
+      <c r="E41" s="117" t="s">
         <v>269</v>
-      </c>
-      <c r="E41" s="117" t="s">
-        <v>270</v>
       </c>
       <c r="F41" s="117" t="s">
         <v>41</v>
       </c>
       <c r="G41" s="117" t="s">
+        <v>298</v>
+      </c>
+      <c r="H41" s="24"/>
+    </row>
+    <row r="42" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B42" s="127"/>
+      <c r="C42" s="26" t="s">
+        <v>266</v>
+      </c>
+      <c r="D42" s="117" t="s">
+        <v>267</v>
+      </c>
+      <c r="E42" s="117" t="s">
+        <v>270</v>
+      </c>
+      <c r="F42" s="117" t="s">
+        <v>137</v>
+      </c>
+      <c r="G42" s="117" t="s">
+        <v>298</v>
+      </c>
+      <c r="H42" s="24"/>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B43" s="143"/>
+      <c r="C43" s="26" t="s">
+        <v>287</v>
+      </c>
+      <c r="D43" s="117" t="s">
+        <v>288</v>
+      </c>
+      <c r="E43" s="117" t="s">
+        <v>289</v>
+      </c>
+      <c r="F43" s="117" t="s">
+        <v>137</v>
+      </c>
+      <c r="G43" s="117" t="s">
         <v>299</v>
       </c>
-      <c r="H41" s="24"/>
-    </row>
-    <row r="42" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B42" s="131"/>
-      <c r="C42" s="26" t="s">
-        <v>267</v>
-      </c>
-      <c r="D42" s="117" t="s">
-        <v>268</v>
-      </c>
-      <c r="E42" s="117" t="s">
+      <c r="H43" s="24"/>
+    </row>
+    <row r="44" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A44" s="125" t="s">
+        <v>319</v>
+      </c>
+      <c r="B44" s="126" t="s">
+        <v>313</v>
+      </c>
+      <c r="C44" s="117" t="s">
+        <v>141</v>
+      </c>
+      <c r="D44" s="117" t="s">
+        <v>142</v>
+      </c>
+      <c r="E44" s="117" t="s">
         <v>271</v>
       </c>
-      <c r="F42" s="117" t="s">
-        <v>138</v>
-      </c>
-      <c r="G42" s="117" t="s">
+      <c r="F44" s="117" t="s">
+        <v>139</v>
+      </c>
+      <c r="G44" s="117" t="s">
         <v>299</v>
-      </c>
-      <c r="H42" s="24"/>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B43" s="132"/>
-      <c r="C43" s="26" t="s">
-        <v>288</v>
-      </c>
-      <c r="D43" s="117" t="s">
-        <v>289</v>
-      </c>
-      <c r="E43" s="117" t="s">
-        <v>290</v>
-      </c>
-      <c r="F43" s="117" t="s">
-        <v>138</v>
-      </c>
-      <c r="G43" s="117" t="s">
-        <v>300</v>
-      </c>
-      <c r="H43" s="24"/>
-    </row>
-    <row r="44" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A44" s="142" t="s">
-        <v>320</v>
-      </c>
-      <c r="B44" s="130" t="s">
-        <v>314</v>
-      </c>
-      <c r="C44" s="117" t="s">
-        <v>142</v>
-      </c>
-      <c r="D44" s="117" t="s">
-        <v>143</v>
-      </c>
-      <c r="E44" s="117" t="s">
-        <v>272</v>
-      </c>
-      <c r="F44" s="117" t="s">
-        <v>140</v>
-      </c>
-      <c r="G44" s="117" t="s">
-        <v>300</v>
       </c>
       <c r="H44" s="30"/>
       <c r="I44" s="28"/>
@@ -3551,22 +3551,22 @@
       <c r="K44" s="28"/>
     </row>
     <row r="45" spans="1:11" s="29" customFormat="1" ht="224.4" x14ac:dyDescent="0.3">
-      <c r="A45" s="142"/>
-      <c r="B45" s="131"/>
+      <c r="A45" s="125"/>
+      <c r="B45" s="127"/>
       <c r="C45" s="117" t="s">
+        <v>143</v>
+      </c>
+      <c r="D45" s="117" t="s">
         <v>144</v>
       </c>
-      <c r="D45" s="117" t="s">
-        <v>145</v>
-      </c>
       <c r="E45" s="117" t="s">
-        <v>363</v>
+        <v>387</v>
       </c>
       <c r="F45" s="26" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G45" s="26" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H45" s="30"/>
       <c r="I45" s="28"/>
@@ -3574,24 +3574,24 @@
       <c r="K45" s="28"/>
     </row>
     <row r="46" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A46" s="142"/>
-      <c r="B46" s="130" t="s">
-        <v>315</v>
+      <c r="A46" s="125"/>
+      <c r="B46" s="126" t="s">
+        <v>314</v>
       </c>
       <c r="C46" s="117" t="s">
+        <v>145</v>
+      </c>
+      <c r="D46" s="117" t="s">
         <v>146</v>
       </c>
-      <c r="D46" s="117" t="s">
-        <v>147</v>
-      </c>
       <c r="E46" s="117" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F46" s="117" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G46" s="117" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H46" s="30"/>
       <c r="I46" s="28"/>
@@ -3599,22 +3599,22 @@
       <c r="K46" s="28"/>
     </row>
     <row r="47" spans="1:11" s="29" customFormat="1" ht="224.4" x14ac:dyDescent="0.3">
-      <c r="A47" s="142"/>
-      <c r="B47" s="131"/>
+      <c r="A47" s="125"/>
+      <c r="B47" s="127"/>
       <c r="C47" s="117" t="s">
+        <v>147</v>
+      </c>
+      <c r="D47" s="117" t="s">
         <v>148</v>
       </c>
-      <c r="D47" s="117" t="s">
-        <v>149</v>
-      </c>
       <c r="E47" s="117" t="s">
-        <v>363</v>
+        <v>387</v>
       </c>
       <c r="F47" s="26" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G47" s="26" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H47" s="30"/>
       <c r="I47" s="28"/>
@@ -3623,23 +3623,23 @@
     </row>
     <row r="48" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A48"/>
-      <c r="B48" s="127" t="s">
+      <c r="B48" s="122" t="s">
+        <v>165</v>
+      </c>
+      <c r="C48" s="36" t="s">
         <v>166</v>
       </c>
-      <c r="C48" s="36" t="s">
+      <c r="D48" s="37" t="s">
         <v>167</v>
       </c>
-      <c r="D48" s="37" t="s">
+      <c r="E48" s="37" t="s">
         <v>168</v>
       </c>
-      <c r="E48" s="37" t="s">
-        <v>169</v>
-      </c>
       <c r="F48" s="36" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G48" s="36" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H48" s="31"/>
       <c r="I48" s="32"/>
@@ -3648,21 +3648,21 @@
     </row>
     <row r="49" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A49"/>
-      <c r="B49" s="129"/>
+      <c r="B49" s="124"/>
       <c r="C49" s="36" t="s">
+        <v>169</v>
+      </c>
+      <c r="D49" s="37" t="s">
         <v>170</v>
       </c>
-      <c r="D49" s="37" t="s">
+      <c r="E49" s="37" t="s">
         <v>171</v>
       </c>
-      <c r="E49" s="37" t="s">
+      <c r="F49" s="36" t="s">
         <v>172</v>
       </c>
-      <c r="F49" s="36" t="s">
-        <v>173</v>
-      </c>
       <c r="G49" s="36" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H49" s="31"/>
       <c r="I49" s="32"/>
@@ -3670,26 +3670,26 @@
       <c r="K49" s="32"/>
     </row>
     <row r="50" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A50" s="142" t="s">
-        <v>321</v>
-      </c>
-      <c r="B50" s="127" t="s">
-        <v>316</v>
+      <c r="A50" s="125" t="s">
+        <v>320</v>
+      </c>
+      <c r="B50" s="122" t="s">
+        <v>315</v>
       </c>
       <c r="C50" s="36" t="s">
+        <v>173</v>
+      </c>
+      <c r="D50" s="37" t="s">
         <v>174</v>
       </c>
-      <c r="D50" s="37" t="s">
+      <c r="E50" s="37" t="s">
         <v>175</v>
       </c>
-      <c r="E50" s="37" t="s">
-        <v>176</v>
-      </c>
       <c r="F50" s="36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G50" s="36" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H50" s="31"/>
       <c r="I50" s="32"/>
@@ -3697,22 +3697,22 @@
       <c r="K50" s="32"/>
     </row>
     <row r="51" spans="1:11" s="33" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="142"/>
-      <c r="B51" s="128"/>
+      <c r="A51" s="125"/>
+      <c r="B51" s="123"/>
       <c r="C51" s="36" t="s">
+        <v>176</v>
+      </c>
+      <c r="D51" s="37" t="s">
         <v>177</v>
       </c>
-      <c r="D51" s="37" t="s">
+      <c r="E51" s="37" t="s">
         <v>178</v>
       </c>
-      <c r="E51" s="37" t="s">
+      <c r="F51" s="36" t="s">
         <v>179</v>
       </c>
-      <c r="F51" s="36" t="s">
-        <v>180</v>
-      </c>
       <c r="G51" s="36" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H51" s="31"/>
       <c r="I51" s="32"/>
@@ -3720,22 +3720,22 @@
       <c r="K51" s="32"/>
     </row>
     <row r="52" spans="1:11" s="33" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.3">
-      <c r="A52" s="142"/>
-      <c r="B52" s="128"/>
+      <c r="A52" s="125"/>
+      <c r="B52" s="123"/>
       <c r="C52" s="36" t="s">
+        <v>180</v>
+      </c>
+      <c r="D52" s="37" t="s">
         <v>181</v>
       </c>
-      <c r="D52" s="37" t="s">
-        <v>182</v>
-      </c>
       <c r="E52" s="37" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="F52" s="36" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G52" s="36" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H52" s="31"/>
       <c r="I52" s="32"/>
@@ -3743,22 +3743,22 @@
       <c r="K52" s="32"/>
     </row>
     <row r="53" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A53" s="142"/>
-      <c r="B53" s="129"/>
+      <c r="A53" s="125"/>
+      <c r="B53" s="124"/>
       <c r="C53" s="36" t="s">
+        <v>182</v>
+      </c>
+      <c r="D53" s="37" t="s">
         <v>183</v>
       </c>
-      <c r="D53" s="37" t="s">
+      <c r="E53" s="37" t="s">
         <v>184</v>
-      </c>
-      <c r="E53" s="37" t="s">
-        <v>185</v>
       </c>
       <c r="F53" s="37" t="s">
         <v>30</v>
       </c>
       <c r="G53" s="36" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H53" s="31"/>
       <c r="I53" s="32"/>
@@ -3766,26 +3766,26 @@
       <c r="K53" s="32"/>
     </row>
     <row r="54" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A54" s="142" t="s">
-        <v>322</v>
-      </c>
-      <c r="B54" s="127" t="s">
-        <v>319</v>
+      <c r="A54" s="125" t="s">
+        <v>321</v>
+      </c>
+      <c r="B54" s="122" t="s">
+        <v>318</v>
       </c>
       <c r="C54" s="36" t="s">
+        <v>185</v>
+      </c>
+      <c r="D54" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="D54" s="37" t="s">
+      <c r="E54" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="E54" s="37" t="s">
-        <v>188</v>
-      </c>
       <c r="F54" s="36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G54" s="36" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H54" s="31"/>
       <c r="I54" s="32"/>
@@ -3793,22 +3793,22 @@
       <c r="K54" s="32"/>
     </row>
     <row r="55" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A55" s="142"/>
-      <c r="B55" s="128"/>
+      <c r="A55" s="125"/>
+      <c r="B55" s="123"/>
       <c r="C55" s="36" t="s">
+        <v>188</v>
+      </c>
+      <c r="D55" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="D55" s="37" t="s">
+      <c r="E55" s="37" t="s">
         <v>190</v>
       </c>
-      <c r="E55" s="37" t="s">
+      <c r="F55" s="36" t="s">
         <v>191</v>
       </c>
-      <c r="F55" s="36" t="s">
-        <v>192</v>
-      </c>
       <c r="G55" s="36" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H55" s="31"/>
       <c r="I55" s="32"/>
@@ -3816,22 +3816,22 @@
       <c r="K55" s="32"/>
     </row>
     <row r="56" spans="1:11" s="33" customFormat="1" ht="356.4" x14ac:dyDescent="0.3">
-      <c r="A56" s="142"/>
-      <c r="B56" s="128"/>
+      <c r="A56" s="125"/>
+      <c r="B56" s="123"/>
       <c r="C56" s="36" t="s">
+        <v>192</v>
+      </c>
+      <c r="D56" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="D56" s="37" t="s">
-        <v>194</v>
-      </c>
       <c r="E56" s="37" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="F56" s="37" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G56" s="36" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H56" s="31"/>
       <c r="I56" s="32"/>
@@ -3839,22 +3839,22 @@
       <c r="K56" s="32"/>
     </row>
     <row r="57" spans="1:11" s="33" customFormat="1" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A57" s="142"/>
-      <c r="B57" s="129"/>
+      <c r="A57" s="125"/>
+      <c r="B57" s="124"/>
       <c r="C57" s="36" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D57" s="37" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E57" s="37" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F57" s="36" t="s">
         <v>30</v>
       </c>
       <c r="G57" s="36" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H57" s="31"/>
       <c r="I57" s="32"/>
@@ -3862,26 +3862,26 @@
       <c r="K57" s="32"/>
     </row>
     <row r="58" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A58" s="142" t="s">
-        <v>321</v>
-      </c>
-      <c r="B58" s="127" t="s">
-        <v>318</v>
+      <c r="A58" s="125" t="s">
+        <v>320</v>
+      </c>
+      <c r="B58" s="122" t="s">
+        <v>317</v>
       </c>
       <c r="C58" s="36" t="s">
+        <v>195</v>
+      </c>
+      <c r="D58" s="37" t="s">
         <v>196</v>
       </c>
-      <c r="D58" s="37" t="s">
+      <c r="E58" s="37" t="s">
         <v>197</v>
       </c>
-      <c r="E58" s="37" t="s">
-        <v>198</v>
-      </c>
       <c r="F58" s="36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G58" s="36" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H58" s="31"/>
       <c r="I58" s="32"/>
@@ -3889,22 +3889,22 @@
       <c r="K58" s="32"/>
     </row>
     <row r="59" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A59" s="142"/>
-      <c r="B59" s="128"/>
+      <c r="A59" s="125"/>
+      <c r="B59" s="123"/>
       <c r="C59" s="36" t="s">
+        <v>198</v>
+      </c>
+      <c r="D59" s="37" t="s">
         <v>199</v>
       </c>
-      <c r="D59" s="37" t="s">
-        <v>200</v>
-      </c>
       <c r="E59" s="37" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F59" s="36" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G59" s="36" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H59" s="31"/>
       <c r="I59" s="32"/>
@@ -3912,22 +3912,22 @@
       <c r="K59" s="32"/>
     </row>
     <row r="60" spans="1:11" s="33" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.3">
-      <c r="A60" s="142"/>
-      <c r="B60" s="128"/>
+      <c r="A60" s="125"/>
+      <c r="B60" s="123"/>
       <c r="C60" s="36" t="s">
+        <v>200</v>
+      </c>
+      <c r="D60" s="37" t="s">
         <v>201</v>
       </c>
-      <c r="D60" s="37" t="s">
-        <v>202</v>
-      </c>
       <c r="E60" s="37" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="F60" s="36" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G60" s="36" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H60" s="31"/>
       <c r="I60" s="32"/>
@@ -3935,22 +3935,22 @@
       <c r="K60" s="32"/>
     </row>
     <row r="61" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A61" s="142"/>
-      <c r="B61" s="129"/>
+      <c r="A61" s="125"/>
+      <c r="B61" s="124"/>
       <c r="C61" s="36" t="s">
+        <v>202</v>
+      </c>
+      <c r="D61" s="37" t="s">
         <v>203</v>
       </c>
-      <c r="D61" s="37" t="s">
-        <v>204</v>
-      </c>
       <c r="E61" s="37" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F61" s="37" t="s">
         <v>30</v>
       </c>
       <c r="G61" s="36" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H61" s="31"/>
       <c r="I61" s="32"/>
@@ -3958,26 +3958,26 @@
       <c r="K61" s="32"/>
     </row>
     <row r="62" spans="1:11" s="33" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="142" t="s">
-        <v>322</v>
-      </c>
-      <c r="B62" s="127" t="s">
-        <v>317</v>
+      <c r="A62" s="125" t="s">
+        <v>321</v>
+      </c>
+      <c r="B62" s="122" t="s">
+        <v>316</v>
       </c>
       <c r="C62" s="36" t="s">
+        <v>204</v>
+      </c>
+      <c r="D62" s="37" t="s">
         <v>205</v>
       </c>
-      <c r="D62" s="37" t="s">
+      <c r="E62" s="37" t="s">
         <v>206</v>
       </c>
-      <c r="E62" s="37" t="s">
-        <v>207</v>
-      </c>
       <c r="F62" s="36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G62" s="36" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H62" s="31"/>
       <c r="I62" s="32"/>
@@ -3985,22 +3985,22 @@
       <c r="K62" s="32"/>
     </row>
     <row r="63" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A63" s="142"/>
-      <c r="B63" s="128"/>
+      <c r="A63" s="125"/>
+      <c r="B63" s="123"/>
       <c r="C63" s="36" t="s">
+        <v>207</v>
+      </c>
+      <c r="D63" s="37" t="s">
         <v>208</v>
       </c>
-      <c r="D63" s="37" t="s">
+      <c r="E63" s="37" t="s">
         <v>209</v>
       </c>
-      <c r="E63" s="37" t="s">
-        <v>210</v>
-      </c>
       <c r="F63" s="36" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G63" s="36" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H63" s="31"/>
       <c r="I63" s="32"/>
@@ -4008,163 +4008,163 @@
       <c r="K63" s="32"/>
     </row>
     <row r="64" spans="1:11" ht="356.4" x14ac:dyDescent="0.3">
-      <c r="A64" s="142"/>
-      <c r="B64" s="128"/>
+      <c r="A64" s="125"/>
+      <c r="B64" s="123"/>
       <c r="C64" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="D64" s="37" t="s">
         <v>211</v>
       </c>
-      <c r="D64" s="37" t="s">
+      <c r="E64" s="37" t="s">
+        <v>383</v>
+      </c>
+      <c r="F64" s="37" t="s">
+        <v>292</v>
+      </c>
+      <c r="G64" s="36" t="s">
+        <v>291</v>
+      </c>
+      <c r="H64" s="12"/>
+    </row>
+    <row r="65" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A65" s="125"/>
+      <c r="B65" s="124"/>
+      <c r="C65" s="36" t="s">
+        <v>357</v>
+      </c>
+      <c r="D65" s="37" t="s">
         <v>212</v>
       </c>
-      <c r="E64" s="37" t="s">
-        <v>387</v>
-      </c>
-      <c r="F64" s="37" t="s">
-        <v>293</v>
-      </c>
-      <c r="G64" s="36" t="s">
-        <v>292</v>
-      </c>
-      <c r="H64" s="12"/>
-    </row>
-    <row r="65" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A65" s="142"/>
-      <c r="B65" s="129"/>
-      <c r="C65" s="36" t="s">
-        <v>358</v>
-      </c>
-      <c r="D65" s="37" t="s">
-        <v>213</v>
-      </c>
       <c r="E65" s="37" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F65" s="36" t="s">
         <v>30</v>
       </c>
       <c r="G65" s="36" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H65" s="12"/>
     </row>
     <row r="66" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B66" s="127" t="s">
-        <v>309</v>
+      <c r="B66" s="122" t="s">
+        <v>308</v>
       </c>
       <c r="C66" s="36" t="s">
+        <v>213</v>
+      </c>
+      <c r="D66" s="37" t="s">
         <v>214</v>
       </c>
-      <c r="D66" s="37" t="s">
+      <c r="E66" s="37" t="s">
+        <v>362</v>
+      </c>
+      <c r="F66" s="36" t="s">
         <v>215</v>
       </c>
-      <c r="E66" s="37" t="s">
-        <v>364</v>
-      </c>
-      <c r="F66" s="36" t="s">
+      <c r="G66" s="36" t="s">
+        <v>299</v>
+      </c>
+      <c r="H66" s="10"/>
+    </row>
+    <row r="67" spans="1:11" ht="93" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B67" s="123"/>
+      <c r="C67" s="36" t="s">
         <v>216</v>
       </c>
-      <c r="G66" s="36" t="s">
-        <v>300</v>
-      </c>
-      <c r="H66" s="10"/>
-    </row>
-    <row r="67" spans="1:11" ht="93" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B67" s="128"/>
-      <c r="C67" s="36" t="s">
+      <c r="D67" s="37" t="s">
         <v>217</v>
       </c>
-      <c r="D67" s="37" t="s">
-        <v>218</v>
-      </c>
       <c r="E67" s="37" t="s">
-        <v>365</v>
+        <v>388</v>
       </c>
       <c r="F67" s="36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G67" s="36" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H67" s="12"/>
     </row>
     <row r="68" spans="1:11" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B68" s="128"/>
+      <c r="B68" s="123"/>
       <c r="C68" s="36" t="s">
+        <v>372</v>
+      </c>
+      <c r="D68" s="37" t="s">
+        <v>374</v>
+      </c>
+      <c r="E68" s="37" t="s">
+        <v>379</v>
+      </c>
+      <c r="F68" s="36" t="s">
         <v>376</v>
       </c>
-      <c r="D68" s="37" t="s">
+      <c r="G68" s="36" t="s">
+        <v>298</v>
+      </c>
+      <c r="H68" s="12"/>
+    </row>
+    <row r="69" spans="1:11" ht="158.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B69" s="123"/>
+      <c r="C69" s="36" t="s">
+        <v>373</v>
+      </c>
+      <c r="D69" s="37" t="s">
+        <v>377</v>
+      </c>
+      <c r="E69" s="37" t="s">
+        <v>380</v>
+      </c>
+      <c r="F69" s="36" t="s">
+        <v>384</v>
+      </c>
+      <c r="G69" s="36" t="s">
+        <v>298</v>
+      </c>
+      <c r="H69" s="12"/>
+    </row>
+    <row r="70" spans="1:11" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B70" s="124"/>
+      <c r="C70" s="36" t="s">
+        <v>375</v>
+      </c>
+      <c r="D70" s="37" t="s">
         <v>378</v>
       </c>
-      <c r="E68" s="37" t="s">
-        <v>383</v>
-      </c>
-      <c r="F68" s="36" t="s">
-        <v>380</v>
-      </c>
-      <c r="G68" s="36" t="s">
-        <v>299</v>
-      </c>
-      <c r="H68" s="12"/>
-    </row>
-    <row r="69" spans="1:11" ht="158.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B69" s="128"/>
-      <c r="C69" s="36" t="s">
-        <v>377</v>
-      </c>
-      <c r="D69" s="37" t="s">
-        <v>381</v>
-      </c>
-      <c r="E69" s="37" t="s">
-        <v>384</v>
-      </c>
-      <c r="F69" s="36" t="s">
-        <v>388</v>
-      </c>
-      <c r="G69" s="36" t="s">
-        <v>299</v>
-      </c>
-      <c r="H69" s="12"/>
-    </row>
-    <row r="70" spans="1:11" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B70" s="129"/>
-      <c r="C70" s="36" t="s">
-        <v>379</v>
-      </c>
-      <c r="D70" s="37" t="s">
-        <v>382</v>
-      </c>
       <c r="E70" s="37" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F70" s="36" t="s">
         <v>30</v>
       </c>
       <c r="G70" s="36" t="s">
+        <v>298</v>
+      </c>
+      <c r="H70" s="12"/>
+    </row>
+    <row r="71" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A71" s="125" t="s">
+        <v>322</v>
+      </c>
+      <c r="B71" s="122" t="s">
+        <v>309</v>
+      </c>
+      <c r="C71" s="36" t="s">
+        <v>218</v>
+      </c>
+      <c r="D71" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="E71" s="37" t="s">
+        <v>220</v>
+      </c>
+      <c r="F71" s="36" t="s">
+        <v>221</v>
+      </c>
+      <c r="G71" s="36" t="s">
         <v>299</v>
-      </c>
-      <c r="H70" s="12"/>
-    </row>
-    <row r="71" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A71" s="142" t="s">
-        <v>323</v>
-      </c>
-      <c r="B71" s="127" t="s">
-        <v>310</v>
-      </c>
-      <c r="C71" s="36" t="s">
-        <v>219</v>
-      </c>
-      <c r="D71" s="37" t="s">
-        <v>220</v>
-      </c>
-      <c r="E71" s="37" t="s">
-        <v>221</v>
-      </c>
-      <c r="F71" s="36" t="s">
-        <v>222</v>
-      </c>
-      <c r="G71" s="36" t="s">
-        <v>300</v>
       </c>
       <c r="H71" s="30"/>
       <c r="I71" s="28"/>
@@ -4172,22 +4172,22 @@
       <c r="K71" s="28"/>
     </row>
     <row r="72" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A72" s="142"/>
-      <c r="B72" s="128"/>
+      <c r="A72" s="125"/>
+      <c r="B72" s="123"/>
       <c r="C72" s="36" t="s">
+        <v>222</v>
+      </c>
+      <c r="D72" s="37" t="s">
         <v>223</v>
       </c>
-      <c r="D72" s="37" t="s">
+      <c r="E72" s="37" t="s">
         <v>224</v>
       </c>
-      <c r="E72" s="37" t="s">
-        <v>225</v>
-      </c>
       <c r="F72" s="36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G72" s="36" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H72" s="30"/>
       <c r="I72" s="28"/>
@@ -4195,22 +4195,22 @@
       <c r="K72" s="28"/>
     </row>
     <row r="73" spans="1:11" s="29" customFormat="1" ht="198" x14ac:dyDescent="0.3">
-      <c r="A73" s="142"/>
-      <c r="B73" s="129"/>
+      <c r="A73" s="125"/>
+      <c r="B73" s="124"/>
       <c r="C73" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="D73" s="37" t="s">
         <v>226</v>
       </c>
-      <c r="D73" s="37" t="s">
-        <v>227</v>
-      </c>
       <c r="E73" s="37" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="F73" s="36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G73" s="36" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H73" s="30"/>
       <c r="I73" s="28"/>
@@ -4218,24 +4218,24 @@
       <c r="K73" s="28"/>
     </row>
     <row r="74" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A74" s="142"/>
-      <c r="B74" s="127" t="s">
-        <v>310</v>
+      <c r="A74" s="125"/>
+      <c r="B74" s="122" t="s">
+        <v>309</v>
       </c>
       <c r="C74" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="D74" s="37" t="s">
         <v>228</v>
       </c>
-      <c r="D74" s="37" t="s">
+      <c r="E74" s="37" t="s">
         <v>229</v>
       </c>
-      <c r="E74" s="37" t="s">
-        <v>230</v>
-      </c>
       <c r="F74" s="36" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G74" s="36" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H74" s="30"/>
       <c r="I74" s="28"/>
@@ -4243,22 +4243,22 @@
       <c r="K74" s="28"/>
     </row>
     <row r="75" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A75" s="142"/>
-      <c r="B75" s="128"/>
+      <c r="A75" s="125"/>
+      <c r="B75" s="123"/>
       <c r="C75" s="36" t="s">
+        <v>230</v>
+      </c>
+      <c r="D75" s="37" t="s">
         <v>231</v>
       </c>
-      <c r="D75" s="37" t="s">
+      <c r="E75" s="37" t="s">
         <v>232</v>
       </c>
-      <c r="E75" s="37" t="s">
-        <v>233</v>
-      </c>
       <c r="F75" s="36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G75" s="36" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H75" s="30"/>
       <c r="I75" s="28"/>
@@ -4266,22 +4266,22 @@
       <c r="K75" s="28"/>
     </row>
     <row r="76" spans="1:11" s="29" customFormat="1" ht="198" x14ac:dyDescent="0.3">
-      <c r="A76" s="142"/>
-      <c r="B76" s="129"/>
+      <c r="A76" s="125"/>
+      <c r="B76" s="124"/>
       <c r="C76" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="D76" s="37" t="s">
         <v>234</v>
       </c>
-      <c r="D76" s="37" t="s">
-        <v>235</v>
-      </c>
       <c r="E76" s="37" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="F76" s="36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G76" s="36" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H76" s="30"/>
       <c r="I76" s="28"/>
@@ -4290,23 +4290,23 @@
     </row>
     <row r="77" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A77"/>
-      <c r="B77" s="127" t="s">
-        <v>311</v>
+      <c r="B77" s="122" t="s">
+        <v>310</v>
       </c>
       <c r="C77" s="118" t="s">
+        <v>235</v>
+      </c>
+      <c r="D77" s="118" t="s">
         <v>236</v>
       </c>
-      <c r="D77" s="118" t="s">
+      <c r="E77" s="118" t="s">
         <v>237</v>
       </c>
-      <c r="E77" s="118" t="s">
-        <v>238</v>
-      </c>
       <c r="F77" s="119" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G77" s="119" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H77" s="30"/>
       <c r="I77" s="28"/>
@@ -4315,21 +4315,21 @@
     </row>
     <row r="78" spans="1:11" s="33" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A78"/>
-      <c r="B78" s="129"/>
+      <c r="B78" s="124"/>
       <c r="C78" s="118" t="s">
+        <v>238</v>
+      </c>
+      <c r="D78" s="118" t="s">
         <v>239</v>
       </c>
-      <c r="D78" s="118" t="s">
-        <v>240</v>
-      </c>
       <c r="E78" s="118" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="F78" s="118" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G78" s="118" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H78" s="31"/>
       <c r="I78" s="32"/>
@@ -4337,26 +4337,26 @@
       <c r="K78" s="32"/>
     </row>
     <row r="79" spans="1:11" s="33" customFormat="1" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="142" t="s">
+      <c r="A79" s="125" t="s">
+        <v>323</v>
+      </c>
+      <c r="B79" s="122" t="s">
         <v>324</v>
       </c>
-      <c r="B79" s="127" t="s">
-        <v>325</v>
-      </c>
       <c r="C79" s="36" t="s">
+        <v>240</v>
+      </c>
+      <c r="D79" s="37" t="s">
         <v>241</v>
       </c>
-      <c r="D79" s="37" t="s">
-        <v>242</v>
-      </c>
       <c r="E79" s="118" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="F79" s="36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G79" s="36" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H79" s="31"/>
       <c r="I79" s="32"/>
@@ -4364,22 +4364,22 @@
       <c r="K79" s="32"/>
     </row>
     <row r="80" spans="1:11" s="33" customFormat="1" ht="78" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="142"/>
-      <c r="B80" s="128"/>
+      <c r="A80" s="125"/>
+      <c r="B80" s="123"/>
       <c r="C80" s="36" t="s">
+        <v>327</v>
+      </c>
+      <c r="D80" s="37" t="s">
         <v>328</v>
       </c>
-      <c r="D80" s="37" t="s">
-        <v>329</v>
-      </c>
       <c r="E80" s="37" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="F80" s="36" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G80" s="36" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H80" s="31"/>
       <c r="I80" s="32"/>
@@ -4387,19 +4387,19 @@
       <c r="K80" s="32"/>
     </row>
     <row r="81" spans="1:11" s="33" customFormat="1" ht="212.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="142"/>
-      <c r="B81" s="129"/>
+      <c r="A81" s="125"/>
+      <c r="B81" s="124"/>
       <c r="C81" s="36" t="s">
+        <v>329</v>
+      </c>
+      <c r="D81" s="37" t="s">
         <v>330</v>
       </c>
-      <c r="D81" s="37" t="s">
+      <c r="E81" s="37" t="s">
+        <v>367</v>
+      </c>
+      <c r="F81" s="36" t="s">
         <v>331</v>
-      </c>
-      <c r="E81" s="37" t="s">
-        <v>370</v>
-      </c>
-      <c r="F81" s="36" t="s">
-        <v>332</v>
       </c>
       <c r="G81" s="36"/>
       <c r="H81" s="31"/>
@@ -4408,26 +4408,26 @@
       <c r="K81" s="32"/>
     </row>
     <row r="82" spans="1:11" s="33" customFormat="1" ht="117" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="142" t="s">
-        <v>324</v>
-      </c>
-      <c r="B82" s="127" t="s">
-        <v>326</v>
+      <c r="A82" s="125" t="s">
+        <v>323</v>
+      </c>
+      <c r="B82" s="122" t="s">
+        <v>325</v>
       </c>
       <c r="C82" s="36" t="s">
+        <v>242</v>
+      </c>
+      <c r="D82" s="37" t="s">
         <v>243</v>
       </c>
-      <c r="D82" s="37" t="s">
-        <v>244</v>
-      </c>
       <c r="E82" s="118" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="F82" s="36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G82" s="36" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H82" s="31"/>
       <c r="I82" s="32"/>
@@ -4435,22 +4435,22 @@
       <c r="K82" s="32"/>
     </row>
     <row r="83" spans="1:11" s="33" customFormat="1" ht="83.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="142"/>
-      <c r="B83" s="128"/>
+      <c r="A83" s="125"/>
+      <c r="B83" s="123"/>
       <c r="C83" s="36" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D83" s="37" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E83" s="37" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="F83" s="36" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G83" s="36" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H83" s="31"/>
       <c r="I83" s="32"/>
@@ -4458,19 +4458,19 @@
       <c r="K83" s="32"/>
     </row>
     <row r="84" spans="1:11" s="33" customFormat="1" ht="199.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="142"/>
-      <c r="B84" s="129"/>
+      <c r="A84" s="125"/>
+      <c r="B84" s="124"/>
       <c r="C84" s="36" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D84" s="37" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E84" s="37" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="F84" s="36" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="G84" s="36"/>
       <c r="H84" s="31"/>
@@ -4479,77 +4479,77 @@
       <c r="K84" s="32"/>
     </row>
     <row r="85" spans="1:11" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="B85" s="127" t="s">
-        <v>312</v>
+      <c r="B85" s="122" t="s">
+        <v>311</v>
       </c>
       <c r="C85" s="36" t="s">
+        <v>252</v>
+      </c>
+      <c r="D85" s="37" t="s">
         <v>253</v>
       </c>
-      <c r="D85" s="37" t="s">
+      <c r="E85" s="118" t="s">
+        <v>371</v>
+      </c>
+      <c r="F85" s="36" t="s">
+        <v>306</v>
+      </c>
+      <c r="G85" s="36" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" ht="118.8" x14ac:dyDescent="0.3">
+      <c r="B86" s="123"/>
+      <c r="C86" s="36" t="s">
         <v>254</v>
       </c>
-      <c r="E85" s="118" t="s">
-        <v>374</v>
-      </c>
-      <c r="F85" s="36" t="s">
-        <v>307</v>
-      </c>
-      <c r="G85" s="36" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="86" spans="1:11" ht="118.8" x14ac:dyDescent="0.3">
-      <c r="B86" s="128"/>
-      <c r="C86" s="36" t="s">
+      <c r="D86" s="37" t="s">
         <v>255</v>
       </c>
-      <c r="D86" s="37" t="s">
+      <c r="E86" s="118" t="s">
+        <v>385</v>
+      </c>
+      <c r="F86" s="36" t="s">
+        <v>137</v>
+      </c>
+      <c r="G86" s="36" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" ht="198" x14ac:dyDescent="0.3">
+      <c r="B87" s="123"/>
+      <c r="C87" s="36" t="s">
         <v>256</v>
       </c>
-      <c r="E86" s="118" t="s">
-        <v>375</v>
-      </c>
-      <c r="F86" s="36" t="s">
-        <v>138</v>
-      </c>
-      <c r="G86" s="36" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="87" spans="1:11" ht="198" x14ac:dyDescent="0.3">
-      <c r="B87" s="128"/>
-      <c r="C87" s="36" t="s">
+      <c r="D87" s="37" t="s">
         <v>257</v>
       </c>
-      <c r="D87" s="37" t="s">
+      <c r="E87" s="118" t="s">
+        <v>381</v>
+      </c>
+      <c r="F87" s="36" t="s">
+        <v>305</v>
+      </c>
+      <c r="G87" s="36" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" ht="66" x14ac:dyDescent="0.3">
+      <c r="B88" s="124"/>
+      <c r="C88" s="36" t="s">
         <v>258</v>
       </c>
-      <c r="E87" s="118" t="s">
-        <v>385</v>
-      </c>
-      <c r="F87" s="36" t="s">
-        <v>306</v>
-      </c>
-      <c r="G87" s="36" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="88" spans="1:11" ht="66" x14ac:dyDescent="0.3">
-      <c r="B88" s="129"/>
-      <c r="C88" s="36" t="s">
+      <c r="D88" s="37" t="s">
         <v>259</v>
       </c>
-      <c r="D88" s="37" t="s">
-        <v>260</v>
-      </c>
       <c r="E88" s="118" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F88" s="36" t="s">
         <v>30</v>
       </c>
       <c r="G88" s="36" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.3">
@@ -4586,6 +4586,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="E17:E26"/>
+    <mergeCell ref="E38:E40"/>
+    <mergeCell ref="B82:B84"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="B54:B57"/>
+    <mergeCell ref="B58:B61"/>
+    <mergeCell ref="B62:B65"/>
+    <mergeCell ref="B66:B70"/>
+    <mergeCell ref="B3:B16"/>
+    <mergeCell ref="B17:B26"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="B30:B40"/>
+    <mergeCell ref="B50:B53"/>
     <mergeCell ref="B85:B88"/>
     <mergeCell ref="A17:A26"/>
     <mergeCell ref="B44:B45"/>
@@ -4602,20 +4616,6 @@
     <mergeCell ref="A79:A81"/>
     <mergeCell ref="B79:B81"/>
     <mergeCell ref="A82:A84"/>
-    <mergeCell ref="B3:B16"/>
-    <mergeCell ref="B17:B26"/>
-    <mergeCell ref="B27:B29"/>
-    <mergeCell ref="B30:B40"/>
-    <mergeCell ref="B50:B53"/>
-    <mergeCell ref="E17:E26"/>
-    <mergeCell ref="E38:E40"/>
-    <mergeCell ref="B82:B84"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="B48:B49"/>
-    <mergeCell ref="B54:B57"/>
-    <mergeCell ref="B58:B61"/>
-    <mergeCell ref="B62:B65"/>
-    <mergeCell ref="B66:B70"/>
   </mergeCells>
   <phoneticPr fontId="29" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4644,7 +4644,7 @@
         <v>28</v>
       </c>
       <c r="B1" s="101" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C1" s="102" t="s">
         <v>33</v>
@@ -4653,7 +4653,7 @@
         <v>37</v>
       </c>
       <c r="E1" s="102" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="F1" s="102" t="s">
         <v>42</v>
@@ -4701,19 +4701,19 @@
         <v>91</v>
       </c>
       <c r="U1" s="103" t="s">
+        <v>277</v>
+      </c>
+      <c r="V1" s="103" t="s">
         <v>278</v>
       </c>
-      <c r="V1" s="103" t="s">
+      <c r="W1" s="103" t="s">
         <v>279</v>
       </c>
-      <c r="W1" s="103" t="s">
+      <c r="X1" s="103" t="s">
         <v>280</v>
       </c>
-      <c r="X1" s="103" t="s">
+      <c r="Y1" s="103" t="s">
         <v>281</v>
-      </c>
-      <c r="Y1" s="103" t="s">
-        <v>282</v>
       </c>
       <c r="Z1" s="104" t="s">
         <v>94</v>
@@ -4743,289 +4743,289 @@
         <v>126</v>
       </c>
       <c r="AI1" s="104" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AJ1" s="104" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AK1" s="104" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="AL1" s="104" t="s">
+        <v>275</v>
+      </c>
+      <c r="AM1" s="104" t="s">
         <v>276</v>
       </c>
-      <c r="AM1" s="104" t="s">
-        <v>277</v>
-      </c>
       <c r="AN1" s="105" t="s">
+        <v>265</v>
+      </c>
+      <c r="AO1" s="105" t="s">
         <v>266</v>
       </c>
-      <c r="AO1" s="105" t="s">
-        <v>267</v>
-      </c>
       <c r="AP1" s="44" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="AQ1" s="44" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AR1" s="44" t="s">
+        <v>140</v>
+      </c>
+      <c r="AS1" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="AS1" s="44" t="s">
-        <v>142</v>
-      </c>
       <c r="AT1" s="44" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="AU1" s="44" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="AV1" s="44" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AW1" s="44" t="s">
+        <v>149</v>
+      </c>
+      <c r="AX1" s="44" t="s">
         <v>150</v>
       </c>
-      <c r="AX1" s="44" t="s">
+      <c r="AY1" s="44" t="s">
         <v>151</v>
       </c>
-      <c r="AY1" s="44" t="s">
+      <c r="AZ1" s="44" t="s">
         <v>152</v>
       </c>
-      <c r="AZ1" s="44" t="s">
+      <c r="BA1" s="44" t="s">
         <v>153</v>
       </c>
-      <c r="BA1" s="44" t="s">
+      <c r="BB1" s="44" t="s">
         <v>154</v>
       </c>
-      <c r="BB1" s="44" t="s">
+      <c r="BC1" s="44" t="s">
         <v>155</v>
       </c>
-      <c r="BC1" s="44" t="s">
+      <c r="BD1" s="44" t="s">
         <v>156</v>
       </c>
-      <c r="BD1" s="44" t="s">
+      <c r="BE1" s="44" t="s">
         <v>157</v>
       </c>
-      <c r="BE1" s="44" t="s">
+      <c r="BF1" s="44" t="s">
         <v>158</v>
       </c>
-      <c r="BF1" s="44" t="s">
+      <c r="BG1" s="44" t="s">
         <v>159</v>
       </c>
-      <c r="BG1" s="44" t="s">
+      <c r="BH1" s="44" t="s">
         <v>160</v>
       </c>
-      <c r="BH1" s="44" t="s">
+      <c r="BI1" s="44" t="s">
         <v>161</v>
       </c>
-      <c r="BI1" s="44" t="s">
+      <c r="BJ1" s="44" t="s">
         <v>162</v>
       </c>
-      <c r="BJ1" s="44" t="s">
+      <c r="BK1" s="44" t="s">
         <v>163</v>
       </c>
-      <c r="BK1" s="44" t="s">
+      <c r="BL1" s="44" t="s">
         <v>164</v>
       </c>
-      <c r="BL1" s="44" t="s">
-        <v>165</v>
-      </c>
       <c r="BM1" s="45" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="BN1" s="45" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="BO1" s="45" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="BP1" s="45" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="BQ1" s="45" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="BR1" s="45" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="BS1" s="45" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="BT1" s="45" t="s">
+        <v>260</v>
+      </c>
+      <c r="BU1" s="45" t="s">
         <v>261</v>
       </c>
-      <c r="BU1" s="45" t="s">
+      <c r="BV1" s="45" t="s">
+        <v>358</v>
+      </c>
+      <c r="BW1" s="45" t="s">
+        <v>195</v>
+      </c>
+      <c r="BX1" s="45" t="s">
+        <v>198</v>
+      </c>
+      <c r="BY1" s="45" t="s">
+        <v>200</v>
+      </c>
+      <c r="BZ1" s="45" t="s">
+        <v>202</v>
+      </c>
+      <c r="CA1" s="45" t="s">
+        <v>204</v>
+      </c>
+      <c r="CB1" s="45" t="s">
         <v>262</v>
       </c>
-      <c r="BV1" s="45" t="s">
+      <c r="CC1" s="45" t="s">
+        <v>263</v>
+      </c>
+      <c r="CD1" s="45" t="s">
         <v>359</v>
       </c>
-      <c r="BW1" s="45" t="s">
-        <v>196</v>
-      </c>
-      <c r="BX1" s="45" t="s">
-        <v>199</v>
-      </c>
-      <c r="BY1" s="45" t="s">
-        <v>201</v>
-      </c>
-      <c r="BZ1" s="45" t="s">
-        <v>203</v>
-      </c>
-      <c r="CA1" s="45" t="s">
-        <v>205</v>
-      </c>
-      <c r="CB1" s="45" t="s">
-        <v>263</v>
-      </c>
-      <c r="CC1" s="45" t="s">
-        <v>264</v>
-      </c>
-      <c r="CD1" s="45" t="s">
-        <v>360</v>
-      </c>
       <c r="CE1" s="45" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="CF1" s="45" t="s">
-        <v>217</v>
-      </c>
-      <c r="CG1" s="143" t="s">
-        <v>376</v>
-      </c>
-      <c r="CH1" s="143" t="s">
-        <v>377</v>
-      </c>
-      <c r="CI1" s="143" t="s">
-        <v>379</v>
+        <v>216</v>
+      </c>
+      <c r="CG1" s="121" t="s">
+        <v>372</v>
+      </c>
+      <c r="CH1" s="121" t="s">
+        <v>373</v>
+      </c>
+      <c r="CI1" s="121" t="s">
+        <v>375</v>
       </c>
       <c r="CJ1" s="45" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="CK1" s="45" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="CL1" s="45" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="CM1" s="45" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="CN1" s="45" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="CO1" s="45" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="CP1" s="45" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="CQ1" s="45" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="CR1" s="45" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="CS1" s="45" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="CT1" s="45" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="CU1" s="45" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="CV1" s="45" t="s">
+        <v>332</v>
+      </c>
+      <c r="CW1" s="45" t="s">
         <v>333</v>
       </c>
-      <c r="CW1" s="45" t="s">
-        <v>334</v>
-      </c>
       <c r="CX1" s="45" t="s">
+        <v>244</v>
+      </c>
+      <c r="CY1" s="45" t="s">
+        <v>336</v>
+      </c>
+      <c r="CZ1" s="45" t="s">
+        <v>344</v>
+      </c>
+      <c r="DA1" s="45" t="s">
         <v>245</v>
       </c>
-      <c r="CY1" s="45" t="s">
+      <c r="DB1" s="45" t="s">
         <v>337</v>
       </c>
-      <c r="CZ1" s="45" t="s">
+      <c r="DC1" s="45" t="s">
         <v>345</v>
       </c>
-      <c r="DA1" s="45" t="s">
+      <c r="DD1" s="45" t="s">
         <v>246</v>
       </c>
-      <c r="DB1" s="45" t="s">
+      <c r="DE1" s="45" t="s">
         <v>338</v>
       </c>
-      <c r="DC1" s="45" t="s">
+      <c r="DF1" s="45" t="s">
         <v>346</v>
       </c>
-      <c r="DD1" s="45" t="s">
+      <c r="DG1" s="45" t="s">
         <v>247</v>
       </c>
-      <c r="DE1" s="45" t="s">
+      <c r="DH1" s="45" t="s">
         <v>339</v>
       </c>
-      <c r="DF1" s="45" t="s">
+      <c r="DI1" s="45" t="s">
         <v>347</v>
       </c>
-      <c r="DG1" s="45" t="s">
+      <c r="DJ1" s="45" t="s">
         <v>248</v>
       </c>
-      <c r="DH1" s="45" t="s">
+      <c r="DK1" s="45" t="s">
         <v>340</v>
       </c>
-      <c r="DI1" s="45" t="s">
+      <c r="DL1" s="45" t="s">
         <v>348</v>
       </c>
-      <c r="DJ1" s="45" t="s">
+      <c r="DM1" s="45" t="s">
         <v>249</v>
       </c>
-      <c r="DK1" s="45" t="s">
+      <c r="DN1" s="45" t="s">
         <v>341</v>
       </c>
-      <c r="DL1" s="45" t="s">
+      <c r="DO1" s="45" t="s">
         <v>349</v>
       </c>
-      <c r="DM1" s="45" t="s">
+      <c r="DP1" s="45" t="s">
         <v>250</v>
       </c>
-      <c r="DN1" s="45" t="s">
+      <c r="DQ1" s="45" t="s">
         <v>342</v>
       </c>
-      <c r="DO1" s="45" t="s">
+      <c r="DR1" s="45" t="s">
         <v>350</v>
       </c>
-      <c r="DP1" s="45" t="s">
+      <c r="DS1" s="45" t="s">
         <v>251</v>
       </c>
-      <c r="DQ1" s="45" t="s">
+      <c r="DT1" s="45" t="s">
         <v>343</v>
       </c>
-      <c r="DR1" s="45" t="s">
+      <c r="DU1" s="45" t="s">
         <v>351</v>
       </c>
-      <c r="DS1" s="45" t="s">
+      <c r="DV1" s="45" t="s">
         <v>252</v>
       </c>
-      <c r="DT1" s="45" t="s">
-        <v>344</v>
-      </c>
-      <c r="DU1" s="45" t="s">
-        <v>352</v>
-      </c>
-      <c r="DV1" s="45" t="s">
-        <v>253</v>
-      </c>
       <c r="DW1" s="45" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="DX1" s="45" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="DY1" s="45" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:129" x14ac:dyDescent="0.3">
@@ -20334,6 +20334,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="42fbd5e6-b175-407a-a25c-5fc6410bf24f" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EE7777BCFCD3E741B5CCCE9A87E98C2C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f7fc7590daec4eb8e38e018938a160ca">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e" xmlns:ns3="42fbd5e6-b175-407a-a25c-5fc6410bf24f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c5ca1b94d4b54616210e83d04e6b3cac" ns2:_="" ns3:_="">
     <xsd:import namespace="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
@@ -20588,27 +20608,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E9485EC-5D88-4A1C-961D-0F4FE84359B8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="42fbd5e6-b175-407a-a25c-5fc6410bf24f"/>
+    <ds:schemaRef ds:uri="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="42fbd5e6-b175-407a-a25c-5fc6410bf24f" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{286F673D-E70D-4002-B8F5-CAC95B029A7E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C9C537E-DFD2-4C38-AC8C-930F122DEFFC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -20625,23 +20644,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{286F673D-E70D-4002-B8F5-CAC95B029A7E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E9485EC-5D88-4A1C-961D-0F4FE84359B8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="42fbd5e6-b175-407a-a25c-5fc6410bf24f"/>
-    <ds:schemaRef ds:uri="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
remove insurance from not elig reason
</commit_message>
<xml_diff>
--- a/data/ALAI UP Client-level Reporting Tool Template_4.7.26.xlsx
+++ b/data/ALAI UP Client-level Reporting Tool Template_4.7.26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kmlab\Desktop\Dashboard\alai_up_local_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64DF2EC6-933B-4F0A-94B4-5096AB6A7C30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1BBBB68-8911-4AF2-9375-25796358C44C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-9840" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{500E2EE0-B1C5-4ACF-BC67-EDC8BDABD2D7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{500E2EE0-B1C5-4ACF-BC67-EDC8BDABD2D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="3" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="388">
   <si>
     <t>INSTRUCTIONS</t>
   </si>
@@ -1396,10 +1396,7 @@
 </t>
   </si>
   <si>
-    <t>1=Currently not suppressed; 2=Known or suspected resistance to cabotegravir or rilpivirine; 3=History of treatment failure; 4=Weighs &lt;35kg; 5=Younger than 12 year; 6=History of visit non-adherence; 7=History of oral ART non-adherence; 8=Buttocks implant; 9=Pregnancy/Family planning; 10 =Not covered by insurance/payor; 20=Other; UNK=Unknown</t>
-  </si>
-  <si>
-    <t>1=Currently not suppressed; 2=Known or suspected resistance to cabotegravir or rilpivirine; 3=History of treatment failure; 4=Weighs &lt;35kg; 5=Younger than 12 year; 6=History of visit non-adherence; 7=History of oral ART non-adherence; 8=Buttocks implant; 9=Pregnancy/Family planning; 10=Not covered by insurance/payor; 20=Other; UNK=Unknown</t>
+    <t>1=Currently not suppressed; 2=Known or suspected resistance to cabotegravir or rilpivirine; 3=History of treatment failure; 4=Weighs &lt;35kg; 5=Younger than 12 year; 6=History of visit non-adherence; 7=History of oral ART non-adherence; 8=Buttocks implant; 9=Pregnancy/Family planning; 20=Other; UNK=Unknown</t>
   </si>
 </sst>
 </file>
@@ -2115,24 +2112,6 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2142,13 +2121,13 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2158,6 +2137,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2178,7 +2166,16 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2741,7 +2738,7 @@
       <c r="K2" s="4"/>
     </row>
     <row r="3" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="134" t="s">
+      <c r="B3" s="128" t="s">
         <v>31</v>
       </c>
       <c r="C3" s="109" t="s">
@@ -2763,7 +2760,7 @@
       <c r="I3" s="8"/>
     </row>
     <row r="4" spans="1:11" ht="67.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="135"/>
+      <c r="B4" s="129"/>
       <c r="C4" s="15" t="s">
         <v>33</v>
       </c>
@@ -2783,7 +2780,7 @@
       <c r="I4" s="8"/>
     </row>
     <row r="5" spans="1:11" ht="44.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="135"/>
+      <c r="B5" s="129"/>
       <c r="C5" s="15" t="s">
         <v>37</v>
       </c>
@@ -2803,7 +2800,7 @@
       <c r="I5" s="17"/>
     </row>
     <row r="6" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B6" s="135"/>
+      <c r="B6" s="129"/>
       <c r="C6" s="15" t="s">
         <v>350</v>
       </c>
@@ -2823,7 +2820,7 @@
     </row>
     <row r="7" spans="1:11" s="19" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A7"/>
-      <c r="B7" s="135"/>
+      <c r="B7" s="129"/>
       <c r="C7" s="15" t="s">
         <v>42</v>
       </c>
@@ -2845,7 +2842,7 @@
       <c r="K7" s="18"/>
     </row>
     <row r="8" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B8" s="135"/>
+      <c r="B8" s="129"/>
       <c r="C8" s="15" t="s">
         <v>46</v>
       </c>
@@ -2864,7 +2861,7 @@
       <c r="H8" s="12"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B9" s="135"/>
+      <c r="B9" s="129"/>
       <c r="C9" s="15" t="s">
         <v>50</v>
       </c>
@@ -2883,7 +2880,7 @@
       <c r="H9" s="12"/>
     </row>
     <row r="10" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B10" s="135"/>
+      <c r="B10" s="129"/>
       <c r="C10" s="15" t="s">
         <v>54</v>
       </c>
@@ -2901,8 +2898,8 @@
       </c>
       <c r="H10" s="12"/>
     </row>
-    <row r="11" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B11" s="135"/>
+    <row r="11" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B11" s="129"/>
       <c r="C11" s="15" t="s">
         <v>58</v>
       </c>
@@ -2921,7 +2918,7 @@
       <c r="H11" s="12"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B12" s="135"/>
+      <c r="B12" s="129"/>
       <c r="C12" s="15" t="s">
         <v>62</v>
       </c>
@@ -2940,7 +2937,7 @@
       <c r="H12" s="12"/>
     </row>
     <row r="13" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B13" s="135"/>
+      <c r="B13" s="129"/>
       <c r="C13" s="15" t="s">
         <v>66</v>
       </c>
@@ -2959,7 +2956,7 @@
       <c r="H13" s="12"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B14" s="135"/>
+      <c r="B14" s="129"/>
       <c r="C14" s="15" t="s">
         <v>70</v>
       </c>
@@ -2978,7 +2975,7 @@
       <c r="H14" s="12"/>
     </row>
     <row r="15" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B15" s="135"/>
+      <c r="B15" s="129"/>
       <c r="C15" s="15" t="s">
         <v>73</v>
       </c>
@@ -2997,7 +2994,7 @@
       <c r="H15" s="20"/>
     </row>
     <row r="16" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B16" s="136"/>
+      <c r="B16" s="130"/>
       <c r="C16" s="15" t="s">
         <v>77</v>
       </c>
@@ -3016,10 +3013,10 @@
       <c r="H16" s="12"/>
     </row>
     <row r="17" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="143" t="s">
+      <c r="A17" s="125" t="s">
         <v>310</v>
       </c>
-      <c r="B17" s="122" t="s">
+      <c r="B17" s="131" t="s">
         <v>81</v>
       </c>
       <c r="C17" s="111" t="s">
@@ -3028,7 +3025,7 @@
       <c r="D17" s="112" t="s">
         <v>83</v>
       </c>
-      <c r="E17" s="122" t="s">
+      <c r="E17" s="131" t="s">
         <v>358</v>
       </c>
       <c r="F17" s="112" t="s">
@@ -3040,15 +3037,15 @@
       <c r="H17" s="12"/>
     </row>
     <row r="18" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="143"/>
-      <c r="B18" s="123"/>
+      <c r="A18" s="125"/>
+      <c r="B18" s="132"/>
       <c r="C18" s="111" t="s">
         <v>85</v>
       </c>
       <c r="D18" s="112" t="s">
         <v>86</v>
       </c>
-      <c r="E18" s="123"/>
+      <c r="E18" s="132"/>
       <c r="F18" s="112" t="s">
         <v>84</v>
       </c>
@@ -3058,15 +3055,15 @@
       <c r="H18" s="12"/>
     </row>
     <row r="19" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="143"/>
-      <c r="B19" s="123"/>
+      <c r="A19" s="125"/>
+      <c r="B19" s="132"/>
       <c r="C19" s="111" t="s">
         <v>87</v>
       </c>
       <c r="D19" s="112" t="s">
         <v>88</v>
       </c>
-      <c r="E19" s="123"/>
+      <c r="E19" s="132"/>
       <c r="F19" s="112" t="s">
         <v>84</v>
       </c>
@@ -3076,15 +3073,15 @@
       <c r="H19" s="12"/>
     </row>
     <row r="20" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A20" s="143"/>
-      <c r="B20" s="123"/>
+      <c r="A20" s="125"/>
+      <c r="B20" s="132"/>
       <c r="C20" s="111" t="s">
         <v>89</v>
       </c>
       <c r="D20" s="112" t="s">
         <v>90</v>
       </c>
-      <c r="E20" s="123"/>
+      <c r="E20" s="132"/>
       <c r="F20" s="112" t="s">
         <v>84</v>
       </c>
@@ -3094,15 +3091,15 @@
       <c r="H20" s="12"/>
     </row>
     <row r="21" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A21" s="143"/>
-      <c r="B21" s="123"/>
+      <c r="A21" s="125"/>
+      <c r="B21" s="132"/>
       <c r="C21" s="111" t="s">
         <v>91</v>
       </c>
       <c r="D21" s="112" t="s">
         <v>92</v>
       </c>
-      <c r="E21" s="123"/>
+      <c r="E21" s="132"/>
       <c r="F21" s="112" t="s">
         <v>84</v>
       </c>
@@ -3112,15 +3109,15 @@
       <c r="H21" s="12"/>
     </row>
     <row r="22" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A22" s="143"/>
-      <c r="B22" s="123"/>
+      <c r="A22" s="125"/>
+      <c r="B22" s="132"/>
       <c r="C22" s="111" t="s">
         <v>277</v>
       </c>
       <c r="D22" s="112" t="s">
         <v>282</v>
       </c>
-      <c r="E22" s="123"/>
+      <c r="E22" s="132"/>
       <c r="F22" s="112" t="s">
         <v>84</v>
       </c>
@@ -3130,15 +3127,15 @@
       <c r="H22" s="12"/>
     </row>
     <row r="23" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A23" s="143"/>
-      <c r="B23" s="123"/>
+      <c r="A23" s="125"/>
+      <c r="B23" s="132"/>
       <c r="C23" s="111" t="s">
         <v>278</v>
       </c>
       <c r="D23" s="112" t="s">
         <v>283</v>
       </c>
-      <c r="E23" s="123"/>
+      <c r="E23" s="132"/>
       <c r="F23" s="112" t="s">
         <v>84</v>
       </c>
@@ -3148,15 +3145,15 @@
       <c r="H23" s="12"/>
     </row>
     <row r="24" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A24" s="143"/>
-      <c r="B24" s="123"/>
+      <c r="A24" s="125"/>
+      <c r="B24" s="132"/>
       <c r="C24" s="111" t="s">
         <v>279</v>
       </c>
       <c r="D24" s="112" t="s">
         <v>284</v>
       </c>
-      <c r="E24" s="123"/>
+      <c r="E24" s="132"/>
       <c r="F24" s="112" t="s">
         <v>84</v>
       </c>
@@ -3166,15 +3163,15 @@
       <c r="H24" s="12"/>
     </row>
     <row r="25" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A25" s="143"/>
-      <c r="B25" s="123"/>
+      <c r="A25" s="125"/>
+      <c r="B25" s="132"/>
       <c r="C25" s="111" t="s">
         <v>280</v>
       </c>
       <c r="D25" s="112" t="s">
         <v>285</v>
       </c>
-      <c r="E25" s="123"/>
+      <c r="E25" s="132"/>
       <c r="F25" s="112" t="s">
         <v>84</v>
       </c>
@@ -3184,15 +3181,15 @@
       <c r="H25" s="12"/>
     </row>
     <row r="26" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A26" s="143"/>
-      <c r="B26" s="124"/>
+      <c r="A26" s="125"/>
+      <c r="B26" s="133"/>
       <c r="C26" s="111" t="s">
         <v>281</v>
       </c>
       <c r="D26" s="112" t="s">
         <v>286</v>
       </c>
-      <c r="E26" s="124"/>
+      <c r="E26" s="133"/>
       <c r="F26" s="112" t="s">
         <v>84</v>
       </c>
@@ -3202,7 +3199,7 @@
       <c r="H26" s="12"/>
     </row>
     <row r="27" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="137" t="s">
+      <c r="B27" s="134" t="s">
         <v>93</v>
       </c>
       <c r="C27" s="113" t="s">
@@ -3223,7 +3220,7 @@
       <c r="H27" s="12"/>
     </row>
     <row r="28" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="138"/>
+      <c r="B28" s="135"/>
       <c r="C28" s="113" t="s">
         <v>98</v>
       </c>
@@ -3242,7 +3239,7 @@
       <c r="H28" s="12"/>
     </row>
     <row r="29" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B29" s="139"/>
+      <c r="B29" s="136"/>
       <c r="C29" s="113" t="s">
         <v>102</v>
       </c>
@@ -3261,7 +3258,7 @@
       <c r="H29" s="12"/>
     </row>
     <row r="30" spans="1:8" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="B30" s="140" t="s">
+      <c r="B30" s="137" t="s">
         <v>106</v>
       </c>
       <c r="C30" s="114" t="s">
@@ -3282,7 +3279,7 @@
       <c r="H30" s="24"/>
     </row>
     <row r="31" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="141"/>
+      <c r="B31" s="138"/>
       <c r="C31" s="114" t="s">
         <v>111</v>
       </c>
@@ -3301,7 +3298,7 @@
       <c r="H31" s="24"/>
     </row>
     <row r="32" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="141"/>
+      <c r="B32" s="138"/>
       <c r="C32" s="114" t="s">
         <v>114</v>
       </c>
@@ -3320,7 +3317,7 @@
       <c r="H32" s="12"/>
     </row>
     <row r="33" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B33" s="141"/>
+      <c r="B33" s="138"/>
       <c r="C33" s="114" t="s">
         <v>118</v>
       </c>
@@ -3339,7 +3336,7 @@
       <c r="H33" s="10"/>
     </row>
     <row r="34" spans="1:11" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="141"/>
+      <c r="B34" s="138"/>
       <c r="C34" s="114" t="s">
         <v>122</v>
       </c>
@@ -3358,7 +3355,7 @@
       <c r="H34" s="12"/>
     </row>
     <row r="35" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B35" s="141"/>
+      <c r="B35" s="138"/>
       <c r="C35" s="114" t="s">
         <v>126</v>
       </c>
@@ -3377,7 +3374,7 @@
       <c r="H35" s="24"/>
     </row>
     <row r="36" spans="1:11" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="141"/>
+      <c r="B36" s="138"/>
       <c r="C36" s="114" t="s">
         <v>129</v>
       </c>
@@ -3396,7 +3393,7 @@
       <c r="H36" s="12"/>
     </row>
     <row r="37" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="B37" s="141"/>
+      <c r="B37" s="138"/>
       <c r="C37" s="114" t="s">
         <v>132</v>
       </c>
@@ -3416,14 +3413,14 @@
     </row>
     <row r="38" spans="1:11" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="95"/>
-      <c r="B38" s="141"/>
+      <c r="B38" s="138"/>
       <c r="C38" s="114" t="s">
         <v>273</v>
       </c>
       <c r="D38" s="115" t="s">
         <v>274</v>
       </c>
-      <c r="E38" s="125" t="s">
+      <c r="E38" s="140" t="s">
         <v>359</v>
       </c>
       <c r="F38" s="115"/>
@@ -3434,14 +3431,14 @@
     </row>
     <row r="39" spans="1:11" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="95"/>
-      <c r="B39" s="141"/>
+      <c r="B39" s="138"/>
       <c r="C39" s="116" t="s">
         <v>275</v>
       </c>
       <c r="D39" s="115" t="s">
         <v>274</v>
       </c>
-      <c r="E39" s="126"/>
+      <c r="E39" s="141"/>
       <c r="F39" s="115"/>
       <c r="G39" s="115" t="s">
         <v>296</v>
@@ -3450,22 +3447,22 @@
     </row>
     <row r="40" spans="1:11" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="95"/>
-      <c r="B40" s="142"/>
+      <c r="B40" s="139"/>
       <c r="C40" s="114" t="s">
         <v>276</v>
       </c>
       <c r="D40" s="115" t="s">
         <v>274</v>
       </c>
-      <c r="E40" s="127"/>
+      <c r="E40" s="142"/>
       <c r="F40" s="115"/>
       <c r="G40" s="115" t="s">
         <v>296</v>
       </c>
       <c r="H40" s="12"/>
     </row>
-    <row r="41" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B41" s="131" t="s">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B41" s="126" t="s">
         <v>305</v>
       </c>
       <c r="C41" s="26" t="s">
@@ -3486,7 +3483,7 @@
       <c r="H41" s="24"/>
     </row>
     <row r="42" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B42" s="132"/>
+      <c r="B42" s="127"/>
       <c r="C42" s="26" t="s">
         <v>266</v>
       </c>
@@ -3505,7 +3502,7 @@
       <c r="H42" s="24"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B43" s="133"/>
+      <c r="B43" s="143"/>
       <c r="C43" s="26" t="s">
         <v>287</v>
       </c>
@@ -3524,10 +3521,10 @@
       <c r="H43" s="24"/>
     </row>
     <row r="44" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A44" s="143" t="s">
+      <c r="A44" s="125" t="s">
         <v>317</v>
       </c>
-      <c r="B44" s="131" t="s">
+      <c r="B44" s="126" t="s">
         <v>311</v>
       </c>
       <c r="C44" s="117" t="s">
@@ -3551,8 +3548,8 @@
       <c r="K44" s="28"/>
     </row>
     <row r="45" spans="1:11" s="29" customFormat="1" ht="224.4" x14ac:dyDescent="0.3">
-      <c r="A45" s="143"/>
-      <c r="B45" s="132"/>
+      <c r="A45" s="125"/>
+      <c r="B45" s="127"/>
       <c r="C45" s="117" t="s">
         <v>143</v>
       </c>
@@ -3574,8 +3571,8 @@
       <c r="K45" s="28"/>
     </row>
     <row r="46" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A46" s="143"/>
-      <c r="B46" s="131" t="s">
+      <c r="A46" s="125"/>
+      <c r="B46" s="126" t="s">
         <v>312</v>
       </c>
       <c r="C46" s="117" t="s">
@@ -3599,8 +3596,8 @@
       <c r="K46" s="28"/>
     </row>
     <row r="47" spans="1:11" s="29" customFormat="1" ht="224.4" x14ac:dyDescent="0.3">
-      <c r="A47" s="143"/>
-      <c r="B47" s="132"/>
+      <c r="A47" s="125"/>
+      <c r="B47" s="127"/>
       <c r="C47" s="117" t="s">
         <v>147</v>
       </c>
@@ -3623,7 +3620,7 @@
     </row>
     <row r="48" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A48"/>
-      <c r="B48" s="128" t="s">
+      <c r="B48" s="122" t="s">
         <v>165</v>
       </c>
       <c r="C48" s="36" t="s">
@@ -3648,7 +3645,7 @@
     </row>
     <row r="49" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A49"/>
-      <c r="B49" s="130"/>
+      <c r="B49" s="124"/>
       <c r="C49" s="36" t="s">
         <v>169</v>
       </c>
@@ -3670,10 +3667,10 @@
       <c r="K49" s="32"/>
     </row>
     <row r="50" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A50" s="143" t="s">
+      <c r="A50" s="125" t="s">
         <v>318</v>
       </c>
-      <c r="B50" s="128" t="s">
+      <c r="B50" s="122" t="s">
         <v>313</v>
       </c>
       <c r="C50" s="36" t="s">
@@ -3697,8 +3694,8 @@
       <c r="K50" s="32"/>
     </row>
     <row r="51" spans="1:11" s="33" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="143"/>
-      <c r="B51" s="129"/>
+      <c r="A51" s="125"/>
+      <c r="B51" s="123"/>
       <c r="C51" s="36" t="s">
         <v>176</v>
       </c>
@@ -3719,9 +3716,9 @@
       <c r="J51" s="32"/>
       <c r="K51" s="32"/>
     </row>
-    <row r="52" spans="1:11" s="33" customFormat="1" ht="316.8" x14ac:dyDescent="0.3">
-      <c r="A52" s="143"/>
-      <c r="B52" s="129"/>
+    <row r="52" spans="1:11" s="33" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.3">
+      <c r="A52" s="125"/>
+      <c r="B52" s="123"/>
       <c r="C52" s="36" t="s">
         <v>180</v>
       </c>
@@ -3743,8 +3740,8 @@
       <c r="K52" s="32"/>
     </row>
     <row r="53" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A53" s="143"/>
-      <c r="B53" s="130"/>
+      <c r="A53" s="125"/>
+      <c r="B53" s="124"/>
       <c r="C53" s="36" t="s">
         <v>182</v>
       </c>
@@ -3766,10 +3763,10 @@
       <c r="K53" s="32"/>
     </row>
     <row r="54" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A54" s="143" t="s">
+      <c r="A54" s="125" t="s">
         <v>319</v>
       </c>
-      <c r="B54" s="128" t="s">
+      <c r="B54" s="122" t="s">
         <v>316</v>
       </c>
       <c r="C54" s="36" t="s">
@@ -3793,8 +3790,8 @@
       <c r="K54" s="32"/>
     </row>
     <row r="55" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A55" s="143"/>
-      <c r="B55" s="129"/>
+      <c r="A55" s="125"/>
+      <c r="B55" s="123"/>
       <c r="C55" s="36" t="s">
         <v>188</v>
       </c>
@@ -3816,8 +3813,8 @@
       <c r="K55" s="32"/>
     </row>
     <row r="56" spans="1:11" s="33" customFormat="1" ht="356.4" x14ac:dyDescent="0.3">
-      <c r="A56" s="143"/>
-      <c r="B56" s="129"/>
+      <c r="A56" s="125"/>
+      <c r="B56" s="123"/>
       <c r="C56" s="36" t="s">
         <v>192</v>
       </c>
@@ -3828,7 +3825,7 @@
         <v>381</v>
       </c>
       <c r="F56" s="37" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="G56" s="36" t="s">
         <v>291</v>
@@ -3839,8 +3836,8 @@
       <c r="K56" s="32"/>
     </row>
     <row r="57" spans="1:11" s="33" customFormat="1" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A57" s="143"/>
-      <c r="B57" s="130"/>
+      <c r="A57" s="125"/>
+      <c r="B57" s="124"/>
       <c r="C57" s="36" t="s">
         <v>354</v>
       </c>
@@ -3862,10 +3859,10 @@
       <c r="K57" s="32"/>
     </row>
     <row r="58" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A58" s="143" t="s">
+      <c r="A58" s="125" t="s">
         <v>318</v>
       </c>
-      <c r="B58" s="128" t="s">
+      <c r="B58" s="122" t="s">
         <v>315</v>
       </c>
       <c r="C58" s="36" t="s">
@@ -3889,8 +3886,8 @@
       <c r="K58" s="32"/>
     </row>
     <row r="59" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A59" s="143"/>
-      <c r="B59" s="129"/>
+      <c r="A59" s="125"/>
+      <c r="B59" s="123"/>
       <c r="C59" s="36" t="s">
         <v>198</v>
       </c>
@@ -3911,9 +3908,9 @@
       <c r="J59" s="32"/>
       <c r="K59" s="32"/>
     </row>
-    <row r="60" spans="1:11" s="33" customFormat="1" ht="316.8" x14ac:dyDescent="0.3">
-      <c r="A60" s="143"/>
-      <c r="B60" s="129"/>
+    <row r="60" spans="1:11" s="33" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.3">
+      <c r="A60" s="125"/>
+      <c r="B60" s="123"/>
       <c r="C60" s="36" t="s">
         <v>200</v>
       </c>
@@ -3935,8 +3932,8 @@
       <c r="K60" s="32"/>
     </row>
     <row r="61" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A61" s="143"/>
-      <c r="B61" s="130"/>
+      <c r="A61" s="125"/>
+      <c r="B61" s="124"/>
       <c r="C61" s="36" t="s">
         <v>202</v>
       </c>
@@ -3958,10 +3955,10 @@
       <c r="K61" s="32"/>
     </row>
     <row r="62" spans="1:11" s="33" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="143" t="s">
+      <c r="A62" s="125" t="s">
         <v>319</v>
       </c>
-      <c r="B62" s="128" t="s">
+      <c r="B62" s="122" t="s">
         <v>314</v>
       </c>
       <c r="C62" s="36" t="s">
@@ -3985,8 +3982,8 @@
       <c r="K62" s="32"/>
     </row>
     <row r="63" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A63" s="143"/>
-      <c r="B63" s="129"/>
+      <c r="A63" s="125"/>
+      <c r="B63" s="123"/>
       <c r="C63" s="36" t="s">
         <v>207</v>
       </c>
@@ -4008,8 +4005,8 @@
       <c r="K63" s="32"/>
     </row>
     <row r="64" spans="1:11" ht="356.4" x14ac:dyDescent="0.3">
-      <c r="A64" s="143"/>
-      <c r="B64" s="129"/>
+      <c r="A64" s="125"/>
+      <c r="B64" s="123"/>
       <c r="C64" s="36" t="s">
         <v>210</v>
       </c>
@@ -4028,8 +4025,8 @@
       <c r="H64" s="12"/>
     </row>
     <row r="65" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A65" s="143"/>
-      <c r="B65" s="130"/>
+      <c r="A65" s="125"/>
+      <c r="B65" s="124"/>
       <c r="C65" s="36" t="s">
         <v>355</v>
       </c>
@@ -4048,7 +4045,7 @@
       <c r="H65" s="12"/>
     </row>
     <row r="66" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B66" s="128" t="s">
+      <c r="B66" s="122" t="s">
         <v>306</v>
       </c>
       <c r="C66" s="36" t="s">
@@ -4069,7 +4066,7 @@
       <c r="H66" s="10"/>
     </row>
     <row r="67" spans="1:11" ht="93" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B67" s="129"/>
+      <c r="B67" s="123"/>
       <c r="C67" s="36" t="s">
         <v>216</v>
       </c>
@@ -4088,7 +4085,7 @@
       <c r="H67" s="12"/>
     </row>
     <row r="68" spans="1:11" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B68" s="129"/>
+      <c r="B68" s="123"/>
       <c r="C68" s="36" t="s">
         <v>370</v>
       </c>
@@ -4107,7 +4104,7 @@
       <c r="H68" s="12"/>
     </row>
     <row r="69" spans="1:11" ht="158.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B69" s="129"/>
+      <c r="B69" s="123"/>
       <c r="C69" s="36" t="s">
         <v>371</v>
       </c>
@@ -4126,7 +4123,7 @@
       <c r="H69" s="12"/>
     </row>
     <row r="70" spans="1:11" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B70" s="130"/>
+      <c r="B70" s="124"/>
       <c r="C70" s="36" t="s">
         <v>373</v>
       </c>
@@ -4145,10 +4142,10 @@
       <c r="H70" s="12"/>
     </row>
     <row r="71" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A71" s="143" t="s">
+      <c r="A71" s="125" t="s">
         <v>320</v>
       </c>
-      <c r="B71" s="128" t="s">
+      <c r="B71" s="122" t="s">
         <v>307</v>
       </c>
       <c r="C71" s="36" t="s">
@@ -4172,8 +4169,8 @@
       <c r="K71" s="28"/>
     </row>
     <row r="72" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A72" s="143"/>
-      <c r="B72" s="129"/>
+      <c r="A72" s="125"/>
+      <c r="B72" s="123"/>
       <c r="C72" s="36" t="s">
         <v>222</v>
       </c>
@@ -4194,9 +4191,9 @@
       <c r="J72" s="28"/>
       <c r="K72" s="28"/>
     </row>
-    <row r="73" spans="1:11" s="29" customFormat="1" ht="198" x14ac:dyDescent="0.3">
-      <c r="A73" s="143"/>
-      <c r="B73" s="130"/>
+    <row r="73" spans="1:11" s="29" customFormat="1" ht="184.8" x14ac:dyDescent="0.3">
+      <c r="A73" s="125"/>
+      <c r="B73" s="124"/>
       <c r="C73" s="36" t="s">
         <v>225</v>
       </c>
@@ -4218,8 +4215,8 @@
       <c r="K73" s="28"/>
     </row>
     <row r="74" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A74" s="143"/>
-      <c r="B74" s="128" t="s">
+      <c r="A74" s="125"/>
+      <c r="B74" s="122" t="s">
         <v>307</v>
       </c>
       <c r="C74" s="36" t="s">
@@ -4243,8 +4240,8 @@
       <c r="K74" s="28"/>
     </row>
     <row r="75" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A75" s="143"/>
-      <c r="B75" s="129"/>
+      <c r="A75" s="125"/>
+      <c r="B75" s="123"/>
       <c r="C75" s="36" t="s">
         <v>230</v>
       </c>
@@ -4265,9 +4262,9 @@
       <c r="J75" s="28"/>
       <c r="K75" s="28"/>
     </row>
-    <row r="76" spans="1:11" s="29" customFormat="1" ht="198" x14ac:dyDescent="0.3">
-      <c r="A76" s="143"/>
-      <c r="B76" s="130"/>
+    <row r="76" spans="1:11" s="29" customFormat="1" ht="184.8" x14ac:dyDescent="0.3">
+      <c r="A76" s="125"/>
+      <c r="B76" s="124"/>
       <c r="C76" s="36" t="s">
         <v>233</v>
       </c>
@@ -4290,7 +4287,7 @@
     </row>
     <row r="77" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A77"/>
-      <c r="B77" s="128" t="s">
+      <c r="B77" s="122" t="s">
         <v>308</v>
       </c>
       <c r="C77" s="118" t="s">
@@ -4315,7 +4312,7 @@
     </row>
     <row r="78" spans="1:11" s="33" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A78"/>
-      <c r="B78" s="130"/>
+      <c r="B78" s="124"/>
       <c r="C78" s="118" t="s">
         <v>238</v>
       </c>
@@ -4337,10 +4334,10 @@
       <c r="K78" s="32"/>
     </row>
     <row r="79" spans="1:11" s="33" customFormat="1" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="143" t="s">
+      <c r="A79" s="125" t="s">
         <v>321</v>
       </c>
-      <c r="B79" s="128" t="s">
+      <c r="B79" s="122" t="s">
         <v>322</v>
       </c>
       <c r="C79" s="36" t="s">
@@ -4364,8 +4361,8 @@
       <c r="K79" s="32"/>
     </row>
     <row r="80" spans="1:11" s="33" customFormat="1" ht="78" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="143"/>
-      <c r="B80" s="129"/>
+      <c r="A80" s="125"/>
+      <c r="B80" s="123"/>
       <c r="C80" s="36" t="s">
         <v>325</v>
       </c>
@@ -4387,8 +4384,8 @@
       <c r="K80" s="32"/>
     </row>
     <row r="81" spans="1:11" s="33" customFormat="1" ht="212.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="143"/>
-      <c r="B81" s="130"/>
+      <c r="A81" s="125"/>
+      <c r="B81" s="124"/>
       <c r="C81" s="36" t="s">
         <v>327</v>
       </c>
@@ -4408,10 +4405,10 @@
       <c r="K81" s="32"/>
     </row>
     <row r="82" spans="1:11" s="33" customFormat="1" ht="117" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="143" t="s">
+      <c r="A82" s="125" t="s">
         <v>321</v>
       </c>
-      <c r="B82" s="128" t="s">
+      <c r="B82" s="122" t="s">
         <v>323</v>
       </c>
       <c r="C82" s="36" t="s">
@@ -4435,8 +4432,8 @@
       <c r="K82" s="32"/>
     </row>
     <row r="83" spans="1:11" s="33" customFormat="1" ht="83.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="143"/>
-      <c r="B83" s="129"/>
+      <c r="A83" s="125"/>
+      <c r="B83" s="123"/>
       <c r="C83" s="36" t="s">
         <v>330</v>
       </c>
@@ -4458,8 +4455,8 @@
       <c r="K83" s="32"/>
     </row>
     <row r="84" spans="1:11" s="33" customFormat="1" ht="199.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="143"/>
-      <c r="B84" s="130"/>
+      <c r="A84" s="125"/>
+      <c r="B84" s="124"/>
       <c r="C84" s="36" t="s">
         <v>331</v>
       </c>
@@ -4479,7 +4476,7 @@
       <c r="K84" s="32"/>
     </row>
     <row r="85" spans="1:11" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="B85" s="128" t="s">
+      <c r="B85" s="122" t="s">
         <v>309</v>
       </c>
       <c r="C85" s="36" t="s">
@@ -4499,7 +4496,7 @@
       </c>
     </row>
     <row r="86" spans="1:11" ht="118.8" x14ac:dyDescent="0.3">
-      <c r="B86" s="129"/>
+      <c r="B86" s="123"/>
       <c r="C86" s="36" t="s">
         <v>254</v>
       </c>
@@ -4516,8 +4513,8 @@
         <v>297</v>
       </c>
     </row>
-    <row r="87" spans="1:11" ht="211.2" x14ac:dyDescent="0.3">
-      <c r="B87" s="129"/>
+    <row r="87" spans="1:11" ht="198" x14ac:dyDescent="0.3">
+      <c r="B87" s="123"/>
       <c r="C87" s="36" t="s">
         <v>256</v>
       </c>
@@ -4535,7 +4532,7 @@
       </c>
     </row>
     <row r="88" spans="1:11" ht="66" x14ac:dyDescent="0.3">
-      <c r="B88" s="130"/>
+      <c r="B88" s="124"/>
       <c r="C88" s="36" t="s">
         <v>258</v>
       </c>
@@ -4586,6 +4583,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="E17:E26"/>
+    <mergeCell ref="E38:E40"/>
+    <mergeCell ref="B82:B84"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="B54:B57"/>
+    <mergeCell ref="B58:B61"/>
+    <mergeCell ref="B62:B65"/>
+    <mergeCell ref="B66:B70"/>
+    <mergeCell ref="B3:B16"/>
+    <mergeCell ref="B17:B26"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="B30:B40"/>
+    <mergeCell ref="B50:B53"/>
     <mergeCell ref="B85:B88"/>
     <mergeCell ref="A17:A26"/>
     <mergeCell ref="B44:B45"/>
@@ -4602,20 +4613,6 @@
     <mergeCell ref="A79:A81"/>
     <mergeCell ref="B79:B81"/>
     <mergeCell ref="A82:A84"/>
-    <mergeCell ref="B3:B16"/>
-    <mergeCell ref="B17:B26"/>
-    <mergeCell ref="B27:B29"/>
-    <mergeCell ref="B30:B40"/>
-    <mergeCell ref="B50:B53"/>
-    <mergeCell ref="E17:E26"/>
-    <mergeCell ref="E38:E40"/>
-    <mergeCell ref="B82:B84"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="B48:B49"/>
-    <mergeCell ref="B54:B57"/>
-    <mergeCell ref="B58:B61"/>
-    <mergeCell ref="B62:B65"/>
-    <mergeCell ref="B66:B70"/>
   </mergeCells>
   <phoneticPr fontId="29" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -20334,6 +20331,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="42fbd5e6-b175-407a-a25c-5fc6410bf24f" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EE7777BCFCD3E741B5CCCE9A87E98C2C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f7fc7590daec4eb8e38e018938a160ca">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e" xmlns:ns3="42fbd5e6-b175-407a-a25c-5fc6410bf24f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c5ca1b94d4b54616210e83d04e6b3cac" ns2:_="" ns3:_="">
     <xsd:import namespace="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
@@ -20588,27 +20605,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E9485EC-5D88-4A1C-961D-0F4FE84359B8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="42fbd5e6-b175-407a-a25c-5fc6410bf24f"/>
+    <ds:schemaRef ds:uri="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="42fbd5e6-b175-407a-a25c-5fc6410bf24f" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{286F673D-E70D-4002-B8F5-CAC95B029A7E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C9C537E-DFD2-4C38-AC8C-930F122DEFFC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -20625,23 +20641,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{286F673D-E70D-4002-B8F5-CAC95B029A7E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E9485EC-5D88-4A1C-961D-0F4FE84359B8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="42fbd5e6-b175-407a-a25c-5fc6410bf24f"/>
-    <ds:schemaRef ds:uri="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
change private insurance option
</commit_message>
<xml_diff>
--- a/data/ALAI UP Client-level Reporting Tool Template_4.7.26.xlsx
+++ b/data/ALAI UP Client-level Reporting Tool Template_4.7.26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kmlab\Desktop\Dashboard\alai_up_local_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1BBBB68-8911-4AF2-9375-25796358C44C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ED1B0B8-1C81-47D7-A585-DB2D553F3B2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{500E2EE0-B1C5-4ACF-BC67-EDC8BDABD2D7}"/>
   </bookViews>
@@ -422,9 +422,6 @@
     <t xml:space="preserve">Report primary source of health care coverage the client had for any part of the reporting period. </t>
   </si>
   <si>
-    <t>1=Private - Employer; 2=Private - Individual; 3=Medicare; 4=Medicaid; 5=Veterans Health Administration; 6=Indian Health Service; 7=Other plan; 8=No insurance/uninsured; UNK=Unknown</t>
-  </si>
-  <si>
     <t>housing_status</t>
   </si>
   <si>
@@ -1397,6 +1394,9 @@
   </si>
   <si>
     <t>1=Currently not suppressed; 2=Known or suspected resistance to cabotegravir or rilpivirine; 3=History of treatment failure; 4=Weighs &lt;35kg; 5=Younger than 12 year; 6=History of visit non-adherence; 7=History of oral ART non-adherence; 8=Buttocks implant; 9=Pregnancy/Family planning; 20=Other; UNK=Unknown</t>
+  </si>
+  <si>
+    <t>1=Private insurance; 2=Medicare; 3=Medicaid; 4=Veterans Health Administration; 5=Indian Health Service; 6=Other plan; 7=No insurance/uninsured; UNK=Unknown</t>
   </si>
 </sst>
 </file>
@@ -2112,6 +2112,24 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2121,13 +2139,13 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2137,15 +2155,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2166,16 +2175,7 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2557,7 +2557,7 @@
     </row>
     <row r="7" spans="2:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="B7" s="87" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.25">
@@ -2567,7 +2567,7 @@
     </row>
     <row r="9" spans="2:2" ht="41.4" x14ac:dyDescent="0.25">
       <c r="B9" s="87" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.25">
@@ -2705,7 +2705,7 @@
         <v>26</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="H1" s="3"/>
       <c r="I1" s="4"/>
@@ -2724,13 +2724,13 @@
         <v>29</v>
       </c>
       <c r="E2" s="108" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F2" s="108" t="s">
         <v>30</v>
       </c>
       <c r="G2" s="108" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="8"/>
@@ -2738,14 +2738,14 @@
       <c r="K2" s="4"/>
     </row>
     <row r="3" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="128" t="s">
+      <c r="B3" s="134" t="s">
         <v>31</v>
       </c>
       <c r="C3" s="109" t="s">
+        <v>299</v>
+      </c>
+      <c r="D3" s="110" t="s">
         <v>300</v>
-      </c>
-      <c r="D3" s="110" t="s">
-        <v>301</v>
       </c>
       <c r="E3" s="110" t="s">
         <v>32</v>
@@ -2754,13 +2754,13 @@
         <v>30</v>
       </c>
       <c r="G3" s="110" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H3" s="12"/>
       <c r="I3" s="8"/>
     </row>
     <row r="4" spans="1:11" ht="67.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="129"/>
+      <c r="B4" s="135"/>
       <c r="C4" s="15" t="s">
         <v>33</v>
       </c>
@@ -2774,13 +2774,13 @@
         <v>36</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H4" s="12"/>
       <c r="I4" s="8"/>
     </row>
     <row r="5" spans="1:11" ht="44.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="129"/>
+      <c r="B5" s="135"/>
       <c r="C5" s="15" t="s">
         <v>37</v>
       </c>
@@ -2794,33 +2794,33 @@
         <v>40</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H5" s="10"/>
       <c r="I5" s="17"/>
     </row>
     <row r="6" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B6" s="129"/>
+      <c r="B6" s="135"/>
       <c r="C6" s="15" t="s">
+        <v>349</v>
+      </c>
+      <c r="D6" s="16" t="s">
         <v>350</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="E6" s="16" t="s">
         <v>351</v>
       </c>
-      <c r="E6" s="16" t="s">
+      <c r="F6" s="16" t="s">
         <v>352</v>
       </c>
-      <c r="F6" s="16" t="s">
-        <v>353</v>
-      </c>
       <c r="G6" s="16" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H6" s="12"/>
     </row>
     <row r="7" spans="1:11" s="19" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A7"/>
-      <c r="B7" s="129"/>
+      <c r="B7" s="135"/>
       <c r="C7" s="15" t="s">
         <v>42</v>
       </c>
@@ -2834,7 +2834,7 @@
         <v>45</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H7" s="10"/>
       <c r="I7" s="18"/>
@@ -2842,7 +2842,7 @@
       <c r="K7" s="18"/>
     </row>
     <row r="8" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B8" s="129"/>
+      <c r="B8" s="135"/>
       <c r="C8" s="15" t="s">
         <v>46</v>
       </c>
@@ -2856,12 +2856,12 @@
         <v>49</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H8" s="12"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B9" s="129"/>
+      <c r="B9" s="135"/>
       <c r="C9" s="15" t="s">
         <v>50</v>
       </c>
@@ -2875,12 +2875,12 @@
         <v>53</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H9" s="12"/>
     </row>
     <row r="10" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B10" s="129"/>
+      <c r="B10" s="135"/>
       <c r="C10" s="15" t="s">
         <v>54</v>
       </c>
@@ -2894,12 +2894,12 @@
         <v>57</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H10" s="12"/>
     </row>
     <row r="11" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B11" s="129"/>
+      <c r="B11" s="135"/>
       <c r="C11" s="15" t="s">
         <v>58</v>
       </c>
@@ -2913,12 +2913,12 @@
         <v>61</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H11" s="12"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B12" s="129"/>
+      <c r="B12" s="135"/>
       <c r="C12" s="15" t="s">
         <v>62</v>
       </c>
@@ -2932,12 +2932,12 @@
         <v>65</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H12" s="12"/>
     </row>
     <row r="13" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B13" s="129"/>
+      <c r="B13" s="135"/>
       <c r="C13" s="15" t="s">
         <v>66</v>
       </c>
@@ -2951,12 +2951,12 @@
         <v>69</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H13" s="12"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B14" s="129"/>
+      <c r="B14" s="135"/>
       <c r="C14" s="15" t="s">
         <v>70</v>
       </c>
@@ -2970,12 +2970,12 @@
         <v>30</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H14" s="12"/>
     </row>
     <row r="15" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B15" s="129"/>
+      <c r="B15" s="135"/>
       <c r="C15" s="15" t="s">
         <v>73</v>
       </c>
@@ -2989,12 +2989,12 @@
         <v>76</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H15" s="20"/>
     </row>
     <row r="16" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B16" s="130"/>
+      <c r="B16" s="136"/>
       <c r="C16" s="15" t="s">
         <v>77</v>
       </c>
@@ -3008,15 +3008,15 @@
         <v>80</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H16" s="12"/>
     </row>
     <row r="17" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="125" t="s">
-        <v>310</v>
-      </c>
-      <c r="B17" s="131" t="s">
+      <c r="A17" s="143" t="s">
+        <v>309</v>
+      </c>
+      <c r="B17" s="122" t="s">
         <v>81</v>
       </c>
       <c r="C17" s="111" t="s">
@@ -3025,181 +3025,181 @@
       <c r="D17" s="112" t="s">
         <v>83</v>
       </c>
-      <c r="E17" s="131" t="s">
-        <v>358</v>
+      <c r="E17" s="122" t="s">
+        <v>357</v>
       </c>
       <c r="F17" s="112" t="s">
         <v>84</v>
       </c>
       <c r="G17" s="112" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H17" s="12"/>
     </row>
     <row r="18" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="125"/>
-      <c r="B18" s="132"/>
+      <c r="A18" s="143"/>
+      <c r="B18" s="123"/>
       <c r="C18" s="111" t="s">
         <v>85</v>
       </c>
       <c r="D18" s="112" t="s">
         <v>86</v>
       </c>
-      <c r="E18" s="132"/>
+      <c r="E18" s="123"/>
       <c r="F18" s="112" t="s">
         <v>84</v>
       </c>
       <c r="G18" s="112" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H18" s="12"/>
     </row>
     <row r="19" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="125"/>
-      <c r="B19" s="132"/>
+      <c r="A19" s="143"/>
+      <c r="B19" s="123"/>
       <c r="C19" s="111" t="s">
         <v>87</v>
       </c>
       <c r="D19" s="112" t="s">
         <v>88</v>
       </c>
-      <c r="E19" s="132"/>
+      <c r="E19" s="123"/>
       <c r="F19" s="112" t="s">
         <v>84</v>
       </c>
       <c r="G19" s="112" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H19" s="12"/>
     </row>
     <row r="20" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A20" s="125"/>
-      <c r="B20" s="132"/>
+      <c r="A20" s="143"/>
+      <c r="B20" s="123"/>
       <c r="C20" s="111" t="s">
         <v>89</v>
       </c>
       <c r="D20" s="112" t="s">
         <v>90</v>
       </c>
-      <c r="E20" s="132"/>
+      <c r="E20" s="123"/>
       <c r="F20" s="112" t="s">
         <v>84</v>
       </c>
       <c r="G20" s="112" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H20" s="12"/>
     </row>
     <row r="21" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A21" s="125"/>
-      <c r="B21" s="132"/>
+      <c r="A21" s="143"/>
+      <c r="B21" s="123"/>
       <c r="C21" s="111" t="s">
         <v>91</v>
       </c>
       <c r="D21" s="112" t="s">
         <v>92</v>
       </c>
-      <c r="E21" s="132"/>
+      <c r="E21" s="123"/>
       <c r="F21" s="112" t="s">
         <v>84</v>
       </c>
       <c r="G21" s="112" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H21" s="12"/>
     </row>
     <row r="22" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A22" s="125"/>
-      <c r="B22" s="132"/>
+      <c r="A22" s="143"/>
+      <c r="B22" s="123"/>
       <c r="C22" s="111" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D22" s="112" t="s">
-        <v>282</v>
-      </c>
-      <c r="E22" s="132"/>
+        <v>281</v>
+      </c>
+      <c r="E22" s="123"/>
       <c r="F22" s="112" t="s">
         <v>84</v>
       </c>
       <c r="G22" s="112" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H22" s="12"/>
     </row>
     <row r="23" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A23" s="125"/>
-      <c r="B23" s="132"/>
+      <c r="A23" s="143"/>
+      <c r="B23" s="123"/>
       <c r="C23" s="111" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D23" s="112" t="s">
-        <v>283</v>
-      </c>
-      <c r="E23" s="132"/>
+        <v>282</v>
+      </c>
+      <c r="E23" s="123"/>
       <c r="F23" s="112" t="s">
         <v>84</v>
       </c>
       <c r="G23" s="112" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H23" s="12"/>
     </row>
     <row r="24" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A24" s="125"/>
-      <c r="B24" s="132"/>
+      <c r="A24" s="143"/>
+      <c r="B24" s="123"/>
       <c r="C24" s="111" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D24" s="112" t="s">
-        <v>284</v>
-      </c>
-      <c r="E24" s="132"/>
+        <v>283</v>
+      </c>
+      <c r="E24" s="123"/>
       <c r="F24" s="112" t="s">
         <v>84</v>
       </c>
       <c r="G24" s="112" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H24" s="12"/>
     </row>
     <row r="25" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A25" s="125"/>
-      <c r="B25" s="132"/>
+      <c r="A25" s="143"/>
+      <c r="B25" s="123"/>
       <c r="C25" s="111" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D25" s="112" t="s">
-        <v>285</v>
-      </c>
-      <c r="E25" s="132"/>
+        <v>284</v>
+      </c>
+      <c r="E25" s="123"/>
       <c r="F25" s="112" t="s">
         <v>84</v>
       </c>
       <c r="G25" s="112" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H25" s="12"/>
     </row>
     <row r="26" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A26" s="125"/>
-      <c r="B26" s="133"/>
+      <c r="A26" s="143"/>
+      <c r="B26" s="124"/>
       <c r="C26" s="111" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D26" s="112" t="s">
-        <v>286</v>
-      </c>
-      <c r="E26" s="133"/>
+        <v>285</v>
+      </c>
+      <c r="E26" s="124"/>
       <c r="F26" s="112" t="s">
         <v>84</v>
       </c>
       <c r="G26" s="112" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H26" s="12"/>
     </row>
     <row r="27" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="134" t="s">
+      <c r="B27" s="137" t="s">
         <v>93</v>
       </c>
       <c r="C27" s="113" t="s">
@@ -3215,12 +3215,12 @@
         <v>97</v>
       </c>
       <c r="G27" s="22" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H27" s="12"/>
     </row>
     <row r="28" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="135"/>
+      <c r="B28" s="138"/>
       <c r="C28" s="113" t="s">
         <v>98</v>
       </c>
@@ -3234,12 +3234,12 @@
         <v>101</v>
       </c>
       <c r="G28" s="22" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H28" s="12"/>
     </row>
     <row r="29" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B29" s="136"/>
+      <c r="B29" s="139"/>
       <c r="C29" s="113" t="s">
         <v>102</v>
       </c>
@@ -3253,12 +3253,12 @@
         <v>105</v>
       </c>
       <c r="G29" s="22" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H29" s="12"/>
     </row>
     <row r="30" spans="1:8" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="B30" s="137" t="s">
+      <c r="B30" s="140" t="s">
         <v>106</v>
       </c>
       <c r="C30" s="114" t="s">
@@ -3271,276 +3271,276 @@
         <v>109</v>
       </c>
       <c r="F30" s="23" t="s">
+        <v>387</v>
+      </c>
+      <c r="G30" s="23" t="s">
+        <v>296</v>
+      </c>
+      <c r="H30" s="24"/>
+    </row>
+    <row r="31" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="141"/>
+      <c r="C31" s="114" t="s">
         <v>110</v>
       </c>
-      <c r="G30" s="23" t="s">
-        <v>297</v>
-      </c>
-      <c r="H30" s="24"/>
-    </row>
-    <row r="31" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="138"/>
-      <c r="C31" s="114" t="s">
+      <c r="D31" s="23" t="s">
         <v>111</v>
       </c>
-      <c r="D31" s="23" t="s">
+      <c r="E31" s="23" t="s">
+        <v>291</v>
+      </c>
+      <c r="F31" s="23" t="s">
         <v>112</v>
       </c>
-      <c r="E31" s="23" t="s">
-        <v>292</v>
-      </c>
-      <c r="F31" s="23" t="s">
+      <c r="G31" s="23" t="s">
+        <v>295</v>
+      </c>
+      <c r="H31" s="24"/>
+    </row>
+    <row r="32" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="141"/>
+      <c r="C32" s="114" t="s">
         <v>113</v>
       </c>
-      <c r="G31" s="23" t="s">
-        <v>296</v>
-      </c>
-      <c r="H31" s="24"/>
-    </row>
-    <row r="32" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="138"/>
-      <c r="C32" s="114" t="s">
+      <c r="D32" s="23" t="s">
         <v>114</v>
       </c>
-      <c r="D32" s="23" t="s">
+      <c r="E32" s="23" t="s">
         <v>115</v>
       </c>
-      <c r="E32" s="23" t="s">
+      <c r="F32" s="23" t="s">
         <v>116</v>
       </c>
-      <c r="F32" s="23" t="s">
+      <c r="G32" s="23" t="s">
+        <v>295</v>
+      </c>
+      <c r="H32" s="12"/>
+    </row>
+    <row r="33" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="B33" s="141"/>
+      <c r="C33" s="114" t="s">
         <v>117</v>
       </c>
-      <c r="G32" s="23" t="s">
-        <v>296</v>
-      </c>
-      <c r="H32" s="12"/>
-    </row>
-    <row r="33" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B33" s="138"/>
-      <c r="C33" s="114" t="s">
+      <c r="D33" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="D33" s="23" t="s">
+      <c r="E33" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="E33" s="23" t="s">
+      <c r="F33" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="F33" s="23" t="s">
+      <c r="G33" s="23" t="s">
+        <v>295</v>
+      </c>
+      <c r="H33" s="10"/>
+    </row>
+    <row r="34" spans="1:11" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="141"/>
+      <c r="C34" s="114" t="s">
         <v>121</v>
       </c>
-      <c r="G33" s="23" t="s">
-        <v>296</v>
-      </c>
-      <c r="H33" s="10"/>
-    </row>
-    <row r="34" spans="1:11" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="138"/>
-      <c r="C34" s="114" t="s">
+      <c r="D34" s="23" t="s">
         <v>122</v>
       </c>
-      <c r="D34" s="23" t="s">
+      <c r="E34" s="23" t="s">
         <v>123</v>
       </c>
-      <c r="E34" s="23" t="s">
+      <c r="F34" s="23" t="s">
         <v>124</v>
       </c>
-      <c r="F34" s="23" t="s">
+      <c r="G34" s="23" t="s">
+        <v>295</v>
+      </c>
+      <c r="H34" s="12"/>
+    </row>
+    <row r="35" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="B35" s="141"/>
+      <c r="C35" s="114" t="s">
         <v>125</v>
       </c>
-      <c r="G34" s="23" t="s">
-        <v>296</v>
-      </c>
-      <c r="H34" s="12"/>
-    </row>
-    <row r="35" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B35" s="138"/>
-      <c r="C35" s="114" t="s">
+      <c r="D35" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="D35" s="23" t="s">
+      <c r="E35" s="23" t="s">
+        <v>383</v>
+      </c>
+      <c r="F35" s="23" t="s">
         <v>127</v>
       </c>
-      <c r="E35" s="23" t="s">
-        <v>384</v>
-      </c>
-      <c r="F35" s="23" t="s">
+      <c r="G35" s="23" t="s">
+        <v>295</v>
+      </c>
+      <c r="H35" s="24"/>
+    </row>
+    <row r="36" spans="1:11" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="141"/>
+      <c r="C36" s="114" t="s">
         <v>128</v>
       </c>
-      <c r="G35" s="23" t="s">
-        <v>296</v>
-      </c>
-      <c r="H35" s="24"/>
-    </row>
-    <row r="36" spans="1:11" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="138"/>
-      <c r="C36" s="114" t="s">
+      <c r="D36" s="23" t="s">
         <v>129</v>
       </c>
-      <c r="D36" s="23" t="s">
+      <c r="E36" s="23" t="s">
         <v>130</v>
-      </c>
-      <c r="E36" s="23" t="s">
-        <v>131</v>
       </c>
       <c r="F36" s="23" t="s">
         <v>30</v>
       </c>
       <c r="G36" s="23" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H36" s="12"/>
     </row>
     <row r="37" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="B37" s="138"/>
+      <c r="B37" s="141"/>
       <c r="C37" s="114" t="s">
+        <v>131</v>
+      </c>
+      <c r="D37" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="D37" s="23" t="s">
+      <c r="E37" s="23" t="s">
         <v>133</v>
       </c>
-      <c r="E37" s="23" t="s">
+      <c r="F37" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="F37" s="23" t="s">
-        <v>135</v>
-      </c>
       <c r="G37" s="23" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H37" s="12"/>
     </row>
     <row r="38" spans="1:11" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="95"/>
-      <c r="B38" s="138"/>
+      <c r="B38" s="141"/>
       <c r="C38" s="114" t="s">
+        <v>272</v>
+      </c>
+      <c r="D38" s="115" t="s">
         <v>273</v>
       </c>
-      <c r="D38" s="115" t="s">
-        <v>274</v>
-      </c>
-      <c r="E38" s="140" t="s">
-        <v>359</v>
+      <c r="E38" s="125" t="s">
+        <v>358</v>
       </c>
       <c r="F38" s="115"/>
       <c r="G38" s="115" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H38" s="12"/>
     </row>
     <row r="39" spans="1:11" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="95"/>
-      <c r="B39" s="138"/>
+      <c r="B39" s="141"/>
       <c r="C39" s="116" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D39" s="115" t="s">
-        <v>274</v>
-      </c>
-      <c r="E39" s="141"/>
+        <v>273</v>
+      </c>
+      <c r="E39" s="126"/>
       <c r="F39" s="115"/>
       <c r="G39" s="115" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H39" s="12"/>
     </row>
     <row r="40" spans="1:11" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="95"/>
-      <c r="B40" s="139"/>
+      <c r="B40" s="142"/>
       <c r="C40" s="114" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D40" s="115" t="s">
-        <v>274</v>
-      </c>
-      <c r="E40" s="142"/>
+        <v>273</v>
+      </c>
+      <c r="E40" s="127"/>
       <c r="F40" s="115"/>
       <c r="G40" s="115" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H40" s="12"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B41" s="126" t="s">
-        <v>305</v>
+      <c r="B41" s="131" t="s">
+        <v>304</v>
       </c>
       <c r="C41" s="26" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D41" s="117" t="s">
+        <v>267</v>
+      </c>
+      <c r="E41" s="117" t="s">
         <v>268</v>
-      </c>
-      <c r="E41" s="117" t="s">
-        <v>269</v>
       </c>
       <c r="F41" s="117" t="s">
         <v>41</v>
       </c>
       <c r="G41" s="117" t="s">
+        <v>295</v>
+      </c>
+      <c r="H41" s="24"/>
+    </row>
+    <row r="42" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B42" s="132"/>
+      <c r="C42" s="26" t="s">
+        <v>265</v>
+      </c>
+      <c r="D42" s="117" t="s">
+        <v>266</v>
+      </c>
+      <c r="E42" s="117" t="s">
+        <v>269</v>
+      </c>
+      <c r="F42" s="117" t="s">
+        <v>136</v>
+      </c>
+      <c r="G42" s="117" t="s">
+        <v>295</v>
+      </c>
+      <c r="H42" s="24"/>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B43" s="133"/>
+      <c r="C43" s="26" t="s">
+        <v>286</v>
+      </c>
+      <c r="D43" s="117" t="s">
+        <v>287</v>
+      </c>
+      <c r="E43" s="117" t="s">
+        <v>288</v>
+      </c>
+      <c r="F43" s="117" t="s">
+        <v>136</v>
+      </c>
+      <c r="G43" s="117" t="s">
         <v>296</v>
       </c>
-      <c r="H41" s="24"/>
-    </row>
-    <row r="42" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B42" s="127"/>
-      <c r="C42" s="26" t="s">
-        <v>266</v>
-      </c>
-      <c r="D42" s="117" t="s">
-        <v>267</v>
-      </c>
-      <c r="E42" s="117" t="s">
+      <c r="H43" s="24"/>
+    </row>
+    <row r="44" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A44" s="143" t="s">
+        <v>316</v>
+      </c>
+      <c r="B44" s="131" t="s">
+        <v>310</v>
+      </c>
+      <c r="C44" s="117" t="s">
+        <v>140</v>
+      </c>
+      <c r="D44" s="117" t="s">
+        <v>141</v>
+      </c>
+      <c r="E44" s="117" t="s">
         <v>270</v>
       </c>
-      <c r="F42" s="117" t="s">
-        <v>137</v>
-      </c>
-      <c r="G42" s="117" t="s">
+      <c r="F44" s="117" t="s">
+        <v>138</v>
+      </c>
+      <c r="G44" s="117" t="s">
         <v>296</v>
-      </c>
-      <c r="H42" s="24"/>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B43" s="143"/>
-      <c r="C43" s="26" t="s">
-        <v>287</v>
-      </c>
-      <c r="D43" s="117" t="s">
-        <v>288</v>
-      </c>
-      <c r="E43" s="117" t="s">
-        <v>289</v>
-      </c>
-      <c r="F43" s="117" t="s">
-        <v>137</v>
-      </c>
-      <c r="G43" s="117" t="s">
-        <v>297</v>
-      </c>
-      <c r="H43" s="24"/>
-    </row>
-    <row r="44" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A44" s="125" t="s">
-        <v>317</v>
-      </c>
-      <c r="B44" s="126" t="s">
-        <v>311</v>
-      </c>
-      <c r="C44" s="117" t="s">
-        <v>141</v>
-      </c>
-      <c r="D44" s="117" t="s">
-        <v>142</v>
-      </c>
-      <c r="E44" s="117" t="s">
-        <v>271</v>
-      </c>
-      <c r="F44" s="117" t="s">
-        <v>139</v>
-      </c>
-      <c r="G44" s="117" t="s">
-        <v>297</v>
       </c>
       <c r="H44" s="30"/>
       <c r="I44" s="28"/>
@@ -3548,22 +3548,22 @@
       <c r="K44" s="28"/>
     </row>
     <row r="45" spans="1:11" s="29" customFormat="1" ht="224.4" x14ac:dyDescent="0.3">
-      <c r="A45" s="125"/>
-      <c r="B45" s="127"/>
+      <c r="A45" s="143"/>
+      <c r="B45" s="132"/>
       <c r="C45" s="117" t="s">
+        <v>142</v>
+      </c>
+      <c r="D45" s="117" t="s">
         <v>143</v>
       </c>
-      <c r="D45" s="117" t="s">
-        <v>144</v>
-      </c>
       <c r="E45" s="117" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F45" s="26" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G45" s="26" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H45" s="30"/>
       <c r="I45" s="28"/>
@@ -3571,24 +3571,24 @@
       <c r="K45" s="28"/>
     </row>
     <row r="46" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A46" s="125"/>
-      <c r="B46" s="126" t="s">
-        <v>312</v>
+      <c r="A46" s="143"/>
+      <c r="B46" s="131" t="s">
+        <v>311</v>
       </c>
       <c r="C46" s="117" t="s">
+        <v>144</v>
+      </c>
+      <c r="D46" s="117" t="s">
         <v>145</v>
       </c>
-      <c r="D46" s="117" t="s">
-        <v>146</v>
-      </c>
       <c r="E46" s="117" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F46" s="117" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G46" s="117" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H46" s="30"/>
       <c r="I46" s="28"/>
@@ -3596,22 +3596,22 @@
       <c r="K46" s="28"/>
     </row>
     <row r="47" spans="1:11" s="29" customFormat="1" ht="224.4" x14ac:dyDescent="0.3">
-      <c r="A47" s="125"/>
-      <c r="B47" s="127"/>
+      <c r="A47" s="143"/>
+      <c r="B47" s="132"/>
       <c r="C47" s="117" t="s">
+        <v>146</v>
+      </c>
+      <c r="D47" s="117" t="s">
         <v>147</v>
       </c>
-      <c r="D47" s="117" t="s">
-        <v>148</v>
-      </c>
       <c r="E47" s="117" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F47" s="26" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G47" s="26" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H47" s="30"/>
       <c r="I47" s="28"/>
@@ -3620,23 +3620,23 @@
     </row>
     <row r="48" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A48"/>
-      <c r="B48" s="122" t="s">
+      <c r="B48" s="128" t="s">
+        <v>164</v>
+      </c>
+      <c r="C48" s="36" t="s">
         <v>165</v>
       </c>
-      <c r="C48" s="36" t="s">
+      <c r="D48" s="37" t="s">
         <v>166</v>
       </c>
-      <c r="D48" s="37" t="s">
+      <c r="E48" s="37" t="s">
         <v>167</v>
       </c>
-      <c r="E48" s="37" t="s">
-        <v>168</v>
-      </c>
       <c r="F48" s="36" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G48" s="36" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H48" s="31"/>
       <c r="I48" s="32"/>
@@ -3645,21 +3645,21 @@
     </row>
     <row r="49" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A49"/>
-      <c r="B49" s="124"/>
+      <c r="B49" s="130"/>
       <c r="C49" s="36" t="s">
+        <v>168</v>
+      </c>
+      <c r="D49" s="37" t="s">
         <v>169</v>
       </c>
-      <c r="D49" s="37" t="s">
+      <c r="E49" s="37" t="s">
         <v>170</v>
       </c>
-      <c r="E49" s="37" t="s">
+      <c r="F49" s="36" t="s">
         <v>171</v>
       </c>
-      <c r="F49" s="36" t="s">
-        <v>172</v>
-      </c>
       <c r="G49" s="36" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H49" s="31"/>
       <c r="I49" s="32"/>
@@ -3667,26 +3667,26 @@
       <c r="K49" s="32"/>
     </row>
     <row r="50" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A50" s="125" t="s">
-        <v>318</v>
-      </c>
-      <c r="B50" s="122" t="s">
-        <v>313</v>
+      <c r="A50" s="143" t="s">
+        <v>317</v>
+      </c>
+      <c r="B50" s="128" t="s">
+        <v>312</v>
       </c>
       <c r="C50" s="36" t="s">
+        <v>172</v>
+      </c>
+      <c r="D50" s="37" t="s">
         <v>173</v>
       </c>
-      <c r="D50" s="37" t="s">
+      <c r="E50" s="37" t="s">
         <v>174</v>
       </c>
-      <c r="E50" s="37" t="s">
-        <v>175</v>
-      </c>
       <c r="F50" s="36" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G50" s="36" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H50" s="31"/>
       <c r="I50" s="32"/>
@@ -3694,22 +3694,22 @@
       <c r="K50" s="32"/>
     </row>
     <row r="51" spans="1:11" s="33" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="125"/>
-      <c r="B51" s="123"/>
+      <c r="A51" s="143"/>
+      <c r="B51" s="129"/>
       <c r="C51" s="36" t="s">
+        <v>175</v>
+      </c>
+      <c r="D51" s="37" t="s">
         <v>176</v>
       </c>
-      <c r="D51" s="37" t="s">
+      <c r="E51" s="37" t="s">
         <v>177</v>
       </c>
-      <c r="E51" s="37" t="s">
+      <c r="F51" s="36" t="s">
         <v>178</v>
       </c>
-      <c r="F51" s="36" t="s">
-        <v>179</v>
-      </c>
       <c r="G51" s="36" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H51" s="31"/>
       <c r="I51" s="32"/>
@@ -3717,22 +3717,22 @@
       <c r="K51" s="32"/>
     </row>
     <row r="52" spans="1:11" s="33" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.3">
-      <c r="A52" s="125"/>
-      <c r="B52" s="123"/>
+      <c r="A52" s="143"/>
+      <c r="B52" s="129"/>
       <c r="C52" s="36" t="s">
+        <v>179</v>
+      </c>
+      <c r="D52" s="37" t="s">
         <v>180</v>
       </c>
-      <c r="D52" s="37" t="s">
-        <v>181</v>
-      </c>
       <c r="E52" s="37" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F52" s="36" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G52" s="36" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H52" s="31"/>
       <c r="I52" s="32"/>
@@ -3740,22 +3740,22 @@
       <c r="K52" s="32"/>
     </row>
     <row r="53" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A53" s="125"/>
-      <c r="B53" s="124"/>
+      <c r="A53" s="143"/>
+      <c r="B53" s="130"/>
       <c r="C53" s="36" t="s">
+        <v>181</v>
+      </c>
+      <c r="D53" s="37" t="s">
         <v>182</v>
       </c>
-      <c r="D53" s="37" t="s">
+      <c r="E53" s="37" t="s">
         <v>183</v>
-      </c>
-      <c r="E53" s="37" t="s">
-        <v>184</v>
       </c>
       <c r="F53" s="37" t="s">
         <v>30</v>
       </c>
       <c r="G53" s="36" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H53" s="31"/>
       <c r="I53" s="32"/>
@@ -3763,26 +3763,26 @@
       <c r="K53" s="32"/>
     </row>
     <row r="54" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A54" s="125" t="s">
-        <v>319</v>
-      </c>
-      <c r="B54" s="122" t="s">
-        <v>316</v>
+      <c r="A54" s="143" t="s">
+        <v>318</v>
+      </c>
+      <c r="B54" s="128" t="s">
+        <v>315</v>
       </c>
       <c r="C54" s="36" t="s">
+        <v>184</v>
+      </c>
+      <c r="D54" s="37" t="s">
         <v>185</v>
       </c>
-      <c r="D54" s="37" t="s">
+      <c r="E54" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="E54" s="37" t="s">
-        <v>187</v>
-      </c>
       <c r="F54" s="36" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G54" s="36" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H54" s="31"/>
       <c r="I54" s="32"/>
@@ -3790,22 +3790,22 @@
       <c r="K54" s="32"/>
     </row>
     <row r="55" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A55" s="125"/>
-      <c r="B55" s="123"/>
+      <c r="A55" s="143"/>
+      <c r="B55" s="129"/>
       <c r="C55" s="36" t="s">
+        <v>187</v>
+      </c>
+      <c r="D55" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="D55" s="37" t="s">
+      <c r="E55" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="E55" s="37" t="s">
+      <c r="F55" s="36" t="s">
         <v>190</v>
       </c>
-      <c r="F55" s="36" t="s">
-        <v>191</v>
-      </c>
       <c r="G55" s="36" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H55" s="31"/>
       <c r="I55" s="32"/>
@@ -3813,22 +3813,22 @@
       <c r="K55" s="32"/>
     </row>
     <row r="56" spans="1:11" s="33" customFormat="1" ht="356.4" x14ac:dyDescent="0.3">
-      <c r="A56" s="125"/>
-      <c r="B56" s="123"/>
+      <c r="A56" s="143"/>
+      <c r="B56" s="129"/>
       <c r="C56" s="36" t="s">
+        <v>191</v>
+      </c>
+      <c r="D56" s="37" t="s">
         <v>192</v>
       </c>
-      <c r="D56" s="37" t="s">
-        <v>193</v>
-      </c>
       <c r="E56" s="37" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="F56" s="37" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="G56" s="36" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H56" s="31"/>
       <c r="I56" s="32"/>
@@ -3836,22 +3836,22 @@
       <c r="K56" s="32"/>
     </row>
     <row r="57" spans="1:11" s="33" customFormat="1" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A57" s="125"/>
-      <c r="B57" s="124"/>
+      <c r="A57" s="143"/>
+      <c r="B57" s="130"/>
       <c r="C57" s="36" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D57" s="37" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E57" s="37" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F57" s="36" t="s">
         <v>30</v>
       </c>
       <c r="G57" s="36" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H57" s="31"/>
       <c r="I57" s="32"/>
@@ -3859,26 +3859,26 @@
       <c r="K57" s="32"/>
     </row>
     <row r="58" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A58" s="125" t="s">
-        <v>318</v>
-      </c>
-      <c r="B58" s="122" t="s">
-        <v>315</v>
+      <c r="A58" s="143" t="s">
+        <v>317</v>
+      </c>
+      <c r="B58" s="128" t="s">
+        <v>314</v>
       </c>
       <c r="C58" s="36" t="s">
+        <v>194</v>
+      </c>
+      <c r="D58" s="37" t="s">
         <v>195</v>
       </c>
-      <c r="D58" s="37" t="s">
+      <c r="E58" s="37" t="s">
         <v>196</v>
       </c>
-      <c r="E58" s="37" t="s">
-        <v>197</v>
-      </c>
       <c r="F58" s="36" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G58" s="36" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H58" s="31"/>
       <c r="I58" s="32"/>
@@ -3886,22 +3886,22 @@
       <c r="K58" s="32"/>
     </row>
     <row r="59" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A59" s="125"/>
-      <c r="B59" s="123"/>
+      <c r="A59" s="143"/>
+      <c r="B59" s="129"/>
       <c r="C59" s="36" t="s">
+        <v>197</v>
+      </c>
+      <c r="D59" s="37" t="s">
         <v>198</v>
       </c>
-      <c r="D59" s="37" t="s">
-        <v>199</v>
-      </c>
       <c r="E59" s="37" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F59" s="36" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G59" s="36" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H59" s="31"/>
       <c r="I59" s="32"/>
@@ -3909,22 +3909,22 @@
       <c r="K59" s="32"/>
     </row>
     <row r="60" spans="1:11" s="33" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.3">
-      <c r="A60" s="125"/>
-      <c r="B60" s="123"/>
+      <c r="A60" s="143"/>
+      <c r="B60" s="129"/>
       <c r="C60" s="36" t="s">
+        <v>199</v>
+      </c>
+      <c r="D60" s="37" t="s">
         <v>200</v>
       </c>
-      <c r="D60" s="37" t="s">
-        <v>201</v>
-      </c>
       <c r="E60" s="37" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F60" s="36" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G60" s="36" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H60" s="31"/>
       <c r="I60" s="32"/>
@@ -3932,22 +3932,22 @@
       <c r="K60" s="32"/>
     </row>
     <row r="61" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A61" s="125"/>
-      <c r="B61" s="124"/>
+      <c r="A61" s="143"/>
+      <c r="B61" s="130"/>
       <c r="C61" s="36" t="s">
+        <v>201</v>
+      </c>
+      <c r="D61" s="37" t="s">
         <v>202</v>
       </c>
-      <c r="D61" s="37" t="s">
-        <v>203</v>
-      </c>
       <c r="E61" s="37" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F61" s="37" t="s">
         <v>30</v>
       </c>
       <c r="G61" s="36" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H61" s="31"/>
       <c r="I61" s="32"/>
@@ -3955,26 +3955,26 @@
       <c r="K61" s="32"/>
     </row>
     <row r="62" spans="1:11" s="33" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="125" t="s">
-        <v>319</v>
-      </c>
-      <c r="B62" s="122" t="s">
-        <v>314</v>
+      <c r="A62" s="143" t="s">
+        <v>318</v>
+      </c>
+      <c r="B62" s="128" t="s">
+        <v>313</v>
       </c>
       <c r="C62" s="36" t="s">
+        <v>203</v>
+      </c>
+      <c r="D62" s="37" t="s">
         <v>204</v>
       </c>
-      <c r="D62" s="37" t="s">
+      <c r="E62" s="37" t="s">
         <v>205</v>
       </c>
-      <c r="E62" s="37" t="s">
-        <v>206</v>
-      </c>
       <c r="F62" s="36" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G62" s="36" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H62" s="31"/>
       <c r="I62" s="32"/>
@@ -3982,22 +3982,22 @@
       <c r="K62" s="32"/>
     </row>
     <row r="63" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A63" s="125"/>
-      <c r="B63" s="123"/>
+      <c r="A63" s="143"/>
+      <c r="B63" s="129"/>
       <c r="C63" s="36" t="s">
+        <v>206</v>
+      </c>
+      <c r="D63" s="37" t="s">
         <v>207</v>
       </c>
-      <c r="D63" s="37" t="s">
+      <c r="E63" s="37" t="s">
         <v>208</v>
       </c>
-      <c r="E63" s="37" t="s">
-        <v>209</v>
-      </c>
       <c r="F63" s="36" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G63" s="36" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H63" s="31"/>
       <c r="I63" s="32"/>
@@ -4005,163 +4005,163 @@
       <c r="K63" s="32"/>
     </row>
     <row r="64" spans="1:11" ht="356.4" x14ac:dyDescent="0.3">
-      <c r="A64" s="125"/>
-      <c r="B64" s="123"/>
+      <c r="A64" s="143"/>
+      <c r="B64" s="129"/>
       <c r="C64" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="D64" s="37" t="s">
         <v>210</v>
       </c>
-      <c r="D64" s="37" t="s">
+      <c r="E64" s="37" t="s">
+        <v>380</v>
+      </c>
+      <c r="F64" s="37" t="s">
+        <v>386</v>
+      </c>
+      <c r="G64" s="36" t="s">
+        <v>290</v>
+      </c>
+      <c r="H64" s="12"/>
+    </row>
+    <row r="65" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A65" s="143"/>
+      <c r="B65" s="130"/>
+      <c r="C65" s="36" t="s">
+        <v>354</v>
+      </c>
+      <c r="D65" s="37" t="s">
         <v>211</v>
       </c>
-      <c r="E64" s="37" t="s">
-        <v>381</v>
-      </c>
-      <c r="F64" s="37" t="s">
-        <v>387</v>
-      </c>
-      <c r="G64" s="36" t="s">
-        <v>291</v>
-      </c>
-      <c r="H64" s="12"/>
-    </row>
-    <row r="65" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A65" s="125"/>
-      <c r="B65" s="124"/>
-      <c r="C65" s="36" t="s">
-        <v>355</v>
-      </c>
-      <c r="D65" s="37" t="s">
-        <v>212</v>
-      </c>
       <c r="E65" s="37" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F65" s="36" t="s">
         <v>30</v>
       </c>
       <c r="G65" s="36" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H65" s="12"/>
     </row>
     <row r="66" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B66" s="122" t="s">
-        <v>306</v>
+      <c r="B66" s="128" t="s">
+        <v>305</v>
       </c>
       <c r="C66" s="36" t="s">
+        <v>212</v>
+      </c>
+      <c r="D66" s="37" t="s">
         <v>213</v>
       </c>
-      <c r="D66" s="37" t="s">
+      <c r="E66" s="37" t="s">
+        <v>359</v>
+      </c>
+      <c r="F66" s="36" t="s">
         <v>214</v>
       </c>
-      <c r="E66" s="37" t="s">
-        <v>360</v>
-      </c>
-      <c r="F66" s="36" t="s">
+      <c r="G66" s="36" t="s">
+        <v>296</v>
+      </c>
+      <c r="H66" s="10"/>
+    </row>
+    <row r="67" spans="1:11" ht="93" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B67" s="129"/>
+      <c r="C67" s="36" t="s">
         <v>215</v>
       </c>
-      <c r="G66" s="36" t="s">
-        <v>297</v>
-      </c>
-      <c r="H66" s="10"/>
-    </row>
-    <row r="67" spans="1:11" ht="93" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B67" s="123"/>
-      <c r="C67" s="36" t="s">
+      <c r="D67" s="37" t="s">
         <v>216</v>
       </c>
-      <c r="D67" s="37" t="s">
-        <v>217</v>
-      </c>
       <c r="E67" s="37" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="F67" s="36" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G67" s="36" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H67" s="12"/>
     </row>
     <row r="68" spans="1:11" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B68" s="123"/>
+      <c r="B68" s="129"/>
       <c r="C68" s="36" t="s">
+        <v>369</v>
+      </c>
+      <c r="D68" s="37" t="s">
+        <v>371</v>
+      </c>
+      <c r="E68" s="37" t="s">
+        <v>376</v>
+      </c>
+      <c r="F68" s="36" t="s">
+        <v>373</v>
+      </c>
+      <c r="G68" s="36" t="s">
+        <v>295</v>
+      </c>
+      <c r="H68" s="12"/>
+    </row>
+    <row r="69" spans="1:11" ht="158.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B69" s="129"/>
+      <c r="C69" s="36" t="s">
         <v>370</v>
       </c>
-      <c r="D68" s="37" t="s">
+      <c r="D69" s="37" t="s">
+        <v>374</v>
+      </c>
+      <c r="E69" s="37" t="s">
+        <v>377</v>
+      </c>
+      <c r="F69" s="36" t="s">
+        <v>381</v>
+      </c>
+      <c r="G69" s="36" t="s">
+        <v>295</v>
+      </c>
+      <c r="H69" s="12"/>
+    </row>
+    <row r="70" spans="1:11" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B70" s="130"/>
+      <c r="C70" s="36" t="s">
         <v>372</v>
       </c>
-      <c r="E68" s="37" t="s">
-        <v>377</v>
-      </c>
-      <c r="F68" s="36" t="s">
-        <v>374</v>
-      </c>
-      <c r="G68" s="36" t="s">
-        <v>296</v>
-      </c>
-      <c r="H68" s="12"/>
-    </row>
-    <row r="69" spans="1:11" ht="158.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B69" s="123"/>
-      <c r="C69" s="36" t="s">
-        <v>371</v>
-      </c>
-      <c r="D69" s="37" t="s">
+      <c r="D70" s="37" t="s">
         <v>375</v>
       </c>
-      <c r="E69" s="37" t="s">
-        <v>378</v>
-      </c>
-      <c r="F69" s="36" t="s">
-        <v>382</v>
-      </c>
-      <c r="G69" s="36" t="s">
-        <v>296</v>
-      </c>
-      <c r="H69" s="12"/>
-    </row>
-    <row r="70" spans="1:11" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B70" s="124"/>
-      <c r="C70" s="36" t="s">
-        <v>373</v>
-      </c>
-      <c r="D70" s="37" t="s">
-        <v>376</v>
-      </c>
       <c r="E70" s="37" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F70" s="36" t="s">
         <v>30</v>
       </c>
       <c r="G70" s="36" t="s">
+        <v>295</v>
+      </c>
+      <c r="H70" s="12"/>
+    </row>
+    <row r="71" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A71" s="143" t="s">
+        <v>319</v>
+      </c>
+      <c r="B71" s="128" t="s">
+        <v>306</v>
+      </c>
+      <c r="C71" s="36" t="s">
+        <v>217</v>
+      </c>
+      <c r="D71" s="37" t="s">
+        <v>218</v>
+      </c>
+      <c r="E71" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="F71" s="36" t="s">
+        <v>220</v>
+      </c>
+      <c r="G71" s="36" t="s">
         <v>296</v>
-      </c>
-      <c r="H70" s="12"/>
-    </row>
-    <row r="71" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A71" s="125" t="s">
-        <v>320</v>
-      </c>
-      <c r="B71" s="122" t="s">
-        <v>307</v>
-      </c>
-      <c r="C71" s="36" t="s">
-        <v>218</v>
-      </c>
-      <c r="D71" s="37" t="s">
-        <v>219</v>
-      </c>
-      <c r="E71" s="37" t="s">
-        <v>220</v>
-      </c>
-      <c r="F71" s="36" t="s">
-        <v>221</v>
-      </c>
-      <c r="G71" s="36" t="s">
-        <v>297</v>
       </c>
       <c r="H71" s="30"/>
       <c r="I71" s="28"/>
@@ -4169,22 +4169,22 @@
       <c r="K71" s="28"/>
     </row>
     <row r="72" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A72" s="125"/>
-      <c r="B72" s="123"/>
+      <c r="A72" s="143"/>
+      <c r="B72" s="129"/>
       <c r="C72" s="36" t="s">
+        <v>221</v>
+      </c>
+      <c r="D72" s="37" t="s">
         <v>222</v>
       </c>
-      <c r="D72" s="37" t="s">
+      <c r="E72" s="37" t="s">
         <v>223</v>
       </c>
-      <c r="E72" s="37" t="s">
-        <v>224</v>
-      </c>
       <c r="F72" s="36" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G72" s="36" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H72" s="30"/>
       <c r="I72" s="28"/>
@@ -4192,22 +4192,22 @@
       <c r="K72" s="28"/>
     </row>
     <row r="73" spans="1:11" s="29" customFormat="1" ht="184.8" x14ac:dyDescent="0.3">
-      <c r="A73" s="125"/>
-      <c r="B73" s="124"/>
+      <c r="A73" s="143"/>
+      <c r="B73" s="130"/>
       <c r="C73" s="36" t="s">
+        <v>224</v>
+      </c>
+      <c r="D73" s="37" t="s">
         <v>225</v>
       </c>
-      <c r="D73" s="37" t="s">
-        <v>226</v>
-      </c>
       <c r="E73" s="37" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="F73" s="36" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G73" s="36" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H73" s="30"/>
       <c r="I73" s="28"/>
@@ -4215,24 +4215,24 @@
       <c r="K73" s="28"/>
     </row>
     <row r="74" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A74" s="125"/>
-      <c r="B74" s="122" t="s">
-        <v>307</v>
+      <c r="A74" s="143"/>
+      <c r="B74" s="128" t="s">
+        <v>306</v>
       </c>
       <c r="C74" s="36" t="s">
+        <v>226</v>
+      </c>
+      <c r="D74" s="37" t="s">
         <v>227</v>
       </c>
-      <c r="D74" s="37" t="s">
+      <c r="E74" s="37" t="s">
         <v>228</v>
       </c>
-      <c r="E74" s="37" t="s">
-        <v>229</v>
-      </c>
       <c r="F74" s="36" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G74" s="36" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H74" s="30"/>
       <c r="I74" s="28"/>
@@ -4240,22 +4240,22 @@
       <c r="K74" s="28"/>
     </row>
     <row r="75" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A75" s="125"/>
-      <c r="B75" s="123"/>
+      <c r="A75" s="143"/>
+      <c r="B75" s="129"/>
       <c r="C75" s="36" t="s">
+        <v>229</v>
+      </c>
+      <c r="D75" s="37" t="s">
         <v>230</v>
       </c>
-      <c r="D75" s="37" t="s">
+      <c r="E75" s="37" t="s">
         <v>231</v>
       </c>
-      <c r="E75" s="37" t="s">
-        <v>232</v>
-      </c>
       <c r="F75" s="36" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G75" s="36" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H75" s="30"/>
       <c r="I75" s="28"/>
@@ -4263,22 +4263,22 @@
       <c r="K75" s="28"/>
     </row>
     <row r="76" spans="1:11" s="29" customFormat="1" ht="184.8" x14ac:dyDescent="0.3">
-      <c r="A76" s="125"/>
-      <c r="B76" s="124"/>
+      <c r="A76" s="143"/>
+      <c r="B76" s="130"/>
       <c r="C76" s="36" t="s">
+        <v>232</v>
+      </c>
+      <c r="D76" s="37" t="s">
         <v>233</v>
       </c>
-      <c r="D76" s="37" t="s">
-        <v>234</v>
-      </c>
       <c r="E76" s="37" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F76" s="36" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G76" s="36" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H76" s="30"/>
       <c r="I76" s="28"/>
@@ -4287,23 +4287,23 @@
     </row>
     <row r="77" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A77"/>
-      <c r="B77" s="122" t="s">
-        <v>308</v>
+      <c r="B77" s="128" t="s">
+        <v>307</v>
       </c>
       <c r="C77" s="118" t="s">
+        <v>234</v>
+      </c>
+      <c r="D77" s="118" t="s">
         <v>235</v>
       </c>
-      <c r="D77" s="118" t="s">
+      <c r="E77" s="118" t="s">
         <v>236</v>
       </c>
-      <c r="E77" s="118" t="s">
-        <v>237</v>
-      </c>
       <c r="F77" s="119" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G77" s="119" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H77" s="30"/>
       <c r="I77" s="28"/>
@@ -4312,21 +4312,21 @@
     </row>
     <row r="78" spans="1:11" s="33" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A78"/>
-      <c r="B78" s="124"/>
+      <c r="B78" s="130"/>
       <c r="C78" s="118" t="s">
+        <v>237</v>
+      </c>
+      <c r="D78" s="118" t="s">
         <v>238</v>
       </c>
-      <c r="D78" s="118" t="s">
-        <v>239</v>
-      </c>
       <c r="E78" s="118" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F78" s="118" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G78" s="118" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H78" s="31"/>
       <c r="I78" s="32"/>
@@ -4334,26 +4334,26 @@
       <c r="K78" s="32"/>
     </row>
     <row r="79" spans="1:11" s="33" customFormat="1" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="125" t="s">
+      <c r="A79" s="143" t="s">
+        <v>320</v>
+      </c>
+      <c r="B79" s="128" t="s">
         <v>321</v>
       </c>
-      <c r="B79" s="122" t="s">
-        <v>322</v>
-      </c>
       <c r="C79" s="36" t="s">
+        <v>239</v>
+      </c>
+      <c r="D79" s="37" t="s">
         <v>240</v>
       </c>
-      <c r="D79" s="37" t="s">
-        <v>241</v>
-      </c>
       <c r="E79" s="118" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="F79" s="36" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G79" s="36" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H79" s="31"/>
       <c r="I79" s="32"/>
@@ -4361,22 +4361,22 @@
       <c r="K79" s="32"/>
     </row>
     <row r="80" spans="1:11" s="33" customFormat="1" ht="78" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="125"/>
-      <c r="B80" s="123"/>
+      <c r="A80" s="143"/>
+      <c r="B80" s="129"/>
       <c r="C80" s="36" t="s">
+        <v>324</v>
+      </c>
+      <c r="D80" s="37" t="s">
         <v>325</v>
       </c>
-      <c r="D80" s="37" t="s">
-        <v>326</v>
-      </c>
       <c r="E80" s="37" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="F80" s="36" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="G80" s="36" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H80" s="31"/>
       <c r="I80" s="32"/>
@@ -4384,19 +4384,19 @@
       <c r="K80" s="32"/>
     </row>
     <row r="81" spans="1:11" s="33" customFormat="1" ht="212.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="125"/>
-      <c r="B81" s="124"/>
+      <c r="A81" s="143"/>
+      <c r="B81" s="130"/>
       <c r="C81" s="36" t="s">
+        <v>326</v>
+      </c>
+      <c r="D81" s="37" t="s">
         <v>327</v>
       </c>
-      <c r="D81" s="37" t="s">
+      <c r="E81" s="37" t="s">
+        <v>364</v>
+      </c>
+      <c r="F81" s="36" t="s">
         <v>328</v>
-      </c>
-      <c r="E81" s="37" t="s">
-        <v>365</v>
-      </c>
-      <c r="F81" s="36" t="s">
-        <v>329</v>
       </c>
       <c r="G81" s="36"/>
       <c r="H81" s="31"/>
@@ -4405,26 +4405,26 @@
       <c r="K81" s="32"/>
     </row>
     <row r="82" spans="1:11" s="33" customFormat="1" ht="117" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="125" t="s">
-        <v>321</v>
-      </c>
-      <c r="B82" s="122" t="s">
-        <v>323</v>
+      <c r="A82" s="143" t="s">
+        <v>320</v>
+      </c>
+      <c r="B82" s="128" t="s">
+        <v>322</v>
       </c>
       <c r="C82" s="36" t="s">
+        <v>241</v>
+      </c>
+      <c r="D82" s="37" t="s">
         <v>242</v>
       </c>
-      <c r="D82" s="37" t="s">
-        <v>243</v>
-      </c>
       <c r="E82" s="118" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="F82" s="36" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G82" s="36" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H82" s="31"/>
       <c r="I82" s="32"/>
@@ -4432,22 +4432,22 @@
       <c r="K82" s="32"/>
     </row>
     <row r="83" spans="1:11" s="33" customFormat="1" ht="83.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="125"/>
-      <c r="B83" s="123"/>
+      <c r="A83" s="143"/>
+      <c r="B83" s="129"/>
       <c r="C83" s="36" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D83" s="37" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="E83" s="37" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="F83" s="36" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="G83" s="36" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H83" s="31"/>
       <c r="I83" s="32"/>
@@ -4455,19 +4455,19 @@
       <c r="K83" s="32"/>
     </row>
     <row r="84" spans="1:11" s="33" customFormat="1" ht="199.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="125"/>
-      <c r="B84" s="124"/>
+      <c r="A84" s="143"/>
+      <c r="B84" s="130"/>
       <c r="C84" s="36" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D84" s="37" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E84" s="37" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="F84" s="36" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="G84" s="36"/>
       <c r="H84" s="31"/>
@@ -4476,77 +4476,77 @@
       <c r="K84" s="32"/>
     </row>
     <row r="85" spans="1:11" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="B85" s="122" t="s">
-        <v>309</v>
+      <c r="B85" s="128" t="s">
+        <v>308</v>
       </c>
       <c r="C85" s="36" t="s">
+        <v>251</v>
+      </c>
+      <c r="D85" s="37" t="s">
         <v>252</v>
       </c>
-      <c r="D85" s="37" t="s">
+      <c r="E85" s="118" t="s">
+        <v>368</v>
+      </c>
+      <c r="F85" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="G85" s="36" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" ht="118.8" x14ac:dyDescent="0.3">
+      <c r="B86" s="129"/>
+      <c r="C86" s="36" t="s">
         <v>253</v>
       </c>
-      <c r="E85" s="118" t="s">
-        <v>369</v>
-      </c>
-      <c r="F85" s="36" t="s">
-        <v>304</v>
-      </c>
-      <c r="G85" s="36" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="86" spans="1:11" ht="118.8" x14ac:dyDescent="0.3">
-      <c r="B86" s="123"/>
-      <c r="C86" s="36" t="s">
+      <c r="D86" s="37" t="s">
         <v>254</v>
       </c>
-      <c r="D86" s="37" t="s">
+      <c r="E86" s="118" t="s">
+        <v>382</v>
+      </c>
+      <c r="F86" s="36" t="s">
+        <v>136</v>
+      </c>
+      <c r="G86" s="36" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" ht="198" x14ac:dyDescent="0.3">
+      <c r="B87" s="129"/>
+      <c r="C87" s="36" t="s">
         <v>255</v>
       </c>
-      <c r="E86" s="118" t="s">
-        <v>383</v>
-      </c>
-      <c r="F86" s="36" t="s">
-        <v>137</v>
-      </c>
-      <c r="G86" s="36" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="87" spans="1:11" ht="198" x14ac:dyDescent="0.3">
-      <c r="B87" s="123"/>
-      <c r="C87" s="36" t="s">
+      <c r="D87" s="37" t="s">
         <v>256</v>
       </c>
-      <c r="D87" s="37" t="s">
+      <c r="E87" s="118" t="s">
+        <v>378</v>
+      </c>
+      <c r="F87" s="36" t="s">
+        <v>302</v>
+      </c>
+      <c r="G87" s="36" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" ht="66" x14ac:dyDescent="0.3">
+      <c r="B88" s="130"/>
+      <c r="C88" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="E87" s="118" t="s">
-        <v>379</v>
-      </c>
-      <c r="F87" s="36" t="s">
-        <v>303</v>
-      </c>
-      <c r="G87" s="36" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="88" spans="1:11" ht="66" x14ac:dyDescent="0.3">
-      <c r="B88" s="124"/>
-      <c r="C88" s="36" t="s">
+      <c r="D88" s="37" t="s">
         <v>258</v>
       </c>
-      <c r="D88" s="37" t="s">
-        <v>259</v>
-      </c>
       <c r="E88" s="118" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F88" s="36" t="s">
         <v>30</v>
       </c>
       <c r="G88" s="36" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.3">
@@ -4583,20 +4583,6 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="E17:E26"/>
-    <mergeCell ref="E38:E40"/>
-    <mergeCell ref="B82:B84"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="B48:B49"/>
-    <mergeCell ref="B54:B57"/>
-    <mergeCell ref="B58:B61"/>
-    <mergeCell ref="B62:B65"/>
-    <mergeCell ref="B66:B70"/>
-    <mergeCell ref="B3:B16"/>
-    <mergeCell ref="B17:B26"/>
-    <mergeCell ref="B27:B29"/>
-    <mergeCell ref="B30:B40"/>
-    <mergeCell ref="B50:B53"/>
     <mergeCell ref="B85:B88"/>
     <mergeCell ref="A17:A26"/>
     <mergeCell ref="B44:B45"/>
@@ -4613,6 +4599,20 @@
     <mergeCell ref="A79:A81"/>
     <mergeCell ref="B79:B81"/>
     <mergeCell ref="A82:A84"/>
+    <mergeCell ref="B3:B16"/>
+    <mergeCell ref="B17:B26"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="B30:B40"/>
+    <mergeCell ref="B50:B53"/>
+    <mergeCell ref="E17:E26"/>
+    <mergeCell ref="E38:E40"/>
+    <mergeCell ref="B82:B84"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="B54:B57"/>
+    <mergeCell ref="B58:B61"/>
+    <mergeCell ref="B62:B65"/>
+    <mergeCell ref="B66:B70"/>
   </mergeCells>
   <phoneticPr fontId="29" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4641,7 +4641,7 @@
         <v>28</v>
       </c>
       <c r="B1" s="101" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C1" s="102" t="s">
         <v>33</v>
@@ -4650,7 +4650,7 @@
         <v>37</v>
       </c>
       <c r="E1" s="102" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="F1" s="102" t="s">
         <v>42</v>
@@ -4698,19 +4698,19 @@
         <v>91</v>
       </c>
       <c r="U1" s="103" t="s">
+        <v>276</v>
+      </c>
+      <c r="V1" s="103" t="s">
         <v>277</v>
       </c>
-      <c r="V1" s="103" t="s">
+      <c r="W1" s="103" t="s">
         <v>278</v>
       </c>
-      <c r="W1" s="103" t="s">
+      <c r="X1" s="103" t="s">
         <v>279</v>
       </c>
-      <c r="X1" s="103" t="s">
+      <c r="Y1" s="103" t="s">
         <v>280</v>
-      </c>
-      <c r="Y1" s="103" t="s">
-        <v>281</v>
       </c>
       <c r="Z1" s="104" t="s">
         <v>94</v>
@@ -4725,304 +4725,304 @@
         <v>107</v>
       </c>
       <c r="AD1" s="104" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AE1" s="104" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="AF1" s="104" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AG1" s="104" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="AH1" s="104" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AI1" s="104" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AJ1" s="104" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="AK1" s="104" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="AL1" s="104" t="s">
+        <v>274</v>
+      </c>
+      <c r="AM1" s="104" t="s">
         <v>275</v>
       </c>
-      <c r="AM1" s="104" t="s">
-        <v>276</v>
-      </c>
       <c r="AN1" s="105" t="s">
+        <v>264</v>
+      </c>
+      <c r="AO1" s="105" t="s">
         <v>265</v>
       </c>
-      <c r="AO1" s="105" t="s">
-        <v>266</v>
-      </c>
       <c r="AP1" s="44" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="AQ1" s="44" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AR1" s="44" t="s">
+        <v>139</v>
+      </c>
+      <c r="AS1" s="44" t="s">
         <v>140</v>
       </c>
-      <c r="AS1" s="44" t="s">
-        <v>141</v>
-      </c>
       <c r="AT1" s="44" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="AU1" s="44" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AV1" s="44" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AW1" s="44" t="s">
+        <v>148</v>
+      </c>
+      <c r="AX1" s="44" t="s">
         <v>149</v>
       </c>
-      <c r="AX1" s="44" t="s">
+      <c r="AY1" s="44" t="s">
         <v>150</v>
       </c>
-      <c r="AY1" s="44" t="s">
+      <c r="AZ1" s="44" t="s">
         <v>151</v>
       </c>
-      <c r="AZ1" s="44" t="s">
+      <c r="BA1" s="44" t="s">
         <v>152</v>
       </c>
-      <c r="BA1" s="44" t="s">
+      <c r="BB1" s="44" t="s">
         <v>153</v>
       </c>
-      <c r="BB1" s="44" t="s">
+      <c r="BC1" s="44" t="s">
         <v>154</v>
       </c>
-      <c r="BC1" s="44" t="s">
+      <c r="BD1" s="44" t="s">
         <v>155</v>
       </c>
-      <c r="BD1" s="44" t="s">
+      <c r="BE1" s="44" t="s">
         <v>156</v>
       </c>
-      <c r="BE1" s="44" t="s">
+      <c r="BF1" s="44" t="s">
         <v>157</v>
       </c>
-      <c r="BF1" s="44" t="s">
+      <c r="BG1" s="44" t="s">
         <v>158</v>
       </c>
-      <c r="BG1" s="44" t="s">
+      <c r="BH1" s="44" t="s">
         <v>159</v>
       </c>
-      <c r="BH1" s="44" t="s">
+      <c r="BI1" s="44" t="s">
         <v>160</v>
       </c>
-      <c r="BI1" s="44" t="s">
+      <c r="BJ1" s="44" t="s">
         <v>161</v>
       </c>
-      <c r="BJ1" s="44" t="s">
+      <c r="BK1" s="44" t="s">
         <v>162</v>
       </c>
-      <c r="BK1" s="44" t="s">
+      <c r="BL1" s="44" t="s">
         <v>163</v>
       </c>
-      <c r="BL1" s="44" t="s">
-        <v>164</v>
-      </c>
       <c r="BM1" s="45" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="BN1" s="45" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="BO1" s="45" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="BP1" s="45" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="BQ1" s="45" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="BR1" s="45" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="BS1" s="45" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="BT1" s="45" t="s">
+        <v>259</v>
+      </c>
+      <c r="BU1" s="45" t="s">
         <v>260</v>
       </c>
-      <c r="BU1" s="45" t="s">
+      <c r="BV1" s="45" t="s">
+        <v>355</v>
+      </c>
+      <c r="BW1" s="45" t="s">
+        <v>194</v>
+      </c>
+      <c r="BX1" s="45" t="s">
+        <v>197</v>
+      </c>
+      <c r="BY1" s="45" t="s">
+        <v>199</v>
+      </c>
+      <c r="BZ1" s="45" t="s">
+        <v>201</v>
+      </c>
+      <c r="CA1" s="45" t="s">
+        <v>203</v>
+      </c>
+      <c r="CB1" s="45" t="s">
         <v>261</v>
       </c>
-      <c r="BV1" s="45" t="s">
+      <c r="CC1" s="45" t="s">
+        <v>262</v>
+      </c>
+      <c r="CD1" s="45" t="s">
         <v>356</v>
       </c>
-      <c r="BW1" s="45" t="s">
-        <v>195</v>
-      </c>
-      <c r="BX1" s="45" t="s">
-        <v>198</v>
-      </c>
-      <c r="BY1" s="45" t="s">
-        <v>200</v>
-      </c>
-      <c r="BZ1" s="45" t="s">
-        <v>202</v>
-      </c>
-      <c r="CA1" s="45" t="s">
-        <v>204</v>
-      </c>
-      <c r="CB1" s="45" t="s">
-        <v>262</v>
-      </c>
-      <c r="CC1" s="45" t="s">
-        <v>263</v>
-      </c>
-      <c r="CD1" s="45" t="s">
-        <v>357</v>
-      </c>
       <c r="CE1" s="45" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="CF1" s="45" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="CG1" s="121" t="s">
+        <v>369</v>
+      </c>
+      <c r="CH1" s="121" t="s">
         <v>370</v>
       </c>
-      <c r="CH1" s="121" t="s">
-        <v>371</v>
-      </c>
       <c r="CI1" s="121" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="CJ1" s="45" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="CK1" s="45" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="CL1" s="45" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="CM1" s="45" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="CN1" s="45" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="CO1" s="45" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="CP1" s="45" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="CQ1" s="45" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="CR1" s="45" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="CS1" s="45" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="CT1" s="45" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="CU1" s="45" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="CV1" s="45" t="s">
+        <v>329</v>
+      </c>
+      <c r="CW1" s="45" t="s">
         <v>330</v>
       </c>
-      <c r="CW1" s="45" t="s">
-        <v>331</v>
-      </c>
       <c r="CX1" s="45" t="s">
+        <v>243</v>
+      </c>
+      <c r="CY1" s="45" t="s">
+        <v>333</v>
+      </c>
+      <c r="CZ1" s="45" t="s">
+        <v>341</v>
+      </c>
+      <c r="DA1" s="45" t="s">
         <v>244</v>
       </c>
-      <c r="CY1" s="45" t="s">
+      <c r="DB1" s="45" t="s">
         <v>334</v>
       </c>
-      <c r="CZ1" s="45" t="s">
+      <c r="DC1" s="45" t="s">
         <v>342</v>
       </c>
-      <c r="DA1" s="45" t="s">
+      <c r="DD1" s="45" t="s">
         <v>245</v>
       </c>
-      <c r="DB1" s="45" t="s">
+      <c r="DE1" s="45" t="s">
         <v>335</v>
       </c>
-      <c r="DC1" s="45" t="s">
+      <c r="DF1" s="45" t="s">
         <v>343</v>
       </c>
-      <c r="DD1" s="45" t="s">
+      <c r="DG1" s="45" t="s">
         <v>246</v>
       </c>
-      <c r="DE1" s="45" t="s">
+      <c r="DH1" s="45" t="s">
         <v>336</v>
       </c>
-      <c r="DF1" s="45" t="s">
+      <c r="DI1" s="45" t="s">
         <v>344</v>
       </c>
-      <c r="DG1" s="45" t="s">
+      <c r="DJ1" s="45" t="s">
         <v>247</v>
       </c>
-      <c r="DH1" s="45" t="s">
+      <c r="DK1" s="45" t="s">
         <v>337</v>
       </c>
-      <c r="DI1" s="45" t="s">
+      <c r="DL1" s="45" t="s">
         <v>345</v>
       </c>
-      <c r="DJ1" s="45" t="s">
+      <c r="DM1" s="45" t="s">
         <v>248</v>
       </c>
-      <c r="DK1" s="45" t="s">
+      <c r="DN1" s="45" t="s">
         <v>338</v>
       </c>
-      <c r="DL1" s="45" t="s">
+      <c r="DO1" s="45" t="s">
         <v>346</v>
       </c>
-      <c r="DM1" s="45" t="s">
+      <c r="DP1" s="45" t="s">
         <v>249</v>
       </c>
-      <c r="DN1" s="45" t="s">
+      <c r="DQ1" s="45" t="s">
         <v>339</v>
       </c>
-      <c r="DO1" s="45" t="s">
+      <c r="DR1" s="45" t="s">
         <v>347</v>
       </c>
-      <c r="DP1" s="45" t="s">
+      <c r="DS1" s="45" t="s">
         <v>250</v>
       </c>
-      <c r="DQ1" s="45" t="s">
+      <c r="DT1" s="45" t="s">
         <v>340</v>
       </c>
-      <c r="DR1" s="45" t="s">
+      <c r="DU1" s="45" t="s">
         <v>348</v>
       </c>
-      <c r="DS1" s="45" t="s">
+      <c r="DV1" s="45" t="s">
         <v>251</v>
       </c>
-      <c r="DT1" s="45" t="s">
-        <v>341</v>
-      </c>
-      <c r="DU1" s="45" t="s">
-        <v>349</v>
-      </c>
-      <c r="DV1" s="45" t="s">
-        <v>252</v>
-      </c>
       <c r="DW1" s="45" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="DX1" s="45" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="DY1" s="45" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" spans="1:129" x14ac:dyDescent="0.3">
@@ -20331,26 +20331,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="42fbd5e6-b175-407a-a25c-5fc6410bf24f" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EE7777BCFCD3E741B5CCCE9A87E98C2C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f7fc7590daec4eb8e38e018938a160ca">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e" xmlns:ns3="42fbd5e6-b175-407a-a25c-5fc6410bf24f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c5ca1b94d4b54616210e83d04e6b3cac" ns2:_="" ns3:_="">
     <xsd:import namespace="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
@@ -20605,26 +20585,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E9485EC-5D88-4A1C-961D-0F4FE84359B8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="42fbd5e6-b175-407a-a25c-5fc6410bf24f"/>
-    <ds:schemaRef ds:uri="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{286F673D-E70D-4002-B8F5-CAC95B029A7E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="42fbd5e6-b175-407a-a25c-5fc6410bf24f" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C9C537E-DFD2-4C38-AC8C-930F122DEFFC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -20641,4 +20622,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{286F673D-E70D-4002-B8F5-CAC95B029A7E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E9485EC-5D88-4A1C-961D-0F4FE84359B8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="42fbd5e6-b175-407a-a25c-5fc6410bf24f"/>
+    <ds:schemaRef ds:uri="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
update instruction for payor var
</commit_message>
<xml_diff>
--- a/data/ALAI UP Client-level Reporting Tool Template_4.7.26.xlsx
+++ b/data/ALAI UP Client-level Reporting Tool Template_4.7.26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kmlab\Desktop\Dashboard\alai_up_local_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{202CCA6C-59A9-443E-B33F-943AD869A990}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D4F2095-0129-452D-8345-560DABCBC696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-9840" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{500E2EE0-B1C5-4ACF-BC67-EDC8BDABD2D7}"/>
   </bookViews>
@@ -1405,10 +1405,10 @@
     <t>Secondary Payor</t>
   </si>
   <si>
-    <t>Report secondary payor of health care coverage, especially as it relates to HIV medications. If there is no secondary payor, this field may be left blank</t>
-  </si>
-  <si>
     <t>1=ADAP; 2=Patient Assistance Program (PAP); 3=Other; UNK=Unknown</t>
+  </si>
+  <si>
+    <t>Report payor of HIV medications if different or supplemental from health care coverage. If there is no secondary payor, this field may be left blank</t>
   </si>
 </sst>
 </file>
@@ -2124,24 +2124,6 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2151,13 +2133,13 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2167,6 +2149,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2187,7 +2178,16 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2750,7 +2750,7 @@
       <c r="K2" s="4"/>
     </row>
     <row r="3" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="134" t="s">
+      <c r="B3" s="128" t="s">
         <v>31</v>
       </c>
       <c r="C3" s="109" t="s">
@@ -2772,7 +2772,7 @@
       <c r="I3" s="8"/>
     </row>
     <row r="4" spans="1:11" ht="67.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="135"/>
+      <c r="B4" s="129"/>
       <c r="C4" s="15" t="s">
         <v>33</v>
       </c>
@@ -2792,7 +2792,7 @@
       <c r="I4" s="8"/>
     </row>
     <row r="5" spans="1:11" ht="44.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="135"/>
+      <c r="B5" s="129"/>
       <c r="C5" s="15" t="s">
         <v>37</v>
       </c>
@@ -2812,7 +2812,7 @@
       <c r="I5" s="17"/>
     </row>
     <row r="6" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B6" s="135"/>
+      <c r="B6" s="129"/>
       <c r="C6" s="15" t="s">
         <v>347</v>
       </c>
@@ -2832,7 +2832,7 @@
     </row>
     <row r="7" spans="1:11" s="19" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A7"/>
-      <c r="B7" s="135"/>
+      <c r="B7" s="129"/>
       <c r="C7" s="15" t="s">
         <v>42</v>
       </c>
@@ -2854,7 +2854,7 @@
       <c r="K7" s="18"/>
     </row>
     <row r="8" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B8" s="135"/>
+      <c r="B8" s="129"/>
       <c r="C8" s="15" t="s">
         <v>46</v>
       </c>
@@ -2873,7 +2873,7 @@
       <c r="H8" s="12"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B9" s="135"/>
+      <c r="B9" s="129"/>
       <c r="C9" s="15" t="s">
         <v>50</v>
       </c>
@@ -2892,7 +2892,7 @@
       <c r="H9" s="12"/>
     </row>
     <row r="10" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B10" s="135"/>
+      <c r="B10" s="129"/>
       <c r="C10" s="15" t="s">
         <v>54</v>
       </c>
@@ -2911,7 +2911,7 @@
       <c r="H10" s="12"/>
     </row>
     <row r="11" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B11" s="135"/>
+      <c r="B11" s="129"/>
       <c r="C11" s="15" t="s">
         <v>58</v>
       </c>
@@ -2930,7 +2930,7 @@
       <c r="H11" s="12"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B12" s="135"/>
+      <c r="B12" s="129"/>
       <c r="C12" s="15" t="s">
         <v>62</v>
       </c>
@@ -2949,7 +2949,7 @@
       <c r="H12" s="12"/>
     </row>
     <row r="13" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B13" s="135"/>
+      <c r="B13" s="129"/>
       <c r="C13" s="15" t="s">
         <v>66</v>
       </c>
@@ -2968,7 +2968,7 @@
       <c r="H13" s="12"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B14" s="135"/>
+      <c r="B14" s="129"/>
       <c r="C14" s="15" t="s">
         <v>70</v>
       </c>
@@ -2987,7 +2987,7 @@
       <c r="H14" s="12"/>
     </row>
     <row r="15" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B15" s="135"/>
+      <c r="B15" s="129"/>
       <c r="C15" s="15" t="s">
         <v>73</v>
       </c>
@@ -3006,7 +3006,7 @@
       <c r="H15" s="20"/>
     </row>
     <row r="16" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B16" s="136"/>
+      <c r="B16" s="130"/>
       <c r="C16" s="15" t="s">
         <v>77</v>
       </c>
@@ -3025,10 +3025,10 @@
       <c r="H16" s="12"/>
     </row>
     <row r="17" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="143" t="s">
+      <c r="A17" s="125" t="s">
         <v>307</v>
       </c>
-      <c r="B17" s="122" t="s">
+      <c r="B17" s="131" t="s">
         <v>81</v>
       </c>
       <c r="C17" s="111" t="s">
@@ -3037,7 +3037,7 @@
       <c r="D17" s="112" t="s">
         <v>83</v>
       </c>
-      <c r="E17" s="122" t="s">
+      <c r="E17" s="131" t="s">
         <v>355</v>
       </c>
       <c r="F17" s="112" t="s">
@@ -3049,15 +3049,15 @@
       <c r="H17" s="12"/>
     </row>
     <row r="18" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="143"/>
-      <c r="B18" s="123"/>
+      <c r="A18" s="125"/>
+      <c r="B18" s="132"/>
       <c r="C18" s="111" t="s">
         <v>85</v>
       </c>
       <c r="D18" s="112" t="s">
         <v>86</v>
       </c>
-      <c r="E18" s="123"/>
+      <c r="E18" s="132"/>
       <c r="F18" s="112" t="s">
         <v>84</v>
       </c>
@@ -3067,15 +3067,15 @@
       <c r="H18" s="12"/>
     </row>
     <row r="19" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="143"/>
-      <c r="B19" s="123"/>
+      <c r="A19" s="125"/>
+      <c r="B19" s="132"/>
       <c r="C19" s="111" t="s">
         <v>87</v>
       </c>
       <c r="D19" s="112" t="s">
         <v>88</v>
       </c>
-      <c r="E19" s="123"/>
+      <c r="E19" s="132"/>
       <c r="F19" s="112" t="s">
         <v>84</v>
       </c>
@@ -3085,15 +3085,15 @@
       <c r="H19" s="12"/>
     </row>
     <row r="20" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A20" s="143"/>
-      <c r="B20" s="123"/>
+      <c r="A20" s="125"/>
+      <c r="B20" s="132"/>
       <c r="C20" s="111" t="s">
         <v>89</v>
       </c>
       <c r="D20" s="112" t="s">
         <v>90</v>
       </c>
-      <c r="E20" s="123"/>
+      <c r="E20" s="132"/>
       <c r="F20" s="112" t="s">
         <v>84</v>
       </c>
@@ -3103,15 +3103,15 @@
       <c r="H20" s="12"/>
     </row>
     <row r="21" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A21" s="143"/>
-      <c r="B21" s="123"/>
+      <c r="A21" s="125"/>
+      <c r="B21" s="132"/>
       <c r="C21" s="111" t="s">
         <v>91</v>
       </c>
       <c r="D21" s="112" t="s">
         <v>92</v>
       </c>
-      <c r="E21" s="123"/>
+      <c r="E21" s="132"/>
       <c r="F21" s="112" t="s">
         <v>84</v>
       </c>
@@ -3121,15 +3121,15 @@
       <c r="H21" s="12"/>
     </row>
     <row r="22" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A22" s="143"/>
-      <c r="B22" s="123"/>
+      <c r="A22" s="125"/>
+      <c r="B22" s="132"/>
       <c r="C22" s="111" t="s">
         <v>274</v>
       </c>
       <c r="D22" s="112" t="s">
         <v>279</v>
       </c>
-      <c r="E22" s="123"/>
+      <c r="E22" s="132"/>
       <c r="F22" s="112" t="s">
         <v>84</v>
       </c>
@@ -3139,15 +3139,15 @@
       <c r="H22" s="12"/>
     </row>
     <row r="23" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A23" s="143"/>
-      <c r="B23" s="123"/>
+      <c r="A23" s="125"/>
+      <c r="B23" s="132"/>
       <c r="C23" s="111" t="s">
         <v>275</v>
       </c>
       <c r="D23" s="112" t="s">
         <v>280</v>
       </c>
-      <c r="E23" s="123"/>
+      <c r="E23" s="132"/>
       <c r="F23" s="112" t="s">
         <v>84</v>
       </c>
@@ -3157,15 +3157,15 @@
       <c r="H23" s="12"/>
     </row>
     <row r="24" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A24" s="143"/>
-      <c r="B24" s="123"/>
+      <c r="A24" s="125"/>
+      <c r="B24" s="132"/>
       <c r="C24" s="111" t="s">
         <v>276</v>
       </c>
       <c r="D24" s="112" t="s">
         <v>281</v>
       </c>
-      <c r="E24" s="123"/>
+      <c r="E24" s="132"/>
       <c r="F24" s="112" t="s">
         <v>84</v>
       </c>
@@ -3175,15 +3175,15 @@
       <c r="H24" s="12"/>
     </row>
     <row r="25" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A25" s="143"/>
-      <c r="B25" s="123"/>
+      <c r="A25" s="125"/>
+      <c r="B25" s="132"/>
       <c r="C25" s="111" t="s">
         <v>277</v>
       </c>
       <c r="D25" s="112" t="s">
         <v>282</v>
       </c>
-      <c r="E25" s="123"/>
+      <c r="E25" s="132"/>
       <c r="F25" s="112" t="s">
         <v>84</v>
       </c>
@@ -3193,15 +3193,15 @@
       <c r="H25" s="12"/>
     </row>
     <row r="26" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A26" s="143"/>
-      <c r="B26" s="124"/>
+      <c r="A26" s="125"/>
+      <c r="B26" s="133"/>
       <c r="C26" s="111" t="s">
         <v>278</v>
       </c>
       <c r="D26" s="112" t="s">
         <v>283</v>
       </c>
-      <c r="E26" s="124"/>
+      <c r="E26" s="133"/>
       <c r="F26" s="112" t="s">
         <v>84</v>
       </c>
@@ -3211,7 +3211,7 @@
       <c r="H26" s="12"/>
     </row>
     <row r="27" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="137" t="s">
+      <c r="B27" s="134" t="s">
         <v>93</v>
       </c>
       <c r="C27" s="113" t="s">
@@ -3232,7 +3232,7 @@
       <c r="H27" s="12"/>
     </row>
     <row r="28" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="138"/>
+      <c r="B28" s="135"/>
       <c r="C28" s="113" t="s">
         <v>98</v>
       </c>
@@ -3251,7 +3251,7 @@
       <c r="H28" s="12"/>
     </row>
     <row r="29" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B29" s="139"/>
+      <c r="B29" s="136"/>
       <c r="C29" s="113" t="s">
         <v>102</v>
       </c>
@@ -3270,7 +3270,7 @@
       <c r="H29" s="12"/>
     </row>
     <row r="30" spans="1:8" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="B30" s="140" t="s">
+      <c r="B30" s="137" t="s">
         <v>106</v>
       </c>
       <c r="C30" s="114" t="s">
@@ -3291,7 +3291,7 @@
       <c r="H30" s="24"/>
     </row>
     <row r="31" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B31" s="141"/>
+      <c r="B31" s="138"/>
       <c r="C31" s="114" t="s">
         <v>388</v>
       </c>
@@ -3299,10 +3299,10 @@
         <v>389</v>
       </c>
       <c r="E31" s="23" t="s">
+        <v>391</v>
+      </c>
+      <c r="F31" s="23" t="s">
         <v>390</v>
-      </c>
-      <c r="F31" s="23" t="s">
-        <v>391</v>
       </c>
       <c r="G31" s="23" t="s">
         <v>293</v>
@@ -3310,7 +3310,7 @@
       <c r="H31" s="24"/>
     </row>
     <row r="32" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="141"/>
+      <c r="B32" s="138"/>
       <c r="C32" s="114" t="s">
         <v>108</v>
       </c>
@@ -3329,7 +3329,7 @@
       <c r="H32" s="24"/>
     </row>
     <row r="33" spans="1:11" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="141"/>
+      <c r="B33" s="138"/>
       <c r="C33" s="114" t="s">
         <v>111</v>
       </c>
@@ -3348,7 +3348,7 @@
       <c r="H33" s="12"/>
     </row>
     <row r="34" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B34" s="141"/>
+      <c r="B34" s="138"/>
       <c r="C34" s="114" t="s">
         <v>115</v>
       </c>
@@ -3367,7 +3367,7 @@
       <c r="H34" s="10"/>
     </row>
     <row r="35" spans="1:11" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="141"/>
+      <c r="B35" s="138"/>
       <c r="C35" s="114" t="s">
         <v>119</v>
       </c>
@@ -3386,7 +3386,7 @@
       <c r="H35" s="12"/>
     </row>
     <row r="36" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B36" s="141"/>
+      <c r="B36" s="138"/>
       <c r="C36" s="114" t="s">
         <v>123</v>
       </c>
@@ -3405,7 +3405,7 @@
       <c r="H36" s="24"/>
     </row>
     <row r="37" spans="1:11" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="141"/>
+      <c r="B37" s="138"/>
       <c r="C37" s="114" t="s">
         <v>126</v>
       </c>
@@ -3424,7 +3424,7 @@
       <c r="H37" s="12"/>
     </row>
     <row r="38" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="B38" s="141"/>
+      <c r="B38" s="138"/>
       <c r="C38" s="114" t="s">
         <v>129</v>
       </c>
@@ -3444,14 +3444,14 @@
     </row>
     <row r="39" spans="1:11" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="95"/>
-      <c r="B39" s="141"/>
+      <c r="B39" s="138"/>
       <c r="C39" s="114" t="s">
         <v>270</v>
       </c>
       <c r="D39" s="115" t="s">
         <v>271</v>
       </c>
-      <c r="E39" s="125" t="s">
+      <c r="E39" s="140" t="s">
         <v>356</v>
       </c>
       <c r="F39" s="115"/>
@@ -3462,14 +3462,14 @@
     </row>
     <row r="40" spans="1:11" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="95"/>
-      <c r="B40" s="141"/>
+      <c r="B40" s="138"/>
       <c r="C40" s="121" t="s">
         <v>106</v>
       </c>
       <c r="D40" s="115" t="s">
         <v>271</v>
       </c>
-      <c r="E40" s="126"/>
+      <c r="E40" s="141"/>
       <c r="F40" s="115"/>
       <c r="G40" s="115" t="s">
         <v>293</v>
@@ -3478,14 +3478,14 @@
     </row>
     <row r="41" spans="1:11" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="95"/>
-      <c r="B41" s="142"/>
+      <c r="B41" s="139"/>
       <c r="C41" s="114" t="s">
         <v>273</v>
       </c>
       <c r="D41" s="115" t="s">
         <v>271</v>
       </c>
-      <c r="E41" s="127"/>
+      <c r="E41" s="142"/>
       <c r="F41" s="115"/>
       <c r="G41" s="115" t="s">
         <v>293</v>
@@ -3493,7 +3493,7 @@
       <c r="H41" s="12"/>
     </row>
     <row r="42" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B42" s="131" t="s">
+      <c r="B42" s="126" t="s">
         <v>302</v>
       </c>
       <c r="C42" s="26" t="s">
@@ -3514,7 +3514,7 @@
       <c r="H42" s="24"/>
     </row>
     <row r="43" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B43" s="132"/>
+      <c r="B43" s="127"/>
       <c r="C43" s="26" t="s">
         <v>263</v>
       </c>
@@ -3533,7 +3533,7 @@
       <c r="H43" s="24"/>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B44" s="133"/>
+      <c r="B44" s="143"/>
       <c r="C44" s="26" t="s">
         <v>284</v>
       </c>
@@ -3552,10 +3552,10 @@
       <c r="H44" s="24"/>
     </row>
     <row r="45" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A45" s="143" t="s">
+      <c r="A45" s="125" t="s">
         <v>314</v>
       </c>
-      <c r="B45" s="131" t="s">
+      <c r="B45" s="126" t="s">
         <v>308</v>
       </c>
       <c r="C45" s="116" t="s">
@@ -3579,8 +3579,8 @@
       <c r="K45" s="28"/>
     </row>
     <row r="46" spans="1:11" s="29" customFormat="1" ht="224.4" x14ac:dyDescent="0.3">
-      <c r="A46" s="143"/>
-      <c r="B46" s="132"/>
+      <c r="A46" s="125"/>
+      <c r="B46" s="127"/>
       <c r="C46" s="116" t="s">
         <v>140</v>
       </c>
@@ -3602,8 +3602,8 @@
       <c r="K46" s="28"/>
     </row>
     <row r="47" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A47" s="143"/>
-      <c r="B47" s="131" t="s">
+      <c r="A47" s="125"/>
+      <c r="B47" s="126" t="s">
         <v>309</v>
       </c>
       <c r="C47" s="116" t="s">
@@ -3627,8 +3627,8 @@
       <c r="K47" s="28"/>
     </row>
     <row r="48" spans="1:11" s="29" customFormat="1" ht="224.4" x14ac:dyDescent="0.3">
-      <c r="A48" s="143"/>
-      <c r="B48" s="132"/>
+      <c r="A48" s="125"/>
+      <c r="B48" s="127"/>
       <c r="C48" s="116" t="s">
         <v>144</v>
       </c>
@@ -3651,7 +3651,7 @@
     </row>
     <row r="49" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A49"/>
-      <c r="B49" s="128" t="s">
+      <c r="B49" s="122" t="s">
         <v>162</v>
       </c>
       <c r="C49" s="36" t="s">
@@ -3676,7 +3676,7 @@
     </row>
     <row r="50" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A50"/>
-      <c r="B50" s="130"/>
+      <c r="B50" s="124"/>
       <c r="C50" s="36" t="s">
         <v>166</v>
       </c>
@@ -3698,10 +3698,10 @@
       <c r="K50" s="32"/>
     </row>
     <row r="51" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A51" s="143" t="s">
+      <c r="A51" s="125" t="s">
         <v>315</v>
       </c>
-      <c r="B51" s="128" t="s">
+      <c r="B51" s="122" t="s">
         <v>310</v>
       </c>
       <c r="C51" s="36" t="s">
@@ -3725,8 +3725,8 @@
       <c r="K51" s="32"/>
     </row>
     <row r="52" spans="1:11" s="33" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="143"/>
-      <c r="B52" s="129"/>
+      <c r="A52" s="125"/>
+      <c r="B52" s="123"/>
       <c r="C52" s="36" t="s">
         <v>173</v>
       </c>
@@ -3748,8 +3748,8 @@
       <c r="K52" s="32"/>
     </row>
     <row r="53" spans="1:11" s="33" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.3">
-      <c r="A53" s="143"/>
-      <c r="B53" s="129"/>
+      <c r="A53" s="125"/>
+      <c r="B53" s="123"/>
       <c r="C53" s="36" t="s">
         <v>177</v>
       </c>
@@ -3771,8 +3771,8 @@
       <c r="K53" s="32"/>
     </row>
     <row r="54" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A54" s="143"/>
-      <c r="B54" s="130"/>
+      <c r="A54" s="125"/>
+      <c r="B54" s="124"/>
       <c r="C54" s="36" t="s">
         <v>179</v>
       </c>
@@ -3794,10 +3794,10 @@
       <c r="K54" s="32"/>
     </row>
     <row r="55" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A55" s="143" t="s">
+      <c r="A55" s="125" t="s">
         <v>316</v>
       </c>
-      <c r="B55" s="128" t="s">
+      <c r="B55" s="122" t="s">
         <v>313</v>
       </c>
       <c r="C55" s="36" t="s">
@@ -3821,8 +3821,8 @@
       <c r="K55" s="32"/>
     </row>
     <row r="56" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A56" s="143"/>
-      <c r="B56" s="129"/>
+      <c r="A56" s="125"/>
+      <c r="B56" s="123"/>
       <c r="C56" s="36" t="s">
         <v>185</v>
       </c>
@@ -3844,8 +3844,8 @@
       <c r="K56" s="32"/>
     </row>
     <row r="57" spans="1:11" s="33" customFormat="1" ht="356.4" x14ac:dyDescent="0.3">
-      <c r="A57" s="143"/>
-      <c r="B57" s="129"/>
+      <c r="A57" s="125"/>
+      <c r="B57" s="123"/>
       <c r="C57" s="36" t="s">
         <v>189</v>
       </c>
@@ -3867,8 +3867,8 @@
       <c r="K57" s="32"/>
     </row>
     <row r="58" spans="1:11" s="33" customFormat="1" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A58" s="143"/>
-      <c r="B58" s="130"/>
+      <c r="A58" s="125"/>
+      <c r="B58" s="124"/>
       <c r="C58" s="36" t="s">
         <v>351</v>
       </c>
@@ -3890,10 +3890,10 @@
       <c r="K58" s="32"/>
     </row>
     <row r="59" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A59" s="143" t="s">
+      <c r="A59" s="125" t="s">
         <v>315</v>
       </c>
-      <c r="B59" s="128" t="s">
+      <c r="B59" s="122" t="s">
         <v>312</v>
       </c>
       <c r="C59" s="36" t="s">
@@ -3917,8 +3917,8 @@
       <c r="K59" s="32"/>
     </row>
     <row r="60" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A60" s="143"/>
-      <c r="B60" s="129"/>
+      <c r="A60" s="125"/>
+      <c r="B60" s="123"/>
       <c r="C60" s="36" t="s">
         <v>195</v>
       </c>
@@ -3940,8 +3940,8 @@
       <c r="K60" s="32"/>
     </row>
     <row r="61" spans="1:11" s="33" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.3">
-      <c r="A61" s="143"/>
-      <c r="B61" s="129"/>
+      <c r="A61" s="125"/>
+      <c r="B61" s="123"/>
       <c r="C61" s="36" t="s">
         <v>197</v>
       </c>
@@ -3963,8 +3963,8 @@
       <c r="K61" s="32"/>
     </row>
     <row r="62" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A62" s="143"/>
-      <c r="B62" s="130"/>
+      <c r="A62" s="125"/>
+      <c r="B62" s="124"/>
       <c r="C62" s="36" t="s">
         <v>199</v>
       </c>
@@ -3986,10 +3986,10 @@
       <c r="K62" s="32"/>
     </row>
     <row r="63" spans="1:11" s="33" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="143" t="s">
+      <c r="A63" s="125" t="s">
         <v>316</v>
       </c>
-      <c r="B63" s="128" t="s">
+      <c r="B63" s="122" t="s">
         <v>311</v>
       </c>
       <c r="C63" s="36" t="s">
@@ -4013,8 +4013,8 @@
       <c r="K63" s="32"/>
     </row>
     <row r="64" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A64" s="143"/>
-      <c r="B64" s="129"/>
+      <c r="A64" s="125"/>
+      <c r="B64" s="123"/>
       <c r="C64" s="36" t="s">
         <v>204</v>
       </c>
@@ -4036,8 +4036,8 @@
       <c r="K64" s="32"/>
     </row>
     <row r="65" spans="1:11" ht="356.4" x14ac:dyDescent="0.3">
-      <c r="A65" s="143"/>
-      <c r="B65" s="129"/>
+      <c r="A65" s="125"/>
+      <c r="B65" s="123"/>
       <c r="C65" s="36" t="s">
         <v>207</v>
       </c>
@@ -4056,8 +4056,8 @@
       <c r="H65" s="12"/>
     </row>
     <row r="66" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A66" s="143"/>
-      <c r="B66" s="130"/>
+      <c r="A66" s="125"/>
+      <c r="B66" s="124"/>
       <c r="C66" s="36" t="s">
         <v>352</v>
       </c>
@@ -4076,7 +4076,7 @@
       <c r="H66" s="12"/>
     </row>
     <row r="67" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B67" s="128" t="s">
+      <c r="B67" s="122" t="s">
         <v>303</v>
       </c>
       <c r="C67" s="36" t="s">
@@ -4097,7 +4097,7 @@
       <c r="H67" s="10"/>
     </row>
     <row r="68" spans="1:11" ht="93" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B68" s="129"/>
+      <c r="B68" s="123"/>
       <c r="C68" s="36" t="s">
         <v>213</v>
       </c>
@@ -4116,7 +4116,7 @@
       <c r="H68" s="12"/>
     </row>
     <row r="69" spans="1:11" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B69" s="129"/>
+      <c r="B69" s="123"/>
       <c r="C69" s="36" t="s">
         <v>367</v>
       </c>
@@ -4135,7 +4135,7 @@
       <c r="H69" s="12"/>
     </row>
     <row r="70" spans="1:11" ht="158.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B70" s="129"/>
+      <c r="B70" s="123"/>
       <c r="C70" s="36" t="s">
         <v>368</v>
       </c>
@@ -4154,7 +4154,7 @@
       <c r="H70" s="12"/>
     </row>
     <row r="71" spans="1:11" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="130"/>
+      <c r="B71" s="124"/>
       <c r="C71" s="36" t="s">
         <v>370</v>
       </c>
@@ -4173,10 +4173,10 @@
       <c r="H71" s="12"/>
     </row>
     <row r="72" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A72" s="143" t="s">
+      <c r="A72" s="125" t="s">
         <v>317</v>
       </c>
-      <c r="B72" s="128" t="s">
+      <c r="B72" s="122" t="s">
         <v>304</v>
       </c>
       <c r="C72" s="36" t="s">
@@ -4200,8 +4200,8 @@
       <c r="K72" s="28"/>
     </row>
     <row r="73" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A73" s="143"/>
-      <c r="B73" s="129"/>
+      <c r="A73" s="125"/>
+      <c r="B73" s="123"/>
       <c r="C73" s="36" t="s">
         <v>219</v>
       </c>
@@ -4223,8 +4223,8 @@
       <c r="K73" s="28"/>
     </row>
     <row r="74" spans="1:11" s="29" customFormat="1" ht="184.8" x14ac:dyDescent="0.3">
-      <c r="A74" s="143"/>
-      <c r="B74" s="130"/>
+      <c r="A74" s="125"/>
+      <c r="B74" s="124"/>
       <c r="C74" s="36" t="s">
         <v>222</v>
       </c>
@@ -4246,8 +4246,8 @@
       <c r="K74" s="28"/>
     </row>
     <row r="75" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A75" s="143"/>
-      <c r="B75" s="128" t="s">
+      <c r="A75" s="125"/>
+      <c r="B75" s="122" t="s">
         <v>304</v>
       </c>
       <c r="C75" s="36" t="s">
@@ -4271,8 +4271,8 @@
       <c r="K75" s="28"/>
     </row>
     <row r="76" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A76" s="143"/>
-      <c r="B76" s="129"/>
+      <c r="A76" s="125"/>
+      <c r="B76" s="123"/>
       <c r="C76" s="36" t="s">
         <v>227</v>
       </c>
@@ -4294,8 +4294,8 @@
       <c r="K76" s="28"/>
     </row>
     <row r="77" spans="1:11" s="29" customFormat="1" ht="184.8" x14ac:dyDescent="0.3">
-      <c r="A77" s="143"/>
-      <c r="B77" s="130"/>
+      <c r="A77" s="125"/>
+      <c r="B77" s="124"/>
       <c r="C77" s="36" t="s">
         <v>230</v>
       </c>
@@ -4318,7 +4318,7 @@
     </row>
     <row r="78" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A78"/>
-      <c r="B78" s="128" t="s">
+      <c r="B78" s="122" t="s">
         <v>305</v>
       </c>
       <c r="C78" s="117" t="s">
@@ -4343,7 +4343,7 @@
     </row>
     <row r="79" spans="1:11" s="33" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A79"/>
-      <c r="B79" s="130"/>
+      <c r="B79" s="124"/>
       <c r="C79" s="117" t="s">
         <v>235</v>
       </c>
@@ -4365,10 +4365,10 @@
       <c r="K79" s="32"/>
     </row>
     <row r="80" spans="1:11" s="33" customFormat="1" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="143" t="s">
+      <c r="A80" s="125" t="s">
         <v>318</v>
       </c>
-      <c r="B80" s="128" t="s">
+      <c r="B80" s="122" t="s">
         <v>319</v>
       </c>
       <c r="C80" s="36" t="s">
@@ -4392,8 +4392,8 @@
       <c r="K80" s="32"/>
     </row>
     <row r="81" spans="1:11" s="33" customFormat="1" ht="78" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="143"/>
-      <c r="B81" s="129"/>
+      <c r="A81" s="125"/>
+      <c r="B81" s="123"/>
       <c r="C81" s="36" t="s">
         <v>322</v>
       </c>
@@ -4415,8 +4415,8 @@
       <c r="K81" s="32"/>
     </row>
     <row r="82" spans="1:11" s="33" customFormat="1" ht="212.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="143"/>
-      <c r="B82" s="130"/>
+      <c r="A82" s="125"/>
+      <c r="B82" s="124"/>
       <c r="C82" s="36" t="s">
         <v>324</v>
       </c>
@@ -4436,10 +4436,10 @@
       <c r="K82" s="32"/>
     </row>
     <row r="83" spans="1:11" s="33" customFormat="1" ht="117" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="143" t="s">
+      <c r="A83" s="125" t="s">
         <v>318</v>
       </c>
-      <c r="B83" s="128" t="s">
+      <c r="B83" s="122" t="s">
         <v>320</v>
       </c>
       <c r="C83" s="36" t="s">
@@ -4463,8 +4463,8 @@
       <c r="K83" s="32"/>
     </row>
     <row r="84" spans="1:11" s="33" customFormat="1" ht="83.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="143"/>
-      <c r="B84" s="129"/>
+      <c r="A84" s="125"/>
+      <c r="B84" s="123"/>
       <c r="C84" s="36" t="s">
         <v>327</v>
       </c>
@@ -4486,8 +4486,8 @@
       <c r="K84" s="32"/>
     </row>
     <row r="85" spans="1:11" s="33" customFormat="1" ht="199.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="143"/>
-      <c r="B85" s="130"/>
+      <c r="A85" s="125"/>
+      <c r="B85" s="124"/>
       <c r="C85" s="36" t="s">
         <v>328</v>
       </c>
@@ -4507,7 +4507,7 @@
       <c r="K85" s="32"/>
     </row>
     <row r="86" spans="1:11" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="B86" s="128" t="s">
+      <c r="B86" s="122" t="s">
         <v>306</v>
       </c>
       <c r="C86" s="36" t="s">
@@ -4527,7 +4527,7 @@
       </c>
     </row>
     <row r="87" spans="1:11" ht="118.8" x14ac:dyDescent="0.3">
-      <c r="B87" s="129"/>
+      <c r="B87" s="123"/>
       <c r="C87" s="36" t="s">
         <v>251</v>
       </c>
@@ -4545,7 +4545,7 @@
       </c>
     </row>
     <row r="88" spans="1:11" ht="198" x14ac:dyDescent="0.3">
-      <c r="B88" s="129"/>
+      <c r="B88" s="123"/>
       <c r="C88" s="36" t="s">
         <v>253</v>
       </c>
@@ -4563,7 +4563,7 @@
       </c>
     </row>
     <row r="89" spans="1:11" ht="66" x14ac:dyDescent="0.3">
-      <c r="B89" s="130"/>
+      <c r="B89" s="124"/>
       <c r="C89" s="36" t="s">
         <v>255</v>
       </c>
@@ -4614,6 +4614,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="E17:E26"/>
+    <mergeCell ref="E39:E41"/>
+    <mergeCell ref="B83:B85"/>
+    <mergeCell ref="B42:B44"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="B55:B58"/>
+    <mergeCell ref="B59:B62"/>
+    <mergeCell ref="B63:B66"/>
+    <mergeCell ref="B67:B71"/>
+    <mergeCell ref="B3:B16"/>
+    <mergeCell ref="B17:B26"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="B30:B41"/>
+    <mergeCell ref="B51:B54"/>
     <mergeCell ref="B86:B89"/>
     <mergeCell ref="A17:A26"/>
     <mergeCell ref="B45:B46"/>
@@ -4630,20 +4644,6 @@
     <mergeCell ref="A80:A82"/>
     <mergeCell ref="B80:B82"/>
     <mergeCell ref="A83:A85"/>
-    <mergeCell ref="B3:B16"/>
-    <mergeCell ref="B17:B26"/>
-    <mergeCell ref="B27:B29"/>
-    <mergeCell ref="B30:B41"/>
-    <mergeCell ref="B51:B54"/>
-    <mergeCell ref="E17:E26"/>
-    <mergeCell ref="E39:E41"/>
-    <mergeCell ref="B83:B85"/>
-    <mergeCell ref="B42:B44"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="B55:B58"/>
-    <mergeCell ref="B59:B62"/>
-    <mergeCell ref="B63:B66"/>
-    <mergeCell ref="B67:B71"/>
   </mergeCells>
   <phoneticPr fontId="29" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -20538,6 +20538,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="42fbd5e6-b175-407a-a25c-5fc6410bf24f" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EE7777BCFCD3E741B5CCCE9A87E98C2C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f7fc7590daec4eb8e38e018938a160ca">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e" xmlns:ns3="42fbd5e6-b175-407a-a25c-5fc6410bf24f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c5ca1b94d4b54616210e83d04e6b3cac" ns2:_="" ns3:_="">
     <xsd:import namespace="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
@@ -20792,27 +20812,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E9485EC-5D88-4A1C-961D-0F4FE84359B8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="42fbd5e6-b175-407a-a25c-5fc6410bf24f"/>
+    <ds:schemaRef ds:uri="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="42fbd5e6-b175-407a-a25c-5fc6410bf24f" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{286F673D-E70D-4002-B8F5-CAC95B029A7E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C9C537E-DFD2-4C38-AC8C-930F122DEFFC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -20829,23 +20848,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{286F673D-E70D-4002-B8F5-CAC95B029A7E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E9485EC-5D88-4A1C-961D-0F4FE84359B8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="42fbd5e6-b175-407a-a25c-5fc6410bf24f"/>
-    <ds:schemaRef ds:uri="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
try to clarify instructions
</commit_message>
<xml_diff>
--- a/data/ALAI UP Client-level Reporting Tool Template_4.7.26.xlsx
+++ b/data/ALAI UP Client-level Reporting Tool Template_4.7.26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kmlab\Desktop\Dashboard\alai_up_local_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D4F2095-0129-452D-8345-560DABCBC696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34E95B5E-2AC0-42F7-A329-2DA90E524A84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-9840" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{500E2EE0-B1C5-4ACF-BC67-EDC8BDABD2D7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{500E2EE0-B1C5-4ACF-BC67-EDC8BDABD2D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="3" r:id="rId1"/>
@@ -2124,6 +2124,24 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2133,13 +2151,13 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2149,15 +2167,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2178,16 +2187,7 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2750,7 +2750,7 @@
       <c r="K2" s="4"/>
     </row>
     <row r="3" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="128" t="s">
+      <c r="B3" s="134" t="s">
         <v>31</v>
       </c>
       <c r="C3" s="109" t="s">
@@ -2772,7 +2772,7 @@
       <c r="I3" s="8"/>
     </row>
     <row r="4" spans="1:11" ht="67.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="129"/>
+      <c r="B4" s="135"/>
       <c r="C4" s="15" t="s">
         <v>33</v>
       </c>
@@ -2792,7 +2792,7 @@
       <c r="I4" s="8"/>
     </row>
     <row r="5" spans="1:11" ht="44.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="129"/>
+      <c r="B5" s="135"/>
       <c r="C5" s="15" t="s">
         <v>37</v>
       </c>
@@ -2812,7 +2812,7 @@
       <c r="I5" s="17"/>
     </row>
     <row r="6" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B6" s="129"/>
+      <c r="B6" s="135"/>
       <c r="C6" s="15" t="s">
         <v>347</v>
       </c>
@@ -2832,7 +2832,7 @@
     </row>
     <row r="7" spans="1:11" s="19" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A7"/>
-      <c r="B7" s="129"/>
+      <c r="B7" s="135"/>
       <c r="C7" s="15" t="s">
         <v>42</v>
       </c>
@@ -2854,7 +2854,7 @@
       <c r="K7" s="18"/>
     </row>
     <row r="8" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B8" s="129"/>
+      <c r="B8" s="135"/>
       <c r="C8" s="15" t="s">
         <v>46</v>
       </c>
@@ -2873,7 +2873,7 @@
       <c r="H8" s="12"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B9" s="129"/>
+      <c r="B9" s="135"/>
       <c r="C9" s="15" t="s">
         <v>50</v>
       </c>
@@ -2892,7 +2892,7 @@
       <c r="H9" s="12"/>
     </row>
     <row r="10" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B10" s="129"/>
+      <c r="B10" s="135"/>
       <c r="C10" s="15" t="s">
         <v>54</v>
       </c>
@@ -2911,7 +2911,7 @@
       <c r="H10" s="12"/>
     </row>
     <row r="11" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B11" s="129"/>
+      <c r="B11" s="135"/>
       <c r="C11" s="15" t="s">
         <v>58</v>
       </c>
@@ -2930,7 +2930,7 @@
       <c r="H11" s="12"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B12" s="129"/>
+      <c r="B12" s="135"/>
       <c r="C12" s="15" t="s">
         <v>62</v>
       </c>
@@ -2949,7 +2949,7 @@
       <c r="H12" s="12"/>
     </row>
     <row r="13" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B13" s="129"/>
+      <c r="B13" s="135"/>
       <c r="C13" s="15" t="s">
         <v>66</v>
       </c>
@@ -2968,7 +2968,7 @@
       <c r="H13" s="12"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B14" s="129"/>
+      <c r="B14" s="135"/>
       <c r="C14" s="15" t="s">
         <v>70</v>
       </c>
@@ -2987,7 +2987,7 @@
       <c r="H14" s="12"/>
     </row>
     <row r="15" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B15" s="129"/>
+      <c r="B15" s="135"/>
       <c r="C15" s="15" t="s">
         <v>73</v>
       </c>
@@ -3006,7 +3006,7 @@
       <c r="H15" s="20"/>
     </row>
     <row r="16" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B16" s="130"/>
+      <c r="B16" s="136"/>
       <c r="C16" s="15" t="s">
         <v>77</v>
       </c>
@@ -3025,10 +3025,10 @@
       <c r="H16" s="12"/>
     </row>
     <row r="17" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="125" t="s">
+      <c r="A17" s="143" t="s">
         <v>307</v>
       </c>
-      <c r="B17" s="131" t="s">
+      <c r="B17" s="122" t="s">
         <v>81</v>
       </c>
       <c r="C17" s="111" t="s">
@@ -3037,7 +3037,7 @@
       <c r="D17" s="112" t="s">
         <v>83</v>
       </c>
-      <c r="E17" s="131" t="s">
+      <c r="E17" s="122" t="s">
         <v>355</v>
       </c>
       <c r="F17" s="112" t="s">
@@ -3049,15 +3049,15 @@
       <c r="H17" s="12"/>
     </row>
     <row r="18" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="125"/>
-      <c r="B18" s="132"/>
+      <c r="A18" s="143"/>
+      <c r="B18" s="123"/>
       <c r="C18" s="111" t="s">
         <v>85</v>
       </c>
       <c r="D18" s="112" t="s">
         <v>86</v>
       </c>
-      <c r="E18" s="132"/>
+      <c r="E18" s="123"/>
       <c r="F18" s="112" t="s">
         <v>84</v>
       </c>
@@ -3067,15 +3067,15 @@
       <c r="H18" s="12"/>
     </row>
     <row r="19" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="125"/>
-      <c r="B19" s="132"/>
+      <c r="A19" s="143"/>
+      <c r="B19" s="123"/>
       <c r="C19" s="111" t="s">
         <v>87</v>
       </c>
       <c r="D19" s="112" t="s">
         <v>88</v>
       </c>
-      <c r="E19" s="132"/>
+      <c r="E19" s="123"/>
       <c r="F19" s="112" t="s">
         <v>84</v>
       </c>
@@ -3085,15 +3085,15 @@
       <c r="H19" s="12"/>
     </row>
     <row r="20" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A20" s="125"/>
-      <c r="B20" s="132"/>
+      <c r="A20" s="143"/>
+      <c r="B20" s="123"/>
       <c r="C20" s="111" t="s">
         <v>89</v>
       </c>
       <c r="D20" s="112" t="s">
         <v>90</v>
       </c>
-      <c r="E20" s="132"/>
+      <c r="E20" s="123"/>
       <c r="F20" s="112" t="s">
         <v>84</v>
       </c>
@@ -3103,15 +3103,15 @@
       <c r="H20" s="12"/>
     </row>
     <row r="21" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A21" s="125"/>
-      <c r="B21" s="132"/>
+      <c r="A21" s="143"/>
+      <c r="B21" s="123"/>
       <c r="C21" s="111" t="s">
         <v>91</v>
       </c>
       <c r="D21" s="112" t="s">
         <v>92</v>
       </c>
-      <c r="E21" s="132"/>
+      <c r="E21" s="123"/>
       <c r="F21" s="112" t="s">
         <v>84</v>
       </c>
@@ -3121,15 +3121,15 @@
       <c r="H21" s="12"/>
     </row>
     <row r="22" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A22" s="125"/>
-      <c r="B22" s="132"/>
+      <c r="A22" s="143"/>
+      <c r="B22" s="123"/>
       <c r="C22" s="111" t="s">
         <v>274</v>
       </c>
       <c r="D22" s="112" t="s">
         <v>279</v>
       </c>
-      <c r="E22" s="132"/>
+      <c r="E22" s="123"/>
       <c r="F22" s="112" t="s">
         <v>84</v>
       </c>
@@ -3139,15 +3139,15 @@
       <c r="H22" s="12"/>
     </row>
     <row r="23" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A23" s="125"/>
-      <c r="B23" s="132"/>
+      <c r="A23" s="143"/>
+      <c r="B23" s="123"/>
       <c r="C23" s="111" t="s">
         <v>275</v>
       </c>
       <c r="D23" s="112" t="s">
         <v>280</v>
       </c>
-      <c r="E23" s="132"/>
+      <c r="E23" s="123"/>
       <c r="F23" s="112" t="s">
         <v>84</v>
       </c>
@@ -3157,15 +3157,15 @@
       <c r="H23" s="12"/>
     </row>
     <row r="24" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A24" s="125"/>
-      <c r="B24" s="132"/>
+      <c r="A24" s="143"/>
+      <c r="B24" s="123"/>
       <c r="C24" s="111" t="s">
         <v>276</v>
       </c>
       <c r="D24" s="112" t="s">
         <v>281</v>
       </c>
-      <c r="E24" s="132"/>
+      <c r="E24" s="123"/>
       <c r="F24" s="112" t="s">
         <v>84</v>
       </c>
@@ -3175,15 +3175,15 @@
       <c r="H24" s="12"/>
     </row>
     <row r="25" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A25" s="125"/>
-      <c r="B25" s="132"/>
+      <c r="A25" s="143"/>
+      <c r="B25" s="123"/>
       <c r="C25" s="111" t="s">
         <v>277</v>
       </c>
       <c r="D25" s="112" t="s">
         <v>282</v>
       </c>
-      <c r="E25" s="132"/>
+      <c r="E25" s="123"/>
       <c r="F25" s="112" t="s">
         <v>84</v>
       </c>
@@ -3193,15 +3193,15 @@
       <c r="H25" s="12"/>
     </row>
     <row r="26" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A26" s="125"/>
-      <c r="B26" s="133"/>
+      <c r="A26" s="143"/>
+      <c r="B26" s="124"/>
       <c r="C26" s="111" t="s">
         <v>278</v>
       </c>
       <c r="D26" s="112" t="s">
         <v>283</v>
       </c>
-      <c r="E26" s="133"/>
+      <c r="E26" s="124"/>
       <c r="F26" s="112" t="s">
         <v>84</v>
       </c>
@@ -3211,7 +3211,7 @@
       <c r="H26" s="12"/>
     </row>
     <row r="27" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="134" t="s">
+      <c r="B27" s="137" t="s">
         <v>93</v>
       </c>
       <c r="C27" s="113" t="s">
@@ -3232,7 +3232,7 @@
       <c r="H27" s="12"/>
     </row>
     <row r="28" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="135"/>
+      <c r="B28" s="138"/>
       <c r="C28" s="113" t="s">
         <v>98</v>
       </c>
@@ -3251,7 +3251,7 @@
       <c r="H28" s="12"/>
     </row>
     <row r="29" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B29" s="136"/>
+      <c r="B29" s="139"/>
       <c r="C29" s="113" t="s">
         <v>102</v>
       </c>
@@ -3270,7 +3270,7 @@
       <c r="H29" s="12"/>
     </row>
     <row r="30" spans="1:8" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="B30" s="137" t="s">
+      <c r="B30" s="140" t="s">
         <v>106</v>
       </c>
       <c r="C30" s="114" t="s">
@@ -3291,7 +3291,7 @@
       <c r="H30" s="24"/>
     </row>
     <row r="31" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B31" s="138"/>
+      <c r="B31" s="141"/>
       <c r="C31" s="114" t="s">
         <v>388</v>
       </c>
@@ -3310,7 +3310,7 @@
       <c r="H31" s="24"/>
     </row>
     <row r="32" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="138"/>
+      <c r="B32" s="141"/>
       <c r="C32" s="114" t="s">
         <v>108</v>
       </c>
@@ -3329,7 +3329,7 @@
       <c r="H32" s="24"/>
     </row>
     <row r="33" spans="1:11" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="138"/>
+      <c r="B33" s="141"/>
       <c r="C33" s="114" t="s">
         <v>111</v>
       </c>
@@ -3348,7 +3348,7 @@
       <c r="H33" s="12"/>
     </row>
     <row r="34" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B34" s="138"/>
+      <c r="B34" s="141"/>
       <c r="C34" s="114" t="s">
         <v>115</v>
       </c>
@@ -3367,7 +3367,7 @@
       <c r="H34" s="10"/>
     </row>
     <row r="35" spans="1:11" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="138"/>
+      <c r="B35" s="141"/>
       <c r="C35" s="114" t="s">
         <v>119</v>
       </c>
@@ -3386,7 +3386,7 @@
       <c r="H35" s="12"/>
     </row>
     <row r="36" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B36" s="138"/>
+      <c r="B36" s="141"/>
       <c r="C36" s="114" t="s">
         <v>123</v>
       </c>
@@ -3405,7 +3405,7 @@
       <c r="H36" s="24"/>
     </row>
     <row r="37" spans="1:11" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="138"/>
+      <c r="B37" s="141"/>
       <c r="C37" s="114" t="s">
         <v>126</v>
       </c>
@@ -3424,7 +3424,7 @@
       <c r="H37" s="12"/>
     </row>
     <row r="38" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="B38" s="138"/>
+      <c r="B38" s="141"/>
       <c r="C38" s="114" t="s">
         <v>129</v>
       </c>
@@ -3444,14 +3444,14 @@
     </row>
     <row r="39" spans="1:11" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="95"/>
-      <c r="B39" s="138"/>
+      <c r="B39" s="141"/>
       <c r="C39" s="114" t="s">
         <v>270</v>
       </c>
       <c r="D39" s="115" t="s">
         <v>271</v>
       </c>
-      <c r="E39" s="140" t="s">
+      <c r="E39" s="125" t="s">
         <v>356</v>
       </c>
       <c r="F39" s="115"/>
@@ -3462,14 +3462,14 @@
     </row>
     <row r="40" spans="1:11" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="95"/>
-      <c r="B40" s="138"/>
+      <c r="B40" s="141"/>
       <c r="C40" s="121" t="s">
         <v>106</v>
       </c>
       <c r="D40" s="115" t="s">
         <v>271</v>
       </c>
-      <c r="E40" s="141"/>
+      <c r="E40" s="126"/>
       <c r="F40" s="115"/>
       <c r="G40" s="115" t="s">
         <v>293</v>
@@ -3478,22 +3478,22 @@
     </row>
     <row r="41" spans="1:11" ht="63" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="95"/>
-      <c r="B41" s="139"/>
+      <c r="B41" s="142"/>
       <c r="C41" s="114" t="s">
         <v>273</v>
       </c>
       <c r="D41" s="115" t="s">
         <v>271</v>
       </c>
-      <c r="E41" s="142"/>
+      <c r="E41" s="127"/>
       <c r="F41" s="115"/>
       <c r="G41" s="115" t="s">
         <v>293</v>
       </c>
       <c r="H41" s="12"/>
     </row>
-    <row r="42" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B42" s="126" t="s">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B42" s="131" t="s">
         <v>302</v>
       </c>
       <c r="C42" s="26" t="s">
@@ -3514,7 +3514,7 @@
       <c r="H42" s="24"/>
     </row>
     <row r="43" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B43" s="127"/>
+      <c r="B43" s="132"/>
       <c r="C43" s="26" t="s">
         <v>263</v>
       </c>
@@ -3533,7 +3533,7 @@
       <c r="H43" s="24"/>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B44" s="143"/>
+      <c r="B44" s="133"/>
       <c r="C44" s="26" t="s">
         <v>284</v>
       </c>
@@ -3552,10 +3552,10 @@
       <c r="H44" s="24"/>
     </row>
     <row r="45" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A45" s="125" t="s">
+      <c r="A45" s="143" t="s">
         <v>314</v>
       </c>
-      <c r="B45" s="126" t="s">
+      <c r="B45" s="131" t="s">
         <v>308</v>
       </c>
       <c r="C45" s="116" t="s">
@@ -3579,8 +3579,8 @@
       <c r="K45" s="28"/>
     </row>
     <row r="46" spans="1:11" s="29" customFormat="1" ht="224.4" x14ac:dyDescent="0.3">
-      <c r="A46" s="125"/>
-      <c r="B46" s="127"/>
+      <c r="A46" s="143"/>
+      <c r="B46" s="132"/>
       <c r="C46" s="116" t="s">
         <v>140</v>
       </c>
@@ -3602,8 +3602,8 @@
       <c r="K46" s="28"/>
     </row>
     <row r="47" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A47" s="125"/>
-      <c r="B47" s="126" t="s">
+      <c r="A47" s="143"/>
+      <c r="B47" s="131" t="s">
         <v>309</v>
       </c>
       <c r="C47" s="116" t="s">
@@ -3627,8 +3627,8 @@
       <c r="K47" s="28"/>
     </row>
     <row r="48" spans="1:11" s="29" customFormat="1" ht="224.4" x14ac:dyDescent="0.3">
-      <c r="A48" s="125"/>
-      <c r="B48" s="127"/>
+      <c r="A48" s="143"/>
+      <c r="B48" s="132"/>
       <c r="C48" s="116" t="s">
         <v>144</v>
       </c>
@@ -3651,7 +3651,7 @@
     </row>
     <row r="49" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A49"/>
-      <c r="B49" s="122" t="s">
+      <c r="B49" s="128" t="s">
         <v>162</v>
       </c>
       <c r="C49" s="36" t="s">
@@ -3676,7 +3676,7 @@
     </row>
     <row r="50" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A50"/>
-      <c r="B50" s="124"/>
+      <c r="B50" s="130"/>
       <c r="C50" s="36" t="s">
         <v>166</v>
       </c>
@@ -3698,10 +3698,10 @@
       <c r="K50" s="32"/>
     </row>
     <row r="51" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A51" s="125" t="s">
+      <c r="A51" s="143" t="s">
         <v>315</v>
       </c>
-      <c r="B51" s="122" t="s">
+      <c r="B51" s="128" t="s">
         <v>310</v>
       </c>
       <c r="C51" s="36" t="s">
@@ -3725,8 +3725,8 @@
       <c r="K51" s="32"/>
     </row>
     <row r="52" spans="1:11" s="33" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="125"/>
-      <c r="B52" s="123"/>
+      <c r="A52" s="143"/>
+      <c r="B52" s="129"/>
       <c r="C52" s="36" t="s">
         <v>173</v>
       </c>
@@ -3748,8 +3748,8 @@
       <c r="K52" s="32"/>
     </row>
     <row r="53" spans="1:11" s="33" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.3">
-      <c r="A53" s="125"/>
-      <c r="B53" s="123"/>
+      <c r="A53" s="143"/>
+      <c r="B53" s="129"/>
       <c r="C53" s="36" t="s">
         <v>177</v>
       </c>
@@ -3771,8 +3771,8 @@
       <c r="K53" s="32"/>
     </row>
     <row r="54" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A54" s="125"/>
-      <c r="B54" s="124"/>
+      <c r="A54" s="143"/>
+      <c r="B54" s="130"/>
       <c r="C54" s="36" t="s">
         <v>179</v>
       </c>
@@ -3794,10 +3794,10 @@
       <c r="K54" s="32"/>
     </row>
     <row r="55" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A55" s="125" t="s">
+      <c r="A55" s="143" t="s">
         <v>316</v>
       </c>
-      <c r="B55" s="122" t="s">
+      <c r="B55" s="128" t="s">
         <v>313</v>
       </c>
       <c r="C55" s="36" t="s">
@@ -3821,8 +3821,8 @@
       <c r="K55" s="32"/>
     </row>
     <row r="56" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A56" s="125"/>
-      <c r="B56" s="123"/>
+      <c r="A56" s="143"/>
+      <c r="B56" s="129"/>
       <c r="C56" s="36" t="s">
         <v>185</v>
       </c>
@@ -3844,8 +3844,8 @@
       <c r="K56" s="32"/>
     </row>
     <row r="57" spans="1:11" s="33" customFormat="1" ht="356.4" x14ac:dyDescent="0.3">
-      <c r="A57" s="125"/>
-      <c r="B57" s="123"/>
+      <c r="A57" s="143"/>
+      <c r="B57" s="129"/>
       <c r="C57" s="36" t="s">
         <v>189</v>
       </c>
@@ -3867,8 +3867,8 @@
       <c r="K57" s="32"/>
     </row>
     <row r="58" spans="1:11" s="33" customFormat="1" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A58" s="125"/>
-      <c r="B58" s="124"/>
+      <c r="A58" s="143"/>
+      <c r="B58" s="130"/>
       <c r="C58" s="36" t="s">
         <v>351</v>
       </c>
@@ -3890,10 +3890,10 @@
       <c r="K58" s="32"/>
     </row>
     <row r="59" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A59" s="125" t="s">
+      <c r="A59" s="143" t="s">
         <v>315</v>
       </c>
-      <c r="B59" s="122" t="s">
+      <c r="B59" s="128" t="s">
         <v>312</v>
       </c>
       <c r="C59" s="36" t="s">
@@ -3917,8 +3917,8 @@
       <c r="K59" s="32"/>
     </row>
     <row r="60" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A60" s="125"/>
-      <c r="B60" s="123"/>
+      <c r="A60" s="143"/>
+      <c r="B60" s="129"/>
       <c r="C60" s="36" t="s">
         <v>195</v>
       </c>
@@ -3940,8 +3940,8 @@
       <c r="K60" s="32"/>
     </row>
     <row r="61" spans="1:11" s="33" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.3">
-      <c r="A61" s="125"/>
-      <c r="B61" s="123"/>
+      <c r="A61" s="143"/>
+      <c r="B61" s="129"/>
       <c r="C61" s="36" t="s">
         <v>197</v>
       </c>
@@ -3963,8 +3963,8 @@
       <c r="K61" s="32"/>
     </row>
     <row r="62" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A62" s="125"/>
-      <c r="B62" s="124"/>
+      <c r="A62" s="143"/>
+      <c r="B62" s="130"/>
       <c r="C62" s="36" t="s">
         <v>199</v>
       </c>
@@ -3986,10 +3986,10 @@
       <c r="K62" s="32"/>
     </row>
     <row r="63" spans="1:11" s="33" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="125" t="s">
+      <c r="A63" s="143" t="s">
         <v>316</v>
       </c>
-      <c r="B63" s="122" t="s">
+      <c r="B63" s="128" t="s">
         <v>311</v>
       </c>
       <c r="C63" s="36" t="s">
@@ -4013,8 +4013,8 @@
       <c r="K63" s="32"/>
     </row>
     <row r="64" spans="1:11" s="33" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A64" s="125"/>
-      <c r="B64" s="123"/>
+      <c r="A64" s="143"/>
+      <c r="B64" s="129"/>
       <c r="C64" s="36" t="s">
         <v>204</v>
       </c>
@@ -4036,8 +4036,8 @@
       <c r="K64" s="32"/>
     </row>
     <row r="65" spans="1:11" ht="356.4" x14ac:dyDescent="0.3">
-      <c r="A65" s="125"/>
-      <c r="B65" s="123"/>
+      <c r="A65" s="143"/>
+      <c r="B65" s="129"/>
       <c r="C65" s="36" t="s">
         <v>207</v>
       </c>
@@ -4056,8 +4056,8 @@
       <c r="H65" s="12"/>
     </row>
     <row r="66" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A66" s="125"/>
-      <c r="B66" s="124"/>
+      <c r="A66" s="143"/>
+      <c r="B66" s="130"/>
       <c r="C66" s="36" t="s">
         <v>352</v>
       </c>
@@ -4076,7 +4076,7 @@
       <c r="H66" s="12"/>
     </row>
     <row r="67" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B67" s="122" t="s">
+      <c r="B67" s="128" t="s">
         <v>303</v>
       </c>
       <c r="C67" s="36" t="s">
@@ -4097,7 +4097,7 @@
       <c r="H67" s="10"/>
     </row>
     <row r="68" spans="1:11" ht="93" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B68" s="123"/>
+      <c r="B68" s="129"/>
       <c r="C68" s="36" t="s">
         <v>213</v>
       </c>
@@ -4116,7 +4116,7 @@
       <c r="H68" s="12"/>
     </row>
     <row r="69" spans="1:11" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B69" s="123"/>
+      <c r="B69" s="129"/>
       <c r="C69" s="36" t="s">
         <v>367</v>
       </c>
@@ -4130,12 +4130,12 @@
         <v>371</v>
       </c>
       <c r="G69" s="36" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="H69" s="12"/>
     </row>
     <row r="70" spans="1:11" ht="158.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B70" s="123"/>
+      <c r="B70" s="129"/>
       <c r="C70" s="36" t="s">
         <v>368</v>
       </c>
@@ -4149,12 +4149,12 @@
         <v>379</v>
       </c>
       <c r="G70" s="36" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="H70" s="12"/>
     </row>
     <row r="71" spans="1:11" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="124"/>
+      <c r="B71" s="130"/>
       <c r="C71" s="36" t="s">
         <v>370</v>
       </c>
@@ -4168,15 +4168,15 @@
         <v>30</v>
       </c>
       <c r="G71" s="36" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="H71" s="12"/>
     </row>
     <row r="72" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A72" s="125" t="s">
+      <c r="A72" s="143" t="s">
         <v>317</v>
       </c>
-      <c r="B72" s="122" t="s">
+      <c r="B72" s="128" t="s">
         <v>304</v>
       </c>
       <c r="C72" s="36" t="s">
@@ -4200,8 +4200,8 @@
       <c r="K72" s="28"/>
     </row>
     <row r="73" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A73" s="125"/>
-      <c r="B73" s="123"/>
+      <c r="A73" s="143"/>
+      <c r="B73" s="129"/>
       <c r="C73" s="36" t="s">
         <v>219</v>
       </c>
@@ -4223,8 +4223,8 @@
       <c r="K73" s="28"/>
     </row>
     <row r="74" spans="1:11" s="29" customFormat="1" ht="184.8" x14ac:dyDescent="0.3">
-      <c r="A74" s="125"/>
-      <c r="B74" s="124"/>
+      <c r="A74" s="143"/>
+      <c r="B74" s="130"/>
       <c r="C74" s="36" t="s">
         <v>222</v>
       </c>
@@ -4246,8 +4246,8 @@
       <c r="K74" s="28"/>
     </row>
     <row r="75" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A75" s="125"/>
-      <c r="B75" s="122" t="s">
+      <c r="A75" s="143"/>
+      <c r="B75" s="128" t="s">
         <v>304</v>
       </c>
       <c r="C75" s="36" t="s">
@@ -4271,8 +4271,8 @@
       <c r="K75" s="28"/>
     </row>
     <row r="76" spans="1:11" s="29" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A76" s="125"/>
-      <c r="B76" s="123"/>
+      <c r="A76" s="143"/>
+      <c r="B76" s="129"/>
       <c r="C76" s="36" t="s">
         <v>227</v>
       </c>
@@ -4294,8 +4294,8 @@
       <c r="K76" s="28"/>
     </row>
     <row r="77" spans="1:11" s="29" customFormat="1" ht="184.8" x14ac:dyDescent="0.3">
-      <c r="A77" s="125"/>
-      <c r="B77" s="124"/>
+      <c r="A77" s="143"/>
+      <c r="B77" s="130"/>
       <c r="C77" s="36" t="s">
         <v>230</v>
       </c>
@@ -4318,7 +4318,7 @@
     </row>
     <row r="78" spans="1:11" s="29" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A78"/>
-      <c r="B78" s="122" t="s">
+      <c r="B78" s="128" t="s">
         <v>305</v>
       </c>
       <c r="C78" s="117" t="s">
@@ -4343,7 +4343,7 @@
     </row>
     <row r="79" spans="1:11" s="33" customFormat="1" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A79"/>
-      <c r="B79" s="124"/>
+      <c r="B79" s="130"/>
       <c r="C79" s="117" t="s">
         <v>235</v>
       </c>
@@ -4365,10 +4365,10 @@
       <c r="K79" s="32"/>
     </row>
     <row r="80" spans="1:11" s="33" customFormat="1" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="125" t="s">
+      <c r="A80" s="143" t="s">
         <v>318</v>
       </c>
-      <c r="B80" s="122" t="s">
+      <c r="B80" s="128" t="s">
         <v>319</v>
       </c>
       <c r="C80" s="36" t="s">
@@ -4392,8 +4392,8 @@
       <c r="K80" s="32"/>
     </row>
     <row r="81" spans="1:11" s="33" customFormat="1" ht="78" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="125"/>
-      <c r="B81" s="123"/>
+      <c r="A81" s="143"/>
+      <c r="B81" s="129"/>
       <c r="C81" s="36" t="s">
         <v>322</v>
       </c>
@@ -4415,8 +4415,8 @@
       <c r="K81" s="32"/>
     </row>
     <row r="82" spans="1:11" s="33" customFormat="1" ht="212.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="125"/>
-      <c r="B82" s="124"/>
+      <c r="A82" s="143"/>
+      <c r="B82" s="130"/>
       <c r="C82" s="36" t="s">
         <v>324</v>
       </c>
@@ -4436,10 +4436,10 @@
       <c r="K82" s="32"/>
     </row>
     <row r="83" spans="1:11" s="33" customFormat="1" ht="117" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="125" t="s">
+      <c r="A83" s="143" t="s">
         <v>318</v>
       </c>
-      <c r="B83" s="122" t="s">
+      <c r="B83" s="128" t="s">
         <v>320</v>
       </c>
       <c r="C83" s="36" t="s">
@@ -4463,8 +4463,8 @@
       <c r="K83" s="32"/>
     </row>
     <row r="84" spans="1:11" s="33" customFormat="1" ht="83.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="125"/>
-      <c r="B84" s="123"/>
+      <c r="A84" s="143"/>
+      <c r="B84" s="129"/>
       <c r="C84" s="36" t="s">
         <v>327</v>
       </c>
@@ -4486,8 +4486,8 @@
       <c r="K84" s="32"/>
     </row>
     <row r="85" spans="1:11" s="33" customFormat="1" ht="199.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="125"/>
-      <c r="B85" s="124"/>
+      <c r="A85" s="143"/>
+      <c r="B85" s="130"/>
       <c r="C85" s="36" t="s">
         <v>328</v>
       </c>
@@ -4507,7 +4507,7 @@
       <c r="K85" s="32"/>
     </row>
     <row r="86" spans="1:11" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="B86" s="122" t="s">
+      <c r="B86" s="128" t="s">
         <v>306</v>
       </c>
       <c r="C86" s="36" t="s">
@@ -4527,7 +4527,7 @@
       </c>
     </row>
     <row r="87" spans="1:11" ht="118.8" x14ac:dyDescent="0.3">
-      <c r="B87" s="123"/>
+      <c r="B87" s="129"/>
       <c r="C87" s="36" t="s">
         <v>251</v>
       </c>
@@ -4545,7 +4545,7 @@
       </c>
     </row>
     <row r="88" spans="1:11" ht="198" x14ac:dyDescent="0.3">
-      <c r="B88" s="123"/>
+      <c r="B88" s="129"/>
       <c r="C88" s="36" t="s">
         <v>253</v>
       </c>
@@ -4563,7 +4563,7 @@
       </c>
     </row>
     <row r="89" spans="1:11" ht="66" x14ac:dyDescent="0.3">
-      <c r="B89" s="124"/>
+      <c r="B89" s="130"/>
       <c r="C89" s="36" t="s">
         <v>255</v>
       </c>
@@ -4614,20 +4614,6 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="E17:E26"/>
-    <mergeCell ref="E39:E41"/>
-    <mergeCell ref="B83:B85"/>
-    <mergeCell ref="B42:B44"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="B55:B58"/>
-    <mergeCell ref="B59:B62"/>
-    <mergeCell ref="B63:B66"/>
-    <mergeCell ref="B67:B71"/>
-    <mergeCell ref="B3:B16"/>
-    <mergeCell ref="B17:B26"/>
-    <mergeCell ref="B27:B29"/>
-    <mergeCell ref="B30:B41"/>
-    <mergeCell ref="B51:B54"/>
     <mergeCell ref="B86:B89"/>
     <mergeCell ref="A17:A26"/>
     <mergeCell ref="B45:B46"/>
@@ -4644,6 +4630,20 @@
     <mergeCell ref="A80:A82"/>
     <mergeCell ref="B80:B82"/>
     <mergeCell ref="A83:A85"/>
+    <mergeCell ref="B3:B16"/>
+    <mergeCell ref="B17:B26"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="B30:B41"/>
+    <mergeCell ref="B51:B54"/>
+    <mergeCell ref="E17:E26"/>
+    <mergeCell ref="E39:E41"/>
+    <mergeCell ref="B83:B85"/>
+    <mergeCell ref="B42:B44"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="B55:B58"/>
+    <mergeCell ref="B59:B62"/>
+    <mergeCell ref="B63:B66"/>
+    <mergeCell ref="B67:B71"/>
   </mergeCells>
   <phoneticPr fontId="29" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -20538,26 +20538,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="42fbd5e6-b175-407a-a25c-5fc6410bf24f" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EE7777BCFCD3E741B5CCCE9A87E98C2C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f7fc7590daec4eb8e38e018938a160ca">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e" xmlns:ns3="42fbd5e6-b175-407a-a25c-5fc6410bf24f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c5ca1b94d4b54616210e83d04e6b3cac" ns2:_="" ns3:_="">
     <xsd:import namespace="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
@@ -20812,26 +20792,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E9485EC-5D88-4A1C-961D-0F4FE84359B8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="42fbd5e6-b175-407a-a25c-5fc6410bf24f"/>
-    <ds:schemaRef ds:uri="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{286F673D-E70D-4002-B8F5-CAC95B029A7E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="42fbd5e6-b175-407a-a25c-5fc6410bf24f" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C9C537E-DFD2-4C38-AC8C-930F122DEFFC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -20848,4 +20829,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{286F673D-E70D-4002-B8F5-CAC95B029A7E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E9485EC-5D88-4A1C-961D-0F4FE84359B8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="42fbd5e6-b175-407a-a25c-5fc6410bf24f"/>
+    <ds:schemaRef ds:uri="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>